<commit_message>
fixed test issue (moved function so it doesn't import state)
</commit_message>
<xml_diff>
--- a/server/assets/translation.xlsx
+++ b/server/assets/translation.xlsx
@@ -375,7 +375,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C453"/>
+  <dimension ref="A1:C459"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1904,111 +1904,108 @@
     </row>
     <row r="159">
       <c r="A159" t="str">
-        <v>settingsTabs.About</v>
+        <v>settingsTabs.Overlay</v>
       </c>
       <c r="B159" t="str">
-        <v>About</v>
-      </c>
-      <c r="C159" t="str">
-        <v>关于</v>
+        <v>Overlay</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="str">
-        <v>settingsTabs.View Data</v>
+        <v>settingsTabs.About</v>
       </c>
       <c r="B160" t="str">
-        <v>View Data</v>
+        <v>About</v>
       </c>
       <c r="C160" t="str">
-        <v>查看数据</v>
+        <v>关于</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="str">
-        <v>settingsTabs.Discussion</v>
+        <v>settingsTabs.View Data</v>
       </c>
       <c r="B161" t="str">
-        <v>Discussion</v>
+        <v>View Data</v>
       </c>
       <c r="C161" t="str">
-        <v>讨论</v>
+        <v>查看数据</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="str">
-        <v>settingsTabs.Warnings</v>
+        <v>settingsTabs.Discussion</v>
       </c>
       <c r="B162" t="str">
-        <v>Warnings</v>
+        <v>Discussion</v>
       </c>
       <c r="C162" t="str">
-        <v>警告</v>
+        <v>讨论</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="str">
-        <v>settingsTabs.Load/Save</v>
+        <v>settingsTabs.Warnings</v>
       </c>
       <c r="B163" t="str">
-        <v>Load/Save</v>
+        <v>Warnings</v>
+      </c>
+      <c r="C163" t="str">
+        <v>警告</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="str">
-        <v>settingsTabs.xAxis</v>
+        <v>settingsTabs.Load/Save</v>
       </c>
       <c r="B164" t="str">
-        <v>X Axis (Age-only)</v>
+        <v>Load/Save</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="str">
-        <v>settingsTabs.yAxis</v>
+        <v>settingsTabs.xAxis</v>
       </c>
       <c r="B165" t="str">
-        <v>Y Axis (Age/Depth)</v>
+        <v>X Axis (Age-only)</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="str">
-        <v>settings.time.interval.top</v>
+        <v>settingsTabs.yAxis</v>
       </c>
       <c r="B166" t="str">
-        <v>Top of Interval</v>
-      </c>
-      <c r="C166" t="str">
-        <v>区间顶部</v>
+        <v>Y Axis (Age/Depth)</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="str">
-        <v>settings.time.interval.base</v>
+        <v>settings.time.interval.top</v>
       </c>
       <c r="B167" t="str">
-        <v>Base of Interval</v>
+        <v>Top of Interval</v>
       </c>
       <c r="C167" t="str">
-        <v>区间底部</v>
+        <v>区间顶部</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="str">
-        <v>settings.time.interval.top-name</v>
+        <v>settings.time.interval.base</v>
       </c>
       <c r="B168" t="str">
-        <v>Top Age/Stage Name</v>
+        <v>Base of Interval</v>
       </c>
       <c r="C168" t="str">
-        <v>年代/阶段 名称</v>
+        <v>区间底部</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="str">
-        <v>settings.time.interval.base-name</v>
+        <v>settings.time.interval.top-name</v>
       </c>
       <c r="B169" t="str">
-        <v>Base Age/Stage Name</v>
+        <v>Top Age/Stage Name</v>
       </c>
       <c r="C169" t="str">
         <v>年代/阶段 名称</v>
@@ -2016,3017 +2013,3068 @@
     </row>
     <row r="170">
       <c r="A170" t="str">
-        <v>settings.time.interval.not-avaliable</v>
+        <v>settings.time.interval.base-name</v>
       </c>
       <c r="B170" t="str">
-        <v>Not Available for this Unit</v>
+        <v>Base Age/Stage Name</v>
       </c>
       <c r="C170" t="str">
-        <v>该时间单位无可选年代</v>
+        <v>年代/阶段 名称</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="str">
-        <v>settings.time.interval.vertical-scale</v>
+        <v>settings.time.interval.not-avaliable</v>
       </c>
       <c r="B171" t="str">
-        <v xml:space="preserve">Vertical Scale (cm per 1 </v>
+        <v>Not Available for this Unit</v>
       </c>
       <c r="C171" t="str">
-        <v>垂直比例（厘米 每 1</v>
+        <v>该时间单位无可选年代</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="str">
-        <v>settings.time.interval.helper-text</v>
+        <v>settings.time.interval.vertical-scale</v>
       </c>
       <c r="B172" t="str">
-        <v>Base age should be older than top age</v>
+        <v xml:space="preserve">Vertical Scale (cm per 1 </v>
       </c>
       <c r="C172" t="str">
-        <v>区间底部年代应大于区间顶部年代</v>
+        <v>垂直比例（厘米 每 1</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="str">
-        <v>settings.time.interval.vertical-scale-header</v>
+        <v>settings.time.interval.helper-text</v>
       </c>
       <c r="B173" t="str">
-        <v>Vertical Scale</v>
+        <v>Base age should be older than top age</v>
+      </c>
+      <c r="C173" t="str">
+        <v>区间底部年代应大于区间顶部年代</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="str">
-        <v>settings.preferences.checkboxs.skip-empty-columns</v>
+        <v>settings.time.interval.vertical-scale-header</v>
       </c>
       <c r="B174" t="str">
-        <v>Gray out (and do not draw) columns which do not have data on the selected time interval</v>
-      </c>
-      <c r="C174" t="str">
-        <v>在已选时间段内没有数据的列将不会被画出</v>
+        <v>Vertical Scale</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="str">
-        <v>settings.preferences.checkboxs.mouse-over-info</v>
+        <v>settings.preferences.checkboxs.skip-empty-columns</v>
       </c>
       <c r="B175" t="str">
-        <v>Add MouseOver info (popups)</v>
+        <v>Gray out (and do not draw) columns which do not have data on the selected time interval</v>
       </c>
       <c r="C175" t="str">
-        <v>鼠标移至目标上时显示详细信息</v>
+        <v>在已选时间段内没有数据的列将不会被画出</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="str">
-        <v>settings.preferences.checkboxs.global-priority</v>
+        <v>settings.preferences.checkboxs.mouse-over-info</v>
       </c>
       <c r="B176" t="str">
-        <v>Enabled Global Priority Filtering for block columns</v>
+        <v>Add MouseOver info (popups)</v>
       </c>
       <c r="C176" t="str">
-        <v>启用优先级过滤</v>
+        <v>鼠标移至目标上时显示详细信息</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="str">
-        <v>settings.preferences.checkboxs.stage-background</v>
+        <v>settings.preferences.checkboxs.global-priority</v>
       </c>
       <c r="B177" t="str">
-        <v>Enabled stage background for event columns</v>
+        <v>Enabled Global Priority Filtering for block columns</v>
       </c>
       <c r="C177" t="str">
-        <v>启用事件列的背景</v>
+        <v>启用优先级过滤</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="str">
-        <v>settings.preferences.checkboxs.enable-legend</v>
+        <v>settings.preferences.checkboxs.stage-background</v>
       </c>
       <c r="B178" t="str">
-        <v>Enable legend for the chart</v>
+        <v>Enabled stage background for event columns</v>
       </c>
       <c r="C178" t="str">
-        <v>启用添加图例</v>
+        <v>启用事件列的背景</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="str">
-        <v>settings.preferences.checkboxs.lithology-auto-indent</v>
+        <v>settings.preferences.checkboxs.enable-legend</v>
       </c>
       <c r="B179" t="str">
-        <v>Do not auto-indent lithology patterns</v>
+        <v>Enable legend for the chart</v>
       </c>
       <c r="C179" t="str">
-        <v>禁用自动缩进岩性图案</v>
+        <v>启用添加图例</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="str">
-        <v>settings.preferences.checkboxs.conserve-chart</v>
+        <v>settings.preferences.checkboxs.lithology-auto-indent</v>
       </c>
       <c r="B180" t="str">
-        <v>Conserve Chart Space in Family Tree Plotting (Not implemented)</v>
+        <v>Do not auto-indent lithology patterns</v>
       </c>
       <c r="C180" t="str">
-        <v>使用家谱绘图时节省图表空间（暂无该功能）</v>
+        <v>禁用自动缩进岩性图案</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="str">
-        <v>settings.preferences.checkboxs.hide-block-labels</v>
+        <v>settings.preferences.checkboxs.conserve-chart</v>
       </c>
       <c r="B181" t="str">
-        <v>Hide block labels based on priority</v>
+        <v>Conserve Chart Space in Family Tree Plotting (Not implemented)</v>
       </c>
       <c r="C181" t="str">
-        <v>根据优先级隐藏组标签</v>
+        <v>使用家谱绘图时节省图表空间（暂无该功能）</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="str">
-        <v>settings.preferences.checkboxs.use-suggested-age-spans</v>
+        <v>settings.preferences.checkboxs.hide-block-labels</v>
       </c>
       <c r="B182" t="str">
-        <v>Do not use the Data-Pack's suggested age span</v>
+        <v>Hide block labels based on priority</v>
       </c>
       <c r="C182" t="str">
-        <v>禁用数据包建议的时间区间</v>
+        <v>根据优先级隐藏组标签</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="str">
-        <v>settings.preferences.settings-file.load</v>
+        <v>settings.preferences.checkboxs.use-suggested-age-spans</v>
       </c>
       <c r="B183" t="str">
-        <v>Load Settings</v>
+        <v>Do not use the Data-Pack's suggested age span</v>
       </c>
       <c r="C183" t="str">
-        <v>上传设置</v>
+        <v>禁用数据包建议的时间区间</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="str">
-        <v>settings.preferences.settings-file.save</v>
+        <v>settings.preferences.settings-file.load</v>
       </c>
       <c r="B184" t="str">
-        <v>Save Settings</v>
+        <v>Load Settings</v>
       </c>
       <c r="C184" t="str">
-        <v>保存设置</v>
+        <v>上传设置</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="str">
-        <v>settings.preferences.settings-file.load-dialog.message</v>
+        <v>settings.preferences.settings-file.save</v>
       </c>
       <c r="B185" t="str">
-        <v>This will overwrite any changes you've made!</v>
+        <v>Save Settings</v>
       </c>
       <c r="C185" t="str">
-        <v>这将覆盖你所做的任何更改！</v>
+        <v>保存设置</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="str">
-        <v>settings.preferences.settings-file.load-dialog.cancel</v>
+        <v>settings.preferences.settings-file.load-dialog.message</v>
       </c>
       <c r="B186" t="str">
-        <v>Cancel</v>
+        <v>This will overwrite any changes you've made!</v>
       </c>
       <c r="C186" t="str">
-        <v>取消</v>
+        <v>这将覆盖你所做的任何更改！</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="str">
-        <v>settings.preferences.settings-file.load-dialog.load</v>
+        <v>settings.preferences.settings-file.load-dialog.cancel</v>
       </c>
       <c r="B187" t="str">
-        <v>Load</v>
+        <v>Cancel</v>
       </c>
       <c r="C187" t="str">
-        <v>上传</v>
+        <v>取消</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="str">
-        <v>settings.preferences.settings-file.save-dialog.message</v>
+        <v>settings.preferences.settings-file.load-dialog.load</v>
       </c>
       <c r="B188" t="str">
-        <v>Please enter the filename below.</v>
+        <v>Load</v>
       </c>
       <c r="C188" t="str">
-        <v>请输入文件名</v>
+        <v>上传</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="str">
-        <v>settings.preferences.settings-file.save-dialog.cancel</v>
+        <v>settings.preferences.settings-file.save-dialog.message</v>
       </c>
       <c r="B189" t="str">
-        <v>Cancel</v>
+        <v>Please enter the filename below.</v>
       </c>
       <c r="C189" t="str">
-        <v>取消</v>
+        <v>请输入文件名</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="str">
-        <v>settings.preferences.settings-file.save-dialog.save</v>
+        <v>settings.preferences.settings-file.save-dialog.cancel</v>
       </c>
       <c r="B190" t="str">
-        <v>Save</v>
+        <v>Cancel</v>
       </c>
       <c r="C190" t="str">
-        <v>保存</v>
+        <v>取消</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="str">
-        <v>settings.column.tooltip.not-in-range</v>
+        <v>settings.preferences.settings-file.save-dialog.save</v>
       </c>
       <c r="B191" t="str">
-        <v>Data not included in time range</v>
+        <v>Save</v>
+      </c>
+      <c r="C191" t="str">
+        <v>保存</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="str">
-        <v>settings.column.tooltip.auto-scale</v>
+        <v>settings.column.tooltip.not-in-range</v>
       </c>
       <c r="B192" t="str">
-        <v>Auto Scale</v>
-      </c>
-      <c r="C192" t="str">
-        <v>自动缩放</v>
+        <v>Data not included in time range</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="str">
-        <v>settings.column.tooltip.flip</v>
+        <v>settings.column.tooltip.auto-scale</v>
       </c>
       <c r="B193" t="str">
-        <v>Flip Range</v>
+        <v>Auto Scale</v>
       </c>
       <c r="C193" t="str">
-        <v>翻转区间</v>
+        <v>自动缩放</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="str">
-        <v>settings.column.titles.column-menu-title</v>
+        <v>settings.column.tooltip.flip</v>
       </c>
       <c r="B194" t="str">
-        <v>Column Customization</v>
+        <v>Flip Range</v>
       </c>
       <c r="C194" t="str">
-        <v>个性化设置列</v>
+        <v>翻转区间</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="str">
-        <v>settings.column.titles.data-mining-title</v>
+        <v>settings.column.titles.column-menu-title</v>
       </c>
       <c r="B195" t="str">
-        <v>Data Mining Settings</v>
+        <v>Column Customization</v>
       </c>
       <c r="C195" t="str">
-        <v>数据挖掘设置</v>
+        <v>个性化设置列</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="str">
-        <v>settings.column.titles.font-option-title</v>
+        <v>settings.column.titles.data-mining-title</v>
       </c>
       <c r="B196" t="str">
-        <v>Font Options for "{{name}}"</v>
+        <v>Data Mining Settings</v>
       </c>
       <c r="C196" t="str">
-        <v>设置"{{name}}"列的字体</v>
+        <v>数据挖掘设置</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="str">
-        <v>settings.column.menu.shift-row</v>
+        <v>settings.column.titles.font-option-title</v>
       </c>
       <c r="B197" t="str">
-        <v>Shift Row Positions</v>
+        <v>Font Options for "{{name}}"</v>
       </c>
       <c r="C197" t="str">
-        <v>移动位置</v>
+        <v>设置"{{name}}"列的字体</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="str">
-        <v>settings.column.menu.edit-name</v>
+        <v>settings.column.menu.shift-row</v>
       </c>
       <c r="B198" t="str">
-        <v>Edit Title</v>
+        <v>Shift Row Positions</v>
       </c>
       <c r="C198" t="str">
-        <v>编辑标题</v>
+        <v>移动位置</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="str">
-        <v>settings.column.menu.background-color</v>
+        <v>settings.column.menu.edit-name</v>
       </c>
       <c r="B199" t="str">
-        <v>Background Color</v>
+        <v>Edit Title</v>
       </c>
       <c r="C199" t="str">
-        <v>背景颜色</v>
+        <v>编辑标题</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="str">
-        <v>settings.column.menu.enable-title</v>
+        <v>settings.column.menu.background-color</v>
       </c>
       <c r="B200" t="str">
-        <v>Enable Title</v>
+        <v>Background Color</v>
       </c>
       <c r="C200" t="str">
-        <v>显示标题</v>
+        <v>背景颜色</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="str">
-        <v>settings.column.menu.show-age-label</v>
+        <v>settings.column.menu.enable-title</v>
       </c>
       <c r="B201" t="str">
-        <v>Show Age Label</v>
+        <v>Enable Title</v>
       </c>
       <c r="C201" t="str">
-        <v>显示年代</v>
+        <v>显示标题</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="str">
-        <v>settings.column.menu.info-box</v>
+        <v>settings.column.menu.show-age-label</v>
       </c>
       <c r="B202" t="str">
-        <v>Information and References</v>
+        <v>Show Age Label</v>
       </c>
       <c r="C202" t="str">
-        <v>信息与参考</v>
+        <v>显示年代</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="str">
-        <v>settings.column.menu.add-blank-column</v>
+        <v>settings.column.menu.info-box</v>
       </c>
       <c r="B203" t="str">
-        <v>Add Blank Column</v>
+        <v>Information and References</v>
       </c>
       <c r="C203" t="str">
-        <v>添加一个空白列</v>
+        <v>信息与参考</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="str">
-        <v>settings.column.menu.add-age-column</v>
+        <v>settings.column.menu.add-blank-column</v>
       </c>
       <c r="B204" t="str">
-        <v>Add Age Column</v>
+        <v>Add Blank Column</v>
       </c>
       <c r="C204" t="str">
-        <v>添加一个年代列</v>
+        <v>添加一个空白列</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="str">
-        <v>settings.column.menu.width</v>
+        <v>settings.column.menu.add-age-column</v>
       </c>
       <c r="B205" t="str">
-        <v>Width</v>
+        <v>Add Age Column</v>
       </c>
       <c r="C205" t="str">
-        <v>宽</v>
+        <v>添加一个年代列</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="str">
-        <v>settings.column.menu.orientation.title</v>
+        <v>settings.column.menu.width</v>
       </c>
       <c r="B206" t="str">
-        <v>Label Orientation</v>
+        <v>Width</v>
       </c>
       <c r="C206" t="str">
-        <v>图标排布</v>
+        <v>宽</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="str">
-        <v>settings.column.menu.orientation.horizontal</v>
+        <v>settings.column.menu.orientation.title</v>
       </c>
       <c r="B207" t="str">
-        <v>Horizontal</v>
+        <v>Label Orientation</v>
       </c>
       <c r="C207" t="str">
-        <v>横向</v>
+        <v>图标排布</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="str">
-        <v>settings.column.menu.orientation.vertical</v>
+        <v>settings.column.menu.orientation.horizontal</v>
       </c>
       <c r="B208" t="str">
-        <v>Vertical</v>
+        <v>Horizontal</v>
       </c>
       <c r="C208" t="str">
-        <v>纵向</v>
+        <v>横向</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="str">
-        <v>settings.column.menu.show-uncertainty</v>
+        <v>settings.column.menu.orientation.vertical</v>
       </c>
       <c r="B209" t="str">
-        <v>Show Uncertainty Labels</v>
+        <v>Vertical</v>
       </c>
       <c r="C209" t="str">
-        <v>显示不确定性</v>
+        <v>纵向</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="str">
-        <v>settings.column.menu.events</v>
+        <v>settings.column.menu.show-uncertainty</v>
       </c>
       <c r="B210" t="str">
-        <v>Events</v>
+        <v>Show Uncertainty Labels</v>
       </c>
       <c r="C210" t="str">
-        <v>事件</v>
+        <v>显示不确定性</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="str">
-        <v>settings.column.menu.ranges</v>
+        <v>settings.column.menu.events</v>
       </c>
       <c r="B211" t="str">
-        <v>Ranges</v>
+        <v>Events</v>
       </c>
       <c r="C211" t="str">
-        <v>范围</v>
+        <v>事件</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="str">
-        <v>settings.column.menu.first-occurrence</v>
+        <v>settings.column.menu.ranges</v>
       </c>
       <c r="B212" t="str">
-        <v>First Occurrence</v>
+        <v>Ranges</v>
       </c>
       <c r="C212" t="str">
-        <v>首先发生的优先</v>
+        <v>范围</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="str">
-        <v>settings.column.menu.last-occurrence</v>
+        <v>settings.column.menu.first-occurrence</v>
       </c>
       <c r="B213" t="str">
-        <v>Last Occurrence</v>
+        <v>First Occurrence</v>
       </c>
       <c r="C213" t="str">
-        <v>最后发生的优先</v>
+        <v>首先发生的优先</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="str">
-        <v>settings.column.menu.alphabetical</v>
+        <v>settings.column.menu.last-occurrence</v>
       </c>
       <c r="B214" t="str">
-        <v>Alphabetical</v>
+        <v>Last Occurrence</v>
       </c>
       <c r="C214" t="str">
-        <v>按字母顺序排列</v>
+        <v>最后发生的优先</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="str">
-        <v>settings.column.menu.ruler.title</v>
+        <v>settings.column.menu.alphabetical</v>
       </c>
       <c r="B215" t="str">
-        <v>Age Ruler Justification</v>
+        <v>Alphabetical</v>
       </c>
       <c r="C215" t="str">
-        <v>调整年代刻度尺</v>
+        <v>按字母顺序排列</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="str">
-        <v>settings.column.menu.ruler.left</v>
+        <v>settings.column.menu.ruler.title</v>
       </c>
       <c r="B216" t="str">
-        <v>Left</v>
+        <v>Age Ruler Justification</v>
       </c>
       <c r="C216" t="str">
-        <v>左对齐</v>
+        <v>调整年代刻度尺</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="str">
-        <v>settings.column.menu.ruler.right</v>
+        <v>settings.column.menu.ruler.left</v>
       </c>
       <c r="B217" t="str">
-        <v>Right</v>
+        <v>Left</v>
       </c>
       <c r="C217" t="str">
-        <v>右对齐</v>
+        <v>左对齐</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="str">
-        <v>settings.column.font-menu.change</v>
+        <v>settings.column.menu.ruler.right</v>
       </c>
       <c r="B218" t="str">
-        <v>Change Font</v>
+        <v>Right</v>
       </c>
       <c r="C218" t="str">
-        <v>更改字体</v>
+        <v>右对齐</v>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="str">
-        <v>settings.column.font-menu.additional</v>
+        <v>settings.column.font-menu.change</v>
       </c>
       <c r="B219" t="str">
-        <v>Additional fonts for child columns</v>
+        <v>Change Font</v>
       </c>
       <c r="C219" t="str">
-        <v>子列的更多字体选项</v>
+        <v>更改字体</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="str">
-        <v>settings.column.datamining-menu.title</v>
+        <v>settings.column.font-menu.additional</v>
       </c>
       <c r="B220" t="str">
-        <v>Data Mining Settings</v>
+        <v>Additional fonts for child columns</v>
       </c>
       <c r="C220" t="str">
-        <v>数据挖掘设置</v>
+        <v>子列的更多字体选项</v>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="str">
-        <v>settings.column.datamining-menu.window-size</v>
+        <v>settings.column.datamining-menu.title</v>
       </c>
       <c r="B221" t="str">
-        <v>Window Size</v>
+        <v>Data Mining Settings</v>
       </c>
       <c r="C221" t="str">
-        <v>窗口大小</v>
+        <v>数据挖掘设置</v>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="str">
-        <v>settings.column.datamining-menu.step-size</v>
+        <v>settings.column.datamining-menu.window-size</v>
       </c>
       <c r="B222" t="str">
-        <v>Step Size</v>
+        <v>Window Size</v>
       </c>
       <c r="C222" t="str">
-        <v>步长</v>
+        <v>窗口大小</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="str">
-        <v>settings.column.datamining-menu.options.frequency</v>
+        <v>settings.column.datamining-menu.step-size</v>
       </c>
       <c r="B223" t="str">
-        <v>Frequency</v>
+        <v>Step Size</v>
       </c>
       <c r="C223" t="str">
-        <v>频率</v>
+        <v>步长</v>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="str">
-        <v>settings.column.datamining-menu.options.max-val</v>
+        <v>settings.column.datamining-menu.options.frequency</v>
       </c>
       <c r="B224" t="str">
-        <v>Maximum Value</v>
+        <v>Frequency</v>
       </c>
       <c r="C224" t="str">
-        <v>最大值</v>
+        <v>频率</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="str">
-        <v>settings.column.datamining-menu.options.min-val</v>
+        <v>settings.column.datamining-menu.options.max-val</v>
       </c>
       <c r="B225" t="str">
-        <v>Minimum Value</v>
+        <v>Maximum Value</v>
       </c>
       <c r="C225" t="str">
-        <v>最小值</v>
+        <v>最大值</v>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="str">
-        <v>settings.column.datamining-menu.options.avg-val</v>
+        <v>settings.column.datamining-menu.options.min-val</v>
       </c>
       <c r="B226" t="str">
-        <v>Average Value</v>
+        <v>Minimum Value</v>
       </c>
       <c r="C226" t="str">
-        <v>平均值</v>
+        <v>最小值</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="str">
-        <v>settings.column.datamining-menu.options.roc</v>
+        <v>settings.column.datamining-menu.options.avg-val</v>
       </c>
       <c r="B227" t="str">
-        <v>Rate of Change</v>
+        <v>Average Value</v>
       </c>
       <c r="C227" t="str">
-        <v>变化率</v>
+        <v>平均值</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="str">
-        <v>settings.column.datamining-menu.options.freq-of-LAD</v>
+        <v>settings.column.datamining-menu.options.roc</v>
       </c>
       <c r="B228" t="str">
-        <v>Frequency of LAD</v>
+        <v>Rate of Change</v>
       </c>
       <c r="C228" t="str">
-        <v>LAD 频率</v>
+        <v>变化率</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="str">
-        <v>settings.column.datamining-menu.options.freq-of-FAD</v>
+        <v>settings.column.datamining-menu.options.freq-of-LAD</v>
       </c>
       <c r="B229" t="str">
-        <v>Frequency of FAD</v>
+        <v>Frequency of LAD</v>
       </c>
       <c r="C229" t="str">
-        <v>FAD 频率</v>
+        <v>LAD 频率</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="str">
-        <v>settings.column.datamining-menu.options.combined-events</v>
+        <v>settings.column.datamining-menu.options.freq-of-FAD</v>
       </c>
       <c r="B230" t="str">
-        <v>Combined Events</v>
+        <v>Frequency of FAD</v>
       </c>
       <c r="C230" t="str">
-        <v>组合事件</v>
+        <v>FAD 频率</v>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="str">
-        <v>settings.column.datamining-menu.options-title.event</v>
+        <v>settings.column.datamining-menu.options.combined-events</v>
       </c>
       <c r="B231" t="str">
-        <v>Event Type</v>
+        <v>Combined Events</v>
       </c>
       <c r="C231" t="str">
-        <v>事件类型</v>
+        <v>组合事件</v>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="str">
-        <v>settings.column.datamining-menu.options-title.chron</v>
+        <v>settings.column.datamining-menu.options-title.event</v>
       </c>
       <c r="B232" t="str">
-        <v>Chron Type</v>
+        <v>Event Type</v>
       </c>
       <c r="C232" t="str">
-        <v>年代类型</v>
+        <v>事件类型</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="str">
-        <v>settings.column.datamining-menu.options-title.plot</v>
+        <v>settings.column.datamining-menu.options-title.chron</v>
       </c>
       <c r="B233" t="str">
-        <v>Data Type to Plot</v>
+        <v>Chron Type</v>
       </c>
       <c r="C233" t="str">
-        <v>绘制数据类型</v>
+        <v>年代类型</v>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="str">
-        <v>settings.column.curve-drawing-menu.title</v>
+        <v>settings.column.datamining-menu.options-title.plot</v>
       </c>
       <c r="B234" t="str">
-        <v>Point Settings</v>
+        <v>Data Type to Plot</v>
       </c>
       <c r="C234" t="str">
-        <v>点设置</v>
+        <v>绘制数据类型</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="str">
-        <v>settings.column.curve-drawing-menu.rod</v>
+        <v>settings.column.curve-drawing-menu.title</v>
       </c>
       <c r="B235" t="str">
-        <v>Range of Data</v>
+        <v>Point Settings</v>
       </c>
       <c r="C235" t="str">
-        <v>数据范围</v>
+        <v>点设置</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="str">
-        <v>settings.column.curve-drawing-menu.lower-range</v>
+        <v>settings.column.curve-drawing-menu.rod</v>
       </c>
       <c r="B236" t="str">
-        <v>Lower Range</v>
+        <v>Range of Data</v>
       </c>
       <c r="C236" t="str">
-        <v>下限</v>
+        <v>数据范围</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="str">
-        <v>settings.column.curve-drawing-menu.upper-range</v>
+        <v>settings.column.curve-drawing-menu.lower-range</v>
       </c>
       <c r="B237" t="str">
-        <v>Upper Range</v>
+        <v>Lower Range</v>
       </c>
       <c r="C237" t="str">
-        <v>上限</v>
+        <v>下限</v>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="str">
-        <v>settings.column.curve-drawing-menu.scale-start</v>
+        <v>settings.column.curve-drawing-menu.upper-range</v>
       </c>
       <c r="B238" t="str">
-        <v>Scale Start</v>
+        <v>Upper Range</v>
       </c>
       <c r="C238" t="str">
-        <v>刻度起点</v>
+        <v>上限</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="str">
-        <v>settings.column.curve-drawing-menu.scale-step</v>
+        <v>settings.column.curve-drawing-menu.scale-start</v>
       </c>
       <c r="B239" t="str">
-        <v>Scale Step</v>
+        <v>Scale Start</v>
       </c>
       <c r="C239" t="str">
-        <v>刻度步长</v>
+        <v>刻度起点</v>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="str">
-        <v>settings.column.curve-drawing-menu.show-scale</v>
+        <v>settings.column.curve-drawing-menu.scale-step</v>
       </c>
       <c r="B240" t="str">
-        <v>Show Scale</v>
+        <v>Scale Step</v>
       </c>
       <c r="C240" t="str">
-        <v>显示刻度</v>
+        <v>刻度步长</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="str">
-        <v>settings.column.curve-drawing-menu.draw-points</v>
+        <v>settings.column.curve-drawing-menu.show-scale</v>
       </c>
       <c r="B241" t="str">
-        <v>Draw Points</v>
+        <v>Show Scale</v>
       </c>
       <c r="C241" t="str">
-        <v>绘制点</v>
+        <v>显示刻度</v>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="str">
-        <v>settings.column.curve-drawing-menu.point-shape</v>
+        <v>settings.column.curve-drawing-menu.draw-points</v>
       </c>
       <c r="B242" t="str">
-        <v>Point Shape</v>
+        <v>Draw Points</v>
       </c>
       <c r="C242" t="str">
-        <v>点形状</v>
+        <v>绘制点</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="str">
-        <v>settings.column.curve-drawing-menu.line</v>
+        <v>settings.column.curve-drawing-menu.point-shape</v>
       </c>
       <c r="B243" t="str">
-        <v>Line</v>
+        <v>Point Shape</v>
       </c>
       <c r="C243" t="str">
-        <v>线条</v>
+        <v>点形状</v>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="str">
-        <v>settings.column.curve-drawing-menu.fill</v>
+        <v>settings.column.curve-drawing-menu.line</v>
       </c>
       <c r="B244" t="str">
-        <v>Fill</v>
+        <v>Line</v>
       </c>
       <c r="C244" t="str">
-        <v>填充</v>
+        <v>线条</v>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="str">
-        <v>settings.column.curve-drawing-menu.background-gradient</v>
+        <v>settings.column.curve-drawing-menu.fill</v>
       </c>
       <c r="B245" t="str">
-        <v>Background Gradient</v>
+        <v>Fill</v>
       </c>
       <c r="C245" t="str">
-        <v>背景渐变</v>
+        <v>填充</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="str">
-        <v>settings.column.curve-drawing-menu.curve-gradient</v>
+        <v>settings.column.curve-drawing-menu.background-gradient</v>
       </c>
       <c r="B246" t="str">
-        <v>Curve Gradient</v>
+        <v>Background Gradient</v>
       </c>
       <c r="C246" t="str">
-        <v>曲线渐变</v>
+        <v>背景渐变</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="str">
-        <v>settings.column.curve-drawing-menu.start</v>
+        <v>settings.column.curve-drawing-menu.curve-gradient</v>
       </c>
       <c r="B247" t="str">
-        <v>Start</v>
+        <v>Curve Gradient</v>
       </c>
       <c r="C247" t="str">
-        <v>起点</v>
+        <v>曲线渐变</v>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="str">
-        <v>settings.column.curve-drawing-menu.end</v>
+        <v>settings.column.curve-drawing-menu.start</v>
       </c>
       <c r="B248" t="str">
-        <v>End</v>
+        <v>Start</v>
       </c>
       <c r="C248" t="str">
-        <v>终点</v>
+        <v>起点</v>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="str">
-        <v>settings.search.search-bar</v>
+        <v>settings.column.curve-drawing-menu.end</v>
       </c>
       <c r="B249" t="str">
-        <v>Search</v>
+        <v>End</v>
       </c>
       <c r="C249" t="str">
-        <v>搜索</v>
+        <v>终点</v>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="str">
-        <v>settings.search.found-result</v>
+        <v>settings.column.overlay-menu.title</v>
       </c>
       <c r="B250" t="str">
-        <v>Found {{count}} Results</v>
-      </c>
-      <c r="C250" t="str">
-        <v>找到 {{count}} 个结果</v>
+        <v>Overlay Settings</v>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="str">
-        <v>settings.search.current-time-settings</v>
+        <v>settings.column.overlay-menu.current-overlay</v>
       </c>
       <c r="B251" t="str">
-        <v>Current Time Settings(Top / Base)</v>
-      </c>
-      <c r="C251" t="str">
-        <v>当前时间区间设置(顶部 / 底部)</v>
+        <v>Current Overlay</v>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="str">
-        <v>settings.search.header.status</v>
+        <v>settings.column.overlay-menu.choose-column-empty</v>
       </c>
       <c r="B252" t="str">
-        <v>Column On?</v>
-      </c>
-      <c r="C252" t="str">
-        <v>是否已选</v>
+        <v>Choose Column &gt;&gt;&gt;</v>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="str">
-        <v>settings.search.header.center</v>
+        <v>settings.column.overlay-menu.display-overlay</v>
       </c>
       <c r="B253" t="str">
-        <v>Center</v>
-      </c>
-      <c r="C253" t="str">
-        <v>居中</v>
+        <v>Display Overlay</v>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="str">
-        <v>settings.search.header.extend</v>
+        <v>settings.column.overlay-menu.choose-second-column</v>
       </c>
       <c r="B254" t="str">
-        <v>Extend</v>
-      </c>
-      <c r="C254" t="str">
-        <v>延展</v>
+        <v>Choose Second Column</v>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="str">
-        <v>settings.search.header.column</v>
+        <v>settings.search.search-bar</v>
       </c>
       <c r="B255" t="str">
-        <v>Column</v>
+        <v>Search</v>
       </c>
       <c r="C255" t="str">
-        <v>列名称</v>
+        <v>搜索</v>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="str">
-        <v>settings.search.header.age</v>
+        <v>settings.search.found-result</v>
       </c>
       <c r="B256" t="str">
-        <v>Age</v>
+        <v>Found {{count}} Results</v>
       </c>
       <c r="C256" t="str">
-        <v>年代</v>
+        <v>找到 {{count}} 个结果</v>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="str">
-        <v>settings.search.header.qualifier</v>
+        <v>settings.search.current-time-settings</v>
       </c>
       <c r="B257" t="str">
-        <v>Type</v>
+        <v>Current Time Settings(Top / Base)</v>
       </c>
       <c r="C257" t="str">
-        <v>类别</v>
+        <v>当前时间区间设置(顶部 / 底部)</v>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="str">
-        <v>settings.search.header.notes</v>
+        <v>settings.search.header.status</v>
       </c>
       <c r="B258" t="str">
-        <v>Notes</v>
+        <v>Column On?</v>
       </c>
       <c r="C258" t="str">
-        <v>注释</v>
+        <v>是否已选</v>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="str">
-        <v>settings.font.notes1</v>
+        <v>settings.search.header.center</v>
       </c>
       <c r="B259" t="str">
-        <v>These are the default systemwide fonts.</v>
+        <v>Center</v>
       </c>
       <c r="C259" t="str">
-        <v>这些是系统默认的全局字体</v>
+        <v>居中</v>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="str">
-        <v>settings.font.notes2</v>
+        <v>settings.search.header.extend</v>
       </c>
       <c r="B260" t="str">
-        <v>Changing one here will affect the entire chart.</v>
+        <v>Extend</v>
       </c>
       <c r="C260" t="str">
-        <v>在此处更改字体会影响整个图表</v>
+        <v>延展</v>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="str">
-        <v>settings.font.notes3</v>
+        <v>settings.search.header.column</v>
       </c>
       <c r="B261" t="str">
-        <v>NOTE: These fonts can be changed on a column by column basis by using the Font button for each column</v>
+        <v>Column</v>
       </c>
       <c r="C261" t="str">
-        <v>注意：可以通过每列的“字体”按钮单独更改每列的字体</v>
+        <v>列名称</v>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="str">
-        <v>settings.map-points.not-avaliable</v>
+        <v>settings.search.header.age</v>
       </c>
       <c r="B262" t="str">
-        <v>No Map Points available for this datapack</v>
+        <v>Age</v>
       </c>
       <c r="C262" t="str">
-        <v>该数据包暂无地图可用</v>
+        <v>年代</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="str">
-        <v>settings.datapacks.see-info-guidance</v>
+        <v>settings.search.header.qualifier</v>
       </c>
       <c r="B263" t="str">
-        <v>Click a datapack to see more information!</v>
+        <v>Type</v>
       </c>
       <c r="C263" t="str">
-        <v>点击数据包以查看更多信息！</v>
+        <v>类别</v>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="str">
-        <v>settings.datapacks.add-datapack-guidance</v>
+        <v>settings.search.header.notes</v>
       </c>
       <c r="B264" t="str">
-        <v>Add a datapack by clicking the checkbox</v>
+        <v>Notes</v>
       </c>
       <c r="C264" t="str">
-        <v>点击加号添加数据包</v>
+        <v>注释</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="str">
-        <v>settings.datapacks.title.private-official</v>
+        <v>settings.font.notes1</v>
       </c>
       <c r="B265" t="str">
-        <v>Private Official Datapacks</v>
+        <v>These are the default systemwide fonts.</v>
+      </c>
+      <c r="C265" t="str">
+        <v>这些是系统默认的全局字体</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="str">
-        <v>settings.datapacks.title.public-official</v>
+        <v>settings.font.notes2</v>
       </c>
       <c r="B266" t="str">
-        <v>Official Datapacks</v>
+        <v>Changing one here will affect the entire chart.</v>
+      </c>
+      <c r="C266" t="str">
+        <v>在此处更改字体会影响整个图表</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="str">
-        <v>settings.datapacks.title.contributed</v>
+        <v>settings.font.notes3</v>
       </c>
       <c r="B267" t="str">
-        <v>User Contributed Datapacks</v>
+        <v>NOTE: These fonts can be changed on a column by column basis by using the Font button for each column</v>
+      </c>
+      <c r="C267" t="str">
+        <v>注意：可以通过每列的“字体”按钮单独更改每列的字体</v>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="str">
-        <v>settings.datapacks.title.workshop</v>
+        <v>settings.map-points.not-avaliable</v>
       </c>
       <c r="B268" t="str">
-        <v>Workshop Datapacks</v>
+        <v>No Map Points available for this datapack</v>
       </c>
       <c r="C268" t="str">
-        <v>工作坊数据包</v>
+        <v>该数据包暂无地图可用</v>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="str">
-        <v>settings.datapacks.title.your</v>
+        <v>settings.datapacks.see-info-guidance</v>
       </c>
       <c r="B269" t="str">
-        <v>Your Datapacks</v>
+        <v>Click a datapack to see more information!</v>
       </c>
       <c r="C269" t="str">
-        <v>你的数据包</v>
+        <v>点击数据包以查看更多信息！</v>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="str">
-        <v>settings.datapacks.no</v>
+        <v>settings.datapacks.add-datapack-guidance</v>
       </c>
       <c r="B270" t="str">
-        <v>No</v>
+        <v>Add a datapack by clicking the checkbox</v>
       </c>
       <c r="C270" t="str">
-        <v>暂无</v>
+        <v>点击加号添加数据包</v>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="str">
-        <v>settings.datapacks.avaliable</v>
+        <v>settings.datapacks.title.private-official</v>
       </c>
       <c r="B271" t="str">
-        <v>Avaliable</v>
-      </c>
-      <c r="C271" t="str">
-        <v>可用</v>
+        <v>Private Official Datapacks</v>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="str">
-        <v>settings.datapacks.upload</v>
+        <v>settings.datapacks.title.public-official</v>
       </c>
       <c r="B272" t="str">
-        <v>Upload Datapack</v>
-      </c>
-      <c r="C272" t="str">
-        <v>上传数据包</v>
+        <v>Official Datapacks</v>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="str">
-        <v>settings.datapacks.pdf-upload</v>
+        <v>settings.datapacks.title.contributed</v>
       </c>
       <c r="B273" t="str">
-        <v>PDF Upload</v>
+        <v>User Contributed Datapacks</v>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="str">
-        <v>settings.datapacks.seeMore</v>
+        <v>settings.datapacks.title.workshop</v>
       </c>
       <c r="B274" t="str">
-        <v>See More...</v>
+        <v>Workshop Datapacks</v>
+      </c>
+      <c r="C274" t="str">
+        <v>工作坊数据包</v>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="str">
-        <v>settings.datapacks.seeLess</v>
+        <v>settings.datapacks.title.your</v>
       </c>
       <c r="B275" t="str">
-        <v>See Less...</v>
+        <v>Your Datapacks</v>
+      </c>
+      <c r="C275" t="str">
+        <v>你的数据包</v>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="str">
-        <v>settings.datapacks.upload-form.title</v>
+        <v>settings.datapacks.no</v>
       </c>
       <c r="B276" t="str">
-        <v>Upload Your Own Datapack</v>
+        <v>No</v>
       </c>
       <c r="C276" t="str">
-        <v>上传你的数据包</v>
+        <v>暂无</v>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="str">
-        <v>settings.datapacks.upload-form.no-file</v>
+        <v>settings.datapacks.avaliable</v>
       </c>
       <c r="B277" t="str">
-        <v>No file selected</v>
+        <v>Avaliable</v>
       </c>
       <c r="C277" t="str">
-        <v>没有选择文件</v>
+        <v>可用</v>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="str">
-        <v>settings.datapacks.upload-form.name</v>
+        <v>settings.datapacks.upload</v>
       </c>
       <c r="B278" t="str">
-        <v>Datapack Name</v>
+        <v>Upload Datapack</v>
       </c>
       <c r="C278" t="str">
-        <v>数据包名称</v>
+        <v>上传数据包</v>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="str">
-        <v>settings.datapacks.upload-form.name-placeholder</v>
+        <v>settings.datapacks.pdf-upload</v>
       </c>
       <c r="B279" t="str">
-        <v>Enter a name for your datapack.</v>
-      </c>
-      <c r="C279" t="str">
-        <v>请为你的数据包输入名称</v>
+        <v>PDF Upload</v>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="str">
-        <v>settings.datapacks.upload-form.author</v>
+        <v>settings.datapacks.seeMore</v>
       </c>
       <c r="B280" t="str">
-        <v>Authored By</v>
-      </c>
-      <c r="C280" t="str">
-        <v>作者</v>
+        <v>See More...</v>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="str">
-        <v>settings.datapacks.upload-form.author-placeholder</v>
+        <v>settings.datapacks.seeLess</v>
       </c>
       <c r="B281" t="str">
-        <v>Credited to...</v>
-      </c>
-      <c r="C281" t="str">
-        <v>作者为...</v>
+        <v>See Less...</v>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="str">
-        <v>settings.datapacks.upload-form.description</v>
+        <v>settings.datapacks.upload-form.title</v>
       </c>
       <c r="B282" t="str">
-        <v>Datapack Description</v>
+        <v>Upload Your Own Datapack</v>
       </c>
       <c r="C282" t="str">
-        <v>数据包概述</v>
+        <v>上传你的数据包</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="str">
-        <v>settings.datapacks.upload-form.description-placeholder</v>
+        <v>settings.datapacks.upload-form.no-file</v>
       </c>
       <c r="B283" t="str">
-        <v>Enter a description for your datapack.</v>
+        <v>No file selected</v>
       </c>
       <c r="C283" t="str">
-        <v>请为你的数据包添加概述</v>
+        <v>没有选择文件</v>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="str">
-        <v>settings.datapacks.upload-form.tags</v>
+        <v>settings.datapacks.upload-form.name</v>
       </c>
       <c r="B284" t="str">
-        <v>Tags</v>
+        <v>Datapack Name</v>
       </c>
       <c r="C284" t="str">
-        <v>标签</v>
+        <v>数据包名称</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="str">
-        <v>settings.datapacks.upload-form.make-public</v>
+        <v>settings.datapacks.upload-form.name-placeholder</v>
       </c>
       <c r="B285" t="str">
-        <v>Make Datapack Publicly Accessible</v>
+        <v>Enter a name for your datapack.</v>
       </c>
       <c r="C285" t="str">
-        <v>使数据包对公共可见</v>
+        <v>请为你的数据包输入名称</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="str">
-        <v>settings.datapacks.upload-form.button.add-ref</v>
+        <v>settings.datapacks.upload-form.author</v>
       </c>
       <c r="B286" t="str">
-        <v>Add Reference</v>
+        <v>Authored By</v>
       </c>
       <c r="C286" t="str">
-        <v>添加引用</v>
+        <v>作者</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="str">
-        <v>settings.datapacks.upload-form.button.more</v>
+        <v>settings.datapacks.upload-form.author-placeholder</v>
       </c>
       <c r="B287" t="str">
-        <v>More Options</v>
+        <v>Credited to...</v>
       </c>
       <c r="C287" t="str">
-        <v>更多选项</v>
+        <v>作者为...</v>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="str">
-        <v>settings.datapacks.upload-form.button.finish</v>
+        <v>settings.datapacks.upload-form.description</v>
       </c>
       <c r="B288" t="str">
-        <v>Finish &amp; Upload</v>
+        <v>Datapack Description</v>
       </c>
       <c r="C288" t="str">
-        <v>完成并上传</v>
+        <v>数据包概述</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="str">
-        <v>settings.datapacks.upload-form.button.startover</v>
+        <v>settings.datapacks.upload-form.description-placeholder</v>
       </c>
       <c r="B289" t="str">
-        <v>Start Over</v>
+        <v>Enter a description for your datapack.</v>
       </c>
       <c r="C289" t="str">
-        <v>重新开始</v>
+        <v>请为你的数据包添加概述</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="str">
-        <v>settings.datapacks.upload-form.reference</v>
+        <v>settings.datapacks.upload-form.tags</v>
       </c>
       <c r="B290" t="str">
-        <v>Reference</v>
+        <v>Tags</v>
       </c>
       <c r="C290" t="str">
-        <v>引用</v>
+        <v>标签</v>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="str">
-        <v>settings.datapacks.upload-form.contact</v>
+        <v>settings.datapacks.upload-form.make-public</v>
       </c>
       <c r="B291" t="str">
-        <v>Contact</v>
+        <v>Make Datapack Publicly Accessible</v>
       </c>
       <c r="C291" t="str">
-        <v>联系方式</v>
+        <v>使数据包对公共可见</v>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="str">
-        <v>settings.datapacks.upload-form.contact-placeholder</v>
+        <v>settings.datapacks.upload-form.button.add-ref</v>
       </c>
       <c r="B292" t="str">
-        <v>Enter your contact information</v>
+        <v>Add Reference</v>
       </c>
       <c r="C292" t="str">
-        <v>输入你的联系方式</v>
+        <v>添加引用</v>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="str">
-        <v>settings.datapacks.upload-form.contact-helper-text</v>
+        <v>settings.datapacks.upload-form.button.more</v>
       </c>
       <c r="B293" t="str">
-        <v>(OPTIONAL) If you would like others to contact you about this datapack</v>
+        <v>More Options</v>
       </c>
       <c r="C293" t="str">
-        <v>如果想要其他用户就此数据包问题联系你，请填写</v>
+        <v>更多选项</v>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="str">
-        <v>settings.datapacks.upload-form.notes</v>
+        <v>settings.datapacks.upload-form.button.finish</v>
       </c>
       <c r="B294" t="str">
-        <v>Notes</v>
+        <v>Finish &amp; Upload</v>
       </c>
       <c r="C294" t="str">
-        <v>注释</v>
+        <v>完成并上传</v>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="str">
-        <v>settings.datapacks.upload-form.notes-placeholder</v>
+        <v>settings.datapacks.upload-form.button.startover</v>
       </c>
       <c r="B295" t="str">
-        <v>Enter notes for the datapack here</v>
+        <v>Start Over</v>
       </c>
       <c r="C295" t="str">
-        <v>为你的数据包添加注释</v>
+        <v>重新开始</v>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="str">
-        <v>settings.datapacks.upload-form.notes-helper-text</v>
+        <v>settings.datapacks.upload-form.reference</v>
       </c>
       <c r="B296" t="str">
-        <v>(OPTIONAL) Generally notes are settings recommendations/How to use your datapack most efficiently</v>
+        <v>Reference</v>
       </c>
       <c r="C296" t="str">
-        <v>如果想要指导其他用户如何有效地使用此数据包，请填写</v>
+        <v>引用</v>
       </c>
     </row>
     <row r="297">
       <c r="A297" t="str">
-        <v>chart.no-chart-yet</v>
+        <v>settings.datapacks.upload-form.contact</v>
       </c>
       <c r="B297" t="str">
-        <v>You have not made a chart yet</v>
+        <v>Contact</v>
       </c>
       <c r="C297" t="str">
-        <v>您还未制作任何图表</v>
+        <v>联系方式</v>
       </c>
     </row>
     <row r="298">
       <c r="A298" t="str">
-        <v>chart.save</v>
+        <v>settings.datapacks.upload-form.contact-placeholder</v>
       </c>
       <c r="B298" t="str">
-        <v>Save Chart</v>
+        <v>Enter your contact information</v>
       </c>
       <c r="C298" t="str">
-        <v>保存图表</v>
+        <v>输入你的联系方式</v>
       </c>
     </row>
     <row r="299">
       <c r="A299" t="str">
-        <v>dialogs.confirm-datapack-change.title</v>
+        <v>settings.datapacks.upload-form.contact-helper-text</v>
       </c>
       <c r="B299" t="str">
-        <v>Confirm Datapack Selection Change</v>
+        <v>(OPTIONAL) If you would like others to contact you about this datapack</v>
       </c>
       <c r="C299" t="str">
-        <v>确认更改数据包</v>
+        <v>如果想要其他用户就此数据包问题联系你，请填写</v>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="str">
-        <v>dialogs.confirm-datapack-change.message</v>
+        <v>settings.datapacks.upload-form.notes</v>
       </c>
       <c r="B300" t="str">
-        <v>You have unsaved changes! Do you want to save your changes?</v>
+        <v>Notes</v>
       </c>
       <c r="C300" t="str">
-        <v>你有未保存的更改! 你想保存你的更改吗?</v>
+        <v>注释</v>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="str">
-        <v>dialogs.confirm-datapack-change.yes</v>
+        <v>settings.datapacks.upload-form.notes-placeholder</v>
       </c>
       <c r="B301" t="str">
-        <v>Save</v>
+        <v>Enter notes for the datapack here</v>
       </c>
       <c r="C301" t="str">
-        <v>保存</v>
+        <v>为你的数据包添加注释</v>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="str">
-        <v>dialogs.confirm-datapack-change.no</v>
+        <v>settings.datapacks.upload-form.notes-helper-text</v>
       </c>
       <c r="B302" t="str">
-        <v>Discard</v>
+        <v>(OPTIONAL) Generally notes are settings recommendations/How to use your datapack most efficiently</v>
       </c>
       <c r="C302" t="str">
-        <v>不保存</v>
+        <v>如果想要指导其他用户如何有效地使用此数据包，请填写</v>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="str">
-        <v>dialogs.default-age.title</v>
+        <v>chart.no-chart-yet</v>
       </c>
       <c r="B303" t="str">
-        <v>Use default age range?</v>
+        <v>You have not made a chart yet</v>
       </c>
       <c r="C303" t="str">
-        <v>使用默认时间区间？</v>
+        <v>您还未制作任何图表</v>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="str">
-        <v>dialogs.confirm-changes.message</v>
+        <v>chart.save</v>
       </c>
       <c r="B304" t="str">
-        <v>Are you sure you want to discard your changes?</v>
+        <v>Save Chart</v>
+      </c>
+      <c r="C304" t="str">
+        <v>保存图表</v>
       </c>
     </row>
     <row r="305">
       <c r="A305" t="str">
-        <v>help.qsg.title</v>
+        <v>dialogs.confirm-datapack-change.title</v>
       </c>
       <c r="B305" t="str">
-        <v>Quick Start Quide</v>
+        <v>Confirm Datapack Selection Change</v>
       </c>
       <c r="C305" t="str">
-        <v>快速指南</v>
+        <v>确认更改数据包</v>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="str">
-        <v>help.qsg.content</v>
+        <v>dialogs.confirm-datapack-change.message</v>
       </c>
       <c r="B306" t="str">
-        <v>Welcome to Time Scale Creator Online! In this Quick Start Guide, you will quickly learn about the functions of each tab on the Nav bar. Click the 'Start QSG' button to begin.</v>
+        <v>You have unsaved changes! Do you want to save your changes?</v>
       </c>
       <c r="C306" t="str">
-        <v>欢迎使用Time Scale Creator在线版！在这个快速指南中，您将迅速了解导航栏上每个标签页的功能。点击“开始快速指南”按钮开始体验。</v>
+        <v>你有未保存的更改! 你想保存你的更改吗?</v>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="str">
-        <v>help.qsg.button</v>
+        <v>dialogs.confirm-datapack-change.yes</v>
       </c>
       <c r="B307" t="str">
-        <v>Start QSG</v>
+        <v>Save</v>
       </c>
       <c r="C307" t="str">
-        <v>开始快速指南</v>
+        <v>保存</v>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="str">
-        <v>help.tour.title</v>
+        <v>dialogs.confirm-datapack-change.no</v>
       </c>
       <c r="B308" t="str">
-        <v>Tour</v>
+        <v>Discard</v>
       </c>
       <c r="C308" t="str">
-        <v>导览</v>
+        <v>不保存</v>
       </c>
     </row>
     <row r="309">
       <c r="A309" t="str">
-        <v>help.tour.content.datapacks</v>
+        <v>dialogs.default-age.title</v>
       </c>
       <c r="B309" t="str">
-        <v>In the datapacks tour you will explore the Datapacks page in depth. Click the button to start your tour!</v>
+        <v>Use default age range?</v>
       </c>
       <c r="C309" t="str">
-        <v>在数据包导览中，您将深入探索数据包页面。点击按钮开始您的导览！</v>
+        <v>使用默认时间区间？</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="str">
-        <v>help.tour.content.settings</v>
+        <v>dialogs.confirm-changes.message</v>
       </c>
       <c r="B310" t="str">
-        <v>In the settings tour you will explore the Settings page in depth. Click the button to start your tour!</v>
-      </c>
-      <c r="C310" t="str">
-        <v>在设置导览中，您将深入探索设置页面。点击按钮开始您的导览！</v>
+        <v>Are you sure you want to discard your changes?</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="str">
-        <v>help.tour.button.datapacks</v>
+        <v>help.qsg.title</v>
       </c>
       <c r="B311" t="str">
-        <v>Start Datapacks Tour</v>
+        <v>Quick Start Quide</v>
       </c>
       <c r="C311" t="str">
-        <v>开始数据包导览</v>
+        <v>快速指南</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="str">
-        <v>help.tour.button.settings</v>
+        <v>help.qsg.content</v>
       </c>
       <c r="B312" t="str">
-        <v>Start Settings Tour</v>
+        <v>Welcome to Time Scale Creator Online! In this Quick Start Guide, you will quickly learn about the functions of each tab on the Nav bar. Click the 'Start QSG' button to begin.</v>
       </c>
       <c r="C312" t="str">
-        <v>开始设置导览</v>
+        <v>欢迎使用Time Scale Creator在线版！在这个快速指南中，您将迅速了解导航栏上每个标签页的功能。点击“开始快速指南”按钮开始体验。</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="str">
-        <v>help.license</v>
+        <v>help.qsg.button</v>
       </c>
       <c r="B313" t="str">
-        <v>Software License</v>
+        <v>Start QSG</v>
       </c>
       <c r="C313" t="str">
-        <v>软件许可</v>
+        <v>开始快速指南</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="str">
-        <v>help.file-format-info.title</v>
+        <v>help.tour.title</v>
       </c>
       <c r="B314" t="str">
-        <v>File Format Info</v>
+        <v>Tour</v>
       </c>
       <c r="C314" t="str">
-        <v>文件格式信息</v>
+        <v>导览</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="str">
-        <v>help.file-format-info.link</v>
+        <v>help.tour.content.datapacks</v>
       </c>
       <c r="B315" t="str">
-        <v>View File Format Info</v>
+        <v>In the datapacks tour you will explore the Datapacks page in depth. Click the button to start your tour!</v>
       </c>
       <c r="C315" t="str">
-        <v>查看文件格式信息</v>
+        <v>在数据包导览中，您将深入探索数据包页面。点击按钮开始您的导览！</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="str">
-        <v>errors.title</v>
+        <v>help.tour.content.settings</v>
       </c>
       <c r="B316" t="str">
-        <v>Error</v>
+        <v>In the settings tour you will explore the Settings page in depth. Click the button to start your tour!</v>
       </c>
       <c r="C316" t="str">
-        <v>错误</v>
+        <v>在设置导览中，您将深入探索设置页面。点击按钮开始您的导览！</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="str">
-        <v>errors.SERVER_RESPONSE_ERROR</v>
+        <v>help.tour.button.datapacks</v>
       </c>
       <c r="B317" t="str">
-        <v>Server response error. Please try again later.</v>
+        <v>Start Datapacks Tour</v>
       </c>
       <c r="C317" t="str">
-        <v>服务器错误。请稍后再试。</v>
+        <v>开始数据包导览</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="str">
-        <v>errors.INVALID_DATAPACK_INFO</v>
+        <v>help.tour.button.settings</v>
       </c>
       <c r="B318" t="str">
-        <v>Invalid datapack info received from server. Please try again later.</v>
+        <v>Start Settings Tour</v>
       </c>
       <c r="C318" t="str">
-        <v>从服务器接收到的数据包信息无效。请稍后再试。</v>
+        <v>开始设置导览</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="str">
-        <v>errors.INVALID_PRESET_INFO</v>
+        <v>help.license</v>
       </c>
       <c r="B319" t="str">
-        <v>Invalid preset info received from server. Please try again later.</v>
+        <v>Software License</v>
       </c>
       <c r="C319" t="str">
-        <v>从服务器接收到的预置无效。请稍后再试。</v>
+        <v>软件许可</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="str">
-        <v>errors.INVALID_PATTERN_INFO</v>
+        <v>help.file-format-info.title</v>
       </c>
       <c r="B320" t="str">
-        <v>Invalid pattern info received from server. Please try again later.</v>
+        <v>File Format Info</v>
       </c>
       <c r="C320" t="str">
-        <v>从服务器接收到的模式信息无效。请稍后再试。</v>
+        <v>文件格式信息</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="str">
-        <v>errors.INVALID_TIME_SCALE</v>
+        <v>help.file-format-info.link</v>
       </c>
       <c r="B321" t="str">
-        <v>Invalid time scale received from server. Please try again later.</v>
+        <v>View File Format Info</v>
       </c>
       <c r="C321" t="str">
-        <v>从服务器收到的时间刻度无效。请稍后再试。</v>
+        <v>查看文件格式信息</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="str">
-        <v>errors.INVALID_DATAPACK_CONFIG</v>
+        <v>errors.title</v>
       </c>
       <c r="B322" t="str">
-        <v>Datapacks were not properly set. Please try again later.</v>
+        <v>Error</v>
       </c>
       <c r="C322" t="str">
-        <v>数据包未正确设置。请稍后再试。</v>
+        <v>错误</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="str">
-        <v>errors.INVALID_SVG_READY_RESPONSE</v>
+        <v>errors.SERVER_RESPONSE_ERROR</v>
       </c>
       <c r="B323" t="str">
-        <v>Invalid SVG ready response received from server. Please try again later.</v>
+        <v>Server response error. Please try again later.</v>
       </c>
       <c r="C323" t="str">
-        <v>从服务器收到的SVG就绪响应无效。请稍后再试。</v>
+        <v>服务器错误。请稍后再试。</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="str">
-        <v>errors.INVALID_SETTINGS_RESPONSE</v>
+        <v>errors.INVALID_DATAPACK_INFO</v>
       </c>
       <c r="B324" t="str">
-        <v>Invalid settings response received from server. Please try again later.</v>
+        <v>Invalid datapack info received from server. Please try again later.</v>
       </c>
       <c r="C324" t="str">
-        <v>从服务器收到的设置响应无效。请稍后再试。</v>
+        <v>从服务器接收到的数据包信息无效。请稍后再试。</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="str">
-        <v>errors.INVALID_CHART_RESPONSE</v>
+        <v>errors.INVALID_PRESET_INFO</v>
       </c>
       <c r="B325" t="str">
-        <v>Invalid chart response received from server. Please try again later.</v>
+        <v>Invalid preset info received from server. Please try again later.</v>
       </c>
       <c r="C325" t="str">
-        <v>从服务器收到的图表响应无效。请稍后再试。</v>
+        <v>从服务器接收到的预置无效。请稍后再试。</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" t="str">
-        <v>errors.INVALID_PATH</v>
+        <v>errors.INVALID_PATTERN_INFO</v>
       </c>
       <c r="B326" t="str">
-        <v>The requested path was invalid. Please ensure the path is correct.</v>
+        <v>Invalid pattern info received from server. Please try again later.</v>
       </c>
       <c r="C326" t="str">
-        <v>请求的文件路径无效。请确保文件路径正确。</v>
+        <v>从服务器接收到的模式信息无效。请稍后再试。</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" t="str">
-        <v>errors.INVALID_DATAPACK_UPLOAD</v>
+        <v>errors.INVALID_TIME_SCALE</v>
       </c>
       <c r="B327" t="str">
-        <v>Invalid datapack upload.</v>
+        <v>Invalid time scale received from server. Please try again later.</v>
       </c>
       <c r="C327" t="str">
-        <v>无效的数据包上传</v>
+        <v>从服务器收到的时间刻度无效。请稍后再试。</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="str">
-        <v>errors.REGULAR_USER_UPLOAD_DATAPACK_TOO_LARGE</v>
+        <v>errors.INVALID_DATAPACK_CONFIG</v>
       </c>
       <c r="B328" t="str">
-        <v>Uploaded datapack is over 3000 characters.</v>
+        <v>Datapacks were not properly set. Please try again later.</v>
+      </c>
+      <c r="C328" t="str">
+        <v>数据包未正确设置。请稍后再试。</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="str">
-        <v>errors.INVALID_USER_DATAPACKS</v>
+        <v>errors.INVALID_SVG_READY_RESPONSE</v>
       </c>
       <c r="B329" t="str">
-        <v>Invalid user datapacks received from server. Please try again later.</v>
+        <v>Invalid SVG ready response received from server. Please try again later.</v>
       </c>
       <c r="C329" t="str">
-        <v>从服务器收到的用户数据包无效。请稍后再试。</v>
+        <v>从服务器收到的SVG就绪响应无效。请稍后再试。</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="str">
-        <v>errors.INVALID_PUBLIC_DATAPACKS</v>
+        <v>errors.INVALID_SETTINGS_RESPONSE</v>
       </c>
       <c r="B330" t="str">
-        <v>Invalid public datapacks received from server. Please try again later.</v>
+        <v>Invalid settings response received from server. Please try again later.</v>
       </c>
       <c r="C330" t="str">
-        <v>从服务器收到的公共数据包无效。请稍后再试。</v>
+        <v>从服务器收到的设置响应无效。请稍后再试。</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="str">
-        <v>errors.NO_DATAPACK_FILE_FOUND</v>
+        <v>errors.INVALID_CHART_RESPONSE</v>
       </c>
       <c r="B331" t="str">
-        <v>No datapack file found. Please upload a datapack file first.</v>
+        <v>Invalid chart response received from server. Please try again later.</v>
       </c>
       <c r="C331" t="str">
-        <v>暂无数据包。请先上传一个数据包。</v>
+        <v>从服务器收到的图表响应无效。请稍后再试。</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="str">
-        <v>errors.DATAPACK_FILE_NAME_TOO_LONG</v>
+        <v>errors.INVALID_PATH</v>
       </c>
       <c r="B332" t="str">
-        <v>Datapack file name is too long. Please shorten the file name.</v>
+        <v>The requested path was invalid. Please ensure the path is correct.</v>
       </c>
       <c r="C332" t="str">
-        <v>数据包名称过长。请缩短名称。</v>
+        <v>请求的文件路径无效。请确保文件路径正确。</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="str">
-        <v>errors.UNRECOGNIZED_DATAPACK_EXTENSION</v>
+        <v>errors.INVALID_DATAPACK_UPLOAD</v>
       </c>
       <c r="B333" t="str">
-        <v>Unrecognized datapack extension. File must be of type .dpk, .mdpk, .map, .txt. Please upload a valid datapack file.</v>
+        <v>Invalid datapack upload.</v>
       </c>
       <c r="C333" t="str">
-        <v>无法识别数据包扩展名。文件必须是 .dpk, .mdpk, .map, .txt格式。请上传有效文件格式。</v>
+        <v>无效的数据包上传</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="str">
-        <v>errors.UNRECOGNIZED_DATAPACK_FILE</v>
+        <v>errors.REGULAR_USER_UPLOAD_DATAPACK_TOO_LARGE</v>
       </c>
       <c r="B334" t="str">
-        <v>Unrecognized datapack file. Please upload a valid datapack file.</v>
-      </c>
-      <c r="C334" t="str">
-        <v>无法识别数据包。请上传有效文件。</v>
+        <v>Uploaded datapack is over 3000 characters.</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="str">
-        <v>errors.UNFINISHED_DATAPACK_UPLOAD_FORM</v>
+        <v>errors.INVALID_USER_DATAPACKS</v>
       </c>
       <c r="B335" t="str">
-        <v>Please finish the datapack upload form before attempting to upload the file.</v>
+        <v>Invalid user datapacks received from server. Please try again later.</v>
       </c>
       <c r="C335" t="str">
-        <v>请完成数据包上传表单后再尝试上传文件。</v>
+        <v>从服务器收到的用户数据包无效。请稍后再试。</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="str">
-        <v>errors.DATAPACK_ALREADY_EXISTS</v>
+        <v>errors.INVALID_PUBLIC_DATAPACKS</v>
       </c>
       <c r="B336" t="str">
-        <v>Datapack already exists. Please upload a datapack with a unique title.</v>
+        <v>Invalid public datapacks received from server. Please try again later.</v>
       </c>
       <c r="C336" t="str">
-        <v>数据包已存在。请上传不重名的数据包。</v>
+        <v>从服务器收到的公共数据包无效。请稍后再试。</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="str">
-        <v>errors.NO_DATAPACKS_SELECTED</v>
+        <v>errors.NO_DATAPACK_FILE_FOUND</v>
       </c>
       <c r="B337" t="str">
-        <v>No datapacks selected. Please select at least one datapack to generate.</v>
+        <v>No datapack file found. Please upload a datapack file first.</v>
       </c>
       <c r="C337" t="str">
-        <v>未选择数据包。请至少选择一个数据包进行绘制。</v>
+        <v>暂无数据包。请先上传一个数据包。</v>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="str">
-        <v>errors.NO_COLUMNS_SELECTED</v>
+        <v>errors.DATAPACK_FILE_NAME_TOO_LONG</v>
       </c>
       <c r="B338" t="str">
-        <v>No columns selected. Please select at least one column to generate.</v>
+        <v>Datapack file name is too long. Please shorten the file name.</v>
       </c>
       <c r="C338" t="str">
-        <v>未选择列。请至少选择一个列进行绘制。</v>
+        <v>数据包名称过长。请缩短名称。</v>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="str">
-        <v>errors.IS_BAD_RANGE</v>
+        <v>errors.UNRECOGNIZED_DATAPACK_EXTENSION</v>
       </c>
       <c r="B339" t="str">
-        <v>Base age must be greater than the top age.</v>
+        <v>Unrecognized datapack extension. File must be of type .dpk, .mdpk, .map, .txt. Please upload a valid datapack file.</v>
       </c>
       <c r="C339" t="str">
-        <v>区间底部年代应大于区间顶部年代。</v>
+        <v>无法识别数据包扩展名。文件必须是 .dpk, .mdpk, .map, .txt格式。请上传有效文件格式。</v>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="str">
-        <v>errors.INVALID_MAPPACK_INFO</v>
+        <v>errors.UNRECOGNIZED_DATAPACK_FILE</v>
       </c>
       <c r="B340" t="str">
-        <v>Invalid mappack info received from server. Please try again later.</v>
+        <v>Unrecognized datapack file. Please upload a valid datapack file.</v>
       </c>
       <c r="C340" t="str">
-        <v>从服务器接收到无效的地图包信息。请稍后再试。</v>
+        <v>无法识别数据包。请上传有效文件。</v>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="str">
-        <v>errors.UNABLE_TO_LOGIN_SERVER</v>
+        <v>errors.UNFINISHED_DATAPACK_UPLOAD_FORM</v>
       </c>
       <c r="B341" t="str">
-        <v>Unable to login due to server error. Please try again later.</v>
+        <v>Please finish the datapack upload form before attempting to upload the file.</v>
       </c>
       <c r="C341" t="str">
-        <v>由于服务器错误无法登陆。请稍后再试。</v>
+        <v>请完成数据包上传表单后再尝试上传文件。</v>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="str">
-        <v>errors.UNABLE_TO_LOGIN_GOOGLE_CREDENTIAL</v>
+        <v>errors.DATAPACK_ALREADY_EXISTS</v>
       </c>
       <c r="B342" t="str">
-        <v>Unable to login with Google credentials. Please try again.</v>
+        <v>Datapack already exists. Please upload a datapack with a unique title.</v>
       </c>
       <c r="C342" t="str">
-        <v>无法使用Google登陆。请稍后再试。</v>
+        <v>数据包已存在。请上传不重名的数据包。</v>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="str">
-        <v>errors.UNABLE_TO_LOGIN_USERNAME_OR_PASSWORD</v>
+        <v>errors.NO_DATAPACKS_SELECTED</v>
       </c>
       <c r="B343" t="str">
-        <v>Invalid username or password. Please try again.</v>
+        <v>No datapacks selected. Please select at least one datapack to generate.</v>
       </c>
       <c r="C343" t="str">
-        <v>无效的用户名或密码。请稍后再试。</v>
+        <v>未选择数据包。请至少选择一个数据包进行绘制。</v>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="str">
-        <v>errors.UNABLE_TO_LOGIN_EXISTING_USER</v>
+        <v>errors.NO_COLUMNS_SELECTED</v>
       </c>
       <c r="B344" t="str">
-        <v>User with that email already exists. Please log in or sign up with a different email.</v>
+        <v>No columns selected. Please select at least one column to generate.</v>
       </c>
       <c r="C344" t="str">
-        <v>已存在使用该电子邮件的用户。请登录或使用其他电子邮件注册。</v>
+        <v>未选择列。请至少选择一个列进行绘制。</v>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="str">
-        <v>errors.UNABLE_TO_LOGOUT</v>
+        <v>errors.IS_BAD_RANGE</v>
       </c>
       <c r="B345" t="str">
-        <v>Unable to logout. Please try again later.</v>
+        <v>Base age must be greater than the top age.</v>
       </c>
       <c r="C345" t="str">
-        <v>无法登出。请稍后再试。</v>
+        <v>区间底部年代应大于区间顶部年代。</v>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="str">
-        <v>errors.UNABLE_TO_SIGNUP_SERVER</v>
+        <v>errors.INVALID_MAPPACK_INFO</v>
       </c>
       <c r="B346" t="str">
-        <v>Unable to sign up due to server error. Please try again later.</v>
+        <v>Invalid mappack info received from server. Please try again later.</v>
       </c>
       <c r="C346" t="str">
-        <v>由于服务器错误无法注册。请稍后再试。</v>
+        <v>从服务器接收到无效的地图包信息。请稍后再试。</v>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="str">
-        <v>errors.UNABLE_TO_SIGNUP_USERNAME_OR_EMAIL</v>
+        <v>errors.UNABLE_TO_LOGIN_SERVER</v>
       </c>
       <c r="B347" t="str">
-        <v>Email or username already exists. Please try again with a different email or username.</v>
+        <v>Unable to login due to server error. Please try again later.</v>
       </c>
       <c r="C347" t="str">
-        <v>电子邮件或用户名已存在。请使用不同的电子邮件或用户名重试。</v>
+        <v>由于服务器错误无法登陆。请稍后再试。</v>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="str">
-        <v>errors.INVALID_FORM</v>
+        <v>errors.UNABLE_TO_LOGIN_GOOGLE_CREDENTIAL</v>
       </c>
       <c r="B348" t="str">
-        <v>Invalid form. Please ensure all fields are filled out correctly.</v>
+        <v>Unable to login with Google credentials. Please try again.</v>
       </c>
       <c r="C348" t="str">
-        <v>表格无效。请确保所有栏目填写正确。</v>
+        <v>无法使用Google登陆。请稍后再试。</v>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="str">
-        <v>errors.UNABLE_TO_VERIFY_ACCOUNT</v>
+        <v>errors.UNABLE_TO_LOGIN_USERNAME_OR_PASSWORD</v>
       </c>
       <c r="B349" t="str">
-        <v>Your email is not verified. Please verify your email first. If you did not receive an email, please resend.</v>
+        <v>Invalid username or password. Please try again.</v>
       </c>
       <c r="C349" t="str">
-        <v>您的电子邮件未经验证。请先验证您的电子邮件。如果您没有收到电子邮件，请重新发送。</v>
+        <v>无效的用户名或密码。请稍后再试。</v>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="str">
-        <v>errors.ALREADY_VERIFIED_ACCOUNT</v>
+        <v>errors.UNABLE_TO_LOGIN_EXISTING_USER</v>
       </c>
       <c r="B350" t="str">
-        <v>Account is already verified. Please log in.</v>
+        <v>User with that email already exists. Please log in or sign up with a different email.</v>
       </c>
       <c r="C350" t="str">
-        <v>帐户已验证。请登录。</v>
+        <v>已存在使用该电子邮件的用户。请登录或使用其他电子邮件注册。</v>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="str">
-        <v>errors.UNABLE_TO_VERIFY_ACCOUNT_SERVER</v>
+        <v>errors.UNABLE_TO_LOGOUT</v>
       </c>
       <c r="B351" t="str">
-        <v>Unable to verify account due to server error. Please try again later.</v>
+        <v>Unable to logout. Please try again later.</v>
       </c>
       <c r="C351" t="str">
-        <v>由于服务器错误，无法验证帐户。请稍后再试。</v>
+        <v>无法登出。请稍后再试。</v>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="str">
-        <v>errors.TOKEN_EXPIRED_OR_INVALID</v>
+        <v>errors.UNABLE_TO_SIGNUP_SERVER</v>
       </c>
       <c r="B352" t="str">
-        <v>Your token is either invalid or has expired. Please request a new verification email.</v>
+        <v>Unable to sign up due to server error. Please try again later.</v>
       </c>
       <c r="C352" t="str">
-        <v>您的令牌无效或已过期。请申请新的验证电子邮件。</v>
+        <v>由于服务器错误无法注册。请稍后再试。</v>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="str">
-        <v>errors.UNABLE_TO_SEND_EMAIL</v>
+        <v>errors.UNABLE_TO_SIGNUP_USERNAME_OR_EMAIL</v>
       </c>
       <c r="B353" t="str">
-        <v>Unable to send email. Please try again later.</v>
+        <v>Email or username already exists. Please try again with a different email or username.</v>
       </c>
       <c r="C353" t="str">
-        <v>无法发送邮件。请稍后再试。</v>
+        <v>电子邮件或用户名已存在。请使用不同的电子邮件或用户名重试。</v>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="str">
-        <v>errors.UNABLE_TO_RESET_PASSWORD</v>
+        <v>errors.INVALID_FORM</v>
       </c>
       <c r="B354" t="str">
-        <v>Unable to reset password. Please try again later.</v>
+        <v>Invalid form. Please ensure all fields are filled out correctly.</v>
       </c>
       <c r="C354" t="str">
-        <v>无法重置密码。请稍后再试。</v>
+        <v>表格无效。请确保所有栏目填写正确。</v>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="str">
-        <v>errors.UNABLE_TO_RESET_EMAIL</v>
+        <v>errors.UNABLE_TO_VERIFY_ACCOUNT</v>
       </c>
       <c r="B355" t="str">
-        <v>Unable to reset email. Please try again later.</v>
+        <v>Your email is not verified. Please verify your email first. If you did not receive an email, please resend.</v>
       </c>
       <c r="C355" t="str">
-        <v>无法重置邮箱。请稍后再试。</v>
+        <v>您的电子邮件未经验证。请先验证您的电子邮件。如果您没有收到电子邮件，请重新发送。</v>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="str">
-        <v>errors.UNABLE_TO_LOGIN_ACCOUNT_LOCKED</v>
+        <v>errors.ALREADY_VERIFIED_ACCOUNT</v>
       </c>
       <c r="B356" t="str">
-        <v>Your account has been locked. Please check your email for more information or contact support.</v>
+        <v>Account is already verified. Please log in.</v>
       </c>
       <c r="C356" t="str">
-        <v>您的账户已被锁定。请查看您的电子邮件以获取更多信息或联系技术支持获得帮助。</v>
+        <v>帐户已验证。请登录。</v>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="str">
-        <v>errors.UNABLE_TO_RECOVER_ACCOUNT</v>
+        <v>errors.UNABLE_TO_VERIFY_ACCOUNT_SERVER</v>
       </c>
       <c r="B357" t="str">
-        <v>Unable to recover account. Please contact support for more information.</v>
+        <v>Unable to verify account due to server error. Please try again later.</v>
       </c>
       <c r="C357" t="str">
-        <v>无法恢复账户。请联系技术支持获取更多信息。</v>
+        <v>由于服务器错误，无法验证帐户。请稍后再试。</v>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="str">
-        <v>errors.NOT_LOGGED_IN</v>
+        <v>errors.TOKEN_EXPIRED_OR_INVALID</v>
       </c>
       <c r="B358" t="str">
-        <v>You are not logged in. Please log in to access this page.</v>
+        <v>Your token is either invalid or has expired. Please request a new verification email.</v>
       </c>
       <c r="C358" t="str">
-        <v>您尚未登录。请登录后访问此页面。</v>
+        <v>您的令牌无效或已过期。请申请新的验证电子邮件。</v>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="str">
-        <v>errors.USER_DATAPACK_FILE_NOT_FOUND_FOR_DOWNLOAD</v>
+        <v>errors.UNABLE_TO_SEND_EMAIL</v>
       </c>
       <c r="B359" t="str">
-        <v>The datapack requested was not found on the server. Please try again later or contact our support team.</v>
+        <v>Unable to send email. Please try again later.</v>
       </c>
       <c r="C359" t="str">
-        <v>服务器上未找到所请求的数据包。请稍后再试，或联系我们的技术支持团队。</v>
+        <v>无法发送邮件。请稍后再试。</v>
       </c>
     </row>
     <row r="360">
       <c r="A360" t="str">
-        <v>errors.INCORRECT_ENCRYPTION_HEADER</v>
+        <v>errors.UNABLE_TO_RESET_PASSWORD</v>
       </c>
       <c r="B360" t="str">
-        <v>Unable to encrypt the file, please try again later.</v>
+        <v>Unable to reset password. Please try again later.</v>
       </c>
       <c r="C360" t="str">
-        <v>无法加密文件。请稍后再试。</v>
+        <v>无法重置密码。请稍后再试。</v>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="str">
-        <v>errors.TOO_MANY_REQUESTS</v>
+        <v>errors.UNABLE_TO_RESET_EMAIL</v>
       </c>
       <c r="B361" t="str">
-        <v>You have made too many requests. Please try again later.</v>
+        <v>Unable to reset email. Please try again later.</v>
       </c>
       <c r="C361" t="str">
-        <v>请求过于频繁。请稍后再试。</v>
+        <v>无法重置邮箱。请稍后再试。</v>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="str">
-        <v>errors.RECAPTCHA_FAILED</v>
+        <v>errors.UNABLE_TO_LOGIN_ACCOUNT_LOCKED</v>
       </c>
       <c r="B362" t="str">
-        <v>Recaptcha failed. Please try again.</v>
+        <v>Your account has been locked. Please check your email for more information or contact support.</v>
       </c>
       <c r="C362" t="str">
-        <v>验证失败. 请稍后再试。</v>
+        <v>您的账户已被锁定。请查看您的电子邮件以获取更多信息或联系技术支持获得帮助。</v>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="str">
-        <v>errors.COOKIE_REJECTED</v>
+        <v>errors.UNABLE_TO_RECOVER_ACCOUNT</v>
       </c>
       <c r="B363" t="str">
-        <v>You must accept cookies to sign in.</v>
+        <v>Unable to recover account. Please contact support for more information.</v>
       </c>
       <c r="C363" t="str">
-        <v>您必须接受 Cookie 才能登录。</v>
+        <v>无法恢复账户。请联系技术支持获取更多信息。</v>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="str">
-        <v>errors.UNRECOGNIZED_IMAGE_FILE</v>
+        <v>errors.NOT_LOGGED_IN</v>
       </c>
       <c r="B364" t="str">
-        <v>Unrecognized image extension. Please upload a valid image file.</v>
+        <v>You are not logged in. Please log in to access this page.</v>
       </c>
       <c r="C364" t="str">
-        <v>图像扩展名无法识别。请上传有效的图像文件。</v>
+        <v>您尚未登录。请登录后访问此页面。</v>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="str">
-        <v>errors.UPLOAD_PROFILE_PICTURE_FAILED</v>
+        <v>errors.USER_DATAPACK_FILE_NOT_FOUND_FOR_DOWNLOAD</v>
       </c>
       <c r="B365" t="str">
-        <v>Unable to upload profile picture. Please try again later.</v>
+        <v>The datapack requested was not found on the server. Please try again later or contact our support team.</v>
       </c>
       <c r="C365" t="str">
-        <v>无法上传个人资料图片。请稍后再试。</v>
+        <v>服务器上未找到所请求的数据包。请稍后再试，或联系我们的技术支持团队。</v>
       </c>
     </row>
     <row r="366">
       <c r="A366" t="str">
-        <v>errors.UNABLE_TO_CHANGE_USERNAME</v>
+        <v>errors.INCORRECT_ENCRYPTION_HEADER</v>
       </c>
       <c r="B366" t="str">
-        <v>Unable to change username. Please try again later.</v>
+        <v>Unable to encrypt the file, please try again later.</v>
       </c>
       <c r="C366" t="str">
-        <v>无法更改用户名。请稍后再试。</v>
+        <v>无法加密文件。请稍后再试。</v>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="str">
-        <v>errors.UNABLE_TO_DELETE_PROFILE</v>
+        <v>errors.TOO_MANY_REQUESTS</v>
       </c>
       <c r="B367" t="str">
-        <v>Unable to delete profile. Please try again later.</v>
+        <v>You have made too many requests. Please try again later.</v>
       </c>
       <c r="C367" t="str">
-        <v>无法删除用户。请稍后再试。</v>
+        <v>请求过于频繁。请稍后再试。</v>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="str">
-        <v>errors.INCORRECT_PASSWORD</v>
+        <v>errors.RECAPTCHA_FAILED</v>
       </c>
       <c r="B368" t="str">
-        <v>Incorrect password. Please try again.</v>
+        <v>Recaptcha failed. Please try again.</v>
       </c>
       <c r="C368" t="str">
-        <v>密码错误。请稍后再试。</v>
+        <v>验证失败. 请稍后再试。</v>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="str">
-        <v>errors.USERNAME_TAKEN</v>
+        <v>errors.COOKIE_REJECTED</v>
       </c>
       <c r="B369" t="str">
-        <v>Username is already taken. Please try a different username.</v>
+        <v>You must accept cookies to sign in.</v>
       </c>
       <c r="C369" t="str">
-        <v>用户名已被使用。请使用一个新的用户名。</v>
+        <v>您必须接受 Cookie 才能登录。</v>
       </c>
     </row>
     <row r="370">
       <c r="A370" t="str">
-        <v>errors.UNABLE_TO_READ_FILE_OR_EMPTY_FILE</v>
+        <v>errors.UNRECOGNIZED_IMAGE_FILE</v>
       </c>
       <c r="B370" t="str">
-        <v>Unable to read file or file is empty. Please try again.</v>
+        <v>Unrecognized image extension. Please upload a valid image file.</v>
       </c>
       <c r="C370" t="str">
-        <v>无法读取文件或文件为空。请稍后再试。</v>
+        <v>图像扩展名无法识别。请上传有效的图像文件。</v>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="str">
-        <v>errors.FETCH_USERS_FAILED</v>
+        <v>errors.UPLOAD_PROFILE_PICTURE_FAILED</v>
       </c>
       <c r="B371" t="str">
-        <v>Unable to fetch users for admin display. Please try again later.</v>
+        <v>Unable to upload profile picture. Please try again later.</v>
       </c>
       <c r="C371" t="str">
-        <v>无法获取用户信息供管理员查阅。请稍后再试。</v>
+        <v>无法上传个人资料图片。请稍后再试。</v>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="str">
-        <v>errors.ADMIN_ADD_USER_FAILED</v>
+        <v>errors.UNABLE_TO_CHANGE_USERNAME</v>
       </c>
       <c r="B372" t="str">
-        <v>Unable to add user. Please try again later.</v>
+        <v>Unable to change username. Please try again later.</v>
       </c>
       <c r="C372" t="str">
-        <v>无法添加用户。请稍后再试。</v>
+        <v>无法更改用户名。请稍后再试。</v>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="str">
-        <v>errors.SERVER_TIMEOUT</v>
+        <v>errors.UNABLE_TO_DELETE_PROFILE</v>
       </c>
       <c r="B373" t="str">
-        <v>Server timed out. Please try again later.</v>
+        <v>Unable to delete profile. Please try again later.</v>
       </c>
       <c r="C373" t="str">
-        <v>服务器超时。请稍后再试。</v>
+        <v>无法删除用户。请稍后再试。</v>
       </c>
     </row>
     <row r="374">
       <c r="A374" t="str">
-        <v>errors.SERVER_BUSY</v>
+        <v>errors.INCORRECT_PASSWORD</v>
       </c>
       <c r="B374" t="str">
-        <v>Server is too busy. Please try again later.</v>
+        <v>Incorrect password. Please try again.</v>
       </c>
       <c r="C374" t="str">
-        <v>服务器忙。请稍后再试。</v>
+        <v>密码错误。请稍后再试。</v>
       </c>
     </row>
     <row r="375">
       <c r="A375" t="str">
-        <v>errors.ADMIN_DELETE_USER_FAILED</v>
+        <v>errors.USERNAME_TAKEN</v>
       </c>
       <c r="B375" t="str">
-        <v>Unable to delete user. Please try again later.</v>
+        <v>Username is already taken. Please try a different username.</v>
       </c>
       <c r="C375" t="str">
-        <v>无法删除用户。请稍后再试。</v>
+        <v>用户名已被使用。请使用一个新的用户名。</v>
       </c>
     </row>
     <row r="376">
       <c r="A376" t="str">
-        <v>errors.UNABLE_TO_FETCH_DATAPACKS</v>
+        <v>errors.UNABLE_TO_READ_FILE_OR_EMPTY_FILE</v>
       </c>
       <c r="B376" t="str">
-        <v>Unable to fetch datapacks. Please try again later.</v>
+        <v>Unable to read file or file is empty. Please try again.</v>
+      </c>
+      <c r="C376" t="str">
+        <v>无法读取文件或文件为空。请稍后再试。</v>
       </c>
     </row>
     <row r="377">
       <c r="A377" t="str">
-        <v>errors.UNABLE_TO_FETCH_USER_DATAPACKS</v>
+        <v>errors.FETCH_USERS_FAILED</v>
       </c>
       <c r="B377" t="str">
-        <v>Unable to fetch user datapacks. Please try again later.</v>
+        <v>Unable to fetch users for admin display. Please try again later.</v>
       </c>
       <c r="C377" t="str">
-        <v>无法获取用户数据包。请稍后再试。</v>
+        <v>无法获取用户信息供管理员查阅。请稍后再试。</v>
       </c>
     </row>
     <row r="378">
       <c r="A378" t="str">
-        <v>errors.CANNOT_DELETE_ROOT_USER</v>
+        <v>errors.ADMIN_ADD_USER_FAILED</v>
       </c>
       <c r="B378" t="str">
-        <v>Cannot delete root user.</v>
+        <v>Unable to add user. Please try again later.</v>
       </c>
       <c r="C378" t="str">
-        <v>不能删除根用户。</v>
+        <v>无法添加用户。请稍后再试。</v>
       </c>
     </row>
     <row r="379">
       <c r="A379" t="str">
-        <v>errors.ADMIN_DELETE_USER_DATAPACK_FAILED</v>
+        <v>errors.SERVER_TIMEOUT</v>
       </c>
       <c r="B379" t="str">
-        <v>Unable to delete user datapack. Please try again later.</v>
+        <v>Server timed out. Please try again later.</v>
       </c>
       <c r="C379" t="str">
-        <v>无法删除用户数据包。请稍后再试。</v>
+        <v>服务器超时。请稍后再试。</v>
       </c>
     </row>
     <row r="380">
       <c r="A380" t="str">
-        <v>errors.ADMIN_DELETE_SERVER_DATAPACK_FAILED</v>
+        <v>errors.SERVER_BUSY</v>
       </c>
       <c r="B380" t="str">
-        <v>Unable to delete server datapack. Please try again later.</v>
+        <v>Server is too busy. Please try again later.</v>
       </c>
       <c r="C380" t="str">
-        <v>无法删除服务器数据包。请稍后再试。</v>
+        <v>服务器忙。请稍后再试。</v>
       </c>
     </row>
     <row r="381">
       <c r="A381" t="str">
-        <v>errors.ADMIN_CANNOT_DELETE_ROOT_DATAPACK</v>
+        <v>errors.ADMIN_DELETE_USER_FAILED</v>
       </c>
       <c r="B381" t="str">
-        <v>Cannot delete root datapack. Ask server admin for assistance.</v>
+        <v>Unable to delete user. Please try again later.</v>
       </c>
       <c r="C381" t="str">
-        <v>无法删除根数据包。请向服务器管理员寻求帮助。</v>
+        <v>无法删除用户。请稍后再试。</v>
       </c>
     </row>
     <row r="382">
       <c r="A382" t="str">
-        <v>errors.INVALID_SERVER_DATAPACK_REQUEST</v>
+        <v>errors.UNABLE_TO_FETCH_DATAPACKS</v>
       </c>
       <c r="B382" t="str">
-        <v>Invalid server datapack request. Please try again later.</v>
-      </c>
-      <c r="C382" t="str">
-        <v>无效的服务器数据包请求。请稍后再试。</v>
+        <v>Unable to fetch datapacks. Please try again later.</v>
       </c>
     </row>
     <row r="383">
       <c r="A383" t="str">
-        <v>errors.SERVER_FILE_METADATA_ERROR</v>
+        <v>errors.UNABLE_TO_FETCH_USER_DATAPACKS</v>
       </c>
       <c r="B383" t="str">
-        <v>Server file metadata error. Please try again later.</v>
+        <v>Unable to fetch user datapacks. Please try again later.</v>
       </c>
       <c r="C383" t="str">
-        <v>服务器文件元数据错误。请稍后再试。</v>
+        <v>无法获取用户数据包。请稍后再试。</v>
       </c>
     </row>
     <row r="384">
       <c r="A384" t="str">
-        <v>errors.USER_DELETE_DATAPACK_FAILED</v>
+        <v>errors.CANNOT_DELETE_ROOT_USER</v>
       </c>
       <c r="B384" t="str">
-        <v>Unable to delete user datapack. Please try again later.</v>
+        <v>Cannot delete root user.</v>
       </c>
       <c r="C384" t="str">
-        <v>无法删除用户数据包。请稍后再试。</v>
+        <v>不能删除根用户。</v>
       </c>
     </row>
     <row r="385">
       <c r="A385" t="str">
-        <v>errors.UNABLE_TO_PROCESS_DATAPACK_CONFIG</v>
+        <v>errors.ADMIN_DELETE_USER_DATAPACK_FAILED</v>
       </c>
       <c r="B385" t="str">
-        <v>Failed to process datapack config. Please try again later.</v>
+        <v>Unable to delete user datapack. Please try again later.</v>
       </c>
       <c r="C385" t="str">
-        <v>处理数据包配置失败。请稍后再试。</v>
+        <v>无法删除用户数据包。请稍后再试。</v>
       </c>
     </row>
     <row r="386">
       <c r="A386" t="str">
-        <v>errors.INVALID_SETTINGS</v>
+        <v>errors.ADMIN_DELETE_SERVER_DATAPACK_FAILED</v>
       </c>
       <c r="B386" t="str">
-        <v>Invalid settings. Please try again.</v>
+        <v>Unable to delete server datapack. Please try again later.</v>
       </c>
       <c r="C386" t="str">
-        <v>无效的设置。请稍后再试。</v>
+        <v>无法删除服务器数据包。请稍后再试。</v>
       </c>
     </row>
     <row r="387">
       <c r="A387" t="str">
-        <v>errors.INTERNAL_ERROR</v>
+        <v>errors.ADMIN_CANNOT_DELETE_ROOT_DATAPACK</v>
       </c>
       <c r="B387" t="str">
-        <v>There was an internal error while generating the chart. Please try again later.</v>
+        <v>Cannot delete root datapack. Ask server admin for assistance.</v>
       </c>
       <c r="C387" t="str">
-        <v>生成图表时出现内部错误。请稍后再试。</v>
+        <v>无法删除根数据包。请向服务器管理员寻求帮助。</v>
       </c>
     </row>
     <row r="388">
       <c r="A388" t="str">
-        <v>errors.ADMIN_ADD_USERS_TO_WORKSHOP_FAILED</v>
+        <v>errors.INVALID_SERVER_DATAPACK_REQUEST</v>
       </c>
       <c r="B388" t="str">
-        <v>Unable to add users to workshop. Please try again later.</v>
+        <v>Invalid server datapack request. Please try again later.</v>
       </c>
       <c r="C388" t="str">
-        <v>无法将用户添加到工作坊。请稍后再试。</v>
+        <v>无效的服务器数据包请求。请稍后再试。</v>
       </c>
     </row>
     <row r="389">
       <c r="A389" t="str">
-        <v>errors.ADMIN_EMAIL_INVALID</v>
+        <v>errors.SERVER_FILE_METADATA_ERROR</v>
       </c>
       <c r="B389" t="str">
-        <v>Invalid email. Please fix the email and try again.</v>
+        <v>Server file metadata error. Please try again later.</v>
       </c>
       <c r="C389" t="str">
-        <v>电子邮件无效。请修复电子邮件并重试。</v>
+        <v>服务器文件元数据错误。请稍后再试。</v>
       </c>
     </row>
     <row r="390">
       <c r="A390" t="str">
-        <v>errors.ADMIN_WORKSHOP_FIELDS_EMPTY</v>
+        <v>errors.USER_DELETE_DATAPACK_FAILED</v>
       </c>
       <c r="B390" t="str">
-        <v>You must provide at least one field to add users to a workshop.</v>
+        <v>Unable to delete user datapack. Please try again later.</v>
       </c>
       <c r="C390" t="str">
-        <v>您必须提供至少一个领域才能将用户添加到工作坊。</v>
+        <v>无法删除用户数据包。请稍后再试。</v>
       </c>
     </row>
     <row r="391">
       <c r="A391" t="str">
-        <v>errors.UNRECOGNIZED_EXCEL_FILE</v>
+        <v>errors.UNABLE_TO_PROCESS_DATAPACK_CONFIG</v>
       </c>
       <c r="B391" t="str">
-        <v>Unrecognized Excel file. Please upload a valid Excel file.</v>
+        <v>Failed to process datapack config. Please try again later.</v>
       </c>
       <c r="C391" t="str">
-        <v>无法识别 Excel 文件。请上传有效的 Excel 文件。</v>
+        <v>处理数据包配置失败。请稍后再试。</v>
       </c>
     </row>
     <row r="392">
       <c r="A392" t="str">
-        <v>errors.SERVER_DATAPACK_ALREADY_EXISTS</v>
+        <v>errors.INVALID_SETTINGS</v>
       </c>
       <c r="B392" t="str">
-        <v>Server datapack already exists. Please upload a unique datapack (different title).</v>
+        <v>Invalid settings. Please try again.</v>
       </c>
       <c r="C392" t="str">
-        <v>服务器数据包已存在。请上传一个独特的数据包（不同的文件名）。</v>
+        <v>无效的设置。请稍后再试。</v>
       </c>
     </row>
     <row r="393">
       <c r="A393" t="str">
-        <v>errors.ADMIN_WORKSHOP_START_AFTER_END</v>
+        <v>errors.INTERNAL_ERROR</v>
       </c>
       <c r="B393" t="str">
-        <v>The start date must be before the end date.</v>
+        <v>There was an internal error while generating the chart. Please try again later.</v>
       </c>
       <c r="C393" t="str">
-        <v>开始日期必须早于结束日期</v>
+        <v>生成图表时出现内部错误。请稍后再试。</v>
       </c>
     </row>
     <row r="394">
       <c r="A394" t="str">
-        <v>errors.ADMIN_CREATE_WORKSHOP_FAILED</v>
+        <v>errors.ADMIN_ADD_USERS_TO_WORKSHOP_FAILED</v>
       </c>
       <c r="B394" t="str">
-        <v>Unable to create workshop. Please try again later.</v>
+        <v>Unable to add users to workshop. Please try again later.</v>
       </c>
       <c r="C394" t="str">
-        <v>无法创建工作坊。请稍后再试。</v>
+        <v>无法将用户添加到工作坊。请稍后再试。</v>
       </c>
     </row>
     <row r="395">
       <c r="A395" t="str">
-        <v>errors.ADMIN_WORKSHOP_ALREADY_EXISTS</v>
+        <v>errors.ADMIN_EMAIL_INVALID</v>
       </c>
       <c r="B395" t="str">
-        <v>Workshop with that title and dates already exists. Please try again.</v>
+        <v>Invalid email. Please fix the email and try again.</v>
       </c>
       <c r="C395" t="str">
-        <v>该工作坊名称已存在。请另选名称。</v>
+        <v>电子邮件无效。请修复电子邮件并重试。</v>
       </c>
     </row>
     <row r="396">
       <c r="A396" t="str">
-        <v>errors.ADMIN_FETCH_WORKSHOPS_FAILED</v>
+        <v>errors.ADMIN_WORKSHOP_FIELDS_EMPTY</v>
       </c>
       <c r="B396" t="str">
-        <v>Unable to fetch workshops. Please try again later.</v>
+        <v>You must provide at least one field to add users to a workshop.</v>
       </c>
       <c r="C396" t="str">
-        <v>无法抓取工作坊。请稍后再试。</v>
+        <v>您必须提供至少一个领域才能将用户添加到工作坊。</v>
       </c>
     </row>
     <row r="397">
       <c r="A397" t="str">
-        <v>errors.ADMIN_DELETE_WORKSHOP_FAILED</v>
+        <v>errors.UNRECOGNIZED_EXCEL_FILE</v>
       </c>
       <c r="B397" t="str">
-        <v>Unable to delete workshop. Please try again later.</v>
+        <v>Unrecognized Excel file. Please upload a valid Excel file.</v>
+      </c>
+      <c r="C397" t="str">
+        <v>无法识别 Excel 文件。请上传有效的 Excel 文件。</v>
       </c>
     </row>
     <row r="398">
       <c r="A398" t="str">
-        <v>errors.ADMIN_WORKSHOP_NOT_FOUND</v>
+        <v>errors.SERVER_DATAPACK_ALREADY_EXISTS</v>
       </c>
       <c r="B398" t="str">
-        <v>Workshop not found on server, it has likely ended or been deleted.</v>
+        <v>Server datapack already exists. Please upload a unique datapack (different title).</v>
       </c>
       <c r="C398" t="str">
-        <v>服务器未找到工作坊。该工作坊可能已结束或被删除。</v>
+        <v>服务器数据包已存在。请上传一个独特的数据包（不同的文件名）。</v>
       </c>
     </row>
     <row r="399">
       <c r="A399" t="str">
-        <v>errors.ADMIN_WORKSHOP_EDIT_FAILED</v>
+        <v>errors.ADMIN_WORKSHOP_START_AFTER_END</v>
       </c>
       <c r="B399" t="str">
-        <v>Unable to edit workshop. Please try again later.</v>
+        <v>The start date must be before the end date.</v>
+      </c>
+      <c r="C399" t="str">
+        <v>开始日期必须早于结束日期</v>
       </c>
     </row>
     <row r="400">
       <c r="A400" t="str">
-        <v>errors.USER_EDIT_DATAPACK_FAILED</v>
+        <v>errors.ADMIN_CREATE_WORKSHOP_FAILED</v>
       </c>
       <c r="B400" t="str">
-        <v>Failed to edit user datapack. Please try again later.</v>
+        <v>Unable to create workshop. Please try again later.</v>
+      </c>
+      <c r="C400" t="str">
+        <v>无法创建工作坊。请稍后再试。</v>
       </c>
     </row>
     <row r="401">
       <c r="A401" t="str">
-        <v>errors.USER_FETCH_DATAPACK_FAILED</v>
+        <v>errors.ADMIN_WORKSHOP_ALREADY_EXISTS</v>
       </c>
       <c r="B401" t="str">
-        <v>Failed to fetch user datapack. Please try again later.</v>
+        <v>Workshop with that title and dates already exists. Please try again.</v>
+      </c>
+      <c r="C401" t="str">
+        <v>该工作坊名称已存在。请另选名称。</v>
       </c>
     </row>
     <row r="402">
       <c r="A402" t="str">
-        <v>errors.USER_REPLACE_DATAPACK_FILE_FAILED</v>
+        <v>errors.ADMIN_FETCH_WORKSHOPS_FAILED</v>
       </c>
       <c r="B402" t="str">
-        <v>Failed to replace user datapack file. Please try again later.</v>
+        <v>Unable to fetch workshops. Please try again later.</v>
+      </c>
+      <c r="C402" t="str">
+        <v>无法抓取工作坊。请稍后再试。</v>
       </c>
     </row>
     <row r="403">
       <c r="A403" t="str">
-        <v>errors.USER_REPLACE_DATAPACK_PROFILE_IMAGE_FAILED</v>
+        <v>errors.ADMIN_DELETE_WORKSHOP_FAILED</v>
       </c>
       <c r="B403" t="str">
-        <v>Failed to replace user datapack profile image. Please try again later.</v>
+        <v>Unable to delete workshop. Please try again later.</v>
       </c>
     </row>
     <row r="404">
       <c r="A404" t="str">
-        <v>errors.DATAPACK_TITLE_LEADING_TRAILING_WHITESPACE</v>
+        <v>errors.ADMIN_WORKSHOP_NOT_FOUND</v>
       </c>
       <c r="B404" t="str">
-        <v>Datapack title cannot have leading or trailing whitespace.</v>
+        <v>Workshop not found on server, it has likely ended or been deleted.</v>
+      </c>
+      <c r="C404" t="str">
+        <v>服务器未找到工作坊。该工作坊可能已结束或被删除。</v>
       </c>
     </row>
     <row r="405">
       <c r="A405" t="str">
-        <v>errors.ADMIN_FETCH_PRIVATE_DATAPACKS_FAILED</v>
+        <v>errors.ADMIN_WORKSHOP_EDIT_FAILED</v>
       </c>
       <c r="B405" t="str">
-        <v>Failed to fetch private datapacks. Please try again later.</v>
+        <v>Unable to edit workshop. Please try again later.</v>
       </c>
     </row>
     <row r="406">
       <c r="A406" t="str">
-        <v>errors.ADMIN_PRIORITY_BATCH_UPDATE_FAILED</v>
+        <v>errors.USER_EDIT_DATAPACK_FAILED</v>
       </c>
       <c r="B406" t="str">
-        <v>Failed to update datapack priorities. Please contact a server admin for assistance.</v>
+        <v>Failed to edit user datapack. Please try again later.</v>
       </c>
     </row>
     <row r="407">
       <c r="A407" t="str">
-        <v>errors.ADMIN_ADD_OFFICIAL_DATAPACK_TO_WORKSHOP_FAILED</v>
+        <v>errors.USER_FETCH_DATAPACK_FAILED</v>
       </c>
       <c r="B407" t="str">
-        <v>Failed to add official datapack to workshop. Please try again later.</v>
+        <v>Failed to fetch user datapack. Please try again later.</v>
       </c>
     </row>
     <row r="408">
       <c r="A408" t="str">
-        <v>errors.ADMIN_SERVER_DATAPACK_ALREADY_EXISTS</v>
+        <v>errors.USER_REPLACE_DATAPACK_FILE_FAILED</v>
       </c>
       <c r="B408" t="str">
-        <v>Server datapack already exists in workshop. Please choose a different datapack.</v>
+        <v>Failed to replace user datapack file. Please try again later.</v>
       </c>
     </row>
     <row r="409">
       <c r="A409" t="str">
-        <v>errors.ADMIN_WORKSHOP_ENDED</v>
+        <v>errors.USER_REPLACE_DATAPACK_PROFILE_IMAGE_FAILED</v>
       </c>
       <c r="B409" t="str">
-        <v>Workshop has ended. You can no longer edit or add datapacks to it.</v>
+        <v>Failed to replace user datapack profile image. Please try again later.</v>
       </c>
     </row>
     <row r="410">
       <c r="A410" t="str">
-        <v>errors.WORKSHOP_FETCH_DATAPACK_FAILED</v>
+        <v>errors.DATAPACK_TITLE_LEADING_TRAILING_WHITESPACE</v>
       </c>
       <c r="B410" t="str">
-        <v>Failed to fetch workshop datapacks. Please try again later.</v>
+        <v>Datapack title cannot have leading or trailing whitespace.</v>
       </c>
     </row>
     <row r="411">
       <c r="A411" t="str">
-        <v>errors.METADATA_NOT_FOUND</v>
+        <v>errors.ADMIN_FETCH_PRIVATE_DATAPACKS_FAILED</v>
       </c>
       <c r="B411" t="str">
-        <v>Metadata not found. Please try again later.</v>
+        <v>Failed to fetch private datapacks. Please try again later.</v>
       </c>
     </row>
     <row r="412">
       <c r="A412" t="str">
-        <v>errors.INVALID_CROSSPLOT_CONVERSION</v>
+        <v>errors.ADMIN_PRIORITY_BATCH_UPDATE_FAILED</v>
       </c>
       <c r="B412" t="str">
-        <v>Invalid crossplot conversion. Please select a valid chart for the Y Axis.</v>
+        <v>Failed to update datapack priorities. Please contact a server admin for assistance.</v>
       </c>
     </row>
     <row r="413">
       <c r="A413" t="str">
-        <v>errors.INVALID_CROSSPLOT_UNITS</v>
+        <v>errors.ADMIN_ADD_OFFICIAL_DATAPACK_TO_WORKSHOP_FAILED</v>
       </c>
       <c r="B413" t="str">
-        <v>Please select a different unit for the Y Axis. This unit cannot be converted.</v>
+        <v>Failed to add official datapack to workshop. Please try again later.</v>
       </c>
     </row>
     <row r="414">
       <c r="A414" t="str">
-        <v>errors.CROSSPLOT_CONVERSION_FAILED</v>
+        <v>errors.ADMIN_SERVER_DATAPACK_ALREADY_EXISTS</v>
       </c>
       <c r="B414" t="str">
-        <v>Crossplot conversion failed. Please try again later.</v>
+        <v>Server datapack already exists in workshop. Please choose a different datapack.</v>
       </c>
     </row>
     <row r="415">
       <c r="A415" t="str">
-        <v>errors.NO_MODELS</v>
+        <v>errors.ADMIN_WORKSHOP_ENDED</v>
       </c>
       <c r="B415" t="str">
-        <v>No models available. Please add a model by clicking the chart in the main view.</v>
+        <v>Workshop has ended. You can no longer edit or add datapacks to it.</v>
       </c>
     </row>
     <row r="416">
       <c r="A416" t="str">
-        <v>errors.CROSSPLOT_SETTINGS_MISMATCH</v>
+        <v>errors.WORKSHOP_FETCH_DATAPACK_FAILED</v>
       </c>
       <c r="B416" t="str">
-        <v>Crossplot settings mismatch. Please generate the crossplot with your most recent changes.</v>
+        <v>Failed to fetch workshop datapacks. Please try again later.</v>
       </c>
     </row>
     <row r="417">
       <c r="A417" t="str">
-        <v>button.generate</v>
+        <v>errors.METADATA_NOT_FOUND</v>
       </c>
       <c r="B417" t="str">
-        <v>Generate</v>
-      </c>
-      <c r="C417" t="str">
-        <v>绘制</v>
+        <v>Metadata not found. Please try again later.</v>
       </c>
     </row>
     <row r="418">
       <c r="A418" t="str">
-        <v>button.generate-chart</v>
+        <v>errors.INVALID_CROSSPLOT_CONVERSION</v>
       </c>
       <c r="B418" t="str">
-        <v>Generate Chart</v>
-      </c>
-      <c r="C418" t="str">
-        <v>绘制图表</v>
+        <v>Invalid crossplot conversion. Please select a valid chart for the Y Axis.</v>
       </c>
     </row>
     <row r="419">
       <c r="A419" t="str">
-        <v>button.remove-cache</v>
+        <v>errors.INVALID_CROSSPLOT_UNITS</v>
       </c>
       <c r="B419" t="str">
-        <v>Remove Cache</v>
-      </c>
-      <c r="C419" t="str">
-        <v>清除缓存</v>
+        <v>Please select a different unit for the Y Axis. This unit cannot be converted.</v>
       </c>
     </row>
     <row r="420">
       <c r="A420" t="str">
-        <v>button.confirm-selection</v>
+        <v>errors.CROSSPLOT_CONVERSION_FAILED</v>
       </c>
       <c r="B420" t="str">
-        <v>Confirm Selection</v>
-      </c>
-      <c r="C420" t="str">
-        <v>确认选择</v>
+        <v>Crossplot conversion failed. Please try again later.</v>
       </c>
     </row>
     <row r="421">
       <c r="A421" t="str">
-        <v>button.generate-cross-plot</v>
+        <v>errors.NO_MODELS</v>
       </c>
       <c r="B421" t="str">
-        <v>Generate Cross Plot</v>
+        <v>No models available. Please add a model by clicking the chart in the main view.</v>
       </c>
     </row>
     <row r="422">
       <c r="A422" t="str">
-        <v>yes</v>
+        <v>errors.CROSSPLOT_SETTINGS_MISMATCH</v>
       </c>
       <c r="B422" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="C422" t="str">
-        <v>是</v>
+        <v>Crossplot settings mismatch. Please generate the crossplot with your most recent changes.</v>
       </c>
     </row>
     <row r="423">
       <c r="A423" t="str">
-        <v>no</v>
+        <v>button.generate</v>
       </c>
       <c r="B423" t="str">
-        <v>No</v>
+        <v>Generate</v>
       </c>
       <c r="C423" t="str">
-        <v>否</v>
+        <v>绘制</v>
       </c>
     </row>
     <row r="424">
       <c r="A424" t="str">
-        <v>languageNames.en-US</v>
+        <v>button.generate-chart</v>
       </c>
       <c r="B424" t="str">
-        <v>English</v>
+        <v>Generate Chart</v>
+      </c>
+      <c r="C424" t="str">
+        <v>绘制图表</v>
       </c>
     </row>
     <row r="425">
       <c r="A425" t="str">
-        <v>languageNames.en</v>
+        <v>button.remove-cache</v>
       </c>
       <c r="B425" t="str">
-        <v>English</v>
+        <v>Remove Cache</v>
+      </c>
+      <c r="C425" t="str">
+        <v>清除缓存</v>
       </c>
     </row>
     <row r="426">
       <c r="A426" t="str">
-        <v>languageNames.zh</v>
+        <v>button.confirm-selection</v>
       </c>
       <c r="B426" t="str">
-        <v>中文</v>
+        <v>Confirm Selection</v>
+      </c>
+      <c r="C426" t="str">
+        <v>确认选择</v>
       </c>
     </row>
     <row r="427">
       <c r="A427" t="str">
-        <v>tours.quit</v>
+        <v>button.generate-cross-plot</v>
       </c>
       <c r="B427" t="str">
-        <v>Quit Tour</v>
-      </c>
-      <c r="C427" t="str">
-        <v>退出导览</v>
+        <v>Generate Cross Plot</v>
       </c>
     </row>
     <row r="428">
       <c r="A428" t="str">
-        <v>tours.finish</v>
+        <v>yes</v>
       </c>
       <c r="B428" t="str">
-        <v>Finish Tour</v>
+        <v>Yes</v>
       </c>
       <c r="C428" t="str">
-        <v>结束导览</v>
+        <v>是</v>
       </c>
     </row>
     <row r="429">
       <c r="A429" t="str">
-        <v>tours.next</v>
+        <v>no</v>
       </c>
       <c r="B429" t="str">
-        <v>Next</v>
+        <v>No</v>
       </c>
       <c r="C429" t="str">
-        <v>下一步</v>
+        <v>否</v>
       </c>
     </row>
     <row r="430">
       <c r="A430" t="str">
-        <v>tours.back</v>
+        <v>languageNames.en-US</v>
       </c>
       <c r="B430" t="str">
-        <v>Back</v>
-      </c>
-      <c r="C430" t="str">
-        <v>上一步</v>
+        <v>English</v>
       </c>
     </row>
     <row r="431">
       <c r="A431" t="str">
-        <v>tours.qsg.step1</v>
+        <v>languageNames.en</v>
       </c>
       <c r="B431" t="str">
-        <v>In the Presets page, we offer pre-configured settings that allow you to rapidly generate specific types of charts without configuring all options from the beginning. Each preset comes equipped with designated data packs, visual styles, and settings, enabling you to create charts with just a single click.</v>
-      </c>
-      <c r="C431" t="str">
-        <v>在预设页面中，我们提供了预设置，允许您快速生成特定类型的图表，无需从头开始配置所有选项。每个预设都配备了指定的数据包、视觉样式和设置，使您能够一键创建图表</v>
+        <v>English</v>
       </c>
     </row>
     <row r="432">
       <c r="A432" t="str">
-        <v>tours.qsg.step2</v>
+        <v>languageNames.zh</v>
       </c>
       <c r="B432" t="str">
-        <v>In the Datapacks page, you can select the datapacks required to generate your charts. We offer nine official data packs, each containing a curated collection of datasets tailored for specific thematic explorations. For more detailed guidance on Datapacks, please refer to the Datapacks Tour under the "Tours" section</v>
-      </c>
-      <c r="C432" t="str">
-        <v>在数据包页面，您可以选择生成图表所需的数据包。我们提供九个官方数据包，每个数据包都包含为特定主题探索量身定制的数据集合集。如需更详细的数据包指导，请参考“导览”部分下的数据包导览。</v>
+        <v>中文</v>
       </c>
     </row>
     <row r="433">
       <c r="A433" t="str">
-        <v>tours.qsg.step3</v>
+        <v>tours.quit</v>
       </c>
       <c r="B433" t="str">
-        <v>In the Chart page, you can view the charts you have created and explore the detailed visualizations of geologic events. Additionally, you have the option to download and save these charts for your reference or further analysis.</v>
+        <v>Quit Tour</v>
       </c>
       <c r="C433" t="str">
-        <v>在图表页面，您可以查看已创建的图表并探索地质事件的详细可视化图。此外，您还可以下载并保存这些图表以供参考或进一步分析。</v>
+        <v>退出导览</v>
       </c>
     </row>
     <row r="434">
       <c r="A434" t="str">
-        <v>tours.qsg.step4</v>
+        <v>tours.finish</v>
       </c>
       <c r="B434" t="str">
-        <v>In the Settings page, you can customize all aspects of your charts. This includes adjusting the scale and time range, selecting which rows to display, setting the background color and font style, etc. Tailor your charts to meet your specific needs and preferences to optimize your visual analysis. For more detailed guidance on Settings, please refer to the Settings Tour under the "Tours" section</v>
+        <v>Finish Tour</v>
       </c>
       <c r="C434" t="str">
-        <v>在设置页面，您可以自定义图表的所有方面。这包括调整比例和时间范围、选择显示哪些行、设置背景色和字体样式等。根据您的具体需求和偏好调整图表，以优化您的视觉分析。如需更详细的设置指导，请参考“导览”部分下的设置导览。</v>
+        <v>结束导览</v>
       </c>
     </row>
     <row r="435">
       <c r="A435" t="str">
-        <v>tours.qsg.step5</v>
+        <v>tours.next</v>
       </c>
       <c r="B435" t="str">
-        <v>In the Help Page, you can find detailed assistance and information on how to use the website.</v>
+        <v>Next</v>
       </c>
       <c r="C435" t="str">
-        <v>在帮助页面，您可以找到关于如何使用网站的详细帮助和信息。</v>
+        <v>下一步</v>
       </c>
     </row>
     <row r="436">
       <c r="A436" t="str">
-        <v>tours.qsg.step6</v>
+        <v>tours.back</v>
       </c>
       <c r="B436" t="str">
-        <v>In the Workshops Page, you can access a range of educational and experimental tutorials that offer in-depth guidance. Here, you can explore the workshops you have registered for, allowing you to engage with the content and enhance your skills in a hands-on learning environment.</v>
+        <v>Back</v>
       </c>
       <c r="C436" t="str">
-        <v>在工作坊页面，您可以访问一系列提供深入指导的教育和实验教程。在这里，您可以探索已注册的研讨会，通过亲身实践的学习环境来提升您的技能。</v>
+        <v>上一步</v>
       </c>
     </row>
     <row r="437">
       <c r="A437" t="str">
-        <v>tours.qsg.step7</v>
+        <v>tours.qsg.step1</v>
       </c>
       <c r="B437" t="str">
-        <v>The About Page provides information about our development team.</v>
+        <v>In the Presets page, we offer pre-configured settings that allow you to rapidly generate specific types of charts without configuring all options from the beginning. Each preset comes equipped with designated data packs, visual styles, and settings, enabling you to create charts with just a single click.</v>
       </c>
       <c r="C437" t="str">
-        <v>关于页面提供了我们开发团队的信息。</v>
+        <v>在预设页面中，我们提供了预设置，允许您快速生成特定类型的图表，无需从头开始配置所有选项。每个预设都配备了指定的数据包、视觉样式和设置，使您能够一键创建图表</v>
       </c>
     </row>
     <row r="438">
       <c r="A438" t="str">
-        <v>tours.qsg.step8</v>
+        <v>tours.qsg.step2</v>
       </c>
       <c r="B438" t="str">
-        <v>Click here to sign in and unlock the features mentioned earlier, such as accessing registered workshops. Once logged in, you will also have the ability to upload datapacks and take full advantage of all functionalities.</v>
+        <v>In the Datapacks page, you can select the datapacks required to generate your charts. We offer nine official data packs, each containing a curated collection of datasets tailored for specific thematic explorations. For more detailed guidance on Datapacks, please refer to the Datapacks Tour under the "Tours" section</v>
       </c>
       <c r="C438" t="str">
-        <v>点击此处登录并解锁前面提到的功能，例如访问工作坊界面。登陆后，您还将能够上传数据包并充分利用所有功能。</v>
+        <v>在数据包页面，您可以选择生成图表所需的数据包。我们提供九个官方数据包，每个数据包都包含为特定主题探索量身定制的数据集合集。如需更详细的数据包指导，请参考“导览”部分下的数据包导览。</v>
       </c>
     </row>
     <row r="439">
       <c r="A439" t="str">
-        <v>tours.datapack.step1</v>
+        <v>tours.qsg.step3</v>
       </c>
       <c r="B439" t="str">
-        <v>Switch between different display types for datapacks: rows, cards, or compact view.</v>
+        <v>In the Chart page, you can view the charts you have created and explore the detailed visualizations of geologic events. Additionally, you have the option to download and save these charts for your reference or further analysis.</v>
       </c>
       <c r="C439" t="str">
-        <v>在数据包显示类型之间切换：行视图、卡片视图或紧凑视图。</v>
+        <v>在图表页面，您可以查看已创建的图表并探索地质事件的详细可视化图。此外，您还可以下载并保存这些图表以供参考或进一步分析。</v>
       </c>
     </row>
     <row r="440">
       <c r="A440" t="str">
-        <v>tours.datapack.step2</v>
+        <v>tours.qsg.step4</v>
       </c>
       <c r="B440" t="str">
-        <v>Add a datapack by clicking the checkbox</v>
+        <v>In the Settings page, you can customize all aspects of your charts. This includes adjusting the scale and time range, selecting which rows to display, setting the background color and font style, etc. Tailor your charts to meet your specific needs and preferences to optimize your visual analysis. For more detailed guidance on Settings, please refer to the Settings Tour under the "Tours" section</v>
       </c>
       <c r="C440" t="str">
-        <v>勾选添加您想要的数据包</v>
+        <v>在设置页面，您可以自定义图表的所有方面。这包括调整比例和时间范围、选择显示哪些行、设置背景色和字体样式等。根据您的具体需求和偏好调整图表，以优化您的视觉分析。如需更详细的设置指导，请参考“导览”部分下的设置导览。</v>
       </c>
     </row>
     <row r="441">
       <c r="A441" t="str">
-        <v>tours.datapack.step3</v>
+        <v>tours.qsg.step5</v>
       </c>
       <c r="B441" t="str">
-        <v>Click the deselect icon to deselect all datapacks</v>
+        <v>In the Help Page, you can find detailed assistance and information on how to use the website.</v>
       </c>
       <c r="C441" t="str">
-        <v>点此取消选择所有数据包</v>
+        <v>在帮助页面，您可以找到关于如何使用网站的详细帮助和信息。</v>
       </c>
     </row>
     <row r="442">
       <c r="A442" t="str">
-        <v>tours.datapack.step4</v>
+        <v>tours.qsg.step6</v>
       </c>
       <c r="B442" t="str">
-        <v>Remember to confirm your selection</v>
+        <v>In the Workshops Page, you can access a range of educational and experimental tutorials that offer in-depth guidance. Here, you can explore the workshops you have registered for, allowing you to engage with the content and enhance your skills in a hands-on learning environment.</v>
       </c>
       <c r="C442" t="str">
-        <v>记得确认您的选择</v>
+        <v>在工作坊页面，您可以访问一系列提供深入指导的教育和实验教程。在这里，您可以探索已注册的研讨会，通过亲身实践的学习环境来提升您的技能。</v>
       </c>
     </row>
     <row r="443">
       <c r="A443" t="str">
-        <v>tours.settings.step1</v>
+        <v>tours.qsg.step7</v>
       </c>
       <c r="B443" t="str">
-        <v>In the Time settings, you can Set the "Top of Interval" and "Base of Interval" for your data. These fields allow you to define the starting and ending ages or stages, which can be adjusted by entering values or using the dropdown selectors. Adjust the vertical scale to change how much vertical space each million years occupies on your charts. For example, setting it higher will spread the intervals further apart, making each period easier to examine closely.</v>
+        <v>The About Page provides information about our development team.</v>
       </c>
       <c r="C443" t="str">
-        <v>在时间设置中，您可以为您的数据设置“时间段顶部”和“时间段底部”。调整这两个值将改变图表的时间跨度，您可以通过输入值或使用下拉选择器进行调整。您还可以调整垂直比例，以改变图表中每百万年占据的垂直空间量。例如，将其设置得更高将使时间间隔进一步分开，使每个时期更易于仔细检查。</v>
+        <v>关于页面提供了我们开发团队的信息。</v>
       </c>
     </row>
     <row r="444">
       <c r="A444" t="str">
-        <v>tours.settings.step2</v>
+        <v>tours.qsg.step8</v>
       </c>
       <c r="B444" t="str">
-        <v>In the Preferences settings, you can customize the display options. For instance, you may choose to gray out columns with no data for selected time periods, add tooltips for additional information, or enable filtering and legend options for charts. Furthermore, you can load your settings from a file or save your current settings to a file. This feature is useful for backing up your configurations, sharing them with others, or quickly applying previously saved configurations to your chart.</v>
+        <v>Click here to sign in and unlock the features mentioned earlier, such as accessing registered workshops. Once logged in, you will also have the ability to upload datapacks and take full advantage of all functionalities.</v>
       </c>
       <c r="C444" t="str">
-        <v>在偏好中，您可以自定义显示选项。例如，您可以选择在选定时间段内将无数据的列显示为灰色，添加工具提示以提供额外信息，或启用图表的筛选和图例选项。此外，您可以从文件加载您的设置或将当前设置保存到文件中。此功能使您可以备份设置、与他人分享或快速应用以前保存的设置到您的图表中。</v>
+        <v>点击此处登录并解锁前面提到的功能，例如访问工作坊界面。登陆后，您还将能够上传数据包并充分利用所有功能。</v>
       </c>
     </row>
     <row r="445">
       <c r="A445" t="str">
-        <v>tours.settings.step3</v>
+        <v>tours.datapack.step1</v>
       </c>
       <c r="B445" t="str">
-        <v>In Column Settings, you can deeply customize the appearance and organization of your charts.In the "Column Customization" area, you can adjust titles and shift row positions to streamline how data is displayed on your charts. Enable or disable specific elements like the chart title and Ma markers to suit your presentation needs. In the "Font Options" section, refine the appearance of your charts by choosing different fonts, sizes, and styles for headers and labels, ensuring important data stands out or meets formatting requirements. Please note that the advanced settings for columns can vary depending on the datapack you are working with, allowing for tailored configurations that best fit the data characteristics.</v>
+        <v>Switch between different display types for datapacks: rows, cards, or compact view.</v>
       </c>
       <c r="C445" t="str">
-        <v>在列设置中，您可以深度自定义图表的外观和组织。在“列自定义”区域，您可以调整标题和移动行位置，以简化图表上数据的显示方式。根据您的展示需求启用或禁用特定元素，如图表标题和百万年标记。在“字体选项”部分，通过选择不同的字体、大小和样式为标题和标签，细化您的图表外观，确保重要数据突出显示或符合格式要求。请注意，列高级设置可能根据您正在使用的数据包而有所不同，每个数据包都有最适合数据特性的列高级设置。</v>
+        <v>在数据包显示类型之间切换：行视图、卡片视图或紧凑视图。</v>
       </c>
     </row>
     <row r="446">
       <c r="A446" t="str">
-        <v>tours.settings.step4</v>
+        <v>tours.datapack.step2</v>
       </c>
       <c r="B446" t="str">
-        <v>In the Search Settings, you can quickly locate specific columns by entering keywords and then directly add them to your chart. Simply enter a term related to the setting you are looking for, and the system will display all relevant results.This feature is particularly useful when managing numerous data points or when you need to make quick adjustments without browsing through extensive lists.</v>
+        <v>Add a datapack by clicking the checkbox</v>
       </c>
       <c r="C446" t="str">
-        <v>在搜索中，您可以通过输入关键词快速定位特定列，然后直接将其添加到您的图表中。只需输入一个与您正在寻找的设置相关的词语，系统便会显示所有相关结果。此功能可以帮助您管理众多数据点，或进行快速调整而无需浏览繁杂列表。请注意目前只支持英文搜索。</v>
+        <v>勾选添加您想要的数据包</v>
       </c>
     </row>
     <row r="447">
       <c r="A447" t="str">
-        <v>tours.settings.step5</v>
+        <v>tours.datapack.step3</v>
       </c>
       <c r="B447" t="str">
-        <v>The Font Settings section allows you to customize the appearance of text within your charts. You can adjust font styles, sizes, and formatting for various elements such as column headers, age labels, and more. Each setting is inheritable, ensuring consistency across related elements unless specified otherwise. Changing a font setting here applies it system-wide, but you can override these for individual columns by using the "Change Font" option within each columns settings.Experiment with different fonts and sizes to enhance readability and visual appeal of your charts.</v>
+        <v>Click the deselect icon to deselect all datapacks</v>
       </c>
       <c r="C447" t="str">
-        <v>在字体设置中您可以自定义图表内的文本外观。您可以为各种元素如列标题、年龄标签等调整字体样式、大小和格式。每项设置都是可继承的，确保相关元素间的一致性，除非另行设置。在这里更改字体设置将系统范围内应用，但您可以使用每个列设置中的“更改字体”选项覆盖这些设置。尝试不同的字体和大小，以增强图表的可读性和视觉吸引力。</v>
+        <v>点此取消选择所有数据包</v>
       </c>
     </row>
     <row r="448">
       <c r="A448" t="str">
-        <v>tours.settings.step6</v>
+        <v>tours.datapack.step4</v>
       </c>
       <c r="B448" t="str">
-        <v>In the Map Points Settings, you can access and manage geographic data points for different locations. This feature allows you to view specific location details directly on the interactive map. You can toggle different map layers and visualize data points with detailed descriptions, like latitude, longitude, and additional notes. Please note, however, that not all datapacks contain map points.</v>
+        <v>Remember to confirm your selection</v>
       </c>
       <c r="C448" t="str">
-        <v>在地图点设置中，您可以访问和管理不同位置的地理数据点。此功能允许您直接在交互式地图上查看特定位置的详细信息。您可以切换不同的地图层，并用详细描述（如纬度、经度和附加说明）可视化数据点。请注意，并非所有数据包都包含地图点。</v>
+        <v>记得确认您的选择</v>
       </c>
     </row>
     <row r="449">
       <c r="A449" t="str">
-        <v>tours.settings.step7</v>
+        <v>tours.settings.step1</v>
       </c>
       <c r="B449" t="str">
-        <v>In the Datapacks Settings, you can select the datapacks you wish to use for generating charts. We offer nine official datapacks, each comprising a curated collection of datasets tailored for specific thematic explorations. You might notice that this page resembles the Datapack page; selections can be configured here or there interchangeably. For more detailed guidance on how to utilize datapacks, please refer to the Datapacks Tour in the Help page "Tours" section.</v>
+        <v>In the Time settings, you can Set the "Top of Interval" and "Base of Interval" for your data. These fields allow you to define the starting and ending ages or stages, which can be adjusted by entering values or using the dropdown selectors. Adjust the vertical scale to change how much vertical space each million years occupies on your charts. For example, setting it higher will spread the intervals further apart, making each period easier to examine closely.</v>
       </c>
       <c r="C449" t="str">
-        <v>在数据包设置中，您可以选择您希望用于生成图表的数据包。我们提供九个官方数据包，每个数据包都包含为特定主题探索量身定制的数据集合。您也许已经注意到，此页面与"数据包"页面内容相同；您在两个地方都可以进行选择和设置。如需更详细的关于如何利用数据包的指导，请参阅帮助页面“导览”部分中的数据包导览。</v>
+        <v>在时间设置中，您可以为您的数据设置“时间段顶部”和“时间段底部”。调整这两个值将改变图表的时间跨度，您可以通过输入值或使用下拉选择器进行调整。您还可以调整垂直比例，以改变图表中每百万年占据的垂直空间量。例如，将其设置得更高将使时间间隔进一步分开，使每个时期更易于仔细检查。</v>
       </c>
     </row>
     <row r="450">
       <c r="A450" t="str">
-        <v>settings.column.tooltip.note-in-range</v>
+        <v>tours.settings.step2</v>
+      </c>
+      <c r="B450" t="str">
+        <v>In the Preferences settings, you can customize the display options. For instance, you may choose to gray out columns with no data for selected time periods, add tooltips for additional information, or enable filtering and legend options for charts. Furthermore, you can load your settings from a file or save your current settings to a file. This feature is useful for backing up your configurations, sharing them with others, or quickly applying previously saved configurations to your chart.</v>
       </c>
       <c r="C450" t="str">
-        <v>数据不在所选时间区间内</v>
+        <v>在偏好中，您可以自定义显示选项。例如，您可以选择在选定时间段内将无数据的列显示为灰色，添加工具提示以提供额外信息，或启用图表的筛选和图例选项。此外，您可以从文件加载您的设置或将当前设置保存到文件中。此功能使您可以备份设置、与他人分享或快速应用以前保存的设置到您的图表中。</v>
       </c>
     </row>
     <row r="451">
       <c r="A451" t="str">
-        <v>language-names.en-US</v>
+        <v>tours.settings.step3</v>
+      </c>
+      <c r="B451" t="str">
+        <v>In Column Settings, you can deeply customize the appearance and organization of your charts.In the "Column Customization" area, you can adjust titles and shift row positions to streamline how data is displayed on your charts. Enable or disable specific elements like the chart title and Ma markers to suit your presentation needs. In the "Font Options" section, refine the appearance of your charts by choosing different fonts, sizes, and styles for headers and labels, ensuring important data stands out or meets formatting requirements. Please note that the advanced settings for columns can vary depending on the datapack you are working with, allowing for tailored configurations that best fit the data characteristics.</v>
       </c>
       <c r="C451" t="str">
-        <v>English</v>
+        <v>在列设置中，您可以深度自定义图表的外观和组织。在“列自定义”区域，您可以调整标题和移动行位置，以简化图表上数据的显示方式。根据您的展示需求启用或禁用特定元素，如图表标题和百万年标记。在“字体选项”部分，通过选择不同的字体、大小和样式为标题和标签，细化您的图表外观，确保重要数据突出显示或符合格式要求。请注意，列高级设置可能根据您正在使用的数据包而有所不同，每个数据包都有最适合数据特性的列高级设置。</v>
       </c>
     </row>
     <row r="452">
       <c r="A452" t="str">
-        <v>language-names.en</v>
+        <v>tours.settings.step4</v>
+      </c>
+      <c r="B452" t="str">
+        <v>In the Search Settings, you can quickly locate specific columns by entering keywords and then directly add them to your chart. Simply enter a term related to the setting you are looking for, and the system will display all relevant results.This feature is particularly useful when managing numerous data points or when you need to make quick adjustments without browsing through extensive lists.</v>
       </c>
       <c r="C452" t="str">
-        <v>English</v>
+        <v>在搜索中，您可以通过输入关键词快速定位特定列，然后直接将其添加到您的图表中。只需输入一个与您正在寻找的设置相关的词语，系统便会显示所有相关结果。此功能可以帮助您管理众多数据点，或进行快速调整而无需浏览繁杂列表。请注意目前只支持英文搜索。</v>
       </c>
     </row>
     <row r="453">
       <c r="A453" t="str">
+        <v>tours.settings.step5</v>
+      </c>
+      <c r="B453" t="str">
+        <v>The Font Settings section allows you to customize the appearance of text within your charts. You can adjust font styles, sizes, and formatting for various elements such as column headers, age labels, and more. Each setting is inheritable, ensuring consistency across related elements unless specified otherwise. Changing a font setting here applies it system-wide, but you can override these for individual columns by using the "Change Font" option within each columns settings.Experiment with different fonts and sizes to enhance readability and visual appeal of your charts.</v>
+      </c>
+      <c r="C453" t="str">
+        <v>在字体设置中您可以自定义图表内的文本外观。您可以为各种元素如列标题、年龄标签等调整字体样式、大小和格式。每项设置都是可继承的，确保相关元素间的一致性，除非另行设置。在这里更改字体设置将系统范围内应用，但您可以使用每个列设置中的“更改字体”选项覆盖这些设置。尝试不同的字体和大小，以增强图表的可读性和视觉吸引力。</v>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="str">
+        <v>tours.settings.step6</v>
+      </c>
+      <c r="B454" t="str">
+        <v>In the Map Points Settings, you can access and manage geographic data points for different locations. This feature allows you to view specific location details directly on the interactive map. You can toggle different map layers and visualize data points with detailed descriptions, like latitude, longitude, and additional notes. Please note, however, that not all datapacks contain map points.</v>
+      </c>
+      <c r="C454" t="str">
+        <v>在地图点设置中，您可以访问和管理不同位置的地理数据点。此功能允许您直接在交互式地图上查看特定位置的详细信息。您可以切换不同的地图层，并用详细描述（如纬度、经度和附加说明）可视化数据点。请注意，并非所有数据包都包含地图点。</v>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="str">
+        <v>tours.settings.step7</v>
+      </c>
+      <c r="B455" t="str">
+        <v>In the Datapacks Settings, you can select the datapacks you wish to use for generating charts. We offer nine official datapacks, each comprising a curated collection of datasets tailored for specific thematic explorations. You might notice that this page resembles the Datapack page; selections can be configured here or there interchangeably. For more detailed guidance on how to utilize datapacks, please refer to the Datapacks Tour in the Help page "Tours" section.</v>
+      </c>
+      <c r="C455" t="str">
+        <v>在数据包设置中，您可以选择您希望用于生成图表的数据包。我们提供九个官方数据包，每个数据包都包含为特定主题探索量身定制的数据集合。您也许已经注意到，此页面与"数据包"页面内容相同；您在两个地方都可以进行选择和设置。如需更详细的关于如何利用数据包的指导，请参阅帮助页面“导览”部分中的数据包导览。</v>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="str">
+        <v>settings.column.tooltip.note-in-range</v>
+      </c>
+      <c r="C456" t="str">
+        <v>数据不在所选时间区间内</v>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="str">
+        <v>language-names.en-US</v>
+      </c>
+      <c r="C457" t="str">
+        <v>English</v>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="str">
+        <v>language-names.en</v>
+      </c>
+      <c r="C458" t="str">
+        <v>English</v>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="str">
         <v>language-names.zh</v>
       </c>
-      <c r="C453" t="str">
+      <c r="C459" t="str">
         <v>中文</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C453"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C459"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
prom, fixed admin edit
</commit_message>
<xml_diff>
--- a/server/assets/translation.xlsx
+++ b/server/assets/translation.xlsx
@@ -375,7 +375,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C453"/>
+  <dimension ref="A1:C454"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4293,439 +4293,439 @@
     </row>
     <row r="380">
       <c r="A380" t="str">
-        <v>errors.ADMIN_DELETE_SERVER_DATAPACK_FAILED</v>
+        <v>errors.ADMIN_MODIFY_USER_FAILED</v>
       </c>
       <c r="B380" t="str">
-        <v>Unable to delete server datapack. Please try again later.</v>
-      </c>
-      <c r="C380" t="str">
-        <v>无法删除服务器数据包。请稍后再试。</v>
+        <v>Unable to modify user. Please try again later.</v>
       </c>
     </row>
     <row r="381">
       <c r="A381" t="str">
-        <v>errors.ADMIN_CANNOT_DELETE_ROOT_DATAPACK</v>
+        <v>errors.ADMIN_DELETE_SERVER_DATAPACK_FAILED</v>
       </c>
       <c r="B381" t="str">
-        <v>Cannot delete root datapack. Ask server admin for assistance.</v>
+        <v>Unable to delete server datapack. Please try again later.</v>
       </c>
       <c r="C381" t="str">
-        <v>无法删除根数据包。请向服务器管理员寻求帮助。</v>
+        <v>无法删除服务器数据包。请稍后再试。</v>
       </c>
     </row>
     <row r="382">
       <c r="A382" t="str">
-        <v>errors.INVALID_SERVER_DATAPACK_REQUEST</v>
+        <v>errors.ADMIN_CANNOT_DELETE_ROOT_DATAPACK</v>
       </c>
       <c r="B382" t="str">
-        <v>Invalid server datapack request. Please try again later.</v>
+        <v>Cannot delete root datapack. Ask server admin for assistance.</v>
       </c>
       <c r="C382" t="str">
-        <v>无效的服务器数据包请求。请稍后再试。</v>
+        <v>无法删除根数据包。请向服务器管理员寻求帮助。</v>
       </c>
     </row>
     <row r="383">
       <c r="A383" t="str">
-        <v>errors.SERVER_FILE_METADATA_ERROR</v>
+        <v>errors.INVALID_SERVER_DATAPACK_REQUEST</v>
       </c>
       <c r="B383" t="str">
-        <v>Server file metadata error. Please try again later.</v>
+        <v>Invalid server datapack request. Please try again later.</v>
       </c>
       <c r="C383" t="str">
-        <v>服务器文件元数据错误。请稍后再试。</v>
+        <v>无效的服务器数据包请求。请稍后再试。</v>
       </c>
     </row>
     <row r="384">
       <c r="A384" t="str">
-        <v>errors.USER_DELETE_DATAPACK_FAILED</v>
+        <v>errors.SERVER_FILE_METADATA_ERROR</v>
       </c>
       <c r="B384" t="str">
-        <v>Unable to delete user datapack. Please try again later.</v>
+        <v>Server file metadata error. Please try again later.</v>
       </c>
       <c r="C384" t="str">
-        <v>无法删除用户数据包。请稍后再试。</v>
+        <v>服务器文件元数据错误。请稍后再试。</v>
       </c>
     </row>
     <row r="385">
       <c r="A385" t="str">
-        <v>errors.UNABLE_TO_PROCESS_DATAPACK_CONFIG</v>
+        <v>errors.USER_DELETE_DATAPACK_FAILED</v>
       </c>
       <c r="B385" t="str">
-        <v>Failed to process datapack config. Please try again later.</v>
+        <v>Unable to delete user datapack. Please try again later.</v>
       </c>
       <c r="C385" t="str">
-        <v>处理数据包配置失败。请稍后再试。</v>
+        <v>无法删除用户数据包。请稍后再试。</v>
       </c>
     </row>
     <row r="386">
       <c r="A386" t="str">
-        <v>errors.INVALID_SETTINGS</v>
+        <v>errors.UNABLE_TO_PROCESS_DATAPACK_CONFIG</v>
       </c>
       <c r="B386" t="str">
-        <v>Invalid settings. Please try again.</v>
+        <v>Failed to process datapack config. Please try again later.</v>
       </c>
       <c r="C386" t="str">
-        <v>无效的设置。请稍后再试。</v>
+        <v>处理数据包配置失败。请稍后再试。</v>
       </c>
     </row>
     <row r="387">
       <c r="A387" t="str">
-        <v>errors.INTERNAL_ERROR</v>
+        <v>errors.INVALID_SETTINGS</v>
       </c>
       <c r="B387" t="str">
-        <v>There was an internal error while generating the chart. Please try again later.</v>
+        <v>Invalid settings. Please try again.</v>
       </c>
       <c r="C387" t="str">
-        <v>生成图表时出现内部错误。请稍后再试。</v>
+        <v>无效的设置。请稍后再试。</v>
       </c>
     </row>
     <row r="388">
       <c r="A388" t="str">
-        <v>errors.ADMIN_ADD_USERS_TO_WORKSHOP_FAILED</v>
+        <v>errors.INTERNAL_ERROR</v>
       </c>
       <c r="B388" t="str">
-        <v>Unable to add users to workshop. Please try again later.</v>
+        <v>There was an internal error while generating the chart. Please try again later.</v>
       </c>
       <c r="C388" t="str">
-        <v>无法将用户添加到工作坊。请稍后再试。</v>
+        <v>生成图表时出现内部错误。请稍后再试。</v>
       </c>
     </row>
     <row r="389">
       <c r="A389" t="str">
-        <v>errors.ADMIN_EMAIL_INVALID</v>
+        <v>errors.ADMIN_ADD_USERS_TO_WORKSHOP_FAILED</v>
       </c>
       <c r="B389" t="str">
-        <v>Invalid email. Please fix the email and try again.</v>
+        <v>Unable to add users to workshop. Please try again later.</v>
       </c>
       <c r="C389" t="str">
-        <v>电子邮件无效。请修复电子邮件并重试。</v>
+        <v>无法将用户添加到工作坊。请稍后再试。</v>
       </c>
     </row>
     <row r="390">
       <c r="A390" t="str">
-        <v>errors.ADMIN_WORKSHOP_FIELDS_EMPTY</v>
+        <v>errors.ADMIN_EMAIL_INVALID</v>
       </c>
       <c r="B390" t="str">
-        <v>You must provide at least one field to add users to a workshop.</v>
+        <v>Invalid email. Please fix the email and try again.</v>
       </c>
       <c r="C390" t="str">
-        <v>您必须提供至少一个领域才能将用户添加到工作坊。</v>
+        <v>电子邮件无效。请修复电子邮件并重试。</v>
       </c>
     </row>
     <row r="391">
       <c r="A391" t="str">
-        <v>errors.UNRECOGNIZED_EXCEL_FILE</v>
+        <v>errors.ADMIN_WORKSHOP_FIELDS_EMPTY</v>
       </c>
       <c r="B391" t="str">
-        <v>Unrecognized Excel file. Please upload a valid Excel file.</v>
+        <v>You must provide at least one field to add users to a workshop.</v>
       </c>
       <c r="C391" t="str">
-        <v>无法识别 Excel 文件。请上传有效的 Excel 文件。</v>
+        <v>您必须提供至少一个领域才能将用户添加到工作坊。</v>
       </c>
     </row>
     <row r="392">
       <c r="A392" t="str">
-        <v>errors.SERVER_DATAPACK_ALREADY_EXISTS</v>
+        <v>errors.UNRECOGNIZED_EXCEL_FILE</v>
       </c>
       <c r="B392" t="str">
-        <v>Server datapack already exists. Please upload a unique datapack (different title).</v>
+        <v>Unrecognized Excel file. Please upload a valid Excel file.</v>
       </c>
       <c r="C392" t="str">
-        <v>服务器数据包已存在。请上传一个独特的数据包（不同的文件名）。</v>
+        <v>无法识别 Excel 文件。请上传有效的 Excel 文件。</v>
       </c>
     </row>
     <row r="393">
       <c r="A393" t="str">
-        <v>errors.ADMIN_WORKSHOP_START_AFTER_END</v>
+        <v>errors.SERVER_DATAPACK_ALREADY_EXISTS</v>
       </c>
       <c r="B393" t="str">
-        <v>The start date must be before the end date.</v>
+        <v>Server datapack already exists. Please upload a unique datapack (different title).</v>
       </c>
       <c r="C393" t="str">
-        <v>开始日期必须早于结束日期</v>
+        <v>服务器数据包已存在。请上传一个独特的数据包（不同的文件名）。</v>
       </c>
     </row>
     <row r="394">
       <c r="A394" t="str">
-        <v>errors.ADMIN_CREATE_WORKSHOP_FAILED</v>
+        <v>errors.ADMIN_WORKSHOP_START_AFTER_END</v>
       </c>
       <c r="B394" t="str">
-        <v>Unable to create workshop. Please try again later.</v>
+        <v>The start date must be before the end date.</v>
       </c>
       <c r="C394" t="str">
-        <v>无法创建工作坊。请稍后再试。</v>
+        <v>开始日期必须早于结束日期</v>
       </c>
     </row>
     <row r="395">
       <c r="A395" t="str">
-        <v>errors.ADMIN_WORKSHOP_ALREADY_EXISTS</v>
+        <v>errors.ADMIN_CREATE_WORKSHOP_FAILED</v>
       </c>
       <c r="B395" t="str">
-        <v>Workshop with that title and dates already exists. Please try again.</v>
+        <v>Unable to create workshop. Please try again later.</v>
       </c>
       <c r="C395" t="str">
-        <v>该工作坊名称已存在。请另选名称。</v>
+        <v>无法创建工作坊。请稍后再试。</v>
       </c>
     </row>
     <row r="396">
       <c r="A396" t="str">
-        <v>errors.ADMIN_FETCH_WORKSHOPS_FAILED</v>
+        <v>errors.ADMIN_WORKSHOP_ALREADY_EXISTS</v>
       </c>
       <c r="B396" t="str">
-        <v>Unable to fetch workshops. Please try again later.</v>
+        <v>Workshop with that title and dates already exists. Please try again.</v>
       </c>
       <c r="C396" t="str">
-        <v>无法抓取工作坊。请稍后再试。</v>
+        <v>该工作坊名称已存在。请另选名称。</v>
       </c>
     </row>
     <row r="397">
       <c r="A397" t="str">
-        <v>errors.ADMIN_DELETE_WORKSHOP_FAILED</v>
+        <v>errors.ADMIN_FETCH_WORKSHOPS_FAILED</v>
       </c>
       <c r="B397" t="str">
-        <v>Unable to delete workshop. Please try again later.</v>
+        <v>Unable to fetch workshops. Please try again later.</v>
+      </c>
+      <c r="C397" t="str">
+        <v>无法抓取工作坊。请稍后再试。</v>
       </c>
     </row>
     <row r="398">
       <c r="A398" t="str">
-        <v>errors.ADMIN_WORKSHOP_NOT_FOUND</v>
+        <v>errors.ADMIN_DELETE_WORKSHOP_FAILED</v>
       </c>
       <c r="B398" t="str">
-        <v>Workshop not found on server, it has likely ended or been deleted.</v>
-      </c>
-      <c r="C398" t="str">
-        <v>服务器未找到工作坊。该工作坊可能已结束或被删除。</v>
+        <v>Unable to delete workshop. Please try again later.</v>
       </c>
     </row>
     <row r="399">
       <c r="A399" t="str">
-        <v>errors.ADMIN_WORKSHOP_EDIT_FAILED</v>
+        <v>errors.ADMIN_WORKSHOP_NOT_FOUND</v>
       </c>
       <c r="B399" t="str">
-        <v>Unable to edit workshop. Please try again later.</v>
+        <v>Workshop not found on server, it has likely ended or been deleted.</v>
+      </c>
+      <c r="C399" t="str">
+        <v>服务器未找到工作坊。该工作坊可能已结束或被删除。</v>
       </c>
     </row>
     <row r="400">
       <c r="A400" t="str">
-        <v>errors.USER_EDIT_DATAPACK_FAILED</v>
+        <v>errors.ADMIN_WORKSHOP_EDIT_FAILED</v>
       </c>
       <c r="B400" t="str">
-        <v>Failed to edit user datapack. Please try again later.</v>
+        <v>Unable to edit workshop. Please try again later.</v>
       </c>
     </row>
     <row r="401">
       <c r="A401" t="str">
-        <v>errors.USER_FETCH_DATAPACK_FAILED</v>
+        <v>errors.USER_EDIT_DATAPACK_FAILED</v>
       </c>
       <c r="B401" t="str">
-        <v>Failed to fetch user datapack. Please try again later.</v>
+        <v>Failed to edit user datapack. Please try again later.</v>
       </c>
     </row>
     <row r="402">
       <c r="A402" t="str">
-        <v>errors.USER_REPLACE_DATAPACK_FILE_FAILED</v>
+        <v>errors.USER_FETCH_DATAPACK_FAILED</v>
       </c>
       <c r="B402" t="str">
-        <v>Failed to replace user datapack file. Please try again later.</v>
+        <v>Failed to fetch user datapack. Please try again later.</v>
       </c>
     </row>
     <row r="403">
       <c r="A403" t="str">
-        <v>errors.USER_REPLACE_DATAPACK_PROFILE_IMAGE_FAILED</v>
+        <v>errors.USER_REPLACE_DATAPACK_FILE_FAILED</v>
       </c>
       <c r="B403" t="str">
-        <v>Failed to replace user datapack profile image. Please try again later.</v>
+        <v>Failed to replace user datapack file. Please try again later.</v>
       </c>
     </row>
     <row r="404">
       <c r="A404" t="str">
-        <v>errors.DATAPACK_TITLE_LEADING_TRAILING_WHITESPACE</v>
+        <v>errors.USER_REPLACE_DATAPACK_PROFILE_IMAGE_FAILED</v>
       </c>
       <c r="B404" t="str">
-        <v>Datapack title cannot have leading or trailing whitespace.</v>
+        <v>Failed to replace user datapack profile image. Please try again later.</v>
       </c>
     </row>
     <row r="405">
       <c r="A405" t="str">
-        <v>errors.ADMIN_FETCH_PRIVATE_DATAPACKS_FAILED</v>
+        <v>errors.DATAPACK_TITLE_LEADING_TRAILING_WHITESPACE</v>
       </c>
       <c r="B405" t="str">
-        <v>Failed to fetch private datapacks. Please try again later.</v>
+        <v>Datapack title cannot have leading or trailing whitespace.</v>
       </c>
     </row>
     <row r="406">
       <c r="A406" t="str">
-        <v>errors.ADMIN_PRIORITY_BATCH_UPDATE_FAILED</v>
+        <v>errors.ADMIN_FETCH_PRIVATE_DATAPACKS_FAILED</v>
       </c>
       <c r="B406" t="str">
-        <v>Failed to update datapack priorities. Please contact a server admin for assistance.</v>
+        <v>Failed to fetch private datapacks. Please try again later.</v>
       </c>
     </row>
     <row r="407">
       <c r="A407" t="str">
-        <v>errors.ADMIN_ADD_OFFICIAL_DATAPACK_TO_WORKSHOP_FAILED</v>
+        <v>errors.ADMIN_PRIORITY_BATCH_UPDATE_FAILED</v>
       </c>
       <c r="B407" t="str">
-        <v>Failed to add official datapack to workshop. Please try again later.</v>
+        <v>Failed to update datapack priorities. Please contact a server admin for assistance.</v>
       </c>
     </row>
     <row r="408">
       <c r="A408" t="str">
-        <v>errors.ADMIN_SERVER_DATAPACK_ALREADY_EXISTS</v>
+        <v>errors.ADMIN_ADD_OFFICIAL_DATAPACK_TO_WORKSHOP_FAILED</v>
       </c>
       <c r="B408" t="str">
-        <v>Server datapack already exists in workshop. Please choose a different datapack.</v>
+        <v>Failed to add official datapack to workshop. Please try again later.</v>
       </c>
     </row>
     <row r="409">
       <c r="A409" t="str">
-        <v>errors.ADMIN_WORKSHOP_ENDED</v>
+        <v>errors.ADMIN_SERVER_DATAPACK_ALREADY_EXISTS</v>
       </c>
       <c r="B409" t="str">
-        <v>Workshop has ended. You can no longer edit or add datapacks to it.</v>
+        <v>Server datapack already exists in workshop. Please choose a different datapack.</v>
       </c>
     </row>
     <row r="410">
       <c r="A410" t="str">
-        <v>errors.WORKSHOP_FETCH_DATAPACK_FAILED</v>
+        <v>errors.ADMIN_WORKSHOP_ENDED</v>
       </c>
       <c r="B410" t="str">
-        <v>Failed to fetch workshop datapacks. Please try again later.</v>
+        <v>Workshop has ended. You can no longer edit or add datapacks to it.</v>
       </c>
     </row>
     <row r="411">
       <c r="A411" t="str">
-        <v>errors.METADATA_NOT_FOUND</v>
+        <v>errors.WORKSHOP_FETCH_DATAPACK_FAILED</v>
       </c>
       <c r="B411" t="str">
-        <v>Metadata not found. Please try again later.</v>
+        <v>Failed to fetch workshop datapacks. Please try again later.</v>
       </c>
     </row>
     <row r="412">
       <c r="A412" t="str">
-        <v>errors.INVALID_CROSSPLOT_CONVERSION</v>
+        <v>errors.METADATA_NOT_FOUND</v>
       </c>
       <c r="B412" t="str">
-        <v>Invalid crossplot conversion. Please select a valid chart for the Y Axis.</v>
+        <v>Metadata not found. Please try again later.</v>
       </c>
     </row>
     <row r="413">
       <c r="A413" t="str">
-        <v>errors.INVALID_CROSSPLOT_UNITS</v>
+        <v>errors.INVALID_CROSSPLOT_CONVERSION</v>
       </c>
       <c r="B413" t="str">
-        <v>Please select a different unit for the Y Axis. This unit cannot be converted.</v>
+        <v>Invalid crossplot conversion. Please select a valid chart for the Y Axis.</v>
       </c>
     </row>
     <row r="414">
       <c r="A414" t="str">
-        <v>errors.CROSSPLOT_CONVERSION_FAILED</v>
+        <v>errors.INVALID_CROSSPLOT_UNITS</v>
       </c>
       <c r="B414" t="str">
-        <v>Crossplot conversion failed. Please try again later.</v>
+        <v>Please select a different unit for the Y Axis. This unit cannot be converted.</v>
       </c>
     </row>
     <row r="415">
       <c r="A415" t="str">
-        <v>errors.NO_MODELS</v>
+        <v>errors.CROSSPLOT_CONVERSION_FAILED</v>
       </c>
       <c r="B415" t="str">
-        <v>No models available. Please add a model by clicking the chart in the main view.</v>
+        <v>Crossplot conversion failed. Please try again later.</v>
       </c>
     </row>
     <row r="416">
       <c r="A416" t="str">
-        <v>errors.CROSSPLOT_SETTINGS_MISMATCH</v>
+        <v>errors.NO_MODELS</v>
       </c>
       <c r="B416" t="str">
-        <v>Crossplot settings mismatch. Please generate the crossplot with your most recent changes.</v>
+        <v>No models available. Please add a model by clicking the chart in the main view.</v>
       </c>
     </row>
     <row r="417">
       <c r="A417" t="str">
-        <v>button.generate</v>
+        <v>errors.CROSSPLOT_SETTINGS_MISMATCH</v>
       </c>
       <c r="B417" t="str">
-        <v>Generate</v>
-      </c>
-      <c r="C417" t="str">
-        <v>绘制</v>
+        <v>Crossplot settings mismatch. Please generate the crossplot with your most recent changes.</v>
       </c>
     </row>
     <row r="418">
       <c r="A418" t="str">
-        <v>button.generate-chart</v>
+        <v>button.generate</v>
       </c>
       <c r="B418" t="str">
-        <v>Generate Chart</v>
+        <v>Generate</v>
       </c>
       <c r="C418" t="str">
-        <v>绘制图表</v>
+        <v>绘制</v>
       </c>
     </row>
     <row r="419">
       <c r="A419" t="str">
-        <v>button.remove-cache</v>
+        <v>button.generate-chart</v>
       </c>
       <c r="B419" t="str">
-        <v>Remove Cache</v>
+        <v>Generate Chart</v>
       </c>
       <c r="C419" t="str">
-        <v>清除缓存</v>
+        <v>绘制图表</v>
       </c>
     </row>
     <row r="420">
       <c r="A420" t="str">
-        <v>button.confirm-selection</v>
+        <v>button.remove-cache</v>
       </c>
       <c r="B420" t="str">
-        <v>Confirm Selection</v>
+        <v>Remove Cache</v>
       </c>
       <c r="C420" t="str">
-        <v>确认选择</v>
+        <v>清除缓存</v>
       </c>
     </row>
     <row r="421">
       <c r="A421" t="str">
-        <v>button.generate-cross-plot</v>
+        <v>button.confirm-selection</v>
       </c>
       <c r="B421" t="str">
-        <v>Generate Cross Plot</v>
+        <v>Confirm Selection</v>
+      </c>
+      <c r="C421" t="str">
+        <v>确认选择</v>
       </c>
     </row>
     <row r="422">
       <c r="A422" t="str">
-        <v>yes</v>
+        <v>button.generate-cross-plot</v>
       </c>
       <c r="B422" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="C422" t="str">
-        <v>是</v>
+        <v>Generate Cross Plot</v>
       </c>
     </row>
     <row r="423">
       <c r="A423" t="str">
-        <v>no</v>
+        <v>yes</v>
       </c>
       <c r="B423" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="C423" t="str">
-        <v>否</v>
+        <v>是</v>
       </c>
     </row>
     <row r="424">
       <c r="A424" t="str">
-        <v>languageNames.en-US</v>
+        <v>no</v>
       </c>
       <c r="B424" t="str">
-        <v>English</v>
+        <v>No</v>
+      </c>
+      <c r="C424" t="str">
+        <v>否</v>
       </c>
     </row>
     <row r="425">
       <c r="A425" t="str">
-        <v>languageNames.en</v>
+        <v>languageNames.en-US</v>
       </c>
       <c r="B425" t="str">
         <v>English</v>
@@ -4733,284 +4733,284 @@
     </row>
     <row r="426">
       <c r="A426" t="str">
-        <v>languageNames.zh</v>
+        <v>languageNames.en</v>
       </c>
       <c r="B426" t="str">
-        <v>中文</v>
+        <v>English</v>
       </c>
     </row>
     <row r="427">
       <c r="A427" t="str">
-        <v>tours.quit</v>
+        <v>languageNames.zh</v>
       </c>
       <c r="B427" t="str">
-        <v>Quit Tour</v>
-      </c>
-      <c r="C427" t="str">
-        <v>退出导览</v>
+        <v>中文</v>
       </c>
     </row>
     <row r="428">
       <c r="A428" t="str">
-        <v>tours.finish</v>
+        <v>tours.quit</v>
       </c>
       <c r="B428" t="str">
-        <v>Finish Tour</v>
+        <v>Quit Tour</v>
       </c>
       <c r="C428" t="str">
-        <v>结束导览</v>
+        <v>退出导览</v>
       </c>
     </row>
     <row r="429">
       <c r="A429" t="str">
-        <v>tours.next</v>
+        <v>tours.finish</v>
       </c>
       <c r="B429" t="str">
-        <v>Next</v>
+        <v>Finish Tour</v>
       </c>
       <c r="C429" t="str">
-        <v>下一步</v>
+        <v>结束导览</v>
       </c>
     </row>
     <row r="430">
       <c r="A430" t="str">
-        <v>tours.back</v>
+        <v>tours.next</v>
       </c>
       <c r="B430" t="str">
-        <v>Back</v>
+        <v>Next</v>
       </c>
       <c r="C430" t="str">
-        <v>上一步</v>
+        <v>下一步</v>
       </c>
     </row>
     <row r="431">
       <c r="A431" t="str">
-        <v>tours.qsg.step1</v>
+        <v>tours.back</v>
       </c>
       <c r="B431" t="str">
-        <v>In the Presets page, we offer pre-configured settings that allow you to rapidly generate specific types of charts without configuring all options from the beginning. Each preset comes equipped with designated data packs, visual styles, and settings, enabling you to create charts with just a single click.</v>
+        <v>Back</v>
       </c>
       <c r="C431" t="str">
-        <v>在预设页面中，我们提供了预设置，允许您快速生成特定类型的图表，无需从头开始配置所有选项。每个预设都配备了指定的数据包、视觉样式和设置，使您能够一键创建图表</v>
+        <v>上一步</v>
       </c>
     </row>
     <row r="432">
       <c r="A432" t="str">
-        <v>tours.qsg.step2</v>
+        <v>tours.qsg.step1</v>
       </c>
       <c r="B432" t="str">
-        <v>In the Datapacks page, you can select the datapacks required to generate your charts. We offer nine official data packs, each containing a curated collection of datasets tailored for specific thematic explorations. For more detailed guidance on Datapacks, please refer to the Datapacks Tour under the "Tours" section</v>
+        <v>In the Presets page, we offer pre-configured settings that allow you to rapidly generate specific types of charts without configuring all options from the beginning. Each preset comes equipped with designated data packs, visual styles, and settings, enabling you to create charts with just a single click.</v>
       </c>
       <c r="C432" t="str">
-        <v>在数据包页面，您可以选择生成图表所需的数据包。我们提供九个官方数据包，每个数据包都包含为特定主题探索量身定制的数据集合集。如需更详细的数据包指导，请参考“导览”部分下的数据包导览。</v>
+        <v>在预设页面中，我们提供了预设置，允许您快速生成特定类型的图表，无需从头开始配置所有选项。每个预设都配备了指定的数据包、视觉样式和设置，使您能够一键创建图表</v>
       </c>
     </row>
     <row r="433">
       <c r="A433" t="str">
-        <v>tours.qsg.step3</v>
+        <v>tours.qsg.step2</v>
       </c>
       <c r="B433" t="str">
-        <v>In the Chart page, you can view the charts you have created and explore the detailed visualizations of geologic events. Additionally, you have the option to download and save these charts for your reference or further analysis.</v>
+        <v>In the Datapacks page, you can select the datapacks required to generate your charts. We offer nine official data packs, each containing a curated collection of datasets tailored for specific thematic explorations. For more detailed guidance on Datapacks, please refer to the Datapacks Tour under the "Tours" section</v>
       </c>
       <c r="C433" t="str">
-        <v>在图表页面，您可以查看已创建的图表并探索地质事件的详细可视化图。此外，您还可以下载并保存这些图表以供参考或进一步分析。</v>
+        <v>在数据包页面，您可以选择生成图表所需的数据包。我们提供九个官方数据包，每个数据包都包含为特定主题探索量身定制的数据集合集。如需更详细的数据包指导，请参考“导览”部分下的数据包导览。</v>
       </c>
     </row>
     <row r="434">
       <c r="A434" t="str">
-        <v>tours.qsg.step4</v>
+        <v>tours.qsg.step3</v>
       </c>
       <c r="B434" t="str">
-        <v>In the Settings page, you can customize all aspects of your charts. This includes adjusting the scale and time range, selecting which rows to display, setting the background color and font style, etc. Tailor your charts to meet your specific needs and preferences to optimize your visual analysis. For more detailed guidance on Settings, please refer to the Settings Tour under the "Tours" section</v>
+        <v>In the Chart page, you can view the charts you have created and explore the detailed visualizations of geologic events. Additionally, you have the option to download and save these charts for your reference or further analysis.</v>
       </c>
       <c r="C434" t="str">
-        <v>在设置页面，您可以自定义图表的所有方面。这包括调整比例和时间范围、选择显示哪些行、设置背景色和字体样式等。根据您的具体需求和偏好调整图表，以优化您的视觉分析。如需更详细的设置指导，请参考“导览”部分下的设置导览。</v>
+        <v>在图表页面，您可以查看已创建的图表并探索地质事件的详细可视化图。此外，您还可以下载并保存这些图表以供参考或进一步分析。</v>
       </c>
     </row>
     <row r="435">
       <c r="A435" t="str">
-        <v>tours.qsg.step5</v>
+        <v>tours.qsg.step4</v>
       </c>
       <c r="B435" t="str">
-        <v>In the Help Page, you can find detailed assistance and information on how to use the website.</v>
+        <v>In the Settings page, you can customize all aspects of your charts. This includes adjusting the scale and time range, selecting which rows to display, setting the background color and font style, etc. Tailor your charts to meet your specific needs and preferences to optimize your visual analysis. For more detailed guidance on Settings, please refer to the Settings Tour under the "Tours" section</v>
       </c>
       <c r="C435" t="str">
-        <v>在帮助页面，您可以找到关于如何使用网站的详细帮助和信息。</v>
+        <v>在设置页面，您可以自定义图表的所有方面。这包括调整比例和时间范围、选择显示哪些行、设置背景色和字体样式等。根据您的具体需求和偏好调整图表，以优化您的视觉分析。如需更详细的设置指导，请参考“导览”部分下的设置导览。</v>
       </c>
     </row>
     <row r="436">
       <c r="A436" t="str">
-        <v>tours.qsg.step6</v>
+        <v>tours.qsg.step5</v>
       </c>
       <c r="B436" t="str">
-        <v>In the Workshops Page, you can access a range of educational and experimental tutorials that offer in-depth guidance. Here, you can explore the workshops you have registered for, allowing you to engage with the content and enhance your skills in a hands-on learning environment.</v>
+        <v>In the Help Page, you can find detailed assistance and information on how to use the website.</v>
       </c>
       <c r="C436" t="str">
-        <v>在工作坊页面，您可以访问一系列提供深入指导的教育和实验教程。在这里，您可以探索已注册的研讨会，通过亲身实践的学习环境来提升您的技能。</v>
+        <v>在帮助页面，您可以找到关于如何使用网站的详细帮助和信息。</v>
       </c>
     </row>
     <row r="437">
       <c r="A437" t="str">
-        <v>tours.qsg.step7</v>
+        <v>tours.qsg.step6</v>
       </c>
       <c r="B437" t="str">
-        <v>The About Page provides information about our development team.</v>
+        <v>In the Workshops Page, you can access a range of educational and experimental tutorials that offer in-depth guidance. Here, you can explore the workshops you have registered for, allowing you to engage with the content and enhance your skills in a hands-on learning environment.</v>
       </c>
       <c r="C437" t="str">
-        <v>关于页面提供了我们开发团队的信息。</v>
+        <v>在工作坊页面，您可以访问一系列提供深入指导的教育和实验教程。在这里，您可以探索已注册的研讨会，通过亲身实践的学习环境来提升您的技能。</v>
       </c>
     </row>
     <row r="438">
       <c r="A438" t="str">
-        <v>tours.qsg.step8</v>
+        <v>tours.qsg.step7</v>
       </c>
       <c r="B438" t="str">
-        <v>Click here to sign in and unlock the features mentioned earlier, such as accessing registered workshops. Once logged in, you will also have the ability to upload datapacks and take full advantage of all functionalities.</v>
+        <v>The About Page provides information about our development team.</v>
       </c>
       <c r="C438" t="str">
-        <v>点击此处登录并解锁前面提到的功能，例如访问工作坊界面。登陆后，您还将能够上传数据包并充分利用所有功能。</v>
+        <v>关于页面提供了我们开发团队的信息。</v>
       </c>
     </row>
     <row r="439">
       <c r="A439" t="str">
-        <v>tours.datapack.step1</v>
+        <v>tours.qsg.step8</v>
       </c>
       <c r="B439" t="str">
-        <v>Switch between different display types for datapacks: rows, cards, or compact view.</v>
+        <v>Click here to sign in and unlock the features mentioned earlier, such as accessing registered workshops. Once logged in, you will also have the ability to upload datapacks and take full advantage of all functionalities.</v>
       </c>
       <c r="C439" t="str">
-        <v>在数据包显示类型之间切换：行视图、卡片视图或紧凑视图。</v>
+        <v>点击此处登录并解锁前面提到的功能，例如访问工作坊界面。登陆后，您还将能够上传数据包并充分利用所有功能。</v>
       </c>
     </row>
     <row r="440">
       <c r="A440" t="str">
-        <v>tours.datapack.step2</v>
+        <v>tours.datapack.step1</v>
       </c>
       <c r="B440" t="str">
-        <v>Add a datapack by clicking the checkbox</v>
+        <v>Switch between different display types for datapacks: rows, cards, or compact view.</v>
       </c>
       <c r="C440" t="str">
-        <v>勾选添加您想要的数据包</v>
+        <v>在数据包显示类型之间切换：行视图、卡片视图或紧凑视图。</v>
       </c>
     </row>
     <row r="441">
       <c r="A441" t="str">
-        <v>tours.datapack.step3</v>
+        <v>tours.datapack.step2</v>
       </c>
       <c r="B441" t="str">
-        <v>Click the deselect icon to deselect all datapacks</v>
+        <v>Add a datapack by clicking the checkbox</v>
       </c>
       <c r="C441" t="str">
-        <v>点此取消选择所有数据包</v>
+        <v>勾选添加您想要的数据包</v>
       </c>
     </row>
     <row r="442">
       <c r="A442" t="str">
-        <v>tours.datapack.step4</v>
+        <v>tours.datapack.step3</v>
       </c>
       <c r="B442" t="str">
-        <v>Remember to confirm your selection</v>
+        <v>Click the deselect icon to deselect all datapacks</v>
       </c>
       <c r="C442" t="str">
-        <v>记得确认您的选择</v>
+        <v>点此取消选择所有数据包</v>
       </c>
     </row>
     <row r="443">
       <c r="A443" t="str">
-        <v>tours.settings.step1</v>
+        <v>tours.datapack.step4</v>
       </c>
       <c r="B443" t="str">
-        <v>In the Time settings, you can Set the "Top of Interval" and "Base of Interval" for your data. These fields allow you to define the starting and ending ages or stages, which can be adjusted by entering values or using the dropdown selectors. Adjust the vertical scale to change how much vertical space each million years occupies on your charts. For example, setting it higher will spread the intervals further apart, making each period easier to examine closely.</v>
+        <v>Remember to confirm your selection</v>
       </c>
       <c r="C443" t="str">
-        <v>在时间设置中，您可以为您的数据设置“时间段顶部”和“时间段底部”。调整这两个值将改变图表的时间跨度，您可以通过输入值或使用下拉选择器进行调整。您还可以调整垂直比例，以改变图表中每百万年占据的垂直空间量。例如，将其设置得更高将使时间间隔进一步分开，使每个时期更易于仔细检查。</v>
+        <v>记得确认您的选择</v>
       </c>
     </row>
     <row r="444">
       <c r="A444" t="str">
-        <v>tours.settings.step2</v>
+        <v>tours.settings.step1</v>
       </c>
       <c r="B444" t="str">
-        <v>In the Preferences settings, you can customize the display options. For instance, you may choose to gray out columns with no data for selected time periods, add tooltips for additional information, or enable filtering and legend options for charts. Furthermore, you can load your settings from a file or save your current settings to a file. This feature is useful for backing up your configurations, sharing them with others, or quickly applying previously saved configurations to your chart.</v>
+        <v>In the Time settings, you can Set the "Top of Interval" and "Base of Interval" for your data. These fields allow you to define the starting and ending ages or stages, which can be adjusted by entering values or using the dropdown selectors. Adjust the vertical scale to change how much vertical space each million years occupies on your charts. For example, setting it higher will spread the intervals further apart, making each period easier to examine closely.</v>
       </c>
       <c r="C444" t="str">
-        <v>在偏好中，您可以自定义显示选项。例如，您可以选择在选定时间段内将无数据的列显示为灰色，添加工具提示以提供额外信息，或启用图表的筛选和图例选项。此外，您可以从文件加载您的设置或将当前设置保存到文件中。此功能使您可以备份设置、与他人分享或快速应用以前保存的设置到您的图表中。</v>
+        <v>在时间设置中，您可以为您的数据设置“时间段顶部”和“时间段底部”。调整这两个值将改变图表的时间跨度，您可以通过输入值或使用下拉选择器进行调整。您还可以调整垂直比例，以改变图表中每百万年占据的垂直空间量。例如，将其设置得更高将使时间间隔进一步分开，使每个时期更易于仔细检查。</v>
       </c>
     </row>
     <row r="445">
       <c r="A445" t="str">
-        <v>tours.settings.step3</v>
+        <v>tours.settings.step2</v>
       </c>
       <c r="B445" t="str">
-        <v>In Column Settings, you can deeply customize the appearance and organization of your charts.In the "Column Customization" area, you can adjust titles and shift row positions to streamline how data is displayed on your charts. Enable or disable specific elements like the chart title and Ma markers to suit your presentation needs. In the "Font Options" section, refine the appearance of your charts by choosing different fonts, sizes, and styles for headers and labels, ensuring important data stands out or meets formatting requirements. Please note that the advanced settings for columns can vary depending on the datapack you are working with, allowing for tailored configurations that best fit the data characteristics.</v>
+        <v>In the Preferences settings, you can customize the display options. For instance, you may choose to gray out columns with no data for selected time periods, add tooltips for additional information, or enable filtering and legend options for charts. Furthermore, you can load your settings from a file or save your current settings to a file. This feature is useful for backing up your configurations, sharing them with others, or quickly applying previously saved configurations to your chart.</v>
       </c>
       <c r="C445" t="str">
-        <v>在列设置中，您可以深度自定义图表的外观和组织。在“列自定义”区域，您可以调整标题和移动行位置，以简化图表上数据的显示方式。根据您的展示需求启用或禁用特定元素，如图表标题和百万年标记。在“字体选项”部分，通过选择不同的字体、大小和样式为标题和标签，细化您的图表外观，确保重要数据突出显示或符合格式要求。请注意，列高级设置可能根据您正在使用的数据包而有所不同，每个数据包都有最适合数据特性的列高级设置。</v>
+        <v>在偏好中，您可以自定义显示选项。例如，您可以选择在选定时间段内将无数据的列显示为灰色，添加工具提示以提供额外信息，或启用图表的筛选和图例选项。此外，您可以从文件加载您的设置或将当前设置保存到文件中。此功能使您可以备份设置、与他人分享或快速应用以前保存的设置到您的图表中。</v>
       </c>
     </row>
     <row r="446">
       <c r="A446" t="str">
-        <v>tours.settings.step4</v>
+        <v>tours.settings.step3</v>
       </c>
       <c r="B446" t="str">
-        <v>In the Search Settings, you can quickly locate specific columns by entering keywords and then directly add them to your chart. Simply enter a term related to the setting you are looking for, and the system will display all relevant results.This feature is particularly useful when managing numerous data points or when you need to make quick adjustments without browsing through extensive lists.</v>
+        <v>In Column Settings, you can deeply customize the appearance and organization of your charts.In the "Column Customization" area, you can adjust titles and shift row positions to streamline how data is displayed on your charts. Enable or disable specific elements like the chart title and Ma markers to suit your presentation needs. In the "Font Options" section, refine the appearance of your charts by choosing different fonts, sizes, and styles for headers and labels, ensuring important data stands out or meets formatting requirements. Please note that the advanced settings for columns can vary depending on the datapack you are working with, allowing for tailored configurations that best fit the data characteristics.</v>
       </c>
       <c r="C446" t="str">
-        <v>在搜索中，您可以通过输入关键词快速定位特定列，然后直接将其添加到您的图表中。只需输入一个与您正在寻找的设置相关的词语，系统便会显示所有相关结果。此功能可以帮助您管理众多数据点，或进行快速调整而无需浏览繁杂列表。请注意目前只支持英文搜索。</v>
+        <v>在列设置中，您可以深度自定义图表的外观和组织。在“列自定义”区域，您可以调整标题和移动行位置，以简化图表上数据的显示方式。根据您的展示需求启用或禁用特定元素，如图表标题和百万年标记。在“字体选项”部分，通过选择不同的字体、大小和样式为标题和标签，细化您的图表外观，确保重要数据突出显示或符合格式要求。请注意，列高级设置可能根据您正在使用的数据包而有所不同，每个数据包都有最适合数据特性的列高级设置。</v>
       </c>
     </row>
     <row r="447">
       <c r="A447" t="str">
-        <v>tours.settings.step5</v>
+        <v>tours.settings.step4</v>
       </c>
       <c r="B447" t="str">
-        <v>The Font Settings section allows you to customize the appearance of text within your charts. You can adjust font styles, sizes, and formatting for various elements such as column headers, age labels, and more. Each setting is inheritable, ensuring consistency across related elements unless specified otherwise. Changing a font setting here applies it system-wide, but you can override these for individual columns by using the "Change Font" option within each columns settings.Experiment with different fonts and sizes to enhance readability and visual appeal of your charts.</v>
+        <v>In the Search Settings, you can quickly locate specific columns by entering keywords and then directly add them to your chart. Simply enter a term related to the setting you are looking for, and the system will display all relevant results.This feature is particularly useful when managing numerous data points or when you need to make quick adjustments without browsing through extensive lists.</v>
       </c>
       <c r="C447" t="str">
-        <v>在字体设置中您可以自定义图表内的文本外观。您可以为各种元素如列标题、年龄标签等调整字体样式、大小和格式。每项设置都是可继承的，确保相关元素间的一致性，除非另行设置。在这里更改字体设置将系统范围内应用，但您可以使用每个列设置中的“更改字体”选项覆盖这些设置。尝试不同的字体和大小，以增强图表的可读性和视觉吸引力。</v>
+        <v>在搜索中，您可以通过输入关键词快速定位特定列，然后直接将其添加到您的图表中。只需输入一个与您正在寻找的设置相关的词语，系统便会显示所有相关结果。此功能可以帮助您管理众多数据点，或进行快速调整而无需浏览繁杂列表。请注意目前只支持英文搜索。</v>
       </c>
     </row>
     <row r="448">
       <c r="A448" t="str">
-        <v>tours.settings.step6</v>
+        <v>tours.settings.step5</v>
       </c>
       <c r="B448" t="str">
-        <v>In the Map Points Settings, you can access and manage geographic data points for different locations. This feature allows you to view specific location details directly on the interactive map. You can toggle different map layers and visualize data points with detailed descriptions, like latitude, longitude, and additional notes. Please note, however, that not all datapacks contain map points.</v>
+        <v>The Font Settings section allows you to customize the appearance of text within your charts. You can adjust font styles, sizes, and formatting for various elements such as column headers, age labels, and more. Each setting is inheritable, ensuring consistency across related elements unless specified otherwise. Changing a font setting here applies it system-wide, but you can override these for individual columns by using the "Change Font" option within each columns settings.Experiment with different fonts and sizes to enhance readability and visual appeal of your charts.</v>
       </c>
       <c r="C448" t="str">
-        <v>在地图点设置中，您可以访问和管理不同位置的地理数据点。此功能允许您直接在交互式地图上查看特定位置的详细信息。您可以切换不同的地图层，并用详细描述（如纬度、经度和附加说明）可视化数据点。请注意，并非所有数据包都包含地图点。</v>
+        <v>在字体设置中您可以自定义图表内的文本外观。您可以为各种元素如列标题、年龄标签等调整字体样式、大小和格式。每项设置都是可继承的，确保相关元素间的一致性，除非另行设置。在这里更改字体设置将系统范围内应用，但您可以使用每个列设置中的“更改字体”选项覆盖这些设置。尝试不同的字体和大小，以增强图表的可读性和视觉吸引力。</v>
       </c>
     </row>
     <row r="449">
       <c r="A449" t="str">
-        <v>tours.settings.step7</v>
+        <v>tours.settings.step6</v>
       </c>
       <c r="B449" t="str">
-        <v>In the Datapacks Settings, you can select the datapacks you wish to use for generating charts. We offer nine official datapacks, each comprising a curated collection of datasets tailored for specific thematic explorations. You might notice that this page resembles the Datapack page; selections can be configured here or there interchangeably. For more detailed guidance on how to utilize datapacks, please refer to the Datapacks Tour in the Help page "Tours" section.</v>
+        <v>In the Map Points Settings, you can access and manage geographic data points for different locations. This feature allows you to view specific location details directly on the interactive map. You can toggle different map layers and visualize data points with detailed descriptions, like latitude, longitude, and additional notes. Please note, however, that not all datapacks contain map points.</v>
       </c>
       <c r="C449" t="str">
-        <v>在数据包设置中，您可以选择您希望用于生成图表的数据包。我们提供九个官方数据包，每个数据包都包含为特定主题探索量身定制的数据集合。您也许已经注意到，此页面与"数据包"页面内容相同；您在两个地方都可以进行选择和设置。如需更详细的关于如何利用数据包的指导，请参阅帮助页面“导览”部分中的数据包导览。</v>
+        <v>在地图点设置中，您可以访问和管理不同位置的地理数据点。此功能允许您直接在交互式地图上查看特定位置的详细信息。您可以切换不同的地图层，并用详细描述（如纬度、经度和附加说明）可视化数据点。请注意，并非所有数据包都包含地图点。</v>
       </c>
     </row>
     <row r="450">
       <c r="A450" t="str">
-        <v>settings.column.tooltip.note-in-range</v>
+        <v>tours.settings.step7</v>
+      </c>
+      <c r="B450" t="str">
+        <v>In the Datapacks Settings, you can select the datapacks you wish to use for generating charts. We offer nine official datapacks, each comprising a curated collection of datasets tailored for specific thematic explorations. You might notice that this page resembles the Datapack page; selections can be configured here or there interchangeably. For more detailed guidance on how to utilize datapacks, please refer to the Datapacks Tour in the Help page "Tours" section.</v>
       </c>
       <c r="C450" t="str">
-        <v>数据不在所选时间区间内</v>
+        <v>在数据包设置中，您可以选择您希望用于生成图表的数据包。我们提供九个官方数据包，每个数据包都包含为特定主题探索量身定制的数据集合。您也许已经注意到，此页面与"数据包"页面内容相同；您在两个地方都可以进行选择和设置。如需更详细的关于如何利用数据包的指导，请参阅帮助页面“导览”部分中的数据包导览。</v>
       </c>
     </row>
     <row r="451">
       <c r="A451" t="str">
-        <v>language-names.en-US</v>
+        <v>settings.column.tooltip.note-in-range</v>
       </c>
       <c r="C451" t="str">
-        <v>English</v>
+        <v>数据不在所选时间区间内</v>
       </c>
     </row>
     <row r="452">
       <c r="A452" t="str">
-        <v>language-names.en</v>
+        <v>language-names.en-US</v>
       </c>
       <c r="C452" t="str">
         <v>English</v>
@@ -5018,15 +5018,23 @@
     </row>
     <row r="453">
       <c r="A453" t="str">
+        <v>language-names.en</v>
+      </c>
+      <c r="C453" t="str">
+        <v>English</v>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="str">
         <v>language-names.zh</v>
       </c>
-      <c r="C453" t="str">
+      <c r="C454" t="str">
         <v>中文</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C453"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C454"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added hasFiles attribute to datapack
</commit_message>
<xml_diff>
--- a/server/assets/translation.xlsx
+++ b/server/assets/translation.xlsx
@@ -375,7 +375,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C473"/>
+  <dimension ref="A1:C453"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1714,82 +1714,82 @@
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v>crossPlot.time.select-unit</v>
+        <v>crossPlot.create-datapack</v>
       </c>
       <c r="B139" t="str">
-        <v>Please select a unit.</v>
+        <v>Create Datapack</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v>crossPlot.time.no-chart-units-available</v>
+        <v>crossPlot.time.no-unit-selected</v>
       </c>
       <c r="B140" t="str">
-        <v>No units available</v>
+        <v>No unit selected</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>crossPlot.time.disabled-unit-reason</v>
+        <v>crossPlot.time.select-unit</v>
       </c>
       <c r="B141" t="str">
-        <v>You cannot change the age unit since it must be on the x-axis.</v>
+        <v>Please select a unit.</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="str">
-        <v>crossPlot.time.select-datapack</v>
+        <v>crossPlot.time.no-chart-units-available</v>
       </c>
       <c r="B142" t="str">
-        <v>Please select a datapack.</v>
+        <v>No units available</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="str">
-        <v>crossPlot.time.no-unit-selected</v>
+        <v>crossPlot.time.disabled-unit-reason</v>
       </c>
       <c r="B143" t="str">
-        <v>No unit selected</v>
+        <v>You cannot change the age unit since it must be on the x-axis.</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="str">
-        <v>crossPlot.time.xAxis</v>
+        <v>crossPlot.time.select-datapack</v>
       </c>
       <c r="B144" t="str">
-        <v>X Axis (Age-only)</v>
+        <v>Please select a datapack.</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="str">
-        <v>crossPlot.time.yAxis</v>
+        <v>crossPlot.time.xAxis</v>
       </c>
       <c r="B145" t="str">
-        <v>Y Axis (Age/Depth)</v>
+        <v>X Axis (Age-only)</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="str">
-        <v>crossPlot.sidebar.no-markers</v>
+        <v>crossPlot.time.yAxis</v>
       </c>
       <c r="B146" t="str">
-        <v xml:space="preserve"> No Markers Available (Please Add a Marker by Clicking the Chart in the Main View)</v>
+        <v>Y Axis (Age/Depth)</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="str">
-        <v>crossPlot.sidebar.no-models</v>
+        <v>crossPlot.sidebar.no-markers</v>
       </c>
       <c r="B147" t="str">
-        <v>No Models Available (Please Add a Model by Clicking the Chart in the Main View)</v>
+        <v xml:space="preserve"> No Markers Available (Please Add a Marker by Clicking the Chart in the Main View)</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="str">
-        <v>crossPlot.create-datapack</v>
+        <v>crossPlot.sidebar.no-models</v>
       </c>
       <c r="B148" t="str">
-        <v>Create Crossplot</v>
+        <v>No Models Available (Please Add a Model by Clicking the Chart in the Main View)</v>
       </c>
     </row>
     <row r="149">
@@ -1904,108 +1904,111 @@
     </row>
     <row r="159">
       <c r="A159" t="str">
-        <v>settingsTabs.Overlay</v>
+        <v>settingsTabs.About</v>
       </c>
       <c r="B159" t="str">
-        <v>Overlay</v>
+        <v>About</v>
+      </c>
+      <c r="C159" t="str">
+        <v>关于</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="str">
-        <v>settingsTabs.About</v>
+        <v>settingsTabs.View Data</v>
       </c>
       <c r="B160" t="str">
-        <v>About</v>
+        <v>View Data</v>
       </c>
       <c r="C160" t="str">
-        <v>关于</v>
+        <v>查看数据</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="str">
-        <v>settingsTabs.View Data</v>
+        <v>settingsTabs.Discussion</v>
       </c>
       <c r="B161" t="str">
-        <v>View Data</v>
+        <v>Discussion</v>
       </c>
       <c r="C161" t="str">
-        <v>查看数据</v>
+        <v>讨论</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="str">
-        <v>settingsTabs.Discussion</v>
+        <v>settingsTabs.Warnings</v>
       </c>
       <c r="B162" t="str">
-        <v>Discussion</v>
+        <v>Warnings</v>
       </c>
       <c r="C162" t="str">
-        <v>讨论</v>
+        <v>警告</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="str">
-        <v>settingsTabs.Warnings</v>
+        <v>settingsTabs.Load/Save</v>
       </c>
       <c r="B163" t="str">
-        <v>Warnings</v>
-      </c>
-      <c r="C163" t="str">
-        <v>警告</v>
+        <v>Load/Save</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="str">
-        <v>settingsTabs.Load/Save</v>
+        <v>settingsTabs.xAxis</v>
       </c>
       <c r="B164" t="str">
-        <v>Load/Save</v>
+        <v>X Axis (Age-only)</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="str">
-        <v>settingsTabs.xAxis</v>
+        <v>settingsTabs.yAxis</v>
       </c>
       <c r="B165" t="str">
-        <v>X Axis (Age-only)</v>
+        <v>Y Axis (Age/Depth)</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="str">
-        <v>settingsTabs.yAxis</v>
+        <v>settings.time.interval.top</v>
       </c>
       <c r="B166" t="str">
-        <v>Y Axis (Age/Depth)</v>
+        <v>Top of Interval</v>
+      </c>
+      <c r="C166" t="str">
+        <v>区间顶部</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="str">
-        <v>settings.time.interval.top</v>
+        <v>settings.time.interval.base</v>
       </c>
       <c r="B167" t="str">
-        <v>Top of Interval</v>
+        <v>Base of Interval</v>
       </c>
       <c r="C167" t="str">
-        <v>区间顶部</v>
+        <v>区间底部</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="str">
-        <v>settings.time.interval.base</v>
+        <v>settings.time.interval.top-name</v>
       </c>
       <c r="B168" t="str">
-        <v>Base of Interval</v>
+        <v>Top Age/Stage Name</v>
       </c>
       <c r="C168" t="str">
-        <v>区间底部</v>
+        <v>年代/阶段 名称</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="str">
-        <v>settings.time.interval.top-name</v>
+        <v>settings.time.interval.base-name</v>
       </c>
       <c r="B169" t="str">
-        <v>Top Age/Stage Name</v>
+        <v>Base Age/Stage Name</v>
       </c>
       <c r="C169" t="str">
         <v>年代/阶段 名称</v>
@@ -2013,3183 +2016,3017 @@
     </row>
     <row r="170">
       <c r="A170" t="str">
-        <v>settings.time.interval.base-name</v>
+        <v>settings.time.interval.not-avaliable</v>
       </c>
       <c r="B170" t="str">
-        <v>Base Age/Stage Name</v>
+        <v>Not Available for this Unit</v>
       </c>
       <c r="C170" t="str">
-        <v>年代/阶段 名称</v>
+        <v>该时间单位无可选年代</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="str">
-        <v>settings.time.interval.not-avaliable</v>
+        <v>settings.time.interval.vertical-scale</v>
       </c>
       <c r="B171" t="str">
-        <v>Not Available for this Unit</v>
+        <v xml:space="preserve">Vertical Scale (cm per 1 </v>
       </c>
       <c r="C171" t="str">
-        <v>该时间单位无可选年代</v>
+        <v>垂直比例（厘米 每 1</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="str">
-        <v>settings.time.interval.vertical-scale</v>
+        <v>settings.time.interval.helper-text</v>
       </c>
       <c r="B172" t="str">
-        <v xml:space="preserve">Vertical Scale (cm per 1 </v>
+        <v>Base age should be older than top age</v>
       </c>
       <c r="C172" t="str">
-        <v>垂直比例（厘米 每 1</v>
+        <v>区间底部年代应大于区间顶部年代</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="str">
-        <v>settings.time.interval.helper-text</v>
+        <v>settings.time.interval.vertical-scale-header</v>
       </c>
       <c r="B173" t="str">
-        <v>Base age should be older than top age</v>
-      </c>
-      <c r="C173" t="str">
-        <v>区间底部年代应大于区间顶部年代</v>
+        <v>Vertical Scale</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="str">
-        <v>settings.time.interval.vertical-scale-header</v>
+        <v>settings.preferences.checkboxs.skip-empty-columns</v>
       </c>
       <c r="B174" t="str">
-        <v>Vertical Scale</v>
+        <v>Gray out (and do not draw) columns which do not have data on the selected time interval</v>
+      </c>
+      <c r="C174" t="str">
+        <v>在已选时间段内没有数据的列将不会被画出</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="str">
-        <v>settings.preferences.checkboxs.skip-empty-columns</v>
+        <v>settings.preferences.checkboxs.mouse-over-info</v>
       </c>
       <c r="B175" t="str">
-        <v>Gray out (and do not draw) columns which do not have data on the selected time interval</v>
+        <v>Add MouseOver info (popups)</v>
       </c>
       <c r="C175" t="str">
-        <v>在已选时间段内没有数据的列将不会被画出</v>
+        <v>鼠标移至目标上时显示详细信息</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="str">
-        <v>settings.preferences.checkboxs.mouse-over-info</v>
+        <v>settings.preferences.checkboxs.global-priority</v>
       </c>
       <c r="B176" t="str">
-        <v>Add MouseOver info (popups)</v>
+        <v>Enabled Global Priority Filtering for block columns</v>
       </c>
       <c r="C176" t="str">
-        <v>鼠标移至目标上时显示详细信息</v>
+        <v>启用优先级过滤</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="str">
-        <v>settings.preferences.checkboxs.global-priority</v>
+        <v>settings.preferences.checkboxs.stage-background</v>
       </c>
       <c r="B177" t="str">
-        <v>Enabled Global Priority Filtering for block columns</v>
+        <v>Enabled stage background for event columns</v>
       </c>
       <c r="C177" t="str">
-        <v>启用优先级过滤</v>
+        <v>启用事件列的背景</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="str">
-        <v>settings.preferences.checkboxs.stage-background</v>
+        <v>settings.preferences.checkboxs.enable-legend</v>
       </c>
       <c r="B178" t="str">
-        <v>Enabled stage background for event columns</v>
+        <v>Enable legend for the chart</v>
       </c>
       <c r="C178" t="str">
-        <v>启用事件列的背景</v>
+        <v>启用添加图例</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="str">
-        <v>settings.preferences.checkboxs.enable-legend</v>
+        <v>settings.preferences.checkboxs.lithology-auto-indent</v>
       </c>
       <c r="B179" t="str">
-        <v>Enable legend for the chart</v>
+        <v>Do not auto-indent lithology patterns</v>
       </c>
       <c r="C179" t="str">
-        <v>启用添加图例</v>
+        <v>禁用自动缩进岩性图案</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="str">
-        <v>settings.preferences.checkboxs.lithology-auto-indent</v>
+        <v>settings.preferences.checkboxs.conserve-chart</v>
       </c>
       <c r="B180" t="str">
-        <v>Do not auto-indent lithology patterns</v>
+        <v>Conserve Chart Space in Family Tree Plotting (Not implemented)</v>
       </c>
       <c r="C180" t="str">
-        <v>禁用自动缩进岩性图案</v>
+        <v>使用家谱绘图时节省图表空间（暂无该功能）</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="str">
-        <v>settings.preferences.checkboxs.conserve-chart</v>
+        <v>settings.preferences.checkboxs.hide-block-labels</v>
       </c>
       <c r="B181" t="str">
-        <v>Conserve Chart Space in Family Tree Plotting (Not implemented)</v>
+        <v>Hide block labels based on priority</v>
       </c>
       <c r="C181" t="str">
-        <v>使用家谱绘图时节省图表空间（暂无该功能）</v>
+        <v>根据优先级隐藏组标签</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="str">
-        <v>settings.preferences.checkboxs.hide-block-labels</v>
+        <v>settings.preferences.checkboxs.use-suggested-age-spans</v>
       </c>
       <c r="B182" t="str">
-        <v>Hide block labels based on priority</v>
+        <v>Do not use the Data-Pack's suggested age span</v>
       </c>
       <c r="C182" t="str">
-        <v>根据优先级隐藏组标签</v>
+        <v>禁用数据包建议的时间区间</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="str">
-        <v>settings.preferences.checkboxs.use-suggested-age-spans</v>
+        <v>settings.preferences.settings-file.load</v>
       </c>
       <c r="B183" t="str">
-        <v>Do not use the Data-Pack's suggested age span</v>
+        <v>Load Settings</v>
       </c>
       <c r="C183" t="str">
-        <v>禁用数据包建议的时间区间</v>
+        <v>上传设置</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="str">
-        <v>settings.preferences.settings-file.load</v>
+        <v>settings.preferences.settings-file.save</v>
       </c>
       <c r="B184" t="str">
-        <v>Load Settings</v>
+        <v>Save Settings</v>
       </c>
       <c r="C184" t="str">
-        <v>上传设置</v>
+        <v>保存设置</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="str">
-        <v>settings.preferences.settings-file.save</v>
+        <v>settings.preferences.settings-file.load-dialog.message</v>
       </c>
       <c r="B185" t="str">
-        <v>Save Settings</v>
+        <v>This will overwrite any changes you've made!</v>
       </c>
       <c r="C185" t="str">
-        <v>保存设置</v>
+        <v>这将覆盖你所做的任何更改！</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="str">
-        <v>settings.preferences.settings-file.load-dialog.message</v>
+        <v>settings.preferences.settings-file.load-dialog.cancel</v>
       </c>
       <c r="B186" t="str">
-        <v>This will overwrite any changes you've made!</v>
+        <v>Cancel</v>
       </c>
       <c r="C186" t="str">
-        <v>这将覆盖你所做的任何更改！</v>
+        <v>取消</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="str">
-        <v>settings.preferences.settings-file.load-dialog.cancel</v>
+        <v>settings.preferences.settings-file.load-dialog.load</v>
       </c>
       <c r="B187" t="str">
-        <v>Cancel</v>
+        <v>Load</v>
       </c>
       <c r="C187" t="str">
-        <v>取消</v>
+        <v>上传</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="str">
-        <v>settings.preferences.settings-file.load-dialog.load</v>
+        <v>settings.preferences.settings-file.save-dialog.message</v>
       </c>
       <c r="B188" t="str">
-        <v>Load</v>
+        <v>Please enter the filename below.</v>
       </c>
       <c r="C188" t="str">
-        <v>上传</v>
+        <v>请输入文件名</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="str">
-        <v>settings.preferences.settings-file.save-dialog.message</v>
+        <v>settings.preferences.settings-file.save-dialog.cancel</v>
       </c>
       <c r="B189" t="str">
-        <v>Please enter the filename below.</v>
+        <v>Cancel</v>
       </c>
       <c r="C189" t="str">
-        <v>请输入文件名</v>
+        <v>取消</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="str">
-        <v>settings.preferences.settings-file.save-dialog.cancel</v>
+        <v>settings.preferences.settings-file.save-dialog.save</v>
       </c>
       <c r="B190" t="str">
-        <v>Cancel</v>
+        <v>Save</v>
       </c>
       <c r="C190" t="str">
-        <v>取消</v>
+        <v>保存</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="str">
-        <v>settings.preferences.settings-file.save-dialog.save</v>
+        <v>settings.column.tooltip.not-in-range</v>
       </c>
       <c r="B191" t="str">
-        <v>Save</v>
-      </c>
-      <c r="C191" t="str">
-        <v>保存</v>
+        <v>Data not included in time range</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="str">
-        <v>settings.column.tooltip.not-in-range</v>
+        <v>settings.column.tooltip.auto-scale</v>
       </c>
       <c r="B192" t="str">
-        <v>Data not included in time range</v>
+        <v>Auto Scale</v>
+      </c>
+      <c r="C192" t="str">
+        <v>自动缩放</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="str">
-        <v>settings.column.tooltip.auto-scale</v>
+        <v>settings.column.tooltip.flip</v>
       </c>
       <c r="B193" t="str">
-        <v>Auto Scale</v>
+        <v>Flip Range</v>
       </c>
       <c r="C193" t="str">
-        <v>自动缩放</v>
+        <v>翻转区间</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="str">
-        <v>settings.column.tooltip.flip</v>
+        <v>settings.column.titles.column-menu-title</v>
       </c>
       <c r="B194" t="str">
-        <v>Flip Range</v>
+        <v>Column Customization</v>
       </c>
       <c r="C194" t="str">
-        <v>翻转区间</v>
+        <v>个性化设置列</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="str">
-        <v>settings.column.titles.column-menu-title</v>
+        <v>settings.column.titles.data-mining-title</v>
       </c>
       <c r="B195" t="str">
-        <v>Column Customization</v>
+        <v>Data Mining Settings</v>
       </c>
       <c r="C195" t="str">
-        <v>个性化设置列</v>
+        <v>数据挖掘设置</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="str">
-        <v>settings.column.titles.data-mining-title</v>
+        <v>settings.column.titles.font-option-title</v>
       </c>
       <c r="B196" t="str">
-        <v>Data Mining Settings</v>
+        <v>Font Options for "{{name}}"</v>
       </c>
       <c r="C196" t="str">
-        <v>数据挖掘设置</v>
+        <v>设置"{{name}}"列的字体</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="str">
-        <v>settings.column.titles.font-option-title</v>
+        <v>settings.column.menu.shift-row</v>
       </c>
       <c r="B197" t="str">
-        <v>Font Options for "{{name}}"</v>
+        <v>Shift Row Positions</v>
       </c>
       <c r="C197" t="str">
-        <v>设置"{{name}}"列的字体</v>
+        <v>移动位置</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="str">
-        <v>settings.column.menu.shift-row</v>
+        <v>settings.column.menu.edit-name</v>
       </c>
       <c r="B198" t="str">
-        <v>Shift Row Positions</v>
+        <v>Edit Title</v>
       </c>
       <c r="C198" t="str">
-        <v>移动位置</v>
+        <v>编辑标题</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="str">
-        <v>settings.column.menu.edit-name</v>
+        <v>settings.column.menu.background-color</v>
       </c>
       <c r="B199" t="str">
-        <v>Edit Title</v>
+        <v>Background Color</v>
       </c>
       <c r="C199" t="str">
-        <v>编辑标题</v>
+        <v>背景颜色</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="str">
-        <v>settings.column.menu.background-color</v>
+        <v>settings.column.menu.enable-title</v>
       </c>
       <c r="B200" t="str">
-        <v>Background Color</v>
+        <v>Enable Title</v>
       </c>
       <c r="C200" t="str">
-        <v>背景颜色</v>
+        <v>显示标题</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="str">
-        <v>settings.column.menu.enable-title</v>
+        <v>settings.column.menu.show-age-label</v>
       </c>
       <c r="B201" t="str">
-        <v>Enable Title</v>
+        <v>Show Age Label</v>
       </c>
       <c r="C201" t="str">
-        <v>显示标题</v>
+        <v>显示年代</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="str">
-        <v>settings.column.menu.show-age-label</v>
+        <v>settings.column.menu.info-box</v>
       </c>
       <c r="B202" t="str">
-        <v>Show Age Label</v>
+        <v>Information and References</v>
       </c>
       <c r="C202" t="str">
-        <v>显示年代</v>
+        <v>信息与参考</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="str">
-        <v>settings.column.menu.info-box</v>
+        <v>settings.column.menu.add-blank-column</v>
       </c>
       <c r="B203" t="str">
-        <v>Information and References</v>
+        <v>Add Blank Column</v>
       </c>
       <c r="C203" t="str">
-        <v>信息与参考</v>
+        <v>添加一个空白列</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="str">
-        <v>settings.column.menu.add-blank-column</v>
+        <v>settings.column.menu.add-age-column</v>
       </c>
       <c r="B204" t="str">
-        <v>Add Blank Column</v>
+        <v>Add Age Column</v>
       </c>
       <c r="C204" t="str">
-        <v>添加一个空白列</v>
+        <v>添加一个年代列</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="str">
-        <v>settings.column.menu.add-age-column</v>
+        <v>settings.column.menu.width</v>
       </c>
       <c r="B205" t="str">
-        <v>Add Age Column</v>
+        <v>Width</v>
       </c>
       <c r="C205" t="str">
-        <v>添加一个年代列</v>
+        <v>宽</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="str">
-        <v>settings.column.menu.width</v>
+        <v>settings.column.menu.orientation.title</v>
       </c>
       <c r="B206" t="str">
-        <v>Width</v>
+        <v>Label Orientation</v>
       </c>
       <c r="C206" t="str">
-        <v>宽</v>
+        <v>图标排布</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="str">
-        <v>settings.column.menu.orientation.title</v>
+        <v>settings.column.menu.orientation.horizontal</v>
       </c>
       <c r="B207" t="str">
-        <v>Label Orientation</v>
+        <v>Horizontal</v>
       </c>
       <c r="C207" t="str">
-        <v>图标排布</v>
+        <v>横向</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="str">
-        <v>settings.column.menu.orientation.horizontal</v>
+        <v>settings.column.menu.orientation.vertical</v>
       </c>
       <c r="B208" t="str">
-        <v>Horizontal</v>
+        <v>Vertical</v>
       </c>
       <c r="C208" t="str">
-        <v>横向</v>
+        <v>纵向</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="str">
-        <v>settings.column.menu.orientation.vertical</v>
+        <v>settings.column.menu.show-uncertainty</v>
       </c>
       <c r="B209" t="str">
-        <v>Vertical</v>
+        <v>Show Uncertainty Labels</v>
       </c>
       <c r="C209" t="str">
-        <v>纵向</v>
+        <v>显示不确定性</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="str">
-        <v>settings.column.menu.show-uncertainty</v>
+        <v>settings.column.menu.events</v>
       </c>
       <c r="B210" t="str">
-        <v>Show Uncertainty Labels</v>
+        <v>Events</v>
       </c>
       <c r="C210" t="str">
-        <v>显示不确定性</v>
+        <v>事件</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="str">
-        <v>settings.column.menu.events</v>
+        <v>settings.column.menu.ranges</v>
       </c>
       <c r="B211" t="str">
-        <v>Events</v>
+        <v>Ranges</v>
       </c>
       <c r="C211" t="str">
-        <v>事件</v>
+        <v>范围</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="str">
-        <v>settings.column.menu.ranges</v>
+        <v>settings.column.menu.first-occurrence</v>
       </c>
       <c r="B212" t="str">
-        <v>Ranges</v>
+        <v>First Occurrence</v>
       </c>
       <c r="C212" t="str">
-        <v>范围</v>
+        <v>首先发生的优先</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="str">
-        <v>settings.column.menu.first-occurrence</v>
+        <v>settings.column.menu.last-occurrence</v>
       </c>
       <c r="B213" t="str">
-        <v>First Occurrence</v>
+        <v>Last Occurrence</v>
       </c>
       <c r="C213" t="str">
-        <v>首先发生的优先</v>
+        <v>最后发生的优先</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="str">
-        <v>settings.column.menu.last-occurrence</v>
+        <v>settings.column.menu.alphabetical</v>
       </c>
       <c r="B214" t="str">
-        <v>Last Occurrence</v>
+        <v>Alphabetical</v>
       </c>
       <c r="C214" t="str">
-        <v>最后发生的优先</v>
+        <v>按字母顺序排列</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="str">
-        <v>settings.column.menu.alphabetical</v>
+        <v>settings.column.menu.ruler.title</v>
       </c>
       <c r="B215" t="str">
-        <v>Alphabetical</v>
+        <v>Age Ruler Justification</v>
       </c>
       <c r="C215" t="str">
-        <v>按字母顺序排列</v>
+        <v>调整年代刻度尺</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="str">
-        <v>settings.column.menu.ruler.title</v>
+        <v>settings.column.menu.ruler.left</v>
       </c>
       <c r="B216" t="str">
-        <v>Age Ruler Justification</v>
+        <v>Left</v>
       </c>
       <c r="C216" t="str">
-        <v>调整年代刻度尺</v>
+        <v>左对齐</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="str">
-        <v>settings.column.menu.ruler.left</v>
+        <v>settings.column.menu.ruler.right</v>
       </c>
       <c r="B217" t="str">
-        <v>Left</v>
+        <v>Right</v>
       </c>
       <c r="C217" t="str">
-        <v>左对齐</v>
+        <v>右对齐</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="str">
-        <v>settings.column.menu.ruler.right</v>
+        <v>settings.column.font-menu.change</v>
       </c>
       <c r="B218" t="str">
-        <v>Right</v>
+        <v>Change Font</v>
       </c>
       <c r="C218" t="str">
-        <v>右对齐</v>
+        <v>更改字体</v>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="str">
-        <v>settings.column.font-menu.change</v>
+        <v>settings.column.font-menu.additional</v>
       </c>
       <c r="B219" t="str">
-        <v>Change Font</v>
+        <v>Additional fonts for child columns</v>
       </c>
       <c r="C219" t="str">
-        <v>更改字体</v>
+        <v>子列的更多字体选项</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="str">
-        <v>settings.column.font-menu.additional</v>
+        <v>settings.column.datamining-menu.title</v>
       </c>
       <c r="B220" t="str">
-        <v>Additional fonts for child columns</v>
+        <v>Data Mining Settings</v>
       </c>
       <c r="C220" t="str">
-        <v>子列的更多字体选项</v>
+        <v>数据挖掘设置</v>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="str">
-        <v>settings.column.datamining-menu.title</v>
+        <v>settings.column.datamining-menu.window-size</v>
       </c>
       <c r="B221" t="str">
-        <v>Data Mining Settings</v>
+        <v>Window Size</v>
       </c>
       <c r="C221" t="str">
-        <v>数据挖掘设置</v>
+        <v>窗口大小</v>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="str">
-        <v>settings.column.datamining-menu.window-size</v>
+        <v>settings.column.datamining-menu.step-size</v>
       </c>
       <c r="B222" t="str">
-        <v>Window Size</v>
+        <v>Step Size</v>
       </c>
       <c r="C222" t="str">
-        <v>窗口大小</v>
+        <v>步长</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="str">
-        <v>settings.column.datamining-menu.step-size</v>
+        <v>settings.column.datamining-menu.options.frequency</v>
       </c>
       <c r="B223" t="str">
-        <v>Step Size</v>
+        <v>Frequency</v>
       </c>
       <c r="C223" t="str">
-        <v>步长</v>
+        <v>频率</v>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="str">
-        <v>settings.column.datamining-menu.options.frequency</v>
+        <v>settings.column.datamining-menu.options.max-val</v>
       </c>
       <c r="B224" t="str">
-        <v>Frequency</v>
+        <v>Maximum Value</v>
       </c>
       <c r="C224" t="str">
-        <v>频率</v>
+        <v>最大值</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="str">
-        <v>settings.column.datamining-menu.options.max-val</v>
+        <v>settings.column.datamining-menu.options.min-val</v>
       </c>
       <c r="B225" t="str">
-        <v>Maximum Value</v>
+        <v>Minimum Value</v>
       </c>
       <c r="C225" t="str">
-        <v>最大值</v>
+        <v>最小值</v>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="str">
-        <v>settings.column.datamining-menu.options.min-val</v>
+        <v>settings.column.datamining-menu.options.avg-val</v>
       </c>
       <c r="B226" t="str">
-        <v>Minimum Value</v>
+        <v>Average Value</v>
       </c>
       <c r="C226" t="str">
-        <v>最小值</v>
+        <v>平均值</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="str">
-        <v>settings.column.datamining-menu.options.avg-val</v>
+        <v>settings.column.datamining-menu.options.roc</v>
       </c>
       <c r="B227" t="str">
-        <v>Average Value</v>
+        <v>Rate of Change</v>
       </c>
       <c r="C227" t="str">
-        <v>平均值</v>
+        <v>变化率</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="str">
-        <v>settings.column.datamining-menu.options.roc</v>
+        <v>settings.column.datamining-menu.options.freq-of-LAD</v>
       </c>
       <c r="B228" t="str">
-        <v>Rate of Change</v>
+        <v>Frequency of LAD</v>
       </c>
       <c r="C228" t="str">
-        <v>变化率</v>
+        <v>LAD 频率</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="str">
-        <v>settings.column.datamining-menu.options.freq-of-LAD</v>
+        <v>settings.column.datamining-menu.options.freq-of-FAD</v>
       </c>
       <c r="B229" t="str">
-        <v>Frequency of LAD</v>
+        <v>Frequency of FAD</v>
       </c>
       <c r="C229" t="str">
-        <v>LAD 频率</v>
+        <v>FAD 频率</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="str">
-        <v>settings.column.datamining-menu.options.freq-of-FAD</v>
+        <v>settings.column.datamining-menu.options.combined-events</v>
       </c>
       <c r="B230" t="str">
-        <v>Frequency of FAD</v>
+        <v>Combined Events</v>
       </c>
       <c r="C230" t="str">
-        <v>FAD 频率</v>
+        <v>组合事件</v>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="str">
-        <v>settings.column.datamining-menu.options.combined-events</v>
+        <v>settings.column.datamining-menu.options-title.event</v>
       </c>
       <c r="B231" t="str">
-        <v>Combined Events</v>
+        <v>Event Type</v>
       </c>
       <c r="C231" t="str">
-        <v>组合事件</v>
+        <v>事件类型</v>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="str">
-        <v>settings.column.datamining-menu.options-title.event</v>
+        <v>settings.column.datamining-menu.options-title.chron</v>
       </c>
       <c r="B232" t="str">
-        <v>Event Type</v>
+        <v>Chron Type</v>
       </c>
       <c r="C232" t="str">
-        <v>事件类型</v>
+        <v>年代类型</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="str">
-        <v>settings.column.datamining-menu.options-title.chron</v>
+        <v>settings.column.datamining-menu.options-title.plot</v>
       </c>
       <c r="B233" t="str">
-        <v>Chron Type</v>
+        <v>Data Type to Plot</v>
       </c>
       <c r="C233" t="str">
-        <v>年代类型</v>
+        <v>绘制数据类型</v>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="str">
-        <v>settings.column.datamining-menu.options-title.plot</v>
+        <v>settings.column.curve-drawing-menu.title</v>
       </c>
       <c r="B234" t="str">
-        <v>Data Type to Plot</v>
+        <v>Point Settings</v>
       </c>
       <c r="C234" t="str">
-        <v>绘制数据类型</v>
+        <v>点设置</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="str">
-        <v>settings.column.curve-drawing-menu.title</v>
+        <v>settings.column.curve-drawing-menu.rod</v>
       </c>
       <c r="B235" t="str">
-        <v>Point Settings</v>
+        <v>Range of Data</v>
       </c>
       <c r="C235" t="str">
-        <v>点设置</v>
+        <v>数据范围</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="str">
-        <v>settings.column.curve-drawing-menu.rod</v>
+        <v>settings.column.curve-drawing-menu.lower-range</v>
       </c>
       <c r="B236" t="str">
-        <v>Range of Data</v>
+        <v>Lower Range</v>
       </c>
       <c r="C236" t="str">
-        <v>数据范围</v>
+        <v>下限</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="str">
-        <v>settings.column.curve-drawing-menu.lower-range</v>
+        <v>settings.column.curve-drawing-menu.upper-range</v>
       </c>
       <c r="B237" t="str">
-        <v>Lower Range</v>
+        <v>Upper Range</v>
       </c>
       <c r="C237" t="str">
-        <v>下限</v>
+        <v>上限</v>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="str">
-        <v>settings.column.curve-drawing-menu.upper-range</v>
+        <v>settings.column.curve-drawing-menu.scale-start</v>
       </c>
       <c r="B238" t="str">
-        <v>Upper Range</v>
+        <v>Scale Start</v>
       </c>
       <c r="C238" t="str">
-        <v>上限</v>
+        <v>刻度起点</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="str">
-        <v>settings.column.curve-drawing-menu.scale-start</v>
+        <v>settings.column.curve-drawing-menu.scale-step</v>
       </c>
       <c r="B239" t="str">
-        <v>Scale Start</v>
+        <v>Scale Step</v>
       </c>
       <c r="C239" t="str">
-        <v>刻度起点</v>
+        <v>刻度步长</v>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="str">
-        <v>settings.column.curve-drawing-menu.scale-step</v>
+        <v>settings.column.curve-drawing-menu.show-scale</v>
       </c>
       <c r="B240" t="str">
-        <v>Scale Step</v>
+        <v>Show Scale</v>
       </c>
       <c r="C240" t="str">
-        <v>刻度步长</v>
+        <v>显示刻度</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="str">
-        <v>settings.column.curve-drawing-menu.show-scale</v>
+        <v>settings.column.curve-drawing-menu.draw-points</v>
       </c>
       <c r="B241" t="str">
-        <v>Show Scale</v>
+        <v>Draw Points</v>
       </c>
       <c r="C241" t="str">
-        <v>显示刻度</v>
+        <v>绘制点</v>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="str">
-        <v>settings.column.curve-drawing-menu.draw-points</v>
+        <v>settings.column.curve-drawing-menu.point-shape</v>
       </c>
       <c r="B242" t="str">
-        <v>Draw Points</v>
+        <v>Point Shape</v>
       </c>
       <c r="C242" t="str">
-        <v>绘制点</v>
+        <v>点形状</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="str">
-        <v>settings.column.curve-drawing-menu.point-shape</v>
+        <v>settings.column.curve-drawing-menu.line</v>
       </c>
       <c r="B243" t="str">
-        <v>Point Shape</v>
+        <v>Line</v>
       </c>
       <c r="C243" t="str">
-        <v>点形状</v>
+        <v>线条</v>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="str">
-        <v>settings.column.curve-drawing-menu.line</v>
+        <v>settings.column.curve-drawing-menu.fill</v>
       </c>
       <c r="B244" t="str">
-        <v>Line</v>
+        <v>Fill</v>
       </c>
       <c r="C244" t="str">
-        <v>线条</v>
+        <v>填充</v>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="str">
-        <v>settings.column.curve-drawing-menu.fill</v>
+        <v>settings.column.curve-drawing-menu.background-gradient</v>
       </c>
       <c r="B245" t="str">
-        <v>Fill</v>
+        <v>Background Gradient</v>
       </c>
       <c r="C245" t="str">
-        <v>填充</v>
+        <v>背景渐变</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="str">
-        <v>settings.column.curve-drawing-menu.background-gradient</v>
+        <v>settings.column.curve-drawing-menu.curve-gradient</v>
       </c>
       <c r="B246" t="str">
-        <v>Background Gradient</v>
+        <v>Curve Gradient</v>
       </c>
       <c r="C246" t="str">
-        <v>背景渐变</v>
+        <v>曲线渐变</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="str">
-        <v>settings.column.curve-drawing-menu.curve-gradient</v>
+        <v>settings.column.curve-drawing-menu.start</v>
       </c>
       <c r="B247" t="str">
-        <v>Curve Gradient</v>
+        <v>Start</v>
       </c>
       <c r="C247" t="str">
-        <v>曲线渐变</v>
+        <v>起点</v>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="str">
-        <v>settings.column.curve-drawing-menu.start</v>
+        <v>settings.column.curve-drawing-menu.end</v>
       </c>
       <c r="B248" t="str">
-        <v>Start</v>
+        <v>End</v>
       </c>
       <c r="C248" t="str">
-        <v>起点</v>
+        <v>终点</v>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="str">
-        <v>settings.column.curve-drawing-menu.end</v>
+        <v>settings.search.search-bar</v>
       </c>
       <c r="B249" t="str">
-        <v>End</v>
+        <v>Search</v>
       </c>
       <c r="C249" t="str">
-        <v>终点</v>
+        <v>搜索</v>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="str">
-        <v>settings.column.overlay-menu.title</v>
+        <v>settings.search.found-result</v>
       </c>
       <c r="B250" t="str">
-        <v>Overlay Settings</v>
+        <v>Found {{count}} Results</v>
+      </c>
+      <c r="C250" t="str">
+        <v>找到 {{count}} 个结果</v>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="str">
-        <v>settings.column.overlay-menu.display-overlay</v>
+        <v>settings.search.current-time-settings</v>
       </c>
       <c r="B251" t="str">
-        <v>Display Overlay</v>
+        <v>Current Time Settings(Top / Base)</v>
+      </c>
+      <c r="C251" t="str">
+        <v>当前时间区间设置(顶部 / 底部)</v>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="str">
-        <v>settings.column.overlay-menu.overlay-column-header</v>
+        <v>settings.search.header.status</v>
       </c>
       <c r="B252" t="str">
-        <v>Overlaying</v>
+        <v>Column On?</v>
+      </c>
+      <c r="C252" t="str">
+        <v>是否已选</v>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="str">
-        <v>settings.column.overlay-menu.overlay-column-preposition</v>
+        <v>settings.search.header.center</v>
       </c>
       <c r="B253" t="str">
-        <v>On</v>
+        <v>Center</v>
+      </c>
+      <c r="C253" t="str">
+        <v>居中</v>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="str">
-        <v>settings.column.overlay-menu.overlay-accordion-caption</v>
+        <v>settings.search.header.extend</v>
       </c>
       <c r="B254" t="str">
-        <v>*Grayed out columns are disabled for Overlay (not Event or Point column)</v>
+        <v>Extend</v>
+      </c>
+      <c r="C254" t="str">
+        <v>延展</v>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="str">
-        <v>settings.column.overlay-menu.invalid-column-mouseover</v>
+        <v>settings.search.header.column</v>
       </c>
       <c r="B255" t="str">
-        <v>Not an Event or Point Column</v>
+        <v>Column</v>
+      </c>
+      <c r="C255" t="str">
+        <v>列名称</v>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="str">
-        <v>settings.column.overlay-menu.column-not-selected</v>
+        <v>settings.search.header.age</v>
       </c>
       <c r="B256" t="str">
-        <v>Select Column from Menu</v>
+        <v>Age</v>
+      </c>
+      <c r="C256" t="str">
+        <v>年代</v>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="str">
-        <v>settings.search.search-bar</v>
+        <v>settings.search.header.qualifier</v>
       </c>
       <c r="B257" t="str">
-        <v>Search</v>
+        <v>Type</v>
       </c>
       <c r="C257" t="str">
-        <v>搜索</v>
+        <v>类别</v>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="str">
-        <v>settings.search.found-result</v>
+        <v>settings.search.header.notes</v>
       </c>
       <c r="B258" t="str">
-        <v>Found {{count}} Results</v>
+        <v>Notes</v>
       </c>
       <c r="C258" t="str">
-        <v>找到 {{count}} 个结果</v>
+        <v>注释</v>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="str">
-        <v>settings.search.current-time-settings</v>
+        <v>settings.font.notes1</v>
       </c>
       <c r="B259" t="str">
-        <v>Current Time Settings(Top / Base)</v>
+        <v>These are the default systemwide fonts.</v>
       </c>
       <c r="C259" t="str">
-        <v>当前时间区间设置(顶部 / 底部)</v>
+        <v>这些是系统默认的全局字体</v>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="str">
-        <v>settings.search.header.status</v>
+        <v>settings.font.notes2</v>
       </c>
       <c r="B260" t="str">
-        <v>Column On?</v>
+        <v>Changing one here will affect the entire chart.</v>
       </c>
       <c r="C260" t="str">
-        <v>是否已选</v>
+        <v>在此处更改字体会影响整个图表</v>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="str">
-        <v>settings.search.header.center</v>
+        <v>settings.font.notes3</v>
       </c>
       <c r="B261" t="str">
-        <v>Center</v>
+        <v>NOTE: These fonts can be changed on a column by column basis by using the Font button for each column</v>
       </c>
       <c r="C261" t="str">
-        <v>居中</v>
+        <v>注意：可以通过每列的“字体”按钮单独更改每列的字体</v>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="str">
-        <v>settings.search.header.extend</v>
+        <v>settings.map-points.not-avaliable</v>
       </c>
       <c r="B262" t="str">
-        <v>Extend</v>
+        <v>No Map Points available for this datapack</v>
       </c>
       <c r="C262" t="str">
-        <v>延展</v>
+        <v>该数据包暂无地图可用</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="str">
-        <v>settings.search.header.column</v>
+        <v>settings.datapacks.see-info-guidance</v>
       </c>
       <c r="B263" t="str">
-        <v>Column</v>
+        <v>Click a datapack to see more information!</v>
       </c>
       <c r="C263" t="str">
-        <v>列名称</v>
+        <v>点击数据包以查看更多信息！</v>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="str">
-        <v>settings.search.header.age</v>
+        <v>settings.datapacks.add-datapack-guidance</v>
       </c>
       <c r="B264" t="str">
-        <v>Age</v>
+        <v>Add a datapack by clicking the checkbox</v>
       </c>
       <c r="C264" t="str">
-        <v>年代</v>
+        <v>点击加号添加数据包</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="str">
-        <v>settings.search.header.qualifier</v>
+        <v>settings.datapacks.title.private-official</v>
       </c>
       <c r="B265" t="str">
-        <v>Type</v>
-      </c>
-      <c r="C265" t="str">
-        <v>类别</v>
+        <v>Private Official Datapacks</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="str">
-        <v>settings.search.header.notes</v>
+        <v>settings.datapacks.title.public-official</v>
       </c>
       <c r="B266" t="str">
-        <v>Notes</v>
-      </c>
-      <c r="C266" t="str">
-        <v>注释</v>
+        <v>Official Datapacks</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="str">
-        <v>settings.font.notes1</v>
+        <v>settings.datapacks.title.contributed</v>
       </c>
       <c r="B267" t="str">
-        <v>These are the default systemwide fonts.</v>
-      </c>
-      <c r="C267" t="str">
-        <v>这些是系统默认的全局字体</v>
+        <v>User Contributed Datapacks</v>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="str">
-        <v>settings.font.notes2</v>
+        <v>settings.datapacks.title.workshop</v>
       </c>
       <c r="B268" t="str">
-        <v>Changing one here will affect the entire chart.</v>
+        <v>Workshop Datapacks</v>
       </c>
       <c r="C268" t="str">
-        <v>在此处更改字体会影响整个图表</v>
+        <v>工作坊数据包</v>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="str">
-        <v>settings.font.notes3</v>
+        <v>settings.datapacks.title.your</v>
       </c>
       <c r="B269" t="str">
-        <v>NOTE: These fonts can be changed on a column by column basis by using the Font button for each column</v>
+        <v>Your Datapacks</v>
       </c>
       <c r="C269" t="str">
-        <v>注意：可以通过每列的“字体”按钮单独更改每列的字体</v>
+        <v>你的数据包</v>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="str">
-        <v>settings.map-points.not-avaliable</v>
+        <v>settings.datapacks.no</v>
       </c>
       <c r="B270" t="str">
-        <v>No Map Points available for this datapack</v>
+        <v>No</v>
       </c>
       <c r="C270" t="str">
-        <v>该数据包暂无地图可用</v>
+        <v>暂无</v>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="str">
-        <v>settings.datapacks.see-info-guidance</v>
+        <v>settings.datapacks.avaliable</v>
       </c>
       <c r="B271" t="str">
-        <v>Click a datapack to see more information!</v>
+        <v>Avaliable</v>
       </c>
       <c r="C271" t="str">
-        <v>点击数据包以查看更多信息！</v>
+        <v>可用</v>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="str">
-        <v>settings.datapacks.add-datapack-guidance</v>
+        <v>settings.datapacks.upload</v>
       </c>
       <c r="B272" t="str">
-        <v>Add a datapack by clicking the checkbox</v>
+        <v>Upload Datapack</v>
       </c>
       <c r="C272" t="str">
-        <v>点击加号添加数据包</v>
+        <v>上传数据包</v>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="str">
-        <v>settings.datapacks.title.private-official</v>
+        <v>settings.datapacks.pdf-upload</v>
       </c>
       <c r="B273" t="str">
-        <v>Private Official Datapacks</v>
+        <v>PDF Upload</v>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="str">
-        <v>settings.datapacks.title.public-official</v>
+        <v>settings.datapacks.seeMore</v>
       </c>
       <c r="B274" t="str">
-        <v>Official Datapacks</v>
+        <v>See More...</v>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="str">
-        <v>settings.datapacks.title.contributed</v>
+        <v>settings.datapacks.seeLess</v>
       </c>
       <c r="B275" t="str">
-        <v>User Contributed Datapacks</v>
+        <v>See Less...</v>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="str">
-        <v>settings.datapacks.title.workshop</v>
+        <v>settings.datapacks.upload-form.title</v>
       </c>
       <c r="B276" t="str">
-        <v>Workshop Datapacks</v>
+        <v>Upload Your Own Datapack</v>
       </c>
       <c r="C276" t="str">
-        <v>工作坊数据包</v>
+        <v>上传你的数据包</v>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="str">
-        <v>settings.datapacks.title.your</v>
+        <v>settings.datapacks.upload-form.no-file</v>
       </c>
       <c r="B277" t="str">
-        <v>Your Datapacks</v>
+        <v>No file selected</v>
       </c>
       <c r="C277" t="str">
-        <v>你的数据包</v>
+        <v>没有选择文件</v>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="str">
-        <v>settings.datapacks.title.treatise</v>
+        <v>settings.datapacks.upload-form.name</v>
       </c>
       <c r="B278" t="str">
-        <v>Treatise Datapacks</v>
+        <v>Datapack Name</v>
+      </c>
+      <c r="C278" t="str">
+        <v>数据包名称</v>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="str">
-        <v>settings.datapacks.no</v>
+        <v>settings.datapacks.upload-form.name-placeholder</v>
       </c>
       <c r="B279" t="str">
-        <v>No</v>
+        <v>Enter a name for your datapack.</v>
       </c>
       <c r="C279" t="str">
-        <v>暂无</v>
+        <v>请为你的数据包输入名称</v>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="str">
-        <v>settings.datapacks.avaliable</v>
+        <v>settings.datapacks.upload-form.author</v>
       </c>
       <c r="B280" t="str">
-        <v>Avaliable</v>
+        <v>Authored By</v>
       </c>
       <c r="C280" t="str">
-        <v>可用</v>
+        <v>作者</v>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="str">
-        <v>settings.datapacks.upload</v>
+        <v>settings.datapacks.upload-form.author-placeholder</v>
       </c>
       <c r="B281" t="str">
-        <v>Upload Datapack</v>
+        <v>Credited to...</v>
       </c>
       <c r="C281" t="str">
-        <v>上传数据包</v>
+        <v>作者为...</v>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="str">
-        <v>settings.datapacks.seeMore</v>
+        <v>settings.datapacks.upload-form.description</v>
       </c>
       <c r="B282" t="str">
-        <v>See More...</v>
+        <v>Datapack Description</v>
+      </c>
+      <c r="C282" t="str">
+        <v>数据包概述</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="str">
-        <v>settings.datapacks.seeLess</v>
+        <v>settings.datapacks.upload-form.description-placeholder</v>
       </c>
       <c r="B283" t="str">
-        <v>See Less...</v>
+        <v>Enter a description for your datapack.</v>
+      </c>
+      <c r="C283" t="str">
+        <v>请为你的数据包添加概述</v>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="str">
-        <v>settings.datapacks.upload-form.title</v>
+        <v>settings.datapacks.upload-form.tags</v>
       </c>
       <c r="B284" t="str">
-        <v>Upload Your Own Datapack</v>
+        <v>Tags</v>
       </c>
       <c r="C284" t="str">
-        <v>上传你的数据包</v>
+        <v>标签</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="str">
-        <v>settings.datapacks.upload-form.no-file</v>
+        <v>settings.datapacks.upload-form.make-public</v>
       </c>
       <c r="B285" t="str">
-        <v>No file selected</v>
+        <v>Make Datapack Publicly Accessible</v>
       </c>
       <c r="C285" t="str">
-        <v>没有选择文件</v>
+        <v>使数据包对公共可见</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="str">
-        <v>settings.datapacks.upload-form.name</v>
+        <v>settings.datapacks.upload-form.button.add-ref</v>
       </c>
       <c r="B286" t="str">
-        <v>Datapack Name</v>
+        <v>Add Reference</v>
       </c>
       <c r="C286" t="str">
-        <v>数据包名称</v>
+        <v>添加引用</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="str">
-        <v>settings.datapacks.upload-form.name-placeholder</v>
+        <v>settings.datapacks.upload-form.button.more</v>
       </c>
       <c r="B287" t="str">
-        <v>Enter a name for your datapack.</v>
+        <v>More Options</v>
       </c>
       <c r="C287" t="str">
-        <v>请为你的数据包输入名称</v>
+        <v>更多选项</v>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="str">
-        <v>settings.datapacks.upload-form.author</v>
+        <v>settings.datapacks.upload-form.button.finish</v>
       </c>
       <c r="B288" t="str">
-        <v>Authored By</v>
+        <v>Finish &amp; Upload</v>
       </c>
       <c r="C288" t="str">
-        <v>作者</v>
+        <v>完成并上传</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="str">
-        <v>settings.datapacks.upload-form.author-placeholder</v>
+        <v>settings.datapacks.upload-form.button.startover</v>
       </c>
       <c r="B289" t="str">
-        <v>Credited to...</v>
+        <v>Start Over</v>
       </c>
       <c r="C289" t="str">
-        <v>作者为...</v>
+        <v>重新开始</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="str">
-        <v>settings.datapacks.upload-form.description</v>
+        <v>settings.datapacks.upload-form.reference</v>
       </c>
       <c r="B290" t="str">
-        <v>Datapack Description</v>
+        <v>Reference</v>
       </c>
       <c r="C290" t="str">
-        <v>数据包概述</v>
+        <v>引用</v>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="str">
-        <v>settings.datapacks.upload-form.description-placeholder</v>
+        <v>settings.datapacks.upload-form.contact</v>
       </c>
       <c r="B291" t="str">
-        <v>Enter a description for your datapack.</v>
+        <v>Contact</v>
       </c>
       <c r="C291" t="str">
-        <v>请为你的数据包添加概述</v>
+        <v>联系方式</v>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="str">
-        <v>settings.datapacks.upload-form.tags</v>
+        <v>settings.datapacks.upload-form.contact-placeholder</v>
       </c>
       <c r="B292" t="str">
-        <v>Tags</v>
+        <v>Enter your contact information</v>
       </c>
       <c r="C292" t="str">
-        <v>标签</v>
+        <v>输入你的联系方式</v>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="str">
-        <v>settings.datapacks.upload-form.make-public</v>
+        <v>settings.datapacks.upload-form.contact-helper-text</v>
       </c>
       <c r="B293" t="str">
-        <v>Make Datapack Publicly Accessible</v>
+        <v>(OPTIONAL) If you would like others to contact you about this datapack</v>
       </c>
       <c r="C293" t="str">
-        <v>使数据包对公共可见</v>
+        <v>如果想要其他用户就此数据包问题联系你，请填写</v>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="str">
-        <v>settings.datapacks.upload-form.button.add-ref</v>
+        <v>settings.datapacks.upload-form.notes</v>
       </c>
       <c r="B294" t="str">
-        <v>Add Reference</v>
+        <v>Notes</v>
       </c>
       <c r="C294" t="str">
-        <v>添加引用</v>
+        <v>注释</v>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="str">
-        <v>settings.datapacks.upload-form.button.more</v>
+        <v>settings.datapacks.upload-form.notes-placeholder</v>
       </c>
       <c r="B295" t="str">
-        <v>More Options</v>
+        <v>Enter notes for the datapack here</v>
       </c>
       <c r="C295" t="str">
-        <v>更多选项</v>
+        <v>为你的数据包添加注释</v>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="str">
-        <v>settings.datapacks.upload-form.button.finish</v>
+        <v>settings.datapacks.upload-form.notes-helper-text</v>
       </c>
       <c r="B296" t="str">
-        <v>Finish &amp; Upload</v>
+        <v>(OPTIONAL) Generally notes are settings recommendations/How to use your datapack most efficiently</v>
       </c>
       <c r="C296" t="str">
-        <v>完成并上传</v>
+        <v>如果想要指导其他用户如何有效地使用此数据包，请填写</v>
       </c>
     </row>
     <row r="297">
       <c r="A297" t="str">
-        <v>settings.datapacks.upload-form.button.startover</v>
+        <v>chart.no-chart-yet</v>
       </c>
       <c r="B297" t="str">
-        <v>Start Over</v>
+        <v>You have not made a chart yet</v>
       </c>
       <c r="C297" t="str">
-        <v>重新开始</v>
+        <v>您还未制作任何图表</v>
       </c>
     </row>
     <row r="298">
       <c r="A298" t="str">
-        <v>settings.datapacks.upload-form.reference</v>
+        <v>chart.save</v>
       </c>
       <c r="B298" t="str">
-        <v>Reference</v>
+        <v>Save Chart</v>
       </c>
       <c r="C298" t="str">
-        <v>引用</v>
+        <v>保存图表</v>
       </c>
     </row>
     <row r="299">
       <c r="A299" t="str">
-        <v>settings.datapacks.upload-form.contact</v>
+        <v>dialogs.confirm-datapack-change.title</v>
       </c>
       <c r="B299" t="str">
-        <v>Contact</v>
+        <v>Confirm Datapack Selection Change</v>
       </c>
       <c r="C299" t="str">
-        <v>联系方式</v>
+        <v>确认更改数据包</v>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="str">
-        <v>settings.datapacks.upload-form.contact-placeholder</v>
+        <v>dialogs.confirm-datapack-change.message</v>
       </c>
       <c r="B300" t="str">
-        <v>Enter your contact information</v>
+        <v>You have unsaved changes! Do you want to save your changes?</v>
       </c>
       <c r="C300" t="str">
-        <v>输入你的联系方式</v>
+        <v>你有未保存的更改! 你想保存你的更改吗?</v>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="str">
-        <v>settings.datapacks.upload-form.contact-helper-text</v>
+        <v>dialogs.confirm-datapack-change.yes</v>
       </c>
       <c r="B301" t="str">
-        <v>(OPTIONAL) If you would like others to contact you about this datapack</v>
+        <v>Save</v>
       </c>
       <c r="C301" t="str">
-        <v>如果想要其他用户就此数据包问题联系你，请填写</v>
+        <v>保存</v>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="str">
-        <v>settings.datapacks.upload-form.notes</v>
+        <v>dialogs.confirm-datapack-change.no</v>
       </c>
       <c r="B302" t="str">
-        <v>Notes</v>
+        <v>Discard</v>
       </c>
       <c r="C302" t="str">
-        <v>注释</v>
+        <v>不保存</v>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="str">
-        <v>settings.datapacks.upload-form.notes-placeholder</v>
+        <v>dialogs.default-age.title</v>
       </c>
       <c r="B303" t="str">
-        <v>Enter notes for the datapack here</v>
+        <v>Use default age range?</v>
       </c>
       <c r="C303" t="str">
-        <v>为你的数据包添加注释</v>
+        <v>使用默认时间区间？</v>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="str">
-        <v>settings.datapacks.upload-form.notes-helper-text</v>
+        <v>dialogs.confirm-changes.message</v>
       </c>
       <c r="B304" t="str">
-        <v>(OPTIONAL) Generally notes are settings recommendations/How to use your datapack most efficiently</v>
-      </c>
-      <c r="C304" t="str">
-        <v>如果想要指导其他用户如何有效地使用此数据包，请填写</v>
+        <v>Are you sure you want to discard your changes?</v>
       </c>
     </row>
     <row r="305">
       <c r="A305" t="str">
-        <v>settings.datapacks.pdf-upload</v>
+        <v>help.qsg.title</v>
       </c>
       <c r="B305" t="str">
-        <v>PDF Upload</v>
+        <v>Quick Start Quide</v>
+      </c>
+      <c r="C305" t="str">
+        <v>快速指南</v>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="str">
-        <v>chart.no-chart-yet</v>
+        <v>help.qsg.content</v>
       </c>
       <c r="B306" t="str">
-        <v>You have not made a chart yet</v>
+        <v>Welcome to Time Scale Creator Online! In this Quick Start Guide, you will quickly learn about the functions of each tab on the Nav bar. Click the 'Start QSG' button to begin.</v>
       </c>
       <c r="C306" t="str">
-        <v>您还未制作任何图表</v>
+        <v>欢迎使用Time Scale Creator在线版！在这个快速指南中，您将迅速了解导航栏上每个标签页的功能。点击“开始快速指南”按钮开始体验。</v>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="str">
-        <v>chart.save</v>
+        <v>help.qsg.button</v>
       </c>
       <c r="B307" t="str">
-        <v>Save Chart</v>
+        <v>Start QSG</v>
       </c>
       <c r="C307" t="str">
-        <v>保存图表</v>
+        <v>开始快速指南</v>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="str">
-        <v>dialogs.confirm-datapack-change.title</v>
+        <v>help.tour.title</v>
       </c>
       <c r="B308" t="str">
-        <v>Confirm Datapack Selection Change</v>
+        <v>Tour</v>
       </c>
       <c r="C308" t="str">
-        <v>确认更改数据包</v>
+        <v>导览</v>
       </c>
     </row>
     <row r="309">
       <c r="A309" t="str">
-        <v>dialogs.confirm-datapack-change.message</v>
+        <v>help.tour.content.datapacks</v>
       </c>
       <c r="B309" t="str">
-        <v>You have unsaved changes! Do you want to save your changes?</v>
+        <v>In the datapacks tour you will explore the Datapacks page in depth. Click the button to start your tour!</v>
       </c>
       <c r="C309" t="str">
-        <v>你有未保存的更改! 你想保存你的更改吗?</v>
+        <v>在数据包导览中，您将深入探索数据包页面。点击按钮开始您的导览！</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="str">
-        <v>dialogs.confirm-datapack-change.yes</v>
+        <v>help.tour.content.settings</v>
       </c>
       <c r="B310" t="str">
-        <v>Save</v>
+        <v>In the settings tour you will explore the Settings page in depth. Click the button to start your tour!</v>
       </c>
       <c r="C310" t="str">
-        <v>保存</v>
+        <v>在设置导览中，您将深入探索设置页面。点击按钮开始您的导览！</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="str">
-        <v>dialogs.confirm-datapack-change.no</v>
+        <v>help.tour.button.datapacks</v>
       </c>
       <c r="B311" t="str">
-        <v>Discard</v>
+        <v>Start Datapacks Tour</v>
       </c>
       <c r="C311" t="str">
-        <v>不保存</v>
+        <v>开始数据包导览</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="str">
-        <v>dialogs.default-age.title</v>
+        <v>help.tour.button.settings</v>
       </c>
       <c r="B312" t="str">
-        <v>Use default age range?</v>
+        <v>Start Settings Tour</v>
       </c>
       <c r="C312" t="str">
-        <v>使用默认时间区间？</v>
+        <v>开始设置导览</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="str">
-        <v>dialogs.confirm-changes.message</v>
+        <v>help.license</v>
       </c>
       <c r="B313" t="str">
-        <v>Are you sure you want to discard your changes?</v>
+        <v>Software License</v>
+      </c>
+      <c r="C313" t="str">
+        <v>软件许可</v>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="str">
-        <v>help.qsg.title</v>
+        <v>help.file-format-info.title</v>
       </c>
       <c r="B314" t="str">
-        <v>Quick Start Quide</v>
+        <v>File Format Info</v>
       </c>
       <c r="C314" t="str">
-        <v>快速指南</v>
+        <v>文件格式信息</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="str">
-        <v>help.qsg.content</v>
+        <v>help.file-format-info.link</v>
       </c>
       <c r="B315" t="str">
-        <v>Welcome to Time Scale Creator Online! In this Quick Start Guide, you will quickly learn about the functions of each tab on the Nav bar. Click the 'Start QSG' button to begin.</v>
+        <v>View File Format Info</v>
       </c>
       <c r="C315" t="str">
-        <v>欢迎使用Time Scale Creator在线版！在这个快速指南中，您将迅速了解导航栏上每个标签页的功能。点击“开始快速指南”按钮开始体验。</v>
+        <v>查看文件格式信息</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="str">
-        <v>help.qsg.button</v>
+        <v>errors.title</v>
       </c>
       <c r="B316" t="str">
-        <v>Start QSG</v>
+        <v>Error</v>
       </c>
       <c r="C316" t="str">
-        <v>开始快速指南</v>
+        <v>错误</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="str">
-        <v>help.tour.title</v>
+        <v>errors.SERVER_RESPONSE_ERROR</v>
       </c>
       <c r="B317" t="str">
-        <v>Tour</v>
+        <v>Server response error. Please try again later.</v>
       </c>
       <c r="C317" t="str">
-        <v>导览</v>
+        <v>服务器错误。请稍后再试。</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="str">
-        <v>help.tour.content.datapacks</v>
+        <v>errors.INVALID_DATAPACK_INFO</v>
       </c>
       <c r="B318" t="str">
-        <v>In the datapacks tour you will explore the Datapacks page in depth. Click the button to start your tour!</v>
+        <v>Invalid datapack info received from server. Please try again later.</v>
       </c>
       <c r="C318" t="str">
-        <v>在数据包导览中，您将深入探索数据包页面。点击按钮开始您的导览！</v>
+        <v>从服务器接收到的数据包信息无效。请稍后再试。</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="str">
-        <v>help.tour.content.settings</v>
+        <v>errors.INVALID_PRESET_INFO</v>
       </c>
       <c r="B319" t="str">
-        <v>In the settings tour you will explore the Settings page in depth. Click the button to start your tour!</v>
+        <v>Invalid preset info received from server. Please try again later.</v>
       </c>
       <c r="C319" t="str">
-        <v>在设置导览中，您将深入探索设置页面。点击按钮开始您的导览！</v>
+        <v>从服务器接收到的预置无效。请稍后再试。</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="str">
-        <v>help.tour.button.datapacks</v>
+        <v>errors.INVALID_PATTERN_INFO</v>
       </c>
       <c r="B320" t="str">
-        <v>Start Datapacks Tour</v>
+        <v>Invalid pattern info received from server. Please try again later.</v>
       </c>
       <c r="C320" t="str">
-        <v>开始数据包导览</v>
+        <v>从服务器接收到的模式信息无效。请稍后再试。</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="str">
-        <v>help.tour.button.settings</v>
+        <v>errors.INVALID_TIME_SCALE</v>
       </c>
       <c r="B321" t="str">
-        <v>Start Settings Tour</v>
+        <v>Invalid time scale received from server. Please try again later.</v>
       </c>
       <c r="C321" t="str">
-        <v>开始设置导览</v>
+        <v>从服务器收到的时间刻度无效。请稍后再试。</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="str">
-        <v>help.license</v>
+        <v>errors.INVALID_DATAPACK_CONFIG</v>
       </c>
       <c r="B322" t="str">
-        <v>Software License</v>
+        <v>Datapacks were not properly set. Please try again later.</v>
       </c>
       <c r="C322" t="str">
-        <v>软件许可</v>
+        <v>数据包未正确设置。请稍后再试。</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="str">
-        <v>help.file-format-info.title</v>
+        <v>errors.INVALID_SVG_READY_RESPONSE</v>
       </c>
       <c r="B323" t="str">
-        <v>File Format Info</v>
+        <v>Invalid SVG ready response received from server. Please try again later.</v>
       </c>
       <c r="C323" t="str">
-        <v>文件格式信息</v>
+        <v>从服务器收到的SVG就绪响应无效。请稍后再试。</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="str">
-        <v>help.file-format-info.link</v>
+        <v>errors.INVALID_SETTINGS_RESPONSE</v>
       </c>
       <c r="B324" t="str">
-        <v>View File Format Info</v>
+        <v>Invalid settings response received from server. Please try again later.</v>
       </c>
       <c r="C324" t="str">
-        <v>查看文件格式信息</v>
+        <v>从服务器收到的设置响应无效。请稍后再试。</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="str">
-        <v>errors.title</v>
+        <v>errors.INVALID_CHART_RESPONSE</v>
       </c>
       <c r="B325" t="str">
-        <v>Error</v>
+        <v>Invalid chart response received from server. Please try again later.</v>
       </c>
       <c r="C325" t="str">
-        <v>错误</v>
+        <v>从服务器收到的图表响应无效。请稍后再试。</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" t="str">
-        <v>errors.SERVER_RESPONSE_ERROR</v>
+        <v>errors.INVALID_PATH</v>
       </c>
       <c r="B326" t="str">
-        <v>Server response error. Please try again later.</v>
+        <v>The requested path was invalid. Please ensure the path is correct.</v>
       </c>
       <c r="C326" t="str">
-        <v>服务器错误。请稍后再试。</v>
+        <v>请求的文件路径无效。请确保文件路径正确。</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" t="str">
-        <v>errors.INVALID_DATAPACK_INFO</v>
+        <v>errors.INVALID_DATAPACK_UPLOAD</v>
       </c>
       <c r="B327" t="str">
-        <v>Invalid datapack info received from server. Please try again later.</v>
+        <v>Invalid datapack upload.</v>
       </c>
       <c r="C327" t="str">
-        <v>从服务器接收到的数据包信息无效。请稍后再试。</v>
+        <v>无效的数据包上传</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="str">
-        <v>errors.INVALID_PRESET_INFO</v>
+        <v>errors.REGULAR_USER_UPLOAD_DATAPACK_TOO_LARGE</v>
       </c>
       <c r="B328" t="str">
-        <v>Invalid preset info received from server. Please try again later.</v>
-      </c>
-      <c r="C328" t="str">
-        <v>从服务器接收到的预置无效。请稍后再试。</v>
+        <v>Uploaded datapack is over 3000 characters.</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="str">
-        <v>errors.INVALID_PATTERN_INFO</v>
+        <v>errors.INVALID_USER_DATAPACKS</v>
       </c>
       <c r="B329" t="str">
-        <v>Invalid pattern info received from server. Please try again later.</v>
+        <v>Invalid user datapacks received from server. Please try again later.</v>
       </c>
       <c r="C329" t="str">
-        <v>从服务器接收到的模式信息无效。请稍后再试。</v>
+        <v>从服务器收到的用户数据包无效。请稍后再试。</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="str">
-        <v>errors.INVALID_TIME_SCALE</v>
+        <v>errors.INVALID_PUBLIC_DATAPACKS</v>
       </c>
       <c r="B330" t="str">
-        <v>Invalid time scale received from server. Please try again later.</v>
+        <v>Invalid public datapacks received from server. Please try again later.</v>
       </c>
       <c r="C330" t="str">
-        <v>从服务器收到的时间刻度无效。请稍后再试。</v>
+        <v>从服务器收到的公共数据包无效。请稍后再试。</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="str">
-        <v>errors.INVALID_DATAPACK_CONFIG</v>
+        <v>errors.NO_DATAPACK_FILE_FOUND</v>
       </c>
       <c r="B331" t="str">
-        <v>Datapacks were not properly set. Please try again later.</v>
+        <v>No datapack file found. Please upload a datapack file first.</v>
       </c>
       <c r="C331" t="str">
-        <v>数据包未正确设置。请稍后再试。</v>
+        <v>暂无数据包。请先上传一个数据包。</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="str">
-        <v>errors.INVALID_SVG_READY_RESPONSE</v>
+        <v>errors.DATAPACK_FILE_NAME_TOO_LONG</v>
       </c>
       <c r="B332" t="str">
-        <v>Invalid SVG ready response received from server. Please try again later.</v>
+        <v>Datapack file name is too long. Please shorten the file name.</v>
       </c>
       <c r="C332" t="str">
-        <v>从服务器收到的SVG就绪响应无效。请稍后再试。</v>
+        <v>数据包名称过长。请缩短名称。</v>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="str">
-        <v>errors.INVALID_SETTINGS_RESPONSE</v>
+        <v>errors.UNRECOGNIZED_DATAPACK_EXTENSION</v>
       </c>
       <c r="B333" t="str">
-        <v>Invalid settings response received from server. Please try again later.</v>
+        <v>Unrecognized datapack extension. File must be of type .dpk, .mdpk, .map, .txt. Please upload a valid datapack file.</v>
       </c>
       <c r="C333" t="str">
-        <v>从服务器收到的设置响应无效。请稍后再试。</v>
+        <v>无法识别数据包扩展名。文件必须是 .dpk, .mdpk, .map, .txt格式。请上传有效文件格式。</v>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="str">
-        <v>errors.INVALID_CHART_RESPONSE</v>
+        <v>errors.UNRECOGNIZED_DATAPACK_FILE</v>
       </c>
       <c r="B334" t="str">
-        <v>Invalid chart response received from server. Please try again later.</v>
+        <v>Unrecognized datapack file. Please upload a valid datapack file.</v>
       </c>
       <c r="C334" t="str">
-        <v>从服务器收到的图表响应无效。请稍后再试。</v>
+        <v>无法识别数据包。请上传有效文件。</v>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="str">
-        <v>errors.INVALID_PATH</v>
+        <v>errors.UNFINISHED_DATAPACK_UPLOAD_FORM</v>
       </c>
       <c r="B335" t="str">
-        <v>The requested path was invalid. Please ensure the path is correct.</v>
+        <v>Please finish the datapack upload form before attempting to upload the file.</v>
       </c>
       <c r="C335" t="str">
-        <v>请求的文件路径无效。请确保文件路径正确。</v>
+        <v>请完成数据包上传表单后再尝试上传文件。</v>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="str">
-        <v>errors.INVALID_DATAPACK_UPLOAD</v>
+        <v>errors.DATAPACK_ALREADY_EXISTS</v>
       </c>
       <c r="B336" t="str">
-        <v>Invalid datapack upload.</v>
+        <v>Datapack already exists. Please upload a datapack with a unique title.</v>
       </c>
       <c r="C336" t="str">
-        <v>无效的数据包上传</v>
+        <v>数据包已存在。请上传不重名的数据包。</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="str">
-        <v>errors.INVALID_DATAPACK_PHYLUM</v>
+        <v>errors.NO_DATAPACKS_SELECTED</v>
       </c>
       <c r="B337" t="str">
-        <v>Invalid treatise datapack phylum provided.</v>
+        <v>No datapacks selected. Please select at least one datapack to generate.</v>
+      </c>
+      <c r="C337" t="str">
+        <v>未选择数据包。请至少选择一个数据包进行绘制。</v>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="str">
-        <v>errors.REGULAR_USER_UPLOAD_DATAPACK_TOO_LARGE</v>
+        <v>errors.NO_COLUMNS_SELECTED</v>
       </c>
       <c r="B338" t="str">
-        <v>Uploaded datapack is over 3000 characters.</v>
+        <v>No columns selected. Please select at least one column to generate.</v>
+      </c>
+      <c r="C338" t="str">
+        <v>未选择列。请至少选择一个列进行绘制。</v>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="str">
-        <v>errors.INVALID_USER_DATAPACKS</v>
+        <v>errors.IS_BAD_RANGE</v>
       </c>
       <c r="B339" t="str">
-        <v>Invalid user datapacks received from server. Please try again later.</v>
+        <v>Base age must be greater than the top age.</v>
       </c>
       <c r="C339" t="str">
-        <v>从服务器收到的用户数据包无效。请稍后再试。</v>
+        <v>区间底部年代应大于区间顶部年代。</v>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="str">
-        <v>errors.INVALID_PUBLIC_DATAPACKS</v>
+        <v>errors.INVALID_MAPPACK_INFO</v>
       </c>
       <c r="B340" t="str">
-        <v>Invalid public datapacks received from server. Please try again later.</v>
+        <v>Invalid mappack info received from server. Please try again later.</v>
       </c>
       <c r="C340" t="str">
-        <v>从服务器收到的公共数据包无效。请稍后再试。</v>
+        <v>从服务器接收到无效的地图包信息。请稍后再试。</v>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="str">
-        <v>errors.NO_DATAPACK_FILE_FOUND</v>
+        <v>errors.UNABLE_TO_LOGIN_SERVER</v>
       </c>
       <c r="B341" t="str">
-        <v>No datapack file found. Please upload a datapack file first.</v>
+        <v>Unable to login due to server error. Please try again later.</v>
       </c>
       <c r="C341" t="str">
-        <v>暂无数据包。请先上传一个数据包。</v>
+        <v>由于服务器错误无法登陆。请稍后再试。</v>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="str">
-        <v>errors.DATAPACK_FILE_NAME_TOO_LONG</v>
+        <v>errors.UNABLE_TO_LOGIN_GOOGLE_CREDENTIAL</v>
       </c>
       <c r="B342" t="str">
-        <v>Datapack file name is too long. Please shorten the file name.</v>
+        <v>Unable to login with Google credentials. Please try again.</v>
       </c>
       <c r="C342" t="str">
-        <v>数据包名称过长。请缩短名称。</v>
+        <v>无法使用Google登陆。请稍后再试。</v>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="str">
-        <v>errors.UNRECOGNIZED_DATAPACK_EXTENSION</v>
+        <v>errors.UNABLE_TO_LOGIN_USERNAME_OR_PASSWORD</v>
       </c>
       <c r="B343" t="str">
-        <v>Unrecognized datapack extension. File must be of type .dpk, .mdpk, .map, .txt. Please upload a valid datapack file.</v>
+        <v>Invalid username or password. Please try again.</v>
       </c>
       <c r="C343" t="str">
-        <v>无法识别数据包扩展名。文件必须是 .dpk, .mdpk, .map, .txt格式。请上传有效文件格式。</v>
+        <v>无效的用户名或密码。请稍后再试。</v>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="str">
-        <v>errors.UNRECOGNIZED_DATAPACK_FILE</v>
+        <v>errors.UNABLE_TO_LOGIN_EXISTING_USER</v>
       </c>
       <c r="B344" t="str">
-        <v>Unrecognized datapack file. Please upload a valid datapack file.</v>
+        <v>User with that email already exists. Please log in or sign up with a different email.</v>
       </c>
       <c r="C344" t="str">
-        <v>无法识别数据包。请上传有效文件。</v>
+        <v>已存在使用该电子邮件的用户。请登录或使用其他电子邮件注册。</v>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="str">
-        <v>errors.UNFINISHED_DATAPACK_UPLOAD_FORM</v>
+        <v>errors.UNABLE_TO_LOGOUT</v>
       </c>
       <c r="B345" t="str">
-        <v>Please finish the datapack upload form before attempting to upload the file.</v>
+        <v>Unable to logout. Please try again later.</v>
       </c>
       <c r="C345" t="str">
-        <v>请完成数据包上传表单后再尝试上传文件。</v>
+        <v>无法登出。请稍后再试。</v>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="str">
-        <v>errors.DATAPACK_ALREADY_EXISTS</v>
+        <v>errors.UNABLE_TO_SIGNUP_SERVER</v>
       </c>
       <c r="B346" t="str">
-        <v>Datapack already exists. Please upload a datapack with a unique title.</v>
+        <v>Unable to sign up due to server error. Please try again later.</v>
       </c>
       <c r="C346" t="str">
-        <v>数据包已存在。请上传不重名的数据包。</v>
+        <v>由于服务器错误无法注册。请稍后再试。</v>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="str">
-        <v>errors.NO_DATAPACKS_SELECTED</v>
+        <v>errors.UNABLE_TO_SIGNUP_USERNAME_OR_EMAIL</v>
       </c>
       <c r="B347" t="str">
-        <v>No datapacks selected. Please select at least one datapack to generate.</v>
+        <v>Email or username already exists. Please try again with a different email or username.</v>
       </c>
       <c r="C347" t="str">
-        <v>未选择数据包。请至少选择一个数据包进行绘制。</v>
+        <v>电子邮件或用户名已存在。请使用不同的电子邮件或用户名重试。</v>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="str">
-        <v>errors.NO_COLUMNS_SELECTED</v>
+        <v>errors.INVALID_FORM</v>
       </c>
       <c r="B348" t="str">
-        <v>No columns selected. Please select at least one column to generate.</v>
+        <v>Invalid form. Please ensure all fields are filled out correctly.</v>
       </c>
       <c r="C348" t="str">
-        <v>未选择列。请至少选择一个列进行绘制。</v>
+        <v>表格无效。请确保所有栏目填写正确。</v>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="str">
-        <v>errors.IS_BAD_RANGE</v>
+        <v>errors.UNABLE_TO_VERIFY_ACCOUNT</v>
       </c>
       <c r="B349" t="str">
-        <v>Base age must be greater than the top age.</v>
+        <v>Your email is not verified. Please verify your email first. If you did not receive an email, please resend.</v>
       </c>
       <c r="C349" t="str">
-        <v>区间底部年代应大于区间顶部年代。</v>
+        <v>您的电子邮件未经验证。请先验证您的电子邮件。如果您没有收到电子邮件，请重新发送。</v>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="str">
-        <v>errors.INVALID_MAPPACK_INFO</v>
+        <v>errors.ALREADY_VERIFIED_ACCOUNT</v>
       </c>
       <c r="B350" t="str">
-        <v>Invalid mappack info received from server. Please try again later.</v>
+        <v>Account is already verified. Please log in.</v>
       </c>
       <c r="C350" t="str">
-        <v>从服务器接收到无效的地图包信息。请稍后再试。</v>
+        <v>帐户已验证。请登录。</v>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="str">
-        <v>errors.UNABLE_TO_LOGIN_SERVER</v>
+        <v>errors.UNABLE_TO_VERIFY_ACCOUNT_SERVER</v>
       </c>
       <c r="B351" t="str">
-        <v>Unable to login due to server error. Please try again later.</v>
+        <v>Unable to verify account due to server error. Please try again later.</v>
       </c>
       <c r="C351" t="str">
-        <v>由于服务器错误无法登陆。请稍后再试。</v>
+        <v>由于服务器错误，无法验证帐户。请稍后再试。</v>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="str">
-        <v>errors.UNABLE_TO_LOGIN_GOOGLE_CREDENTIAL</v>
+        <v>errors.TOKEN_EXPIRED_OR_INVALID</v>
       </c>
       <c r="B352" t="str">
-        <v>Unable to login with Google credentials. Please try again.</v>
+        <v>Your token is either invalid or has expired. Please request a new verification email.</v>
       </c>
       <c r="C352" t="str">
-        <v>无法使用Google登陆。请稍后再试。</v>
+        <v>您的令牌无效或已过期。请申请新的验证电子邮件。</v>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="str">
-        <v>errors.UNABLE_TO_LOGIN_USERNAME_OR_PASSWORD</v>
+        <v>errors.UNABLE_TO_SEND_EMAIL</v>
       </c>
       <c r="B353" t="str">
-        <v>Invalid username or password. Please try again.</v>
+        <v>Unable to send email. Please try again later.</v>
       </c>
       <c r="C353" t="str">
-        <v>无效的用户名或密码。请稍后再试。</v>
+        <v>无法发送邮件。请稍后再试。</v>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="str">
-        <v>errors.UNABLE_TO_LOGIN_EXISTING_USER</v>
+        <v>errors.UNABLE_TO_RESET_PASSWORD</v>
       </c>
       <c r="B354" t="str">
-        <v>User with that email already exists. Please log in or sign up with a different email.</v>
+        <v>Unable to reset password. Please try again later.</v>
       </c>
       <c r="C354" t="str">
-        <v>已存在使用该电子邮件的用户。请登录或使用其他电子邮件注册。</v>
+        <v>无法重置密码。请稍后再试。</v>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="str">
-        <v>errors.UNABLE_TO_LOGOUT</v>
+        <v>errors.UNABLE_TO_RESET_EMAIL</v>
       </c>
       <c r="B355" t="str">
-        <v>Unable to logout. Please try again later.</v>
+        <v>Unable to reset email. Please try again later.</v>
       </c>
       <c r="C355" t="str">
-        <v>无法登出。请稍后再试。</v>
+        <v>无法重置邮箱。请稍后再试。</v>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="str">
-        <v>errors.UNABLE_TO_SIGNUP_SERVER</v>
+        <v>errors.UNABLE_TO_LOGIN_ACCOUNT_LOCKED</v>
       </c>
       <c r="B356" t="str">
-        <v>Unable to sign up due to server error. Please try again later.</v>
+        <v>Your account has been locked. Please check your email for more information or contact support.</v>
       </c>
       <c r="C356" t="str">
-        <v>由于服务器错误无法注册。请稍后再试。</v>
+        <v>您的账户已被锁定。请查看您的电子邮件以获取更多信息或联系技术支持获得帮助。</v>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="str">
-        <v>errors.UNABLE_TO_SIGNUP_USERNAME_OR_EMAIL</v>
+        <v>errors.UNABLE_TO_RECOVER_ACCOUNT</v>
       </c>
       <c r="B357" t="str">
-        <v>Email or username already exists. Please try again with a different email or username.</v>
+        <v>Unable to recover account. Please contact support for more information.</v>
       </c>
       <c r="C357" t="str">
-        <v>电子邮件或用户名已存在。请使用不同的电子邮件或用户名重试。</v>
+        <v>无法恢复账户。请联系技术支持获取更多信息。</v>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="str">
-        <v>errors.INVALID_FORM</v>
+        <v>errors.NOT_LOGGED_IN</v>
       </c>
       <c r="B358" t="str">
-        <v>Invalid form. Please ensure all fields are filled out correctly.</v>
+        <v>You are not logged in. Please log in to access this page.</v>
       </c>
       <c r="C358" t="str">
-        <v>表格无效。请确保所有栏目填写正确。</v>
+        <v>您尚未登录。请登录后访问此页面。</v>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="str">
-        <v>errors.UNABLE_TO_VERIFY_ACCOUNT</v>
+        <v>errors.USER_DATAPACK_FILE_NOT_FOUND_FOR_DOWNLOAD</v>
       </c>
       <c r="B359" t="str">
-        <v>Your email is not verified. Please verify your email first. If you did not receive an email, please resend.</v>
+        <v>The datapack requested was not found on the server. Please try again later or contact our support team.</v>
       </c>
       <c r="C359" t="str">
-        <v>您的电子邮件未经验证。请先验证您的电子邮件。如果您没有收到电子邮件，请重新发送。</v>
+        <v>服务器上未找到所请求的数据包。请稍后再试，或联系我们的技术支持团队。</v>
       </c>
     </row>
     <row r="360">
       <c r="A360" t="str">
-        <v>errors.ALREADY_VERIFIED_ACCOUNT</v>
+        <v>errors.INCORRECT_ENCRYPTION_HEADER</v>
       </c>
       <c r="B360" t="str">
-        <v>Account is already verified. Please log in.</v>
+        <v>Unable to encrypt the file, please try again later.</v>
       </c>
       <c r="C360" t="str">
-        <v>帐户已验证。请登录。</v>
+        <v>无法加密文件。请稍后再试。</v>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="str">
-        <v>errors.UNABLE_TO_VERIFY_ACCOUNT_SERVER</v>
+        <v>errors.TOO_MANY_REQUESTS</v>
       </c>
       <c r="B361" t="str">
-        <v>Unable to verify account due to server error. Please try again later.</v>
+        <v>You have made too many requests. Please try again later.</v>
       </c>
       <c r="C361" t="str">
-        <v>由于服务器错误，无法验证帐户。请稍后再试。</v>
+        <v>请求过于频繁。请稍后再试。</v>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="str">
-        <v>errors.TOKEN_EXPIRED_OR_INVALID</v>
+        <v>errors.RECAPTCHA_FAILED</v>
       </c>
       <c r="B362" t="str">
-        <v>Your token is either invalid or has expired. Please request a new verification email.</v>
+        <v>Recaptcha failed. Please try again.</v>
       </c>
       <c r="C362" t="str">
-        <v>您的令牌无效或已过期。请申请新的验证电子邮件。</v>
+        <v>验证失败. 请稍后再试。</v>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="str">
-        <v>errors.UNABLE_TO_SEND_EMAIL</v>
+        <v>errors.COOKIE_REJECTED</v>
       </c>
       <c r="B363" t="str">
-        <v>Unable to send email. Please try again later.</v>
+        <v>You must accept cookies to sign in.</v>
       </c>
       <c r="C363" t="str">
-        <v>无法发送邮件。请稍后再试。</v>
+        <v>您必须接受 Cookie 才能登录。</v>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="str">
-        <v>errors.UNABLE_TO_RESET_PASSWORD</v>
+        <v>errors.UNRECOGNIZED_IMAGE_FILE</v>
       </c>
       <c r="B364" t="str">
-        <v>Unable to reset password. Please try again later.</v>
+        <v>Unrecognized image extension. Please upload a valid image file.</v>
       </c>
       <c r="C364" t="str">
-        <v>无法重置密码。请稍后再试。</v>
+        <v>图像扩展名无法识别。请上传有效的图像文件。</v>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="str">
-        <v>errors.UNABLE_TO_RESET_EMAIL</v>
+        <v>errors.UPLOAD_PROFILE_PICTURE_FAILED</v>
       </c>
       <c r="B365" t="str">
-        <v>Unable to reset email. Please try again later.</v>
+        <v>Unable to upload profile picture. Please try again later.</v>
       </c>
       <c r="C365" t="str">
-        <v>无法重置邮箱。请稍后再试。</v>
+        <v>无法上传个人资料图片。请稍后再试。</v>
       </c>
     </row>
     <row r="366">
       <c r="A366" t="str">
-        <v>errors.UNABLE_TO_LOGIN_ACCOUNT_LOCKED</v>
+        <v>errors.UNABLE_TO_CHANGE_USERNAME</v>
       </c>
       <c r="B366" t="str">
-        <v>Your account has been locked. Please check your email for more information or contact support.</v>
+        <v>Unable to change username. Please try again later.</v>
       </c>
       <c r="C366" t="str">
-        <v>您的账户已被锁定。请查看您的电子邮件以获取更多信息或联系技术支持获得帮助。</v>
+        <v>无法更改用户名。请稍后再试。</v>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="str">
-        <v>errors.UNABLE_TO_RECOVER_ACCOUNT</v>
+        <v>errors.UNABLE_TO_DELETE_PROFILE</v>
       </c>
       <c r="B367" t="str">
-        <v>Unable to recover account. Please contact support for more information.</v>
+        <v>Unable to delete profile. Please try again later.</v>
       </c>
       <c r="C367" t="str">
-        <v>无法恢复账户。请联系技术支持获取更多信息。</v>
+        <v>无法删除用户。请稍后再试。</v>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="str">
-        <v>errors.NOT_LOGGED_IN</v>
+        <v>errors.INCORRECT_PASSWORD</v>
       </c>
       <c r="B368" t="str">
-        <v>You are not logged in. Please log in to access this page.</v>
+        <v>Incorrect password. Please try again.</v>
       </c>
       <c r="C368" t="str">
-        <v>您尚未登录。请登录后访问此页面。</v>
+        <v>密码错误。请稍后再试。</v>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="str">
-        <v>errors.USER_DATAPACK_FILE_NOT_FOUND_FOR_DOWNLOAD</v>
+        <v>errors.USERNAME_TAKEN</v>
       </c>
       <c r="B369" t="str">
-        <v>The datapack requested was not found on the server. Please try again later or contact our support team.</v>
+        <v>Username is already taken. Please try a different username.</v>
       </c>
       <c r="C369" t="str">
-        <v>服务器上未找到所请求的数据包。请稍后再试，或联系我们的技术支持团队。</v>
+        <v>用户名已被使用。请使用一个新的用户名。</v>
       </c>
     </row>
     <row r="370">
       <c r="A370" t="str">
-        <v>errors.INCORRECT_ENCRYPTION_HEADER</v>
+        <v>errors.UNABLE_TO_READ_FILE_OR_EMPTY_FILE</v>
       </c>
       <c r="B370" t="str">
-        <v>Unable to encrypt the file, please try again later.</v>
+        <v>Unable to read file or file is empty. Please try again.</v>
       </c>
       <c r="C370" t="str">
-        <v>无法加密文件。请稍后再试。</v>
+        <v>无法读取文件或文件为空。请稍后再试。</v>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="str">
-        <v>errors.TOO_MANY_REQUESTS</v>
+        <v>errors.FETCH_USERS_FAILED</v>
       </c>
       <c r="B371" t="str">
-        <v>You have made too many requests. Please try again later.</v>
+        <v>Unable to fetch users for admin display. Please try again later.</v>
       </c>
       <c r="C371" t="str">
-        <v>请求过于频繁。请稍后再试。</v>
+        <v>无法获取用户信息供管理员查阅。请稍后再试。</v>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="str">
-        <v>errors.RECAPTCHA_FAILED</v>
+        <v>errors.ADMIN_ADD_USER_FAILED</v>
       </c>
       <c r="B372" t="str">
-        <v>Recaptcha failed. Please try again.</v>
+        <v>Unable to add user. Please try again later.</v>
       </c>
       <c r="C372" t="str">
-        <v>验证失败. 请稍后再试。</v>
+        <v>无法添加用户。请稍后再试。</v>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="str">
-        <v>errors.COOKIE_REJECTED</v>
+        <v>errors.SERVER_TIMEOUT</v>
       </c>
       <c r="B373" t="str">
-        <v>You must accept cookies to sign in.</v>
+        <v>Server timed out. Please try again later.</v>
       </c>
       <c r="C373" t="str">
-        <v>您必须接受 Cookie 才能登录。</v>
+        <v>服务器超时。请稍后再试。</v>
       </c>
     </row>
     <row r="374">
       <c r="A374" t="str">
-        <v>errors.UNRECOGNIZED_IMAGE_FILE</v>
+        <v>errors.SERVER_BUSY</v>
       </c>
       <c r="B374" t="str">
-        <v>Unrecognized image extension. Please upload a valid image file.</v>
+        <v>Server is too busy. Please try again later.</v>
       </c>
       <c r="C374" t="str">
-        <v>图像扩展名无法识别。请上传有效的图像文件。</v>
+        <v>服务器忙。请稍后再试。</v>
       </c>
     </row>
     <row r="375">
       <c r="A375" t="str">
-        <v>errors.UPLOAD_PROFILE_PICTURE_FAILED</v>
+        <v>errors.ADMIN_DELETE_USER_FAILED</v>
       </c>
       <c r="B375" t="str">
-        <v>Unable to upload profile picture. Please try again later.</v>
+        <v>Unable to delete user. Please try again later.</v>
       </c>
       <c r="C375" t="str">
-        <v>无法上传个人资料图片。请稍后再试。</v>
+        <v>无法删除用户。请稍后再试。</v>
       </c>
     </row>
     <row r="376">
       <c r="A376" t="str">
-        <v>errors.UNABLE_TO_CHANGE_USERNAME</v>
+        <v>errors.UNABLE_TO_FETCH_DATAPACKS</v>
       </c>
       <c r="B376" t="str">
-        <v>Unable to change username. Please try again later.</v>
-      </c>
-      <c r="C376" t="str">
-        <v>无法更改用户名。请稍后再试。</v>
+        <v>Unable to fetch datapacks. Please try again later.</v>
       </c>
     </row>
     <row r="377">
       <c r="A377" t="str">
-        <v>errors.UNABLE_TO_DELETE_PROFILE</v>
+        <v>errors.UNABLE_TO_FETCH_USER_DATAPACKS</v>
       </c>
       <c r="B377" t="str">
-        <v>Unable to delete profile. Please try again later.</v>
+        <v>Unable to fetch user datapacks. Please try again later.</v>
       </c>
       <c r="C377" t="str">
-        <v>无法删除用户。请稍后再试。</v>
+        <v>无法获取用户数据包。请稍后再试。</v>
       </c>
     </row>
     <row r="378">
       <c r="A378" t="str">
-        <v>errors.INCORRECT_PASSWORD</v>
+        <v>errors.CANNOT_DELETE_ROOT_USER</v>
       </c>
       <c r="B378" t="str">
-        <v>Incorrect password. Please try again.</v>
+        <v>Cannot delete root user.</v>
       </c>
       <c r="C378" t="str">
-        <v>密码错误。请稍后再试。</v>
+        <v>不能删除根用户。</v>
       </c>
     </row>
     <row r="379">
       <c r="A379" t="str">
-        <v>errors.USERNAME_TAKEN</v>
+        <v>errors.ADMIN_DELETE_USER_DATAPACK_FAILED</v>
       </c>
       <c r="B379" t="str">
-        <v>Username is already taken. Please try a different username.</v>
+        <v>Unable to delete user datapack. Please try again later.</v>
       </c>
       <c r="C379" t="str">
-        <v>用户名已被使用。请使用一个新的用户名。</v>
+        <v>无法删除用户数据包。请稍后再试。</v>
       </c>
     </row>
     <row r="380">
       <c r="A380" t="str">
-        <v>errors.UNABLE_TO_READ_FILE_OR_EMPTY_FILE</v>
+        <v>errors.ADMIN_DELETE_SERVER_DATAPACK_FAILED</v>
       </c>
       <c r="B380" t="str">
-        <v>Unable to read file or file is empty. Please try again.</v>
+        <v>Unable to delete server datapack. Please try again later.</v>
       </c>
       <c r="C380" t="str">
-        <v>无法读取文件或文件为空。请稍后再试。</v>
+        <v>无法删除服务器数据包。请稍后再试。</v>
       </c>
     </row>
     <row r="381">
       <c r="A381" t="str">
-        <v>errors.FETCH_USERS_FAILED</v>
+        <v>errors.ADMIN_CANNOT_DELETE_ROOT_DATAPACK</v>
       </c>
       <c r="B381" t="str">
-        <v>Unable to fetch users for admin display. Please try again later.</v>
+        <v>Cannot delete root datapack. Ask server admin for assistance.</v>
       </c>
       <c r="C381" t="str">
-        <v>无法获取用户信息供管理员查阅。请稍后再试。</v>
+        <v>无法删除根数据包。请向服务器管理员寻求帮助。</v>
       </c>
     </row>
     <row r="382">
       <c r="A382" t="str">
-        <v>errors.ADMIN_ADD_USER_FAILED</v>
+        <v>errors.INVALID_SERVER_DATAPACK_REQUEST</v>
       </c>
       <c r="B382" t="str">
-        <v>Unable to add user. Please try again later.</v>
+        <v>Invalid server datapack request. Please try again later.</v>
       </c>
       <c r="C382" t="str">
-        <v>无法添加用户。请稍后再试。</v>
+        <v>无效的服务器数据包请求。请稍后再试。</v>
       </c>
     </row>
     <row r="383">
       <c r="A383" t="str">
-        <v>errors.SERVER_TIMEOUT</v>
+        <v>errors.SERVER_FILE_METADATA_ERROR</v>
       </c>
       <c r="B383" t="str">
-        <v>Server timed out. Please try again later.</v>
+        <v>Server file metadata error. Please try again later.</v>
       </c>
       <c r="C383" t="str">
-        <v>服务器超时。请稍后再试。</v>
+        <v>服务器文件元数据错误。请稍后再试。</v>
       </c>
     </row>
     <row r="384">
       <c r="A384" t="str">
-        <v>errors.SERVER_BUSY</v>
+        <v>errors.USER_DELETE_DATAPACK_FAILED</v>
       </c>
       <c r="B384" t="str">
-        <v>Server is too busy. Please try again later.</v>
+        <v>Unable to delete user datapack. Please try again later.</v>
       </c>
       <c r="C384" t="str">
-        <v>服务器忙。请稍后再试。</v>
+        <v>无法删除用户数据包。请稍后再试。</v>
       </c>
     </row>
     <row r="385">
       <c r="A385" t="str">
-        <v>errors.ADMIN_DELETE_USER_FAILED</v>
+        <v>errors.UNABLE_TO_PROCESS_DATAPACK_CONFIG</v>
       </c>
       <c r="B385" t="str">
-        <v>Unable to delete user. Please try again later.</v>
+        <v>Failed to process datapack config. Please try again later.</v>
       </c>
       <c r="C385" t="str">
-        <v>无法删除用户。请稍后再试。</v>
+        <v>处理数据包配置失败。请稍后再试。</v>
       </c>
     </row>
     <row r="386">
       <c r="A386" t="str">
-        <v>errors.UNABLE_TO_FETCH_DATAPACKS</v>
+        <v>errors.INVALID_SETTINGS</v>
       </c>
       <c r="B386" t="str">
-        <v>Unable to fetch datapacks. Please try again later.</v>
+        <v>Invalid settings. Please try again.</v>
+      </c>
+      <c r="C386" t="str">
+        <v>无效的设置。请稍后再试。</v>
       </c>
     </row>
     <row r="387">
       <c r="A387" t="str">
-        <v>errors.UNABLE_TO_FETCH_USER_DATAPACKS</v>
+        <v>errors.INTERNAL_ERROR</v>
       </c>
       <c r="B387" t="str">
-        <v>Unable to fetch user datapacks. Please try again later.</v>
+        <v>There was an internal error while generating the chart. Please try again later.</v>
       </c>
       <c r="C387" t="str">
-        <v>无法获取用户数据包。请稍后再试。</v>
+        <v>生成图表时出现内部错误。请稍后再试。</v>
       </c>
     </row>
     <row r="388">
       <c r="A388" t="str">
-        <v>errors.CANNOT_DELETE_ROOT_USER</v>
+        <v>errors.ADMIN_ADD_USERS_TO_WORKSHOP_FAILED</v>
       </c>
       <c r="B388" t="str">
-        <v>Cannot delete root user.</v>
+        <v>Unable to add users to workshop. Please try again later.</v>
       </c>
       <c r="C388" t="str">
-        <v>不能删除根用户。</v>
+        <v>无法将用户添加到工作坊。请稍后再试。</v>
       </c>
     </row>
     <row r="389">
       <c r="A389" t="str">
-        <v>errors.ADMIN_DELETE_USER_DATAPACK_FAILED</v>
+        <v>errors.ADMIN_EMAIL_INVALID</v>
       </c>
       <c r="B389" t="str">
-        <v>Unable to delete user datapack. Please try again later.</v>
+        <v>Invalid email. Please fix the email and try again.</v>
       </c>
       <c r="C389" t="str">
-        <v>无法删除用户数据包。请稍后再试。</v>
+        <v>电子邮件无效。请修复电子邮件并重试。</v>
       </c>
     </row>
     <row r="390">
       <c r="A390" t="str">
-        <v>errors.ADMIN_MODIFY_USER_FAILED</v>
+        <v>errors.ADMIN_WORKSHOP_FIELDS_EMPTY</v>
       </c>
       <c r="B390" t="str">
-        <v>Unable to modify user. Please try again later.</v>
+        <v>You must provide at least one field to add users to a workshop.</v>
+      </c>
+      <c r="C390" t="str">
+        <v>您必须提供至少一个领域才能将用户添加到工作坊。</v>
       </c>
     </row>
     <row r="391">
       <c r="A391" t="str">
-        <v>errors.ADMIN_DELETE_SERVER_DATAPACK_FAILED</v>
+        <v>errors.UNRECOGNIZED_EXCEL_FILE</v>
       </c>
       <c r="B391" t="str">
-        <v>Unable to delete server datapack. Please try again later.</v>
+        <v>Unrecognized Excel file. Please upload a valid Excel file.</v>
       </c>
       <c r="C391" t="str">
-        <v>无法删除服务器数据包。请稍后再试。</v>
+        <v>无法识别 Excel 文件。请上传有效的 Excel 文件。</v>
       </c>
     </row>
     <row r="392">
       <c r="A392" t="str">
-        <v>errors.ADMIN_CANNOT_DELETE_ROOT_DATAPACK</v>
+        <v>errors.SERVER_DATAPACK_ALREADY_EXISTS</v>
       </c>
       <c r="B392" t="str">
-        <v>Cannot delete root datapack. Ask server admin for assistance.</v>
+        <v>Server datapack already exists. Please upload a unique datapack (different title).</v>
       </c>
       <c r="C392" t="str">
-        <v>无法删除根数据包。请向服务器管理员寻求帮助。</v>
+        <v>服务器数据包已存在。请上传一个独特的数据包（不同的文件名）。</v>
       </c>
     </row>
     <row r="393">
       <c r="A393" t="str">
-        <v>errors.INVALID_SERVER_DATAPACK_REQUEST</v>
+        <v>errors.ADMIN_WORKSHOP_START_AFTER_END</v>
       </c>
       <c r="B393" t="str">
-        <v>Invalid server datapack request. Please try again later.</v>
+        <v>The start date must be before the end date.</v>
       </c>
       <c r="C393" t="str">
-        <v>无效的服务器数据包请求。请稍后再试。</v>
+        <v>开始日期必须早于结束日期</v>
       </c>
     </row>
     <row r="394">
       <c r="A394" t="str">
-        <v>errors.SERVER_FILE_METADATA_ERROR</v>
+        <v>errors.ADMIN_CREATE_WORKSHOP_FAILED</v>
       </c>
       <c r="B394" t="str">
-        <v>Server file metadata error. Please try again later.</v>
+        <v>Unable to create workshop. Please try again later.</v>
       </c>
       <c r="C394" t="str">
-        <v>服务器文件元数据错误。请稍后再试。</v>
+        <v>无法创建工作坊。请稍后再试。</v>
       </c>
     </row>
     <row r="395">
       <c r="A395" t="str">
-        <v>errors.USER_DELETE_DATAPACK_FAILED</v>
+        <v>errors.ADMIN_WORKSHOP_ALREADY_EXISTS</v>
       </c>
       <c r="B395" t="str">
-        <v>Unable to delete user datapack. Please try again later.</v>
+        <v>Workshop with that title and dates already exists. Please try again.</v>
       </c>
       <c r="C395" t="str">
-        <v>无法删除用户数据包。请稍后再试。</v>
+        <v>该工作坊名称已存在。请另选名称。</v>
       </c>
     </row>
     <row r="396">
       <c r="A396" t="str">
-        <v>errors.UNABLE_TO_PROCESS_DATAPACK_CONFIG</v>
+        <v>errors.ADMIN_FETCH_WORKSHOPS_FAILED</v>
       </c>
       <c r="B396" t="str">
-        <v>Failed to process datapack config. Please try again later.</v>
+        <v>Unable to fetch workshops. Please try again later.</v>
       </c>
       <c r="C396" t="str">
-        <v>处理数据包配置失败。请稍后再试。</v>
+        <v>无法抓取工作坊。请稍后再试。</v>
       </c>
     </row>
     <row r="397">
       <c r="A397" t="str">
-        <v>errors.INVALID_SETTINGS</v>
+        <v>errors.ADMIN_DELETE_WORKSHOP_FAILED</v>
       </c>
       <c r="B397" t="str">
-        <v>Invalid settings. Please try again.</v>
-      </c>
-      <c r="C397" t="str">
-        <v>无效的设置。请稍后再试。</v>
+        <v>Unable to delete workshop. Please try again later.</v>
       </c>
     </row>
     <row r="398">
       <c r="A398" t="str">
-        <v>errors.INTERNAL_ERROR</v>
+        <v>errors.ADMIN_WORKSHOP_NOT_FOUND</v>
       </c>
       <c r="B398" t="str">
-        <v>There was an internal error while generating the chart. Please try again later.</v>
+        <v>Workshop not found on server, it has likely ended or been deleted.</v>
       </c>
       <c r="C398" t="str">
-        <v>生成图表时出现内部错误。请稍后再试。</v>
+        <v>服务器未找到工作坊。该工作坊可能已结束或被删除。</v>
       </c>
     </row>
     <row r="399">
       <c r="A399" t="str">
-        <v>errors.ADMIN_ADD_USERS_TO_WORKSHOP_FAILED</v>
+        <v>errors.ADMIN_WORKSHOP_EDIT_FAILED</v>
       </c>
       <c r="B399" t="str">
-        <v>Unable to add users to workshop. Please try again later.</v>
-      </c>
-      <c r="C399" t="str">
-        <v>无法将用户添加到工作坊。请稍后再试。</v>
+        <v>Unable to edit workshop. Please try again later.</v>
       </c>
     </row>
     <row r="400">
       <c r="A400" t="str">
-        <v>errors.ADMIN_EMAIL_INVALID</v>
+        <v>errors.USER_EDIT_DATAPACK_FAILED</v>
       </c>
       <c r="B400" t="str">
-        <v>Invalid email. Please fix the email and try again.</v>
-      </c>
-      <c r="C400" t="str">
-        <v>电子邮件无效。请修复电子邮件并重试。</v>
+        <v>Failed to edit user datapack. Please try again later.</v>
       </c>
     </row>
     <row r="401">
       <c r="A401" t="str">
-        <v>errors.ADMIN_WORKSHOP_FIELDS_EMPTY</v>
+        <v>errors.USER_FETCH_DATAPACK_FAILED</v>
       </c>
       <c r="B401" t="str">
-        <v>You must provide at least one field to add users to a workshop.</v>
-      </c>
-      <c r="C401" t="str">
-        <v>您必须提供至少一个领域才能将用户添加到工作坊。</v>
+        <v>Failed to fetch user datapack. Please try again later.</v>
       </c>
     </row>
     <row r="402">
       <c r="A402" t="str">
-        <v>errors.UNRECOGNIZED_EXCEL_FILE</v>
+        <v>errors.USER_REPLACE_DATAPACK_FILE_FAILED</v>
       </c>
       <c r="B402" t="str">
-        <v>Unrecognized Excel file. Please upload a valid Excel file.</v>
-      </c>
-      <c r="C402" t="str">
-        <v>无法识别 Excel 文件。请上传有效的 Excel 文件。</v>
+        <v>Failed to replace user datapack file. Please try again later.</v>
       </c>
     </row>
     <row r="403">
       <c r="A403" t="str">
-        <v>errors.SERVER_DATAPACK_ALREADY_EXISTS</v>
+        <v>errors.USER_REPLACE_DATAPACK_PROFILE_IMAGE_FAILED</v>
       </c>
       <c r="B403" t="str">
-        <v>Server datapack already exists. Please upload a unique datapack (different title).</v>
-      </c>
-      <c r="C403" t="str">
-        <v>服务器数据包已存在。请上传一个独特的数据包（不同的文件名）。</v>
+        <v>Failed to replace user datapack profile image. Please try again later.</v>
       </c>
     </row>
     <row r="404">
       <c r="A404" t="str">
-        <v>errors.ADMIN_WORKSHOP_START_AFTER_END</v>
+        <v>errors.DATAPACK_TITLE_LEADING_TRAILING_WHITESPACE</v>
       </c>
       <c r="B404" t="str">
-        <v>The start date must be before the end date.</v>
-      </c>
-      <c r="C404" t="str">
-        <v>开始日期必须早于结束日期</v>
+        <v>Datapack title cannot have leading or trailing whitespace.</v>
       </c>
     </row>
     <row r="405">
       <c r="A405" t="str">
-        <v>errors.ADMIN_CREATE_WORKSHOP_FAILED</v>
+        <v>errors.ADMIN_FETCH_PRIVATE_DATAPACKS_FAILED</v>
       </c>
       <c r="B405" t="str">
-        <v>Unable to create workshop. Please try again later.</v>
-      </c>
-      <c r="C405" t="str">
-        <v>无法创建工作坊。请稍后再试。</v>
+        <v>Failed to fetch private datapacks. Please try again later.</v>
       </c>
     </row>
     <row r="406">
       <c r="A406" t="str">
-        <v>errors.ADMIN_WORKSHOP_ALREADY_EXISTS</v>
+        <v>errors.ADMIN_PRIORITY_BATCH_UPDATE_FAILED</v>
       </c>
       <c r="B406" t="str">
-        <v>Workshop with that title and dates already exists. Please try again.</v>
-      </c>
-      <c r="C406" t="str">
-        <v>该工作坊名称已存在。请另选名称。</v>
+        <v>Failed to update datapack priorities. Please contact a server admin for assistance.</v>
       </c>
     </row>
     <row r="407">
       <c r="A407" t="str">
-        <v>errors.ADMIN_FETCH_WORKSHOPS_FAILED</v>
+        <v>errors.ADMIN_ADD_OFFICIAL_DATAPACK_TO_WORKSHOP_FAILED</v>
       </c>
       <c r="B407" t="str">
-        <v>Unable to fetch workshops. Please try again later.</v>
-      </c>
-      <c r="C407" t="str">
-        <v>无法抓取工作坊。请稍后再试。</v>
+        <v>Failed to add official datapack to workshop. Please try again later.</v>
       </c>
     </row>
     <row r="408">
       <c r="A408" t="str">
-        <v>errors.ADMIN_DELETE_WORKSHOP_FAILED</v>
+        <v>errors.ADMIN_SERVER_DATAPACK_ALREADY_EXISTS</v>
       </c>
       <c r="B408" t="str">
-        <v>Unable to delete workshop. Please try again later.</v>
+        <v>Server datapack already exists in workshop. Please choose a different datapack.</v>
       </c>
     </row>
     <row r="409">
       <c r="A409" t="str">
-        <v>errors.ADMIN_WORKSHOP_NOT_FOUND</v>
+        <v>errors.ADMIN_WORKSHOP_ENDED</v>
       </c>
       <c r="B409" t="str">
-        <v>Workshop not found on server, it has likely ended or been deleted.</v>
-      </c>
-      <c r="C409" t="str">
-        <v>服务器未找到工作坊。该工作坊可能已结束或被删除。</v>
+        <v>Workshop has ended. You can no longer edit or add datapacks to it.</v>
       </c>
     </row>
     <row r="410">
       <c r="A410" t="str">
-        <v>errors.ADMIN_WORKSHOP_EDIT_FAILED</v>
+        <v>errors.WORKSHOP_FETCH_DATAPACK_FAILED</v>
       </c>
       <c r="B410" t="str">
-        <v>Unable to edit workshop. Please try again later.</v>
+        <v>Failed to fetch workshop datapacks. Please try again later.</v>
       </c>
     </row>
     <row r="411">
       <c r="A411" t="str">
-        <v>errors.USER_EDIT_DATAPACK_FAILED</v>
+        <v>errors.METADATA_NOT_FOUND</v>
       </c>
       <c r="B411" t="str">
-        <v>Failed to edit user datapack. Please try again later.</v>
+        <v>Metadata not found. Please try again later.</v>
       </c>
     </row>
     <row r="412">
       <c r="A412" t="str">
-        <v>errors.USER_FETCH_DATAPACK_FAILED</v>
+        <v>errors.INVALID_CROSSPLOT_CONVERSION</v>
       </c>
       <c r="B412" t="str">
-        <v>Failed to fetch user datapack. Please try again later.</v>
+        <v>Invalid crossplot conversion. Please select a valid chart for the Y Axis.</v>
       </c>
     </row>
     <row r="413">
       <c r="A413" t="str">
-        <v>errors.USER_REPLACE_DATAPACK_FILE_FAILED</v>
+        <v>errors.INVALID_CROSSPLOT_UNITS</v>
       </c>
       <c r="B413" t="str">
-        <v>Failed to replace user datapack file. Please try again later.</v>
+        <v>Please select a different unit for the Y Axis. This unit cannot be converted.</v>
       </c>
     </row>
     <row r="414">
       <c r="A414" t="str">
-        <v>errors.USER_REPLACE_DATAPACK_PROFILE_IMAGE_FAILED</v>
+        <v>errors.CROSSPLOT_CONVERSION_FAILED</v>
       </c>
       <c r="B414" t="str">
-        <v>Failed to replace user datapack profile image. Please try again later.</v>
+        <v>Crossplot conversion failed. Please try again later.</v>
       </c>
     </row>
     <row r="415">
       <c r="A415" t="str">
-        <v>errors.DATAPACK_TITLE_LEADING_TRAILING_WHITESPACE</v>
+        <v>errors.NO_MODELS</v>
       </c>
       <c r="B415" t="str">
-        <v>Datapack title cannot have leading or trailing whitespace.</v>
+        <v>No models available. Please add a model by clicking the chart in the main view.</v>
       </c>
     </row>
     <row r="416">
       <c r="A416" t="str">
-        <v>errors.ADMIN_FETCH_PRIVATE_DATAPACKS_FAILED</v>
+        <v>errors.CROSSPLOT_SETTINGS_MISMATCH</v>
       </c>
       <c r="B416" t="str">
-        <v>Failed to fetch private datapacks. Please try again later.</v>
+        <v>Crossplot settings mismatch. Please generate the crossplot with your most recent changes.</v>
       </c>
     </row>
     <row r="417">
       <c r="A417" t="str">
-        <v>errors.ADMIN_PRIORITY_BATCH_UPDATE_FAILED</v>
+        <v>button.generate</v>
       </c>
       <c r="B417" t="str">
-        <v>Failed to update datapack priorities. Please contact a server admin for assistance.</v>
+        <v>Generate</v>
+      </c>
+      <c r="C417" t="str">
+        <v>绘制</v>
       </c>
     </row>
     <row r="418">
       <c r="A418" t="str">
-        <v>errors.ADMIN_ADD_OFFICIAL_DATAPACK_TO_WORKSHOP_FAILED</v>
+        <v>button.generate-chart</v>
       </c>
       <c r="B418" t="str">
-        <v>Failed to add official datapack to workshop. Please try again later.</v>
+        <v>Generate Chart</v>
+      </c>
+      <c r="C418" t="str">
+        <v>绘制图表</v>
       </c>
     </row>
     <row r="419">
       <c r="A419" t="str">
-        <v>errors.ADMIN_SERVER_DATAPACK_ALREADY_EXISTS</v>
+        <v>button.remove-cache</v>
       </c>
       <c r="B419" t="str">
-        <v>Server datapack already exists in workshop. Please choose a different datapack.</v>
+        <v>Remove Cache</v>
+      </c>
+      <c r="C419" t="str">
+        <v>清除缓存</v>
       </c>
     </row>
     <row r="420">
       <c r="A420" t="str">
-        <v>errors.ADMIN_WORKSHOP_ENDED</v>
+        <v>button.confirm-selection</v>
       </c>
       <c r="B420" t="str">
-        <v>Workshop has ended. You can no longer edit or add datapacks to it.</v>
+        <v>Confirm Selection</v>
+      </c>
+      <c r="C420" t="str">
+        <v>确认选择</v>
       </c>
     </row>
     <row r="421">
       <c r="A421" t="str">
-        <v>errors.WORKSHOP_FETCH_DATAPACK_FAILED</v>
+        <v>button.generate-cross-plot</v>
       </c>
       <c r="B421" t="str">
-        <v>Failed to fetch workshop datapacks. Please try again later.</v>
+        <v>Generate Cross Plot</v>
       </c>
     </row>
     <row r="422">
       <c r="A422" t="str">
-        <v>errors.METADATA_NOT_FOUND</v>
+        <v>yes</v>
       </c>
       <c r="B422" t="str">
-        <v>Metadata not found. Please try again later.</v>
+        <v>Yes</v>
+      </c>
+      <c r="C422" t="str">
+        <v>是</v>
       </c>
     </row>
     <row r="423">
       <c r="A423" t="str">
-        <v>errors.INVALID_CROSSPLOT_CONVERSION</v>
+        <v>no</v>
       </c>
       <c r="B423" t="str">
-        <v>Invalid crossplot conversion. Please select a valid chart for the Y Axis.</v>
+        <v>No</v>
+      </c>
+      <c r="C423" t="str">
+        <v>否</v>
       </c>
     </row>
     <row r="424">
       <c r="A424" t="str">
-        <v>errors.INVALID_CROSSPLOT_UNITS</v>
+        <v>languageNames.en-US</v>
       </c>
       <c r="B424" t="str">
-        <v>Please select a different unit for the Y Axis. This unit cannot be converted.</v>
+        <v>English</v>
       </c>
     </row>
     <row r="425">
       <c r="A425" t="str">
-        <v>errors.CROSSPLOT_CONVERSION_FAILED</v>
+        <v>languageNames.en</v>
       </c>
       <c r="B425" t="str">
-        <v>Crossplot conversion failed. Please try again later.</v>
+        <v>English</v>
       </c>
     </row>
     <row r="426">
       <c r="A426" t="str">
-        <v>errors.NO_MODELS</v>
+        <v>languageNames.zh</v>
       </c>
       <c r="B426" t="str">
-        <v>At least 2 models are required for conversion. Please add a model by clicking the chart in the main view.</v>
+        <v>中文</v>
       </c>
     </row>
     <row r="427">
       <c r="A427" t="str">
-        <v>errors.CROSSPLOT_SETTINGS_MISMATCH</v>
+        <v>tours.quit</v>
       </c>
       <c r="B427" t="str">
-        <v>Crossplot settings mismatch. Please generate the crossplot with your most recent changes.</v>
+        <v>Quit Tour</v>
+      </c>
+      <c r="C427" t="str">
+        <v>退出导览</v>
       </c>
     </row>
     <row r="428">
       <c r="A428" t="str">
-        <v>errors.ADMIN_ADD_FILES_TO_WORKSHOP_FAILED</v>
+        <v>tours.finish</v>
       </c>
       <c r="B428" t="str">
-        <v>Failed to add files to workshop</v>
+        <v>Finish Tour</v>
+      </c>
+      <c r="C428" t="str">
+        <v>结束导览</v>
       </c>
     </row>
     <row r="429">
       <c r="A429" t="str">
-        <v>errors.ADMIN_ADD_COVER_TO_WORKSHOP_FAILED</v>
+        <v>tours.next</v>
       </c>
       <c r="B429" t="str">
-        <v>Failed to add cover to workshop</v>
+        <v>Next</v>
+      </c>
+      <c r="C429" t="str">
+        <v>下一步</v>
       </c>
     </row>
     <row r="430">
       <c r="A430" t="str">
-        <v>errors.INVALID_FILE_FORMAT</v>
+        <v>tours.back</v>
       </c>
       <c r="B430" t="str">
-        <v>Invalid file format.</v>
+        <v>Back</v>
+      </c>
+      <c r="C430" t="str">
+        <v>上一步</v>
       </c>
     </row>
     <row r="431">
       <c r="A431" t="str">
-        <v>errors.USER_WORKSHOP_FILE_NOT_FOUND_FOR_DOWNLOAD</v>
+        <v>tours.qsg.step1</v>
       </c>
       <c r="B431" t="str">
-        <v>The workshop file requested was not found on the server. Please try again later or contact our support team.</v>
+        <v>In the Presets page, we offer pre-configured settings that allow you to rapidly generate specific types of charts without configuring all options from the beginning. Each preset comes equipped with designated data packs, visual styles, and settings, enabling you to create charts with just a single click.</v>
       </c>
       <c r="C431" t="str">
-        <v>请求文件不存在，请稍后再试或联系开发团队</v>
+        <v>在预设页面中，我们提供了预设置，允许您快速生成特定类型的图表，无需从头开始配置所有选项。每个预设都配备了指定的数据包、视觉样式和设置，使您能够一键创建图表</v>
       </c>
     </row>
     <row r="432">
       <c r="A432" t="str">
-        <v>errors.INVALID_DATAPACK_HASH</v>
+        <v>tours.qsg.step2</v>
       </c>
       <c r="B432" t="str">
-        <v>Invalid treatise datapack hash provided.</v>
+        <v>In the Datapacks page, you can select the datapacks required to generate your charts. We offer nine official data packs, each containing a curated collection of datasets tailored for specific thematic explorations. For more detailed guidance on Datapacks, please refer to the Datapacks Tour under the "Tours" section</v>
+      </c>
+      <c r="C432" t="str">
+        <v>在数据包页面，您可以选择生成图表所需的数据包。我们提供九个官方数据包，每个数据包都包含为特定主题探索量身定制的数据集合集。如需更详细的数据包指导，请参考“导览”部分下的数据包导览。</v>
       </c>
     </row>
     <row r="433">
       <c r="A433" t="str">
-        <v>errors.USER_FETCH_HISTORY_FAILED</v>
+        <v>tours.qsg.step3</v>
       </c>
       <c r="B433" t="str">
-        <v>Failed to fetch user history. Please try again later.</v>
+        <v>In the Chart page, you can view the charts you have created and explore the detailed visualizations of geologic events. Additionally, you have the option to download and save these charts for your reference or further analysis.</v>
+      </c>
+      <c r="C433" t="str">
+        <v>在图表页面，您可以查看已创建的图表并探索地质事件的详细可视化图。此外，您还可以下载并保存这些图表以供参考或进一步分析。</v>
       </c>
     </row>
     <row r="434">
       <c r="A434" t="str">
-        <v>errors.USER_DELETE_HISTORY_FAILED</v>
+        <v>tours.qsg.step4</v>
       </c>
       <c r="B434" t="str">
-        <v>Failed to delete user history. Please try again later</v>
+        <v>In the Settings page, you can customize all aspects of your charts. This includes adjusting the scale and time range, selecting which rows to display, setting the background color and font style, etc. Tailor your charts to meet your specific needs and preferences to optimize your visual analysis. For more detailed guidance on Settings, please refer to the Settings Tour under the "Tours" section</v>
+      </c>
+      <c r="C434" t="str">
+        <v>在设置页面，您可以自定义图表的所有方面。这包括调整比例和时间范围、选择显示哪些行、设置背景色和字体样式等。根据您的具体需求和偏好调整图表，以优化您的视觉分析。如需更详细的设置指导，请参考“导览”部分下的设置导览。</v>
       </c>
     </row>
     <row r="435">
       <c r="A435" t="str">
-        <v>errors.USER_FETCH_HISTORY_METADATA_FAILED</v>
+        <v>tours.qsg.step5</v>
       </c>
       <c r="B435" t="str">
-        <v>Failed to fetch user history metadata. Please try again later</v>
+        <v>In the Help Page, you can find detailed assistance and information on how to use the website.</v>
+      </c>
+      <c r="C435" t="str">
+        <v>在帮助页面，您可以找到关于如何使用网站的详细帮助和信息。</v>
       </c>
     </row>
     <row r="436">
       <c r="A436" t="str">
-        <v>errors.USER_FETCH_HISTORY_FAILED_DATAPACKS_MISSING</v>
+        <v>tours.qsg.step6</v>
       </c>
       <c r="B436" t="str">
-        <v>This chart entry couldn't be loaded due to missing files and has been removed from your history.</v>
+        <v>In the Workshops Page, you can access a range of educational and experimental tutorials that offer in-depth guidance. Here, you can explore the workshops you have registered for, allowing you to engage with the content and enhance your skills in a hands-on learning environment.</v>
+      </c>
+      <c r="C436" t="str">
+        <v>在工作坊页面，您可以访问一系列提供深入指导的教育和实验教程。在这里，您可以探索已注册的研讨会，通过亲身实践的学习环境来提升您的技能。</v>
       </c>
     </row>
     <row r="437">
       <c r="A437" t="str">
-        <v>button.generate</v>
+        <v>tours.qsg.step7</v>
       </c>
       <c r="B437" t="str">
-        <v>Generate</v>
+        <v>The About Page provides information about our development team.</v>
       </c>
       <c r="C437" t="str">
-        <v>绘制</v>
+        <v>关于页面提供了我们开发团队的信息。</v>
       </c>
     </row>
     <row r="438">
       <c r="A438" t="str">
-        <v>button.generate-chart</v>
+        <v>tours.qsg.step8</v>
       </c>
       <c r="B438" t="str">
-        <v>Generate Chart</v>
+        <v>Click here to sign in and unlock the features mentioned earlier, such as accessing registered workshops. Once logged in, you will also have the ability to upload datapacks and take full advantage of all functionalities.</v>
       </c>
       <c r="C438" t="str">
-        <v>绘制图表</v>
+        <v>点击此处登录并解锁前面提到的功能，例如访问工作坊界面。登陆后，您还将能够上传数据包并充分利用所有功能。</v>
       </c>
     </row>
     <row r="439">
       <c r="A439" t="str">
-        <v>button.remove-cache</v>
+        <v>tours.datapack.step1</v>
       </c>
       <c r="B439" t="str">
-        <v>Remove Cache</v>
+        <v>Switch between different display types for datapacks: rows, cards, or compact view.</v>
       </c>
       <c r="C439" t="str">
-        <v>清除缓存</v>
+        <v>在数据包显示类型之间切换：行视图、卡片视图或紧凑视图。</v>
       </c>
     </row>
     <row r="440">
       <c r="A440" t="str">
-        <v>button.confirm-selection</v>
+        <v>tours.datapack.step2</v>
       </c>
       <c r="B440" t="str">
-        <v>Confirm Selection</v>
+        <v>Add a datapack by clicking the checkbox</v>
       </c>
       <c r="C440" t="str">
-        <v>确认选择</v>
+        <v>勾选添加您想要的数据包</v>
       </c>
     </row>
     <row r="441">
       <c r="A441" t="str">
-        <v>button.generate-cross-plot</v>
+        <v>tours.datapack.step3</v>
       </c>
       <c r="B441" t="str">
-        <v>Generate Cross Plot</v>
+        <v>Click the deselect icon to deselect all datapacks</v>
+      </c>
+      <c r="C441" t="str">
+        <v>点此取消选择所有数据包</v>
       </c>
     </row>
     <row r="442">
       <c r="A442" t="str">
-        <v>yes</v>
+        <v>tours.datapack.step4</v>
       </c>
       <c r="B442" t="str">
-        <v>Yes</v>
+        <v>Remember to confirm your selection</v>
       </c>
       <c r="C442" t="str">
-        <v>是</v>
+        <v>记得确认您的选择</v>
       </c>
     </row>
     <row r="443">
       <c r="A443" t="str">
-        <v>no</v>
+        <v>tours.settings.step1</v>
       </c>
       <c r="B443" t="str">
-        <v>No</v>
+        <v>In the Time settings, you can Set the "Top of Interval" and "Base of Interval" for your data. These fields allow you to define the starting and ending ages or stages, which can be adjusted by entering values or using the dropdown selectors. Adjust the vertical scale to change how much vertical space each million years occupies on your charts. For example, setting it higher will spread the intervals further apart, making each period easier to examine closely.</v>
       </c>
       <c r="C443" t="str">
-        <v>否</v>
+        <v>在时间设置中，您可以为您的数据设置“时间段顶部”和“时间段底部”。调整这两个值将改变图表的时间跨度，您可以通过输入值或使用下拉选择器进行调整。您还可以调整垂直比例，以改变图表中每百万年占据的垂直空间量。例如，将其设置得更高将使时间间隔进一步分开，使每个时期更易于仔细检查。</v>
       </c>
     </row>
     <row r="444">
       <c r="A444" t="str">
-        <v>languageNames.en-US</v>
+        <v>tours.settings.step2</v>
       </c>
       <c r="B444" t="str">
-        <v>English</v>
+        <v>In the Preferences settings, you can customize the display options. For instance, you may choose to gray out columns with no data for selected time periods, add tooltips for additional information, or enable filtering and legend options for charts. Furthermore, you can load your settings from a file or save your current settings to a file. This feature is useful for backing up your configurations, sharing them with others, or quickly applying previously saved configurations to your chart.</v>
+      </c>
+      <c r="C444" t="str">
+        <v>在偏好中，您可以自定义显示选项。例如，您可以选择在选定时间段内将无数据的列显示为灰色，添加工具提示以提供额外信息，或启用图表的筛选和图例选项。此外，您可以从文件加载您的设置或将当前设置保存到文件中。此功能使您可以备份设置、与他人分享或快速应用以前保存的设置到您的图表中。</v>
       </c>
     </row>
     <row r="445">
       <c r="A445" t="str">
-        <v>languageNames.en</v>
+        <v>tours.settings.step3</v>
       </c>
       <c r="B445" t="str">
-        <v>English</v>
+        <v>In Column Settings, you can deeply customize the appearance and organization of your charts.In the "Column Customization" area, you can adjust titles and shift row positions to streamline how data is displayed on your charts. Enable or disable specific elements like the chart title and Ma markers to suit your presentation needs. In the "Font Options" section, refine the appearance of your charts by choosing different fonts, sizes, and styles for headers and labels, ensuring important data stands out or meets formatting requirements. Please note that the advanced settings for columns can vary depending on the datapack you are working with, allowing for tailored configurations that best fit the data characteristics.</v>
+      </c>
+      <c r="C445" t="str">
+        <v>在列设置中，您可以深度自定义图表的外观和组织。在“列自定义”区域，您可以调整标题和移动行位置，以简化图表上数据的显示方式。根据您的展示需求启用或禁用特定元素，如图表标题和百万年标记。在“字体选项”部分，通过选择不同的字体、大小和样式为标题和标签，细化您的图表外观，确保重要数据突出显示或符合格式要求。请注意，列高级设置可能根据您正在使用的数据包而有所不同，每个数据包都有最适合数据特性的列高级设置。</v>
       </c>
     </row>
     <row r="446">
       <c r="A446" t="str">
-        <v>languageNames.zh</v>
+        <v>tours.settings.step4</v>
       </c>
       <c r="B446" t="str">
-        <v>中文</v>
+        <v>In the Search Settings, you can quickly locate specific columns by entering keywords and then directly add them to your chart. Simply enter a term related to the setting you are looking for, and the system will display all relevant results.This feature is particularly useful when managing numerous data points or when you need to make quick adjustments without browsing through extensive lists.</v>
+      </c>
+      <c r="C446" t="str">
+        <v>在搜索中，您可以通过输入关键词快速定位特定列，然后直接将其添加到您的图表中。只需输入一个与您正在寻找的设置相关的词语，系统便会显示所有相关结果。此功能可以帮助您管理众多数据点，或进行快速调整而无需浏览繁杂列表。请注意目前只支持英文搜索。</v>
       </c>
     </row>
     <row r="447">
       <c r="A447" t="str">
-        <v>tours.quit</v>
+        <v>tours.settings.step5</v>
       </c>
       <c r="B447" t="str">
-        <v>Quit Tour</v>
+        <v>The Font Settings section allows you to customize the appearance of text within your charts. You can adjust font styles, sizes, and formatting for various elements such as column headers, age labels, and more. Each setting is inheritable, ensuring consistency across related elements unless specified otherwise. Changing a font setting here applies it system-wide, but you can override these for individual columns by using the "Change Font" option within each columns settings.Experiment with different fonts and sizes to enhance readability and visual appeal of your charts.</v>
       </c>
       <c r="C447" t="str">
-        <v>退出导览</v>
+        <v>在字体设置中您可以自定义图表内的文本外观。您可以为各种元素如列标题、年龄标签等调整字体样式、大小和格式。每项设置都是可继承的，确保相关元素间的一致性，除非另行设置。在这里更改字体设置将系统范围内应用，但您可以使用每个列设置中的“更改字体”选项覆盖这些设置。尝试不同的字体和大小，以增强图表的可读性和视觉吸引力。</v>
       </c>
     </row>
     <row r="448">
       <c r="A448" t="str">
-        <v>tours.finish</v>
+        <v>tours.settings.step6</v>
       </c>
       <c r="B448" t="str">
-        <v>Finish Tour</v>
+        <v>In the Map Points Settings, you can access and manage geographic data points for different locations. This feature allows you to view specific location details directly on the interactive map. You can toggle different map layers and visualize data points with detailed descriptions, like latitude, longitude, and additional notes. Please note, however, that not all datapacks contain map points.</v>
       </c>
       <c r="C448" t="str">
-        <v>结束导览</v>
+        <v>在地图点设置中，您可以访问和管理不同位置的地理数据点。此功能允许您直接在交互式地图上查看特定位置的详细信息。您可以切换不同的地图层，并用详细描述（如纬度、经度和附加说明）可视化数据点。请注意，并非所有数据包都包含地图点。</v>
       </c>
     </row>
     <row r="449">
       <c r="A449" t="str">
-        <v>tours.next</v>
+        <v>tours.settings.step7</v>
       </c>
       <c r="B449" t="str">
-        <v>Next</v>
+        <v>In the Datapacks Settings, you can select the datapacks you wish to use for generating charts. We offer nine official datapacks, each comprising a curated collection of datasets tailored for specific thematic explorations. You might notice that this page resembles the Datapack page; selections can be configured here or there interchangeably. For more detailed guidance on how to utilize datapacks, please refer to the Datapacks Tour in the Help page "Tours" section.</v>
       </c>
       <c r="C449" t="str">
-        <v>下一步</v>
+        <v>在数据包设置中，您可以选择您希望用于生成图表的数据包。我们提供九个官方数据包，每个数据包都包含为特定主题探索量身定制的数据集合。您也许已经注意到，此页面与"数据包"页面内容相同；您在两个地方都可以进行选择和设置。如需更详细的关于如何利用数据包的指导，请参阅帮助页面“导览”部分中的数据包导览。</v>
       </c>
     </row>
     <row r="450">
       <c r="A450" t="str">
-        <v>tours.back</v>
-      </c>
-      <c r="B450" t="str">
-        <v>Back</v>
+        <v>settings.column.tooltip.note-in-range</v>
       </c>
       <c r="C450" t="str">
-        <v>上一步</v>
+        <v>数据不在所选时间区间内</v>
       </c>
     </row>
     <row r="451">
       <c r="A451" t="str">
-        <v>tours.qsg.step1</v>
-      </c>
-      <c r="B451" t="str">
-        <v>In the Presets page, we offer pre-configured settings that allow you to rapidly generate specific types of charts without configuring all options from the beginning. Each preset comes equipped with designated data packs, visual styles, and settings, enabling you to create charts with just a single click.</v>
+        <v>language-names.en-US</v>
       </c>
       <c r="C451" t="str">
-        <v>在预设页面中，我们提供了预设置，允许您快速生成特定类型的图表，无需从头开始配置所有选项。每个预设都配备了指定的数据包、视觉样式和设置，使您能够一键创建图表</v>
+        <v>English</v>
       </c>
     </row>
     <row r="452">
       <c r="A452" t="str">
-        <v>tours.qsg.step2</v>
-      </c>
-      <c r="B452" t="str">
-        <v>In the Datapacks page, you can select the datapacks required to generate your charts. We offer nine official data packs, each containing a curated collection of datasets tailored for specific thematic explorations. For more detailed guidance on Datapacks, please refer to the Datapacks Tour under the "Tours" section</v>
+        <v>language-names.en</v>
       </c>
       <c r="C452" t="str">
-        <v>在数据包页面，您可以选择生成图表所需的数据包。我们提供九个官方数据包，每个数据包都包含为特定主题探索量身定制的数据集合集。如需更详细的数据包指导，请参考“导览”部分下的数据包导览。</v>
+        <v>English</v>
       </c>
     </row>
     <row r="453">
       <c r="A453" t="str">
-        <v>tours.qsg.step3</v>
-      </c>
-      <c r="B453" t="str">
-        <v>In the Chart page, you can view the charts you have created and explore the detailed visualizations of geologic events. Additionally, you have the option to download and save these charts for your reference or further analysis.</v>
+        <v>language-names.zh</v>
       </c>
       <c r="C453" t="str">
-        <v>在图表页面，您可以查看已创建的图表并探索地质事件的详细可视化图。此外，您还可以下载并保存这些图表以供参考或进一步分析。</v>
-      </c>
-    </row>
-    <row r="454">
-      <c r="A454" t="str">
-        <v>tours.qsg.step4</v>
-      </c>
-      <c r="B454" t="str">
-        <v>In the Settings page, you can customize all aspects of your charts. This includes adjusting the scale and time range, selecting which rows to display, setting the background color and font style, etc. Tailor your charts to meet your specific needs and preferences to optimize your visual analysis. For more detailed guidance on Settings, please refer to the Settings Tour under the "Tours" section</v>
-      </c>
-      <c r="C454" t="str">
-        <v>在设置页面，您可以自定义图表的所有方面。这包括调整比例和时间范围、选择显示哪些行、设置背景色和字体样式等。根据您的具体需求和偏好调整图表，以优化您的视觉分析。如需更详细的设置指导，请参考“导览”部分下的设置导览。</v>
-      </c>
-    </row>
-    <row r="455">
-      <c r="A455" t="str">
-        <v>tours.qsg.step5</v>
-      </c>
-      <c r="B455" t="str">
-        <v>In the Help Page, you can find detailed assistance and information on how to use the website.</v>
-      </c>
-      <c r="C455" t="str">
-        <v>在帮助页面，您可以找到关于如何使用网站的详细帮助和信息。</v>
-      </c>
-    </row>
-    <row r="456">
-      <c r="A456" t="str">
-        <v>tours.qsg.step6</v>
-      </c>
-      <c r="B456" t="str">
-        <v>In the Workshops Page, you can access a range of educational and experimental tutorials that offer in-depth guidance. Here, you can explore the workshops you have registered for, allowing you to engage with the content and enhance your skills in a hands-on learning environment.</v>
-      </c>
-      <c r="C456" t="str">
-        <v>在工作坊页面，您可以访问一系列提供深入指导的教育和实验教程。在这里，您可以探索已注册的研讨会，通过亲身实践的学习环境来提升您的技能。</v>
-      </c>
-    </row>
-    <row r="457">
-      <c r="A457" t="str">
-        <v>tours.qsg.step7</v>
-      </c>
-      <c r="B457" t="str">
-        <v>The About Page provides information about our development team.</v>
-      </c>
-      <c r="C457" t="str">
-        <v>关于页面提供了我们开发团队的信息。</v>
-      </c>
-    </row>
-    <row r="458">
-      <c r="A458" t="str">
-        <v>tours.qsg.step8</v>
-      </c>
-      <c r="B458" t="str">
-        <v>Click here to sign in and unlock the features mentioned earlier, such as accessing registered workshops. Once logged in, you will also have the ability to upload datapacks and take full advantage of all functionalities.</v>
-      </c>
-      <c r="C458" t="str">
-        <v>点击此处登录并解锁前面提到的功能，例如访问工作坊界面。登陆后，您还将能够上传数据包并充分利用所有功能。</v>
-      </c>
-    </row>
-    <row r="459">
-      <c r="A459" t="str">
-        <v>tours.datapack.step1</v>
-      </c>
-      <c r="B459" t="str">
-        <v>Switch between different display types for datapacks: rows, cards, or compact view.</v>
-      </c>
-      <c r="C459" t="str">
-        <v>在数据包显示类型之间切换：行视图、卡片视图或紧凑视图。</v>
-      </c>
-    </row>
-    <row r="460">
-      <c r="A460" t="str">
-        <v>tours.datapack.step2</v>
-      </c>
-      <c r="B460" t="str">
-        <v>Add a datapack by clicking the checkbox</v>
-      </c>
-      <c r="C460" t="str">
-        <v>勾选添加您想要的数据包</v>
-      </c>
-    </row>
-    <row r="461">
-      <c r="A461" t="str">
-        <v>tours.datapack.step3</v>
-      </c>
-      <c r="B461" t="str">
-        <v>Click the deselect icon to deselect all datapacks</v>
-      </c>
-      <c r="C461" t="str">
-        <v>点此取消选择所有数据包</v>
-      </c>
-    </row>
-    <row r="462">
-      <c r="A462" t="str">
-        <v>tours.datapack.step4</v>
-      </c>
-      <c r="B462" t="str">
-        <v>Remember to confirm your selection</v>
-      </c>
-      <c r="C462" t="str">
-        <v>记得确认您的选择</v>
-      </c>
-    </row>
-    <row r="463">
-      <c r="A463" t="str">
-        <v>tours.settings.step1</v>
-      </c>
-      <c r="B463" t="str">
-        <v>In the Time settings, you can Set the "Top of Interval" and "Base of Interval" for your data. These fields allow you to define the starting and ending ages or stages, which can be adjusted by entering values or using the dropdown selectors. Adjust the vertical scale to change how much vertical space each million years occupies on your charts. For example, setting it higher will spread the intervals further apart, making each period easier to examine closely.</v>
-      </c>
-      <c r="C463" t="str">
-        <v>在时间设置中，您可以为您的数据设置“时间段顶部”和“时间段底部”。调整这两个值将改变图表的时间跨度，您可以通过输入值或使用下拉选择器进行调整。您还可以调整垂直比例，以改变图表中每百万年占据的垂直空间量。例如，将其设置得更高将使时间间隔进一步分开，使每个时期更易于仔细检查。</v>
-      </c>
-    </row>
-    <row r="464">
-      <c r="A464" t="str">
-        <v>tours.settings.step2</v>
-      </c>
-      <c r="B464" t="str">
-        <v>In the Preferences settings, you can customize the display options. For instance, you may choose to gray out columns with no data for selected time periods, add tooltips for additional information, or enable filtering and legend options for charts. Furthermore, you can load your settings from a file or save your current settings to a file. This feature is useful for backing up your configurations, sharing them with others, or quickly applying previously saved configurations to your chart.</v>
-      </c>
-      <c r="C464" t="str">
-        <v>在偏好中，您可以自定义显示选项。例如，您可以选择在选定时间段内将无数据的列显示为灰色，添加工具提示以提供额外信息，或启用图表的筛选和图例选项。此外，您可以从文件加载您的设置或将当前设置保存到文件中。此功能使您可以备份设置、与他人分享或快速应用以前保存的设置到您的图表中。</v>
-      </c>
-    </row>
-    <row r="465">
-      <c r="A465" t="str">
-        <v>tours.settings.step3</v>
-      </c>
-      <c r="B465" t="str">
-        <v>In Column Settings, you can deeply customize the appearance and organization of your charts.In the "Column Customization" area, you can adjust titles and shift row positions to streamline how data is displayed on your charts. Enable or disable specific elements like the chart title and Ma markers to suit your presentation needs. In the "Font Options" section, refine the appearance of your charts by choosing different fonts, sizes, and styles for headers and labels, ensuring important data stands out or meets formatting requirements. Please note that the advanced settings for columns can vary depending on the datapack you are working with, allowing for tailored configurations that best fit the data characteristics.</v>
-      </c>
-      <c r="C465" t="str">
-        <v>在列设置中，您可以深度自定义图表的外观和组织。在“列自定义”区域，您可以调整标题和移动行位置，以简化图表上数据的显示方式。根据您的展示需求启用或禁用特定元素，如图表标题和百万年标记。在“字体选项”部分，通过选择不同的字体、大小和样式为标题和标签，细化您的图表外观，确保重要数据突出显示或符合格式要求。请注意，列高级设置可能根据您正在使用的数据包而有所不同，每个数据包都有最适合数据特性的列高级设置。</v>
-      </c>
-    </row>
-    <row r="466">
-      <c r="A466" t="str">
-        <v>tours.settings.step4</v>
-      </c>
-      <c r="B466" t="str">
-        <v>In the Search Settings, you can quickly locate specific columns by entering keywords and then directly add them to your chart. Simply enter a term related to the setting you are looking for, and the system will display all relevant results.This feature is particularly useful when managing numerous data points or when you need to make quick adjustments without browsing through extensive lists.</v>
-      </c>
-      <c r="C466" t="str">
-        <v>在搜索中，您可以通过输入关键词快速定位特定列，然后直接将其添加到您的图表中。只需输入一个与您正在寻找的设置相关的词语，系统便会显示所有相关结果。此功能可以帮助您管理众多数据点，或进行快速调整而无需浏览繁杂列表。请注意目前只支持英文搜索。</v>
-      </c>
-    </row>
-    <row r="467">
-      <c r="A467" t="str">
-        <v>tours.settings.step5</v>
-      </c>
-      <c r="B467" t="str">
-        <v>The Font Settings section allows you to customize the appearance of text within your charts. You can adjust font styles, sizes, and formatting for various elements such as column headers, age labels, and more. Each setting is inheritable, ensuring consistency across related elements unless specified otherwise. Changing a font setting here applies it system-wide, but you can override these for individual columns by using the "Change Font" option within each columns settings.Experiment with different fonts and sizes to enhance readability and visual appeal of your charts.</v>
-      </c>
-      <c r="C467" t="str">
-        <v>在字体设置中您可以自定义图表内的文本外观。您可以为各种元素如列标题、年龄标签等调整字体样式、大小和格式。每项设置都是可继承的，确保相关元素间的一致性，除非另行设置。在这里更改字体设置将系统范围内应用，但您可以使用每个列设置中的“更改字体”选项覆盖这些设置。尝试不同的字体和大小，以增强图表的可读性和视觉吸引力。</v>
-      </c>
-    </row>
-    <row r="468">
-      <c r="A468" t="str">
-        <v>tours.settings.step6</v>
-      </c>
-      <c r="B468" t="str">
-        <v>In the Map Points Settings, you can access and manage geographic data points for different locations. This feature allows you to view specific location details directly on the interactive map. You can toggle different map layers and visualize data points with detailed descriptions, like latitude, longitude, and additional notes. Please note, however, that not all datapacks contain map points.</v>
-      </c>
-      <c r="C468" t="str">
-        <v>在地图点设置中，您可以访问和管理不同位置的地理数据点。此功能允许您直接在交互式地图上查看特定位置的详细信息。您可以切换不同的地图层，并用详细描述（如纬度、经度和附加说明）可视化数据点。请注意，并非所有数据包都包含地图点。</v>
-      </c>
-    </row>
-    <row r="469">
-      <c r="A469" t="str">
-        <v>tours.settings.step7</v>
-      </c>
-      <c r="B469" t="str">
-        <v>In the Datapacks Settings, you can select the datapacks you wish to use for generating charts. We offer nine official datapacks, each comprising a curated collection of datasets tailored for specific thematic explorations. You might notice that this page resembles the Datapack page; selections can be configured here or there interchangeably. For more detailed guidance on how to utilize datapacks, please refer to the Datapacks Tour in the Help page "Tours" section.</v>
-      </c>
-      <c r="C469" t="str">
-        <v>在数据包设置中，您可以选择您希望用于生成图表的数据包。我们提供九个官方数据包，每个数据包都包含为特定主题探索量身定制的数据集合。您也许已经注意到，此页面与"数据包"页面内容相同；您在两个地方都可以进行选择和设置。如需更详细的关于如何利用数据包的指导，请参阅帮助页面“导览”部分中的数据包导览。</v>
-      </c>
-    </row>
-    <row r="470">
-      <c r="A470" t="str">
-        <v>settings.column.tooltip.note-in-range</v>
-      </c>
-      <c r="C470" t="str">
-        <v>数据不在所选时间区间内</v>
-      </c>
-    </row>
-    <row r="471">
-      <c r="A471" t="str">
-        <v>language-names.en-US</v>
-      </c>
-      <c r="C471" t="str">
-        <v>English</v>
-      </c>
-    </row>
-    <row r="472">
-      <c r="A472" t="str">
-        <v>language-names.en</v>
-      </c>
-      <c r="C472" t="str">
-        <v>English</v>
-      </c>
-    </row>
-    <row r="473">
-      <c r="A473" t="str">
-        <v>language-names.zh</v>
-      </c>
-      <c r="C473" t="str">
         <v>中文</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C473"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C453"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added frontend and backend for loading chart history
</commit_message>
<xml_diff>
--- a/server/assets/translation.xlsx
+++ b/server/assets/translation.xlsx
@@ -375,7 +375,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C453"/>
+  <dimension ref="A1:C454"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4643,89 +4643,89 @@
     </row>
     <row r="417">
       <c r="A417" t="str">
-        <v>button.generate</v>
+        <v>errors.USER_FETCH_HISTORY_FAILED</v>
       </c>
       <c r="B417" t="str">
-        <v>Generate</v>
-      </c>
-      <c r="C417" t="str">
-        <v>绘制</v>
+        <v>Failed to fetch user history. Please try again later.</v>
       </c>
     </row>
     <row r="418">
       <c r="A418" t="str">
-        <v>button.generate-chart</v>
+        <v>button.generate</v>
       </c>
       <c r="B418" t="str">
-        <v>Generate Chart</v>
+        <v>Generate</v>
       </c>
       <c r="C418" t="str">
-        <v>绘制图表</v>
+        <v>绘制</v>
       </c>
     </row>
     <row r="419">
       <c r="A419" t="str">
-        <v>button.remove-cache</v>
+        <v>button.generate-chart</v>
       </c>
       <c r="B419" t="str">
-        <v>Remove Cache</v>
+        <v>Generate Chart</v>
       </c>
       <c r="C419" t="str">
-        <v>清除缓存</v>
+        <v>绘制图表</v>
       </c>
     </row>
     <row r="420">
       <c r="A420" t="str">
-        <v>button.confirm-selection</v>
+        <v>button.remove-cache</v>
       </c>
       <c r="B420" t="str">
-        <v>Confirm Selection</v>
+        <v>Remove Cache</v>
       </c>
       <c r="C420" t="str">
-        <v>确认选择</v>
+        <v>清除缓存</v>
       </c>
     </row>
     <row r="421">
       <c r="A421" t="str">
-        <v>button.generate-cross-plot</v>
+        <v>button.confirm-selection</v>
       </c>
       <c r="B421" t="str">
-        <v>Generate Cross Plot</v>
+        <v>Confirm Selection</v>
+      </c>
+      <c r="C421" t="str">
+        <v>确认选择</v>
       </c>
     </row>
     <row r="422">
       <c r="A422" t="str">
-        <v>yes</v>
+        <v>button.generate-cross-plot</v>
       </c>
       <c r="B422" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="C422" t="str">
-        <v>是</v>
+        <v>Generate Cross Plot</v>
       </c>
     </row>
     <row r="423">
       <c r="A423" t="str">
-        <v>no</v>
+        <v>yes</v>
       </c>
       <c r="B423" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="C423" t="str">
-        <v>否</v>
+        <v>是</v>
       </c>
     </row>
     <row r="424">
       <c r="A424" t="str">
-        <v>languageNames.en-US</v>
+        <v>no</v>
       </c>
       <c r="B424" t="str">
-        <v>English</v>
+        <v>No</v>
+      </c>
+      <c r="C424" t="str">
+        <v>否</v>
       </c>
     </row>
     <row r="425">
       <c r="A425" t="str">
-        <v>languageNames.en</v>
+        <v>languageNames.en-US</v>
       </c>
       <c r="B425" t="str">
         <v>English</v>
@@ -4733,284 +4733,284 @@
     </row>
     <row r="426">
       <c r="A426" t="str">
-        <v>languageNames.zh</v>
+        <v>languageNames.en</v>
       </c>
       <c r="B426" t="str">
-        <v>中文</v>
+        <v>English</v>
       </c>
     </row>
     <row r="427">
       <c r="A427" t="str">
-        <v>tours.quit</v>
+        <v>languageNames.zh</v>
       </c>
       <c r="B427" t="str">
-        <v>Quit Tour</v>
-      </c>
-      <c r="C427" t="str">
-        <v>退出导览</v>
+        <v>中文</v>
       </c>
     </row>
     <row r="428">
       <c r="A428" t="str">
-        <v>tours.finish</v>
+        <v>tours.quit</v>
       </c>
       <c r="B428" t="str">
-        <v>Finish Tour</v>
+        <v>Quit Tour</v>
       </c>
       <c r="C428" t="str">
-        <v>结束导览</v>
+        <v>退出导览</v>
       </c>
     </row>
     <row r="429">
       <c r="A429" t="str">
-        <v>tours.next</v>
+        <v>tours.finish</v>
       </c>
       <c r="B429" t="str">
-        <v>Next</v>
+        <v>Finish Tour</v>
       </c>
       <c r="C429" t="str">
-        <v>下一步</v>
+        <v>结束导览</v>
       </c>
     </row>
     <row r="430">
       <c r="A430" t="str">
-        <v>tours.back</v>
+        <v>tours.next</v>
       </c>
       <c r="B430" t="str">
-        <v>Back</v>
+        <v>Next</v>
       </c>
       <c r="C430" t="str">
-        <v>上一步</v>
+        <v>下一步</v>
       </c>
     </row>
     <row r="431">
       <c r="A431" t="str">
-        <v>tours.qsg.step1</v>
+        <v>tours.back</v>
       </c>
       <c r="B431" t="str">
-        <v>In the Presets page, we offer pre-configured settings that allow you to rapidly generate specific types of charts without configuring all options from the beginning. Each preset comes equipped with designated data packs, visual styles, and settings, enabling you to create charts with just a single click.</v>
+        <v>Back</v>
       </c>
       <c r="C431" t="str">
-        <v>在预设页面中，我们提供了预设置，允许您快速生成特定类型的图表，无需从头开始配置所有选项。每个预设都配备了指定的数据包、视觉样式和设置，使您能够一键创建图表</v>
+        <v>上一步</v>
       </c>
     </row>
     <row r="432">
       <c r="A432" t="str">
-        <v>tours.qsg.step2</v>
+        <v>tours.qsg.step1</v>
       </c>
       <c r="B432" t="str">
-        <v>In the Datapacks page, you can select the datapacks required to generate your charts. We offer nine official data packs, each containing a curated collection of datasets tailored for specific thematic explorations. For more detailed guidance on Datapacks, please refer to the Datapacks Tour under the "Tours" section</v>
+        <v>In the Presets page, we offer pre-configured settings that allow you to rapidly generate specific types of charts without configuring all options from the beginning. Each preset comes equipped with designated data packs, visual styles, and settings, enabling you to create charts with just a single click.</v>
       </c>
       <c r="C432" t="str">
-        <v>在数据包页面，您可以选择生成图表所需的数据包。我们提供九个官方数据包，每个数据包都包含为特定主题探索量身定制的数据集合集。如需更详细的数据包指导，请参考“导览”部分下的数据包导览。</v>
+        <v>在预设页面中，我们提供了预设置，允许您快速生成特定类型的图表，无需从头开始配置所有选项。每个预设都配备了指定的数据包、视觉样式和设置，使您能够一键创建图表</v>
       </c>
     </row>
     <row r="433">
       <c r="A433" t="str">
-        <v>tours.qsg.step3</v>
+        <v>tours.qsg.step2</v>
       </c>
       <c r="B433" t="str">
-        <v>In the Chart page, you can view the charts you have created and explore the detailed visualizations of geologic events. Additionally, you have the option to download and save these charts for your reference or further analysis.</v>
+        <v>In the Datapacks page, you can select the datapacks required to generate your charts. We offer nine official data packs, each containing a curated collection of datasets tailored for specific thematic explorations. For more detailed guidance on Datapacks, please refer to the Datapacks Tour under the "Tours" section</v>
       </c>
       <c r="C433" t="str">
-        <v>在图表页面，您可以查看已创建的图表并探索地质事件的详细可视化图。此外，您还可以下载并保存这些图表以供参考或进一步分析。</v>
+        <v>在数据包页面，您可以选择生成图表所需的数据包。我们提供九个官方数据包，每个数据包都包含为特定主题探索量身定制的数据集合集。如需更详细的数据包指导，请参考“导览”部分下的数据包导览。</v>
       </c>
     </row>
     <row r="434">
       <c r="A434" t="str">
-        <v>tours.qsg.step4</v>
+        <v>tours.qsg.step3</v>
       </c>
       <c r="B434" t="str">
-        <v>In the Settings page, you can customize all aspects of your charts. This includes adjusting the scale and time range, selecting which rows to display, setting the background color and font style, etc. Tailor your charts to meet your specific needs and preferences to optimize your visual analysis. For more detailed guidance on Settings, please refer to the Settings Tour under the "Tours" section</v>
+        <v>In the Chart page, you can view the charts you have created and explore the detailed visualizations of geologic events. Additionally, you have the option to download and save these charts for your reference or further analysis.</v>
       </c>
       <c r="C434" t="str">
-        <v>在设置页面，您可以自定义图表的所有方面。这包括调整比例和时间范围、选择显示哪些行、设置背景色和字体样式等。根据您的具体需求和偏好调整图表，以优化您的视觉分析。如需更详细的设置指导，请参考“导览”部分下的设置导览。</v>
+        <v>在图表页面，您可以查看已创建的图表并探索地质事件的详细可视化图。此外，您还可以下载并保存这些图表以供参考或进一步分析。</v>
       </c>
     </row>
     <row r="435">
       <c r="A435" t="str">
-        <v>tours.qsg.step5</v>
+        <v>tours.qsg.step4</v>
       </c>
       <c r="B435" t="str">
-        <v>In the Help Page, you can find detailed assistance and information on how to use the website.</v>
+        <v>In the Settings page, you can customize all aspects of your charts. This includes adjusting the scale and time range, selecting which rows to display, setting the background color and font style, etc. Tailor your charts to meet your specific needs and preferences to optimize your visual analysis. For more detailed guidance on Settings, please refer to the Settings Tour under the "Tours" section</v>
       </c>
       <c r="C435" t="str">
-        <v>在帮助页面，您可以找到关于如何使用网站的详细帮助和信息。</v>
+        <v>在设置页面，您可以自定义图表的所有方面。这包括调整比例和时间范围、选择显示哪些行、设置背景色和字体样式等。根据您的具体需求和偏好调整图表，以优化您的视觉分析。如需更详细的设置指导，请参考“导览”部分下的设置导览。</v>
       </c>
     </row>
     <row r="436">
       <c r="A436" t="str">
-        <v>tours.qsg.step6</v>
+        <v>tours.qsg.step5</v>
       </c>
       <c r="B436" t="str">
-        <v>In the Workshops Page, you can access a range of educational and experimental tutorials that offer in-depth guidance. Here, you can explore the workshops you have registered for, allowing you to engage with the content and enhance your skills in a hands-on learning environment.</v>
+        <v>In the Help Page, you can find detailed assistance and information on how to use the website.</v>
       </c>
       <c r="C436" t="str">
-        <v>在工作坊页面，您可以访问一系列提供深入指导的教育和实验教程。在这里，您可以探索已注册的研讨会，通过亲身实践的学习环境来提升您的技能。</v>
+        <v>在帮助页面，您可以找到关于如何使用网站的详细帮助和信息。</v>
       </c>
     </row>
     <row r="437">
       <c r="A437" t="str">
-        <v>tours.qsg.step7</v>
+        <v>tours.qsg.step6</v>
       </c>
       <c r="B437" t="str">
-        <v>The About Page provides information about our development team.</v>
+        <v>In the Workshops Page, you can access a range of educational and experimental tutorials that offer in-depth guidance. Here, you can explore the workshops you have registered for, allowing you to engage with the content and enhance your skills in a hands-on learning environment.</v>
       </c>
       <c r="C437" t="str">
-        <v>关于页面提供了我们开发团队的信息。</v>
+        <v>在工作坊页面，您可以访问一系列提供深入指导的教育和实验教程。在这里，您可以探索已注册的研讨会，通过亲身实践的学习环境来提升您的技能。</v>
       </c>
     </row>
     <row r="438">
       <c r="A438" t="str">
-        <v>tours.qsg.step8</v>
+        <v>tours.qsg.step7</v>
       </c>
       <c r="B438" t="str">
-        <v>Click here to sign in and unlock the features mentioned earlier, such as accessing registered workshops. Once logged in, you will also have the ability to upload datapacks and take full advantage of all functionalities.</v>
+        <v>The About Page provides information about our development team.</v>
       </c>
       <c r="C438" t="str">
-        <v>点击此处登录并解锁前面提到的功能，例如访问工作坊界面。登陆后，您还将能够上传数据包并充分利用所有功能。</v>
+        <v>关于页面提供了我们开发团队的信息。</v>
       </c>
     </row>
     <row r="439">
       <c r="A439" t="str">
-        <v>tours.datapack.step1</v>
+        <v>tours.qsg.step8</v>
       </c>
       <c r="B439" t="str">
-        <v>Switch between different display types for datapacks: rows, cards, or compact view.</v>
+        <v>Click here to sign in and unlock the features mentioned earlier, such as accessing registered workshops. Once logged in, you will also have the ability to upload datapacks and take full advantage of all functionalities.</v>
       </c>
       <c r="C439" t="str">
-        <v>在数据包显示类型之间切换：行视图、卡片视图或紧凑视图。</v>
+        <v>点击此处登录并解锁前面提到的功能，例如访问工作坊界面。登陆后，您还将能够上传数据包并充分利用所有功能。</v>
       </c>
     </row>
     <row r="440">
       <c r="A440" t="str">
-        <v>tours.datapack.step2</v>
+        <v>tours.datapack.step1</v>
       </c>
       <c r="B440" t="str">
-        <v>Add a datapack by clicking the checkbox</v>
+        <v>Switch between different display types for datapacks: rows, cards, or compact view.</v>
       </c>
       <c r="C440" t="str">
-        <v>勾选添加您想要的数据包</v>
+        <v>在数据包显示类型之间切换：行视图、卡片视图或紧凑视图。</v>
       </c>
     </row>
     <row r="441">
       <c r="A441" t="str">
-        <v>tours.datapack.step3</v>
+        <v>tours.datapack.step2</v>
       </c>
       <c r="B441" t="str">
-        <v>Click the deselect icon to deselect all datapacks</v>
+        <v>Add a datapack by clicking the checkbox</v>
       </c>
       <c r="C441" t="str">
-        <v>点此取消选择所有数据包</v>
+        <v>勾选添加您想要的数据包</v>
       </c>
     </row>
     <row r="442">
       <c r="A442" t="str">
-        <v>tours.datapack.step4</v>
+        <v>tours.datapack.step3</v>
       </c>
       <c r="B442" t="str">
-        <v>Remember to confirm your selection</v>
+        <v>Click the deselect icon to deselect all datapacks</v>
       </c>
       <c r="C442" t="str">
-        <v>记得确认您的选择</v>
+        <v>点此取消选择所有数据包</v>
       </c>
     </row>
     <row r="443">
       <c r="A443" t="str">
-        <v>tours.settings.step1</v>
+        <v>tours.datapack.step4</v>
       </c>
       <c r="B443" t="str">
-        <v>In the Time settings, you can Set the "Top of Interval" and "Base of Interval" for your data. These fields allow you to define the starting and ending ages or stages, which can be adjusted by entering values or using the dropdown selectors. Adjust the vertical scale to change how much vertical space each million years occupies on your charts. For example, setting it higher will spread the intervals further apart, making each period easier to examine closely.</v>
+        <v>Remember to confirm your selection</v>
       </c>
       <c r="C443" t="str">
-        <v>在时间设置中，您可以为您的数据设置“时间段顶部”和“时间段底部”。调整这两个值将改变图表的时间跨度，您可以通过输入值或使用下拉选择器进行调整。您还可以调整垂直比例，以改变图表中每百万年占据的垂直空间量。例如，将其设置得更高将使时间间隔进一步分开，使每个时期更易于仔细检查。</v>
+        <v>记得确认您的选择</v>
       </c>
     </row>
     <row r="444">
       <c r="A444" t="str">
-        <v>tours.settings.step2</v>
+        <v>tours.settings.step1</v>
       </c>
       <c r="B444" t="str">
-        <v>In the Preferences settings, you can customize the display options. For instance, you may choose to gray out columns with no data for selected time periods, add tooltips for additional information, or enable filtering and legend options for charts. Furthermore, you can load your settings from a file or save your current settings to a file. This feature is useful for backing up your configurations, sharing them with others, or quickly applying previously saved configurations to your chart.</v>
+        <v>In the Time settings, you can Set the "Top of Interval" and "Base of Interval" for your data. These fields allow you to define the starting and ending ages or stages, which can be adjusted by entering values or using the dropdown selectors. Adjust the vertical scale to change how much vertical space each million years occupies on your charts. For example, setting it higher will spread the intervals further apart, making each period easier to examine closely.</v>
       </c>
       <c r="C444" t="str">
-        <v>在偏好中，您可以自定义显示选项。例如，您可以选择在选定时间段内将无数据的列显示为灰色，添加工具提示以提供额外信息，或启用图表的筛选和图例选项。此外，您可以从文件加载您的设置或将当前设置保存到文件中。此功能使您可以备份设置、与他人分享或快速应用以前保存的设置到您的图表中。</v>
+        <v>在时间设置中，您可以为您的数据设置“时间段顶部”和“时间段底部”。调整这两个值将改变图表的时间跨度，您可以通过输入值或使用下拉选择器进行调整。您还可以调整垂直比例，以改变图表中每百万年占据的垂直空间量。例如，将其设置得更高将使时间间隔进一步分开，使每个时期更易于仔细检查。</v>
       </c>
     </row>
     <row r="445">
       <c r="A445" t="str">
-        <v>tours.settings.step3</v>
+        <v>tours.settings.step2</v>
       </c>
       <c r="B445" t="str">
-        <v>In Column Settings, you can deeply customize the appearance and organization of your charts.In the "Column Customization" area, you can adjust titles and shift row positions to streamline how data is displayed on your charts. Enable or disable specific elements like the chart title and Ma markers to suit your presentation needs. In the "Font Options" section, refine the appearance of your charts by choosing different fonts, sizes, and styles for headers and labels, ensuring important data stands out or meets formatting requirements. Please note that the advanced settings for columns can vary depending on the datapack you are working with, allowing for tailored configurations that best fit the data characteristics.</v>
+        <v>In the Preferences settings, you can customize the display options. For instance, you may choose to gray out columns with no data for selected time periods, add tooltips for additional information, or enable filtering and legend options for charts. Furthermore, you can load your settings from a file or save your current settings to a file. This feature is useful for backing up your configurations, sharing them with others, or quickly applying previously saved configurations to your chart.</v>
       </c>
       <c r="C445" t="str">
-        <v>在列设置中，您可以深度自定义图表的外观和组织。在“列自定义”区域，您可以调整标题和移动行位置，以简化图表上数据的显示方式。根据您的展示需求启用或禁用特定元素，如图表标题和百万年标记。在“字体选项”部分，通过选择不同的字体、大小和样式为标题和标签，细化您的图表外观，确保重要数据突出显示或符合格式要求。请注意，列高级设置可能根据您正在使用的数据包而有所不同，每个数据包都有最适合数据特性的列高级设置。</v>
+        <v>在偏好中，您可以自定义显示选项。例如，您可以选择在选定时间段内将无数据的列显示为灰色，添加工具提示以提供额外信息，或启用图表的筛选和图例选项。此外，您可以从文件加载您的设置或将当前设置保存到文件中。此功能使您可以备份设置、与他人分享或快速应用以前保存的设置到您的图表中。</v>
       </c>
     </row>
     <row r="446">
       <c r="A446" t="str">
-        <v>tours.settings.step4</v>
+        <v>tours.settings.step3</v>
       </c>
       <c r="B446" t="str">
-        <v>In the Search Settings, you can quickly locate specific columns by entering keywords and then directly add them to your chart. Simply enter a term related to the setting you are looking for, and the system will display all relevant results.This feature is particularly useful when managing numerous data points or when you need to make quick adjustments without browsing through extensive lists.</v>
+        <v>In Column Settings, you can deeply customize the appearance and organization of your charts.In the "Column Customization" area, you can adjust titles and shift row positions to streamline how data is displayed on your charts. Enable or disable specific elements like the chart title and Ma markers to suit your presentation needs. In the "Font Options" section, refine the appearance of your charts by choosing different fonts, sizes, and styles for headers and labels, ensuring important data stands out or meets formatting requirements. Please note that the advanced settings for columns can vary depending on the datapack you are working with, allowing for tailored configurations that best fit the data characteristics.</v>
       </c>
       <c r="C446" t="str">
-        <v>在搜索中，您可以通过输入关键词快速定位特定列，然后直接将其添加到您的图表中。只需输入一个与您正在寻找的设置相关的词语，系统便会显示所有相关结果。此功能可以帮助您管理众多数据点，或进行快速调整而无需浏览繁杂列表。请注意目前只支持英文搜索。</v>
+        <v>在列设置中，您可以深度自定义图表的外观和组织。在“列自定义”区域，您可以调整标题和移动行位置，以简化图表上数据的显示方式。根据您的展示需求启用或禁用特定元素，如图表标题和百万年标记。在“字体选项”部分，通过选择不同的字体、大小和样式为标题和标签，细化您的图表外观，确保重要数据突出显示或符合格式要求。请注意，列高级设置可能根据您正在使用的数据包而有所不同，每个数据包都有最适合数据特性的列高级设置。</v>
       </c>
     </row>
     <row r="447">
       <c r="A447" t="str">
-        <v>tours.settings.step5</v>
+        <v>tours.settings.step4</v>
       </c>
       <c r="B447" t="str">
-        <v>The Font Settings section allows you to customize the appearance of text within your charts. You can adjust font styles, sizes, and formatting for various elements such as column headers, age labels, and more. Each setting is inheritable, ensuring consistency across related elements unless specified otherwise. Changing a font setting here applies it system-wide, but you can override these for individual columns by using the "Change Font" option within each columns settings.Experiment with different fonts and sizes to enhance readability and visual appeal of your charts.</v>
+        <v>In the Search Settings, you can quickly locate specific columns by entering keywords and then directly add them to your chart. Simply enter a term related to the setting you are looking for, and the system will display all relevant results.This feature is particularly useful when managing numerous data points or when you need to make quick adjustments without browsing through extensive lists.</v>
       </c>
       <c r="C447" t="str">
-        <v>在字体设置中您可以自定义图表内的文本外观。您可以为各种元素如列标题、年龄标签等调整字体样式、大小和格式。每项设置都是可继承的，确保相关元素间的一致性，除非另行设置。在这里更改字体设置将系统范围内应用，但您可以使用每个列设置中的“更改字体”选项覆盖这些设置。尝试不同的字体和大小，以增强图表的可读性和视觉吸引力。</v>
+        <v>在搜索中，您可以通过输入关键词快速定位特定列，然后直接将其添加到您的图表中。只需输入一个与您正在寻找的设置相关的词语，系统便会显示所有相关结果。此功能可以帮助您管理众多数据点，或进行快速调整而无需浏览繁杂列表。请注意目前只支持英文搜索。</v>
       </c>
     </row>
     <row r="448">
       <c r="A448" t="str">
-        <v>tours.settings.step6</v>
+        <v>tours.settings.step5</v>
       </c>
       <c r="B448" t="str">
-        <v>In the Map Points Settings, you can access and manage geographic data points for different locations. This feature allows you to view specific location details directly on the interactive map. You can toggle different map layers and visualize data points with detailed descriptions, like latitude, longitude, and additional notes. Please note, however, that not all datapacks contain map points.</v>
+        <v>The Font Settings section allows you to customize the appearance of text within your charts. You can adjust font styles, sizes, and formatting for various elements such as column headers, age labels, and more. Each setting is inheritable, ensuring consistency across related elements unless specified otherwise. Changing a font setting here applies it system-wide, but you can override these for individual columns by using the "Change Font" option within each columns settings.Experiment with different fonts and sizes to enhance readability and visual appeal of your charts.</v>
       </c>
       <c r="C448" t="str">
-        <v>在地图点设置中，您可以访问和管理不同位置的地理数据点。此功能允许您直接在交互式地图上查看特定位置的详细信息。您可以切换不同的地图层，并用详细描述（如纬度、经度和附加说明）可视化数据点。请注意，并非所有数据包都包含地图点。</v>
+        <v>在字体设置中您可以自定义图表内的文本外观。您可以为各种元素如列标题、年龄标签等调整字体样式、大小和格式。每项设置都是可继承的，确保相关元素间的一致性，除非另行设置。在这里更改字体设置将系统范围内应用，但您可以使用每个列设置中的“更改字体”选项覆盖这些设置。尝试不同的字体和大小，以增强图表的可读性和视觉吸引力。</v>
       </c>
     </row>
     <row r="449">
       <c r="A449" t="str">
-        <v>tours.settings.step7</v>
+        <v>tours.settings.step6</v>
       </c>
       <c r="B449" t="str">
-        <v>In the Datapacks Settings, you can select the datapacks you wish to use for generating charts. We offer nine official datapacks, each comprising a curated collection of datasets tailored for specific thematic explorations. You might notice that this page resembles the Datapack page; selections can be configured here or there interchangeably. For more detailed guidance on how to utilize datapacks, please refer to the Datapacks Tour in the Help page "Tours" section.</v>
+        <v>In the Map Points Settings, you can access and manage geographic data points for different locations. This feature allows you to view specific location details directly on the interactive map. You can toggle different map layers and visualize data points with detailed descriptions, like latitude, longitude, and additional notes. Please note, however, that not all datapacks contain map points.</v>
       </c>
       <c r="C449" t="str">
-        <v>在数据包设置中，您可以选择您希望用于生成图表的数据包。我们提供九个官方数据包，每个数据包都包含为特定主题探索量身定制的数据集合。您也许已经注意到，此页面与"数据包"页面内容相同；您在两个地方都可以进行选择和设置。如需更详细的关于如何利用数据包的指导，请参阅帮助页面“导览”部分中的数据包导览。</v>
+        <v>在地图点设置中，您可以访问和管理不同位置的地理数据点。此功能允许您直接在交互式地图上查看特定位置的详细信息。您可以切换不同的地图层，并用详细描述（如纬度、经度和附加说明）可视化数据点。请注意，并非所有数据包都包含地图点。</v>
       </c>
     </row>
     <row r="450">
       <c r="A450" t="str">
-        <v>settings.column.tooltip.note-in-range</v>
+        <v>tours.settings.step7</v>
+      </c>
+      <c r="B450" t="str">
+        <v>In the Datapacks Settings, you can select the datapacks you wish to use for generating charts. We offer nine official datapacks, each comprising a curated collection of datasets tailored for specific thematic explorations. You might notice that this page resembles the Datapack page; selections can be configured here or there interchangeably. For more detailed guidance on how to utilize datapacks, please refer to the Datapacks Tour in the Help page "Tours" section.</v>
       </c>
       <c r="C450" t="str">
-        <v>数据不在所选时间区间内</v>
+        <v>在数据包设置中，您可以选择您希望用于生成图表的数据包。我们提供九个官方数据包，每个数据包都包含为特定主题探索量身定制的数据集合。您也许已经注意到，此页面与"数据包"页面内容相同；您在两个地方都可以进行选择和设置。如需更详细的关于如何利用数据包的指导，请参阅帮助页面“导览”部分中的数据包导览。</v>
       </c>
     </row>
     <row r="451">
       <c r="A451" t="str">
-        <v>language-names.en-US</v>
+        <v>settings.column.tooltip.note-in-range</v>
       </c>
       <c r="C451" t="str">
-        <v>English</v>
+        <v>数据不在所选时间区间内</v>
       </c>
     </row>
     <row r="452">
       <c r="A452" t="str">
-        <v>language-names.en</v>
+        <v>language-names.en-US</v>
       </c>
       <c r="C452" t="str">
         <v>English</v>
@@ -5018,15 +5018,23 @@
     </row>
     <row r="453">
       <c r="A453" t="str">
+        <v>language-names.en</v>
+      </c>
+      <c r="C453" t="str">
+        <v>English</v>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="str">
         <v>language-names.zh</v>
       </c>
-      <c r="C453" t="str">
+      <c r="C454" t="str">
         <v>中文</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C453"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C454"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added ability to delete history
</commit_message>
<xml_diff>
--- a/server/assets/translation.xlsx
+++ b/server/assets/translation.xlsx
@@ -375,7 +375,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C454"/>
+  <dimension ref="A1:C455"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4651,89 +4651,89 @@
     </row>
     <row r="418">
       <c r="A418" t="str">
-        <v>button.generate</v>
+        <v>errors.USER_DELETE_HISTORY_FAILED</v>
       </c>
       <c r="B418" t="str">
-        <v>Generate</v>
-      </c>
-      <c r="C418" t="str">
-        <v>绘制</v>
+        <v>Failed to delete user history. Please try again later</v>
       </c>
     </row>
     <row r="419">
       <c r="A419" t="str">
-        <v>button.generate-chart</v>
+        <v>button.generate</v>
       </c>
       <c r="B419" t="str">
-        <v>Generate Chart</v>
+        <v>Generate</v>
       </c>
       <c r="C419" t="str">
-        <v>绘制图表</v>
+        <v>绘制</v>
       </c>
     </row>
     <row r="420">
       <c r="A420" t="str">
-        <v>button.remove-cache</v>
+        <v>button.generate-chart</v>
       </c>
       <c r="B420" t="str">
-        <v>Remove Cache</v>
+        <v>Generate Chart</v>
       </c>
       <c r="C420" t="str">
-        <v>清除缓存</v>
+        <v>绘制图表</v>
       </c>
     </row>
     <row r="421">
       <c r="A421" t="str">
-        <v>button.confirm-selection</v>
+        <v>button.remove-cache</v>
       </c>
       <c r="B421" t="str">
-        <v>Confirm Selection</v>
+        <v>Remove Cache</v>
       </c>
       <c r="C421" t="str">
-        <v>确认选择</v>
+        <v>清除缓存</v>
       </c>
     </row>
     <row r="422">
       <c r="A422" t="str">
-        <v>button.generate-cross-plot</v>
+        <v>button.confirm-selection</v>
       </c>
       <c r="B422" t="str">
-        <v>Generate Cross Plot</v>
+        <v>Confirm Selection</v>
+      </c>
+      <c r="C422" t="str">
+        <v>确认选择</v>
       </c>
     </row>
     <row r="423">
       <c r="A423" t="str">
-        <v>yes</v>
+        <v>button.generate-cross-plot</v>
       </c>
       <c r="B423" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="C423" t="str">
-        <v>是</v>
+        <v>Generate Cross Plot</v>
       </c>
     </row>
     <row r="424">
       <c r="A424" t="str">
-        <v>no</v>
+        <v>yes</v>
       </c>
       <c r="B424" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="C424" t="str">
-        <v>否</v>
+        <v>是</v>
       </c>
     </row>
     <row r="425">
       <c r="A425" t="str">
-        <v>languageNames.en-US</v>
+        <v>no</v>
       </c>
       <c r="B425" t="str">
-        <v>English</v>
+        <v>No</v>
+      </c>
+      <c r="C425" t="str">
+        <v>否</v>
       </c>
     </row>
     <row r="426">
       <c r="A426" t="str">
-        <v>languageNames.en</v>
+        <v>languageNames.en-US</v>
       </c>
       <c r="B426" t="str">
         <v>English</v>
@@ -4741,284 +4741,284 @@
     </row>
     <row r="427">
       <c r="A427" t="str">
-        <v>languageNames.zh</v>
+        <v>languageNames.en</v>
       </c>
       <c r="B427" t="str">
-        <v>中文</v>
+        <v>English</v>
       </c>
     </row>
     <row r="428">
       <c r="A428" t="str">
-        <v>tours.quit</v>
+        <v>languageNames.zh</v>
       </c>
       <c r="B428" t="str">
-        <v>Quit Tour</v>
-      </c>
-      <c r="C428" t="str">
-        <v>退出导览</v>
+        <v>中文</v>
       </c>
     </row>
     <row r="429">
       <c r="A429" t="str">
-        <v>tours.finish</v>
+        <v>tours.quit</v>
       </c>
       <c r="B429" t="str">
-        <v>Finish Tour</v>
+        <v>Quit Tour</v>
       </c>
       <c r="C429" t="str">
-        <v>结束导览</v>
+        <v>退出导览</v>
       </c>
     </row>
     <row r="430">
       <c r="A430" t="str">
-        <v>tours.next</v>
+        <v>tours.finish</v>
       </c>
       <c r="B430" t="str">
-        <v>Next</v>
+        <v>Finish Tour</v>
       </c>
       <c r="C430" t="str">
-        <v>下一步</v>
+        <v>结束导览</v>
       </c>
     </row>
     <row r="431">
       <c r="A431" t="str">
-        <v>tours.back</v>
+        <v>tours.next</v>
       </c>
       <c r="B431" t="str">
-        <v>Back</v>
+        <v>Next</v>
       </c>
       <c r="C431" t="str">
-        <v>上一步</v>
+        <v>下一步</v>
       </c>
     </row>
     <row r="432">
       <c r="A432" t="str">
-        <v>tours.qsg.step1</v>
+        <v>tours.back</v>
       </c>
       <c r="B432" t="str">
-        <v>In the Presets page, we offer pre-configured settings that allow you to rapidly generate specific types of charts without configuring all options from the beginning. Each preset comes equipped with designated data packs, visual styles, and settings, enabling you to create charts with just a single click.</v>
+        <v>Back</v>
       </c>
       <c r="C432" t="str">
-        <v>在预设页面中，我们提供了预设置，允许您快速生成特定类型的图表，无需从头开始配置所有选项。每个预设都配备了指定的数据包、视觉样式和设置，使您能够一键创建图表</v>
+        <v>上一步</v>
       </c>
     </row>
     <row r="433">
       <c r="A433" t="str">
-        <v>tours.qsg.step2</v>
+        <v>tours.qsg.step1</v>
       </c>
       <c r="B433" t="str">
-        <v>In the Datapacks page, you can select the datapacks required to generate your charts. We offer nine official data packs, each containing a curated collection of datasets tailored for specific thematic explorations. For more detailed guidance on Datapacks, please refer to the Datapacks Tour under the "Tours" section</v>
+        <v>In the Presets page, we offer pre-configured settings that allow you to rapidly generate specific types of charts without configuring all options from the beginning. Each preset comes equipped with designated data packs, visual styles, and settings, enabling you to create charts with just a single click.</v>
       </c>
       <c r="C433" t="str">
-        <v>在数据包页面，您可以选择生成图表所需的数据包。我们提供九个官方数据包，每个数据包都包含为特定主题探索量身定制的数据集合集。如需更详细的数据包指导，请参考“导览”部分下的数据包导览。</v>
+        <v>在预设页面中，我们提供了预设置，允许您快速生成特定类型的图表，无需从头开始配置所有选项。每个预设都配备了指定的数据包、视觉样式和设置，使您能够一键创建图表</v>
       </c>
     </row>
     <row r="434">
       <c r="A434" t="str">
-        <v>tours.qsg.step3</v>
+        <v>tours.qsg.step2</v>
       </c>
       <c r="B434" t="str">
-        <v>In the Chart page, you can view the charts you have created and explore the detailed visualizations of geologic events. Additionally, you have the option to download and save these charts for your reference or further analysis.</v>
+        <v>In the Datapacks page, you can select the datapacks required to generate your charts. We offer nine official data packs, each containing a curated collection of datasets tailored for specific thematic explorations. For more detailed guidance on Datapacks, please refer to the Datapacks Tour under the "Tours" section</v>
       </c>
       <c r="C434" t="str">
-        <v>在图表页面，您可以查看已创建的图表并探索地质事件的详细可视化图。此外，您还可以下载并保存这些图表以供参考或进一步分析。</v>
+        <v>在数据包页面，您可以选择生成图表所需的数据包。我们提供九个官方数据包，每个数据包都包含为特定主题探索量身定制的数据集合集。如需更详细的数据包指导，请参考“导览”部分下的数据包导览。</v>
       </c>
     </row>
     <row r="435">
       <c r="A435" t="str">
-        <v>tours.qsg.step4</v>
+        <v>tours.qsg.step3</v>
       </c>
       <c r="B435" t="str">
-        <v>In the Settings page, you can customize all aspects of your charts. This includes adjusting the scale and time range, selecting which rows to display, setting the background color and font style, etc. Tailor your charts to meet your specific needs and preferences to optimize your visual analysis. For more detailed guidance on Settings, please refer to the Settings Tour under the "Tours" section</v>
+        <v>In the Chart page, you can view the charts you have created and explore the detailed visualizations of geologic events. Additionally, you have the option to download and save these charts for your reference or further analysis.</v>
       </c>
       <c r="C435" t="str">
-        <v>在设置页面，您可以自定义图表的所有方面。这包括调整比例和时间范围、选择显示哪些行、设置背景色和字体样式等。根据您的具体需求和偏好调整图表，以优化您的视觉分析。如需更详细的设置指导，请参考“导览”部分下的设置导览。</v>
+        <v>在图表页面，您可以查看已创建的图表并探索地质事件的详细可视化图。此外，您还可以下载并保存这些图表以供参考或进一步分析。</v>
       </c>
     </row>
     <row r="436">
       <c r="A436" t="str">
-        <v>tours.qsg.step5</v>
+        <v>tours.qsg.step4</v>
       </c>
       <c r="B436" t="str">
-        <v>In the Help Page, you can find detailed assistance and information on how to use the website.</v>
+        <v>In the Settings page, you can customize all aspects of your charts. This includes adjusting the scale and time range, selecting which rows to display, setting the background color and font style, etc. Tailor your charts to meet your specific needs and preferences to optimize your visual analysis. For more detailed guidance on Settings, please refer to the Settings Tour under the "Tours" section</v>
       </c>
       <c r="C436" t="str">
-        <v>在帮助页面，您可以找到关于如何使用网站的详细帮助和信息。</v>
+        <v>在设置页面，您可以自定义图表的所有方面。这包括调整比例和时间范围、选择显示哪些行、设置背景色和字体样式等。根据您的具体需求和偏好调整图表，以优化您的视觉分析。如需更详细的设置指导，请参考“导览”部分下的设置导览。</v>
       </c>
     </row>
     <row r="437">
       <c r="A437" t="str">
-        <v>tours.qsg.step6</v>
+        <v>tours.qsg.step5</v>
       </c>
       <c r="B437" t="str">
-        <v>In the Workshops Page, you can access a range of educational and experimental tutorials that offer in-depth guidance. Here, you can explore the workshops you have registered for, allowing you to engage with the content and enhance your skills in a hands-on learning environment.</v>
+        <v>In the Help Page, you can find detailed assistance and information on how to use the website.</v>
       </c>
       <c r="C437" t="str">
-        <v>在工作坊页面，您可以访问一系列提供深入指导的教育和实验教程。在这里，您可以探索已注册的研讨会，通过亲身实践的学习环境来提升您的技能。</v>
+        <v>在帮助页面，您可以找到关于如何使用网站的详细帮助和信息。</v>
       </c>
     </row>
     <row r="438">
       <c r="A438" t="str">
-        <v>tours.qsg.step7</v>
+        <v>tours.qsg.step6</v>
       </c>
       <c r="B438" t="str">
-        <v>The About Page provides information about our development team.</v>
+        <v>In the Workshops Page, you can access a range of educational and experimental tutorials that offer in-depth guidance. Here, you can explore the workshops you have registered for, allowing you to engage with the content and enhance your skills in a hands-on learning environment.</v>
       </c>
       <c r="C438" t="str">
-        <v>关于页面提供了我们开发团队的信息。</v>
+        <v>在工作坊页面，您可以访问一系列提供深入指导的教育和实验教程。在这里，您可以探索已注册的研讨会，通过亲身实践的学习环境来提升您的技能。</v>
       </c>
     </row>
     <row r="439">
       <c r="A439" t="str">
-        <v>tours.qsg.step8</v>
+        <v>tours.qsg.step7</v>
       </c>
       <c r="B439" t="str">
-        <v>Click here to sign in and unlock the features mentioned earlier, such as accessing registered workshops. Once logged in, you will also have the ability to upload datapacks and take full advantage of all functionalities.</v>
+        <v>The About Page provides information about our development team.</v>
       </c>
       <c r="C439" t="str">
-        <v>点击此处登录并解锁前面提到的功能，例如访问工作坊界面。登陆后，您还将能够上传数据包并充分利用所有功能。</v>
+        <v>关于页面提供了我们开发团队的信息。</v>
       </c>
     </row>
     <row r="440">
       <c r="A440" t="str">
-        <v>tours.datapack.step1</v>
+        <v>tours.qsg.step8</v>
       </c>
       <c r="B440" t="str">
-        <v>Switch between different display types for datapacks: rows, cards, or compact view.</v>
+        <v>Click here to sign in and unlock the features mentioned earlier, such as accessing registered workshops. Once logged in, you will also have the ability to upload datapacks and take full advantage of all functionalities.</v>
       </c>
       <c r="C440" t="str">
-        <v>在数据包显示类型之间切换：行视图、卡片视图或紧凑视图。</v>
+        <v>点击此处登录并解锁前面提到的功能，例如访问工作坊界面。登陆后，您还将能够上传数据包并充分利用所有功能。</v>
       </c>
     </row>
     <row r="441">
       <c r="A441" t="str">
-        <v>tours.datapack.step2</v>
+        <v>tours.datapack.step1</v>
       </c>
       <c r="B441" t="str">
-        <v>Add a datapack by clicking the checkbox</v>
+        <v>Switch between different display types for datapacks: rows, cards, or compact view.</v>
       </c>
       <c r="C441" t="str">
-        <v>勾选添加您想要的数据包</v>
+        <v>在数据包显示类型之间切换：行视图、卡片视图或紧凑视图。</v>
       </c>
     </row>
     <row r="442">
       <c r="A442" t="str">
-        <v>tours.datapack.step3</v>
+        <v>tours.datapack.step2</v>
       </c>
       <c r="B442" t="str">
-        <v>Click the deselect icon to deselect all datapacks</v>
+        <v>Add a datapack by clicking the checkbox</v>
       </c>
       <c r="C442" t="str">
-        <v>点此取消选择所有数据包</v>
+        <v>勾选添加您想要的数据包</v>
       </c>
     </row>
     <row r="443">
       <c r="A443" t="str">
-        <v>tours.datapack.step4</v>
+        <v>tours.datapack.step3</v>
       </c>
       <c r="B443" t="str">
-        <v>Remember to confirm your selection</v>
+        <v>Click the deselect icon to deselect all datapacks</v>
       </c>
       <c r="C443" t="str">
-        <v>记得确认您的选择</v>
+        <v>点此取消选择所有数据包</v>
       </c>
     </row>
     <row r="444">
       <c r="A444" t="str">
-        <v>tours.settings.step1</v>
+        <v>tours.datapack.step4</v>
       </c>
       <c r="B444" t="str">
-        <v>In the Time settings, you can Set the "Top of Interval" and "Base of Interval" for your data. These fields allow you to define the starting and ending ages or stages, which can be adjusted by entering values or using the dropdown selectors. Adjust the vertical scale to change how much vertical space each million years occupies on your charts. For example, setting it higher will spread the intervals further apart, making each period easier to examine closely.</v>
+        <v>Remember to confirm your selection</v>
       </c>
       <c r="C444" t="str">
-        <v>在时间设置中，您可以为您的数据设置“时间段顶部”和“时间段底部”。调整这两个值将改变图表的时间跨度，您可以通过输入值或使用下拉选择器进行调整。您还可以调整垂直比例，以改变图表中每百万年占据的垂直空间量。例如，将其设置得更高将使时间间隔进一步分开，使每个时期更易于仔细检查。</v>
+        <v>记得确认您的选择</v>
       </c>
     </row>
     <row r="445">
       <c r="A445" t="str">
-        <v>tours.settings.step2</v>
+        <v>tours.settings.step1</v>
       </c>
       <c r="B445" t="str">
-        <v>In the Preferences settings, you can customize the display options. For instance, you may choose to gray out columns with no data for selected time periods, add tooltips for additional information, or enable filtering and legend options for charts. Furthermore, you can load your settings from a file or save your current settings to a file. This feature is useful for backing up your configurations, sharing them with others, or quickly applying previously saved configurations to your chart.</v>
+        <v>In the Time settings, you can Set the "Top of Interval" and "Base of Interval" for your data. These fields allow you to define the starting and ending ages or stages, which can be adjusted by entering values or using the dropdown selectors. Adjust the vertical scale to change how much vertical space each million years occupies on your charts. For example, setting it higher will spread the intervals further apart, making each period easier to examine closely.</v>
       </c>
       <c r="C445" t="str">
-        <v>在偏好中，您可以自定义显示选项。例如，您可以选择在选定时间段内将无数据的列显示为灰色，添加工具提示以提供额外信息，或启用图表的筛选和图例选项。此外，您可以从文件加载您的设置或将当前设置保存到文件中。此功能使您可以备份设置、与他人分享或快速应用以前保存的设置到您的图表中。</v>
+        <v>在时间设置中，您可以为您的数据设置“时间段顶部”和“时间段底部”。调整这两个值将改变图表的时间跨度，您可以通过输入值或使用下拉选择器进行调整。您还可以调整垂直比例，以改变图表中每百万年占据的垂直空间量。例如，将其设置得更高将使时间间隔进一步分开，使每个时期更易于仔细检查。</v>
       </c>
     </row>
     <row r="446">
       <c r="A446" t="str">
-        <v>tours.settings.step3</v>
+        <v>tours.settings.step2</v>
       </c>
       <c r="B446" t="str">
-        <v>In Column Settings, you can deeply customize the appearance and organization of your charts.In the "Column Customization" area, you can adjust titles and shift row positions to streamline how data is displayed on your charts. Enable or disable specific elements like the chart title and Ma markers to suit your presentation needs. In the "Font Options" section, refine the appearance of your charts by choosing different fonts, sizes, and styles for headers and labels, ensuring important data stands out or meets formatting requirements. Please note that the advanced settings for columns can vary depending on the datapack you are working with, allowing for tailored configurations that best fit the data characteristics.</v>
+        <v>In the Preferences settings, you can customize the display options. For instance, you may choose to gray out columns with no data for selected time periods, add tooltips for additional information, or enable filtering and legend options for charts. Furthermore, you can load your settings from a file or save your current settings to a file. This feature is useful for backing up your configurations, sharing them with others, or quickly applying previously saved configurations to your chart.</v>
       </c>
       <c r="C446" t="str">
-        <v>在列设置中，您可以深度自定义图表的外观和组织。在“列自定义”区域，您可以调整标题和移动行位置，以简化图表上数据的显示方式。根据您的展示需求启用或禁用特定元素，如图表标题和百万年标记。在“字体选项”部分，通过选择不同的字体、大小和样式为标题和标签，细化您的图表外观，确保重要数据突出显示或符合格式要求。请注意，列高级设置可能根据您正在使用的数据包而有所不同，每个数据包都有最适合数据特性的列高级设置。</v>
+        <v>在偏好中，您可以自定义显示选项。例如，您可以选择在选定时间段内将无数据的列显示为灰色，添加工具提示以提供额外信息，或启用图表的筛选和图例选项。此外，您可以从文件加载您的设置或将当前设置保存到文件中。此功能使您可以备份设置、与他人分享或快速应用以前保存的设置到您的图表中。</v>
       </c>
     </row>
     <row r="447">
       <c r="A447" t="str">
-        <v>tours.settings.step4</v>
+        <v>tours.settings.step3</v>
       </c>
       <c r="B447" t="str">
-        <v>In the Search Settings, you can quickly locate specific columns by entering keywords and then directly add them to your chart. Simply enter a term related to the setting you are looking for, and the system will display all relevant results.This feature is particularly useful when managing numerous data points or when you need to make quick adjustments without browsing through extensive lists.</v>
+        <v>In Column Settings, you can deeply customize the appearance and organization of your charts.In the "Column Customization" area, you can adjust titles and shift row positions to streamline how data is displayed on your charts. Enable or disable specific elements like the chart title and Ma markers to suit your presentation needs. In the "Font Options" section, refine the appearance of your charts by choosing different fonts, sizes, and styles for headers and labels, ensuring important data stands out or meets formatting requirements. Please note that the advanced settings for columns can vary depending on the datapack you are working with, allowing for tailored configurations that best fit the data characteristics.</v>
       </c>
       <c r="C447" t="str">
-        <v>在搜索中，您可以通过输入关键词快速定位特定列，然后直接将其添加到您的图表中。只需输入一个与您正在寻找的设置相关的词语，系统便会显示所有相关结果。此功能可以帮助您管理众多数据点，或进行快速调整而无需浏览繁杂列表。请注意目前只支持英文搜索。</v>
+        <v>在列设置中，您可以深度自定义图表的外观和组织。在“列自定义”区域，您可以调整标题和移动行位置，以简化图表上数据的显示方式。根据您的展示需求启用或禁用特定元素，如图表标题和百万年标记。在“字体选项”部分，通过选择不同的字体、大小和样式为标题和标签，细化您的图表外观，确保重要数据突出显示或符合格式要求。请注意，列高级设置可能根据您正在使用的数据包而有所不同，每个数据包都有最适合数据特性的列高级设置。</v>
       </c>
     </row>
     <row r="448">
       <c r="A448" t="str">
-        <v>tours.settings.step5</v>
+        <v>tours.settings.step4</v>
       </c>
       <c r="B448" t="str">
-        <v>The Font Settings section allows you to customize the appearance of text within your charts. You can adjust font styles, sizes, and formatting for various elements such as column headers, age labels, and more. Each setting is inheritable, ensuring consistency across related elements unless specified otherwise. Changing a font setting here applies it system-wide, but you can override these for individual columns by using the "Change Font" option within each columns settings.Experiment with different fonts and sizes to enhance readability and visual appeal of your charts.</v>
+        <v>In the Search Settings, you can quickly locate specific columns by entering keywords and then directly add them to your chart. Simply enter a term related to the setting you are looking for, and the system will display all relevant results.This feature is particularly useful when managing numerous data points or when you need to make quick adjustments without browsing through extensive lists.</v>
       </c>
       <c r="C448" t="str">
-        <v>在字体设置中您可以自定义图表内的文本外观。您可以为各种元素如列标题、年龄标签等调整字体样式、大小和格式。每项设置都是可继承的，确保相关元素间的一致性，除非另行设置。在这里更改字体设置将系统范围内应用，但您可以使用每个列设置中的“更改字体”选项覆盖这些设置。尝试不同的字体和大小，以增强图表的可读性和视觉吸引力。</v>
+        <v>在搜索中，您可以通过输入关键词快速定位特定列，然后直接将其添加到您的图表中。只需输入一个与您正在寻找的设置相关的词语，系统便会显示所有相关结果。此功能可以帮助您管理众多数据点，或进行快速调整而无需浏览繁杂列表。请注意目前只支持英文搜索。</v>
       </c>
     </row>
     <row r="449">
       <c r="A449" t="str">
-        <v>tours.settings.step6</v>
+        <v>tours.settings.step5</v>
       </c>
       <c r="B449" t="str">
-        <v>In the Map Points Settings, you can access and manage geographic data points for different locations. This feature allows you to view specific location details directly on the interactive map. You can toggle different map layers and visualize data points with detailed descriptions, like latitude, longitude, and additional notes. Please note, however, that not all datapacks contain map points.</v>
+        <v>The Font Settings section allows you to customize the appearance of text within your charts. You can adjust font styles, sizes, and formatting for various elements such as column headers, age labels, and more. Each setting is inheritable, ensuring consistency across related elements unless specified otherwise. Changing a font setting here applies it system-wide, but you can override these for individual columns by using the "Change Font" option within each columns settings.Experiment with different fonts and sizes to enhance readability and visual appeal of your charts.</v>
       </c>
       <c r="C449" t="str">
-        <v>在地图点设置中，您可以访问和管理不同位置的地理数据点。此功能允许您直接在交互式地图上查看特定位置的详细信息。您可以切换不同的地图层，并用详细描述（如纬度、经度和附加说明）可视化数据点。请注意，并非所有数据包都包含地图点。</v>
+        <v>在字体设置中您可以自定义图表内的文本外观。您可以为各种元素如列标题、年龄标签等调整字体样式、大小和格式。每项设置都是可继承的，确保相关元素间的一致性，除非另行设置。在这里更改字体设置将系统范围内应用，但您可以使用每个列设置中的“更改字体”选项覆盖这些设置。尝试不同的字体和大小，以增强图表的可读性和视觉吸引力。</v>
       </c>
     </row>
     <row r="450">
       <c r="A450" t="str">
-        <v>tours.settings.step7</v>
+        <v>tours.settings.step6</v>
       </c>
       <c r="B450" t="str">
-        <v>In the Datapacks Settings, you can select the datapacks you wish to use for generating charts. We offer nine official datapacks, each comprising a curated collection of datasets tailored for specific thematic explorations. You might notice that this page resembles the Datapack page; selections can be configured here or there interchangeably. For more detailed guidance on how to utilize datapacks, please refer to the Datapacks Tour in the Help page "Tours" section.</v>
+        <v>In the Map Points Settings, you can access and manage geographic data points for different locations. This feature allows you to view specific location details directly on the interactive map. You can toggle different map layers and visualize data points with detailed descriptions, like latitude, longitude, and additional notes. Please note, however, that not all datapacks contain map points.</v>
       </c>
       <c r="C450" t="str">
-        <v>在数据包设置中，您可以选择您希望用于生成图表的数据包。我们提供九个官方数据包，每个数据包都包含为特定主题探索量身定制的数据集合。您也许已经注意到，此页面与"数据包"页面内容相同；您在两个地方都可以进行选择和设置。如需更详细的关于如何利用数据包的指导，请参阅帮助页面“导览”部分中的数据包导览。</v>
+        <v>在地图点设置中，您可以访问和管理不同位置的地理数据点。此功能允许您直接在交互式地图上查看特定位置的详细信息。您可以切换不同的地图层，并用详细描述（如纬度、经度和附加说明）可视化数据点。请注意，并非所有数据包都包含地图点。</v>
       </c>
     </row>
     <row r="451">
       <c r="A451" t="str">
-        <v>settings.column.tooltip.note-in-range</v>
+        <v>tours.settings.step7</v>
+      </c>
+      <c r="B451" t="str">
+        <v>In the Datapacks Settings, you can select the datapacks you wish to use for generating charts. We offer nine official datapacks, each comprising a curated collection of datasets tailored for specific thematic explorations. You might notice that this page resembles the Datapack page; selections can be configured here or there interchangeably. For more detailed guidance on how to utilize datapacks, please refer to the Datapacks Tour in the Help page "Tours" section.</v>
       </c>
       <c r="C451" t="str">
-        <v>数据不在所选时间区间内</v>
+        <v>在数据包设置中，您可以选择您希望用于生成图表的数据包。我们提供九个官方数据包，每个数据包都包含为特定主题探索量身定制的数据集合。您也许已经注意到，此页面与"数据包"页面内容相同；您在两个地方都可以进行选择和设置。如需更详细的关于如何利用数据包的指导，请参阅帮助页面“导览”部分中的数据包导览。</v>
       </c>
     </row>
     <row r="452">
       <c r="A452" t="str">
-        <v>language-names.en-US</v>
+        <v>settings.column.tooltip.note-in-range</v>
       </c>
       <c r="C452" t="str">
-        <v>English</v>
+        <v>数据不在所选时间区间内</v>
       </c>
     </row>
     <row r="453">
       <c r="A453" t="str">
-        <v>language-names.en</v>
+        <v>language-names.en-US</v>
       </c>
       <c r="C453" t="str">
         <v>English</v>
@@ -5026,15 +5026,23 @@
     </row>
     <row r="454">
       <c r="A454" t="str">
+        <v>language-names.en</v>
+      </c>
+      <c r="C454" t="str">
+        <v>English</v>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="str">
         <v>language-names.zh</v>
       </c>
-      <c r="C454" t="str">
+      <c r="C455" t="str">
         <v>中文</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C454"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C455"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added fetching chart history metadata on chart generation
</commit_message>
<xml_diff>
--- a/server/assets/translation.xlsx
+++ b/server/assets/translation.xlsx
@@ -375,7 +375,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C455"/>
+  <dimension ref="A1:C456"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4659,89 +4659,89 @@
     </row>
     <row r="419">
       <c r="A419" t="str">
-        <v>button.generate</v>
+        <v>errors.USER_FETCH_HISTORY_METADATA_FAILED</v>
       </c>
       <c r="B419" t="str">
-        <v>Generate</v>
-      </c>
-      <c r="C419" t="str">
-        <v>绘制</v>
+        <v>Failed to fetch user history metadata. Please try again later</v>
       </c>
     </row>
     <row r="420">
       <c r="A420" t="str">
-        <v>button.generate-chart</v>
+        <v>button.generate</v>
       </c>
       <c r="B420" t="str">
-        <v>Generate Chart</v>
+        <v>Generate</v>
       </c>
       <c r="C420" t="str">
-        <v>绘制图表</v>
+        <v>绘制</v>
       </c>
     </row>
     <row r="421">
       <c r="A421" t="str">
-        <v>button.remove-cache</v>
+        <v>button.generate-chart</v>
       </c>
       <c r="B421" t="str">
-        <v>Remove Cache</v>
+        <v>Generate Chart</v>
       </c>
       <c r="C421" t="str">
-        <v>清除缓存</v>
+        <v>绘制图表</v>
       </c>
     </row>
     <row r="422">
       <c r="A422" t="str">
-        <v>button.confirm-selection</v>
+        <v>button.remove-cache</v>
       </c>
       <c r="B422" t="str">
-        <v>Confirm Selection</v>
+        <v>Remove Cache</v>
       </c>
       <c r="C422" t="str">
-        <v>确认选择</v>
+        <v>清除缓存</v>
       </c>
     </row>
     <row r="423">
       <c r="A423" t="str">
-        <v>button.generate-cross-plot</v>
+        <v>button.confirm-selection</v>
       </c>
       <c r="B423" t="str">
-        <v>Generate Cross Plot</v>
+        <v>Confirm Selection</v>
+      </c>
+      <c r="C423" t="str">
+        <v>确认选择</v>
       </c>
     </row>
     <row r="424">
       <c r="A424" t="str">
-        <v>yes</v>
+        <v>button.generate-cross-plot</v>
       </c>
       <c r="B424" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="C424" t="str">
-        <v>是</v>
+        <v>Generate Cross Plot</v>
       </c>
     </row>
     <row r="425">
       <c r="A425" t="str">
-        <v>no</v>
+        <v>yes</v>
       </c>
       <c r="B425" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="C425" t="str">
-        <v>否</v>
+        <v>是</v>
       </c>
     </row>
     <row r="426">
       <c r="A426" t="str">
-        <v>languageNames.en-US</v>
+        <v>no</v>
       </c>
       <c r="B426" t="str">
-        <v>English</v>
+        <v>No</v>
+      </c>
+      <c r="C426" t="str">
+        <v>否</v>
       </c>
     </row>
     <row r="427">
       <c r="A427" t="str">
-        <v>languageNames.en</v>
+        <v>languageNames.en-US</v>
       </c>
       <c r="B427" t="str">
         <v>English</v>
@@ -4749,284 +4749,284 @@
     </row>
     <row r="428">
       <c r="A428" t="str">
-        <v>languageNames.zh</v>
+        <v>languageNames.en</v>
       </c>
       <c r="B428" t="str">
-        <v>中文</v>
+        <v>English</v>
       </c>
     </row>
     <row r="429">
       <c r="A429" t="str">
-        <v>tours.quit</v>
+        <v>languageNames.zh</v>
       </c>
       <c r="B429" t="str">
-        <v>Quit Tour</v>
-      </c>
-      <c r="C429" t="str">
-        <v>退出导览</v>
+        <v>中文</v>
       </c>
     </row>
     <row r="430">
       <c r="A430" t="str">
-        <v>tours.finish</v>
+        <v>tours.quit</v>
       </c>
       <c r="B430" t="str">
-        <v>Finish Tour</v>
+        <v>Quit Tour</v>
       </c>
       <c r="C430" t="str">
-        <v>结束导览</v>
+        <v>退出导览</v>
       </c>
     </row>
     <row r="431">
       <c r="A431" t="str">
-        <v>tours.next</v>
+        <v>tours.finish</v>
       </c>
       <c r="B431" t="str">
-        <v>Next</v>
+        <v>Finish Tour</v>
       </c>
       <c r="C431" t="str">
-        <v>下一步</v>
+        <v>结束导览</v>
       </c>
     </row>
     <row r="432">
       <c r="A432" t="str">
-        <v>tours.back</v>
+        <v>tours.next</v>
       </c>
       <c r="B432" t="str">
-        <v>Back</v>
+        <v>Next</v>
       </c>
       <c r="C432" t="str">
-        <v>上一步</v>
+        <v>下一步</v>
       </c>
     </row>
     <row r="433">
       <c r="A433" t="str">
-        <v>tours.qsg.step1</v>
+        <v>tours.back</v>
       </c>
       <c r="B433" t="str">
-        <v>In the Presets page, we offer pre-configured settings that allow you to rapidly generate specific types of charts without configuring all options from the beginning. Each preset comes equipped with designated data packs, visual styles, and settings, enabling you to create charts with just a single click.</v>
+        <v>Back</v>
       </c>
       <c r="C433" t="str">
-        <v>在预设页面中，我们提供了预设置，允许您快速生成特定类型的图表，无需从头开始配置所有选项。每个预设都配备了指定的数据包、视觉样式和设置，使您能够一键创建图表</v>
+        <v>上一步</v>
       </c>
     </row>
     <row r="434">
       <c r="A434" t="str">
-        <v>tours.qsg.step2</v>
+        <v>tours.qsg.step1</v>
       </c>
       <c r="B434" t="str">
-        <v>In the Datapacks page, you can select the datapacks required to generate your charts. We offer nine official data packs, each containing a curated collection of datasets tailored for specific thematic explorations. For more detailed guidance on Datapacks, please refer to the Datapacks Tour under the "Tours" section</v>
+        <v>In the Presets page, we offer pre-configured settings that allow you to rapidly generate specific types of charts without configuring all options from the beginning. Each preset comes equipped with designated data packs, visual styles, and settings, enabling you to create charts with just a single click.</v>
       </c>
       <c r="C434" t="str">
-        <v>在数据包页面，您可以选择生成图表所需的数据包。我们提供九个官方数据包，每个数据包都包含为特定主题探索量身定制的数据集合集。如需更详细的数据包指导，请参考“导览”部分下的数据包导览。</v>
+        <v>在预设页面中，我们提供了预设置，允许您快速生成特定类型的图表，无需从头开始配置所有选项。每个预设都配备了指定的数据包、视觉样式和设置，使您能够一键创建图表</v>
       </c>
     </row>
     <row r="435">
       <c r="A435" t="str">
-        <v>tours.qsg.step3</v>
+        <v>tours.qsg.step2</v>
       </c>
       <c r="B435" t="str">
-        <v>In the Chart page, you can view the charts you have created and explore the detailed visualizations of geologic events. Additionally, you have the option to download and save these charts for your reference or further analysis.</v>
+        <v>In the Datapacks page, you can select the datapacks required to generate your charts. We offer nine official data packs, each containing a curated collection of datasets tailored for specific thematic explorations. For more detailed guidance on Datapacks, please refer to the Datapacks Tour under the "Tours" section</v>
       </c>
       <c r="C435" t="str">
-        <v>在图表页面，您可以查看已创建的图表并探索地质事件的详细可视化图。此外，您还可以下载并保存这些图表以供参考或进一步分析。</v>
+        <v>在数据包页面，您可以选择生成图表所需的数据包。我们提供九个官方数据包，每个数据包都包含为特定主题探索量身定制的数据集合集。如需更详细的数据包指导，请参考“导览”部分下的数据包导览。</v>
       </c>
     </row>
     <row r="436">
       <c r="A436" t="str">
-        <v>tours.qsg.step4</v>
+        <v>tours.qsg.step3</v>
       </c>
       <c r="B436" t="str">
-        <v>In the Settings page, you can customize all aspects of your charts. This includes adjusting the scale and time range, selecting which rows to display, setting the background color and font style, etc. Tailor your charts to meet your specific needs and preferences to optimize your visual analysis. For more detailed guidance on Settings, please refer to the Settings Tour under the "Tours" section</v>
+        <v>In the Chart page, you can view the charts you have created and explore the detailed visualizations of geologic events. Additionally, you have the option to download and save these charts for your reference or further analysis.</v>
       </c>
       <c r="C436" t="str">
-        <v>在设置页面，您可以自定义图表的所有方面。这包括调整比例和时间范围、选择显示哪些行、设置背景色和字体样式等。根据您的具体需求和偏好调整图表，以优化您的视觉分析。如需更详细的设置指导，请参考“导览”部分下的设置导览。</v>
+        <v>在图表页面，您可以查看已创建的图表并探索地质事件的详细可视化图。此外，您还可以下载并保存这些图表以供参考或进一步分析。</v>
       </c>
     </row>
     <row r="437">
       <c r="A437" t="str">
-        <v>tours.qsg.step5</v>
+        <v>tours.qsg.step4</v>
       </c>
       <c r="B437" t="str">
-        <v>In the Help Page, you can find detailed assistance and information on how to use the website.</v>
+        <v>In the Settings page, you can customize all aspects of your charts. This includes adjusting the scale and time range, selecting which rows to display, setting the background color and font style, etc. Tailor your charts to meet your specific needs and preferences to optimize your visual analysis. For more detailed guidance on Settings, please refer to the Settings Tour under the "Tours" section</v>
       </c>
       <c r="C437" t="str">
-        <v>在帮助页面，您可以找到关于如何使用网站的详细帮助和信息。</v>
+        <v>在设置页面，您可以自定义图表的所有方面。这包括调整比例和时间范围、选择显示哪些行、设置背景色和字体样式等。根据您的具体需求和偏好调整图表，以优化您的视觉分析。如需更详细的设置指导，请参考“导览”部分下的设置导览。</v>
       </c>
     </row>
     <row r="438">
       <c r="A438" t="str">
-        <v>tours.qsg.step6</v>
+        <v>tours.qsg.step5</v>
       </c>
       <c r="B438" t="str">
-        <v>In the Workshops Page, you can access a range of educational and experimental tutorials that offer in-depth guidance. Here, you can explore the workshops you have registered for, allowing you to engage with the content and enhance your skills in a hands-on learning environment.</v>
+        <v>In the Help Page, you can find detailed assistance and information on how to use the website.</v>
       </c>
       <c r="C438" t="str">
-        <v>在工作坊页面，您可以访问一系列提供深入指导的教育和实验教程。在这里，您可以探索已注册的研讨会，通过亲身实践的学习环境来提升您的技能。</v>
+        <v>在帮助页面，您可以找到关于如何使用网站的详细帮助和信息。</v>
       </c>
     </row>
     <row r="439">
       <c r="A439" t="str">
-        <v>tours.qsg.step7</v>
+        <v>tours.qsg.step6</v>
       </c>
       <c r="B439" t="str">
-        <v>The About Page provides information about our development team.</v>
+        <v>In the Workshops Page, you can access a range of educational and experimental tutorials that offer in-depth guidance. Here, you can explore the workshops you have registered for, allowing you to engage with the content and enhance your skills in a hands-on learning environment.</v>
       </c>
       <c r="C439" t="str">
-        <v>关于页面提供了我们开发团队的信息。</v>
+        <v>在工作坊页面，您可以访问一系列提供深入指导的教育和实验教程。在这里，您可以探索已注册的研讨会，通过亲身实践的学习环境来提升您的技能。</v>
       </c>
     </row>
     <row r="440">
       <c r="A440" t="str">
-        <v>tours.qsg.step8</v>
+        <v>tours.qsg.step7</v>
       </c>
       <c r="B440" t="str">
-        <v>Click here to sign in and unlock the features mentioned earlier, such as accessing registered workshops. Once logged in, you will also have the ability to upload datapacks and take full advantage of all functionalities.</v>
+        <v>The About Page provides information about our development team.</v>
       </c>
       <c r="C440" t="str">
-        <v>点击此处登录并解锁前面提到的功能，例如访问工作坊界面。登陆后，您还将能够上传数据包并充分利用所有功能。</v>
+        <v>关于页面提供了我们开发团队的信息。</v>
       </c>
     </row>
     <row r="441">
       <c r="A441" t="str">
-        <v>tours.datapack.step1</v>
+        <v>tours.qsg.step8</v>
       </c>
       <c r="B441" t="str">
-        <v>Switch between different display types for datapacks: rows, cards, or compact view.</v>
+        <v>Click here to sign in and unlock the features mentioned earlier, such as accessing registered workshops. Once logged in, you will also have the ability to upload datapacks and take full advantage of all functionalities.</v>
       </c>
       <c r="C441" t="str">
-        <v>在数据包显示类型之间切换：行视图、卡片视图或紧凑视图。</v>
+        <v>点击此处登录并解锁前面提到的功能，例如访问工作坊界面。登陆后，您还将能够上传数据包并充分利用所有功能。</v>
       </c>
     </row>
     <row r="442">
       <c r="A442" t="str">
-        <v>tours.datapack.step2</v>
+        <v>tours.datapack.step1</v>
       </c>
       <c r="B442" t="str">
-        <v>Add a datapack by clicking the checkbox</v>
+        <v>Switch between different display types for datapacks: rows, cards, or compact view.</v>
       </c>
       <c r="C442" t="str">
-        <v>勾选添加您想要的数据包</v>
+        <v>在数据包显示类型之间切换：行视图、卡片视图或紧凑视图。</v>
       </c>
     </row>
     <row r="443">
       <c r="A443" t="str">
-        <v>tours.datapack.step3</v>
+        <v>tours.datapack.step2</v>
       </c>
       <c r="B443" t="str">
-        <v>Click the deselect icon to deselect all datapacks</v>
+        <v>Add a datapack by clicking the checkbox</v>
       </c>
       <c r="C443" t="str">
-        <v>点此取消选择所有数据包</v>
+        <v>勾选添加您想要的数据包</v>
       </c>
     </row>
     <row r="444">
       <c r="A444" t="str">
-        <v>tours.datapack.step4</v>
+        <v>tours.datapack.step3</v>
       </c>
       <c r="B444" t="str">
-        <v>Remember to confirm your selection</v>
+        <v>Click the deselect icon to deselect all datapacks</v>
       </c>
       <c r="C444" t="str">
-        <v>记得确认您的选择</v>
+        <v>点此取消选择所有数据包</v>
       </c>
     </row>
     <row r="445">
       <c r="A445" t="str">
-        <v>tours.settings.step1</v>
+        <v>tours.datapack.step4</v>
       </c>
       <c r="B445" t="str">
-        <v>In the Time settings, you can Set the "Top of Interval" and "Base of Interval" for your data. These fields allow you to define the starting and ending ages or stages, which can be adjusted by entering values or using the dropdown selectors. Adjust the vertical scale to change how much vertical space each million years occupies on your charts. For example, setting it higher will spread the intervals further apart, making each period easier to examine closely.</v>
+        <v>Remember to confirm your selection</v>
       </c>
       <c r="C445" t="str">
-        <v>在时间设置中，您可以为您的数据设置“时间段顶部”和“时间段底部”。调整这两个值将改变图表的时间跨度，您可以通过输入值或使用下拉选择器进行调整。您还可以调整垂直比例，以改变图表中每百万年占据的垂直空间量。例如，将其设置得更高将使时间间隔进一步分开，使每个时期更易于仔细检查。</v>
+        <v>记得确认您的选择</v>
       </c>
     </row>
     <row r="446">
       <c r="A446" t="str">
-        <v>tours.settings.step2</v>
+        <v>tours.settings.step1</v>
       </c>
       <c r="B446" t="str">
-        <v>In the Preferences settings, you can customize the display options. For instance, you may choose to gray out columns with no data for selected time periods, add tooltips for additional information, or enable filtering and legend options for charts. Furthermore, you can load your settings from a file or save your current settings to a file. This feature is useful for backing up your configurations, sharing them with others, or quickly applying previously saved configurations to your chart.</v>
+        <v>In the Time settings, you can Set the "Top of Interval" and "Base of Interval" for your data. These fields allow you to define the starting and ending ages or stages, which can be adjusted by entering values or using the dropdown selectors. Adjust the vertical scale to change how much vertical space each million years occupies on your charts. For example, setting it higher will spread the intervals further apart, making each period easier to examine closely.</v>
       </c>
       <c r="C446" t="str">
-        <v>在偏好中，您可以自定义显示选项。例如，您可以选择在选定时间段内将无数据的列显示为灰色，添加工具提示以提供额外信息，或启用图表的筛选和图例选项。此外，您可以从文件加载您的设置或将当前设置保存到文件中。此功能使您可以备份设置、与他人分享或快速应用以前保存的设置到您的图表中。</v>
+        <v>在时间设置中，您可以为您的数据设置“时间段顶部”和“时间段底部”。调整这两个值将改变图表的时间跨度，您可以通过输入值或使用下拉选择器进行调整。您还可以调整垂直比例，以改变图表中每百万年占据的垂直空间量。例如，将其设置得更高将使时间间隔进一步分开，使每个时期更易于仔细检查。</v>
       </c>
     </row>
     <row r="447">
       <c r="A447" t="str">
-        <v>tours.settings.step3</v>
+        <v>tours.settings.step2</v>
       </c>
       <c r="B447" t="str">
-        <v>In Column Settings, you can deeply customize the appearance and organization of your charts.In the "Column Customization" area, you can adjust titles and shift row positions to streamline how data is displayed on your charts. Enable or disable specific elements like the chart title and Ma markers to suit your presentation needs. In the "Font Options" section, refine the appearance of your charts by choosing different fonts, sizes, and styles for headers and labels, ensuring important data stands out or meets formatting requirements. Please note that the advanced settings for columns can vary depending on the datapack you are working with, allowing for tailored configurations that best fit the data characteristics.</v>
+        <v>In the Preferences settings, you can customize the display options. For instance, you may choose to gray out columns with no data for selected time periods, add tooltips for additional information, or enable filtering and legend options for charts. Furthermore, you can load your settings from a file or save your current settings to a file. This feature is useful for backing up your configurations, sharing them with others, or quickly applying previously saved configurations to your chart.</v>
       </c>
       <c r="C447" t="str">
-        <v>在列设置中，您可以深度自定义图表的外观和组织。在“列自定义”区域，您可以调整标题和移动行位置，以简化图表上数据的显示方式。根据您的展示需求启用或禁用特定元素，如图表标题和百万年标记。在“字体选项”部分，通过选择不同的字体、大小和样式为标题和标签，细化您的图表外观，确保重要数据突出显示或符合格式要求。请注意，列高级设置可能根据您正在使用的数据包而有所不同，每个数据包都有最适合数据特性的列高级设置。</v>
+        <v>在偏好中，您可以自定义显示选项。例如，您可以选择在选定时间段内将无数据的列显示为灰色，添加工具提示以提供额外信息，或启用图表的筛选和图例选项。此外，您可以从文件加载您的设置或将当前设置保存到文件中。此功能使您可以备份设置、与他人分享或快速应用以前保存的设置到您的图表中。</v>
       </c>
     </row>
     <row r="448">
       <c r="A448" t="str">
-        <v>tours.settings.step4</v>
+        <v>tours.settings.step3</v>
       </c>
       <c r="B448" t="str">
-        <v>In the Search Settings, you can quickly locate specific columns by entering keywords and then directly add them to your chart. Simply enter a term related to the setting you are looking for, and the system will display all relevant results.This feature is particularly useful when managing numerous data points or when you need to make quick adjustments without browsing through extensive lists.</v>
+        <v>In Column Settings, you can deeply customize the appearance and organization of your charts.In the "Column Customization" area, you can adjust titles and shift row positions to streamline how data is displayed on your charts. Enable or disable specific elements like the chart title and Ma markers to suit your presentation needs. In the "Font Options" section, refine the appearance of your charts by choosing different fonts, sizes, and styles for headers and labels, ensuring important data stands out or meets formatting requirements. Please note that the advanced settings for columns can vary depending on the datapack you are working with, allowing for tailored configurations that best fit the data characteristics.</v>
       </c>
       <c r="C448" t="str">
-        <v>在搜索中，您可以通过输入关键词快速定位特定列，然后直接将其添加到您的图表中。只需输入一个与您正在寻找的设置相关的词语，系统便会显示所有相关结果。此功能可以帮助您管理众多数据点，或进行快速调整而无需浏览繁杂列表。请注意目前只支持英文搜索。</v>
+        <v>在列设置中，您可以深度自定义图表的外观和组织。在“列自定义”区域，您可以调整标题和移动行位置，以简化图表上数据的显示方式。根据您的展示需求启用或禁用特定元素，如图表标题和百万年标记。在“字体选项”部分，通过选择不同的字体、大小和样式为标题和标签，细化您的图表外观，确保重要数据突出显示或符合格式要求。请注意，列高级设置可能根据您正在使用的数据包而有所不同，每个数据包都有最适合数据特性的列高级设置。</v>
       </c>
     </row>
     <row r="449">
       <c r="A449" t="str">
-        <v>tours.settings.step5</v>
+        <v>tours.settings.step4</v>
       </c>
       <c r="B449" t="str">
-        <v>The Font Settings section allows you to customize the appearance of text within your charts. You can adjust font styles, sizes, and formatting for various elements such as column headers, age labels, and more. Each setting is inheritable, ensuring consistency across related elements unless specified otherwise. Changing a font setting here applies it system-wide, but you can override these for individual columns by using the "Change Font" option within each columns settings.Experiment with different fonts and sizes to enhance readability and visual appeal of your charts.</v>
+        <v>In the Search Settings, you can quickly locate specific columns by entering keywords and then directly add them to your chart. Simply enter a term related to the setting you are looking for, and the system will display all relevant results.This feature is particularly useful when managing numerous data points or when you need to make quick adjustments without browsing through extensive lists.</v>
       </c>
       <c r="C449" t="str">
-        <v>在字体设置中您可以自定义图表内的文本外观。您可以为各种元素如列标题、年龄标签等调整字体样式、大小和格式。每项设置都是可继承的，确保相关元素间的一致性，除非另行设置。在这里更改字体设置将系统范围内应用，但您可以使用每个列设置中的“更改字体”选项覆盖这些设置。尝试不同的字体和大小，以增强图表的可读性和视觉吸引力。</v>
+        <v>在搜索中，您可以通过输入关键词快速定位特定列，然后直接将其添加到您的图表中。只需输入一个与您正在寻找的设置相关的词语，系统便会显示所有相关结果。此功能可以帮助您管理众多数据点，或进行快速调整而无需浏览繁杂列表。请注意目前只支持英文搜索。</v>
       </c>
     </row>
     <row r="450">
       <c r="A450" t="str">
-        <v>tours.settings.step6</v>
+        <v>tours.settings.step5</v>
       </c>
       <c r="B450" t="str">
-        <v>In the Map Points Settings, you can access and manage geographic data points for different locations. This feature allows you to view specific location details directly on the interactive map. You can toggle different map layers and visualize data points with detailed descriptions, like latitude, longitude, and additional notes. Please note, however, that not all datapacks contain map points.</v>
+        <v>The Font Settings section allows you to customize the appearance of text within your charts. You can adjust font styles, sizes, and formatting for various elements such as column headers, age labels, and more. Each setting is inheritable, ensuring consistency across related elements unless specified otherwise. Changing a font setting here applies it system-wide, but you can override these for individual columns by using the "Change Font" option within each columns settings.Experiment with different fonts and sizes to enhance readability and visual appeal of your charts.</v>
       </c>
       <c r="C450" t="str">
-        <v>在地图点设置中，您可以访问和管理不同位置的地理数据点。此功能允许您直接在交互式地图上查看特定位置的详细信息。您可以切换不同的地图层，并用详细描述（如纬度、经度和附加说明）可视化数据点。请注意，并非所有数据包都包含地图点。</v>
+        <v>在字体设置中您可以自定义图表内的文本外观。您可以为各种元素如列标题、年龄标签等调整字体样式、大小和格式。每项设置都是可继承的，确保相关元素间的一致性，除非另行设置。在这里更改字体设置将系统范围内应用，但您可以使用每个列设置中的“更改字体”选项覆盖这些设置。尝试不同的字体和大小，以增强图表的可读性和视觉吸引力。</v>
       </c>
     </row>
     <row r="451">
       <c r="A451" t="str">
-        <v>tours.settings.step7</v>
+        <v>tours.settings.step6</v>
       </c>
       <c r="B451" t="str">
-        <v>In the Datapacks Settings, you can select the datapacks you wish to use for generating charts. We offer nine official datapacks, each comprising a curated collection of datasets tailored for specific thematic explorations. You might notice that this page resembles the Datapack page; selections can be configured here or there interchangeably. For more detailed guidance on how to utilize datapacks, please refer to the Datapacks Tour in the Help page "Tours" section.</v>
+        <v>In the Map Points Settings, you can access and manage geographic data points for different locations. This feature allows you to view specific location details directly on the interactive map. You can toggle different map layers and visualize data points with detailed descriptions, like latitude, longitude, and additional notes. Please note, however, that not all datapacks contain map points.</v>
       </c>
       <c r="C451" t="str">
-        <v>在数据包设置中，您可以选择您希望用于生成图表的数据包。我们提供九个官方数据包，每个数据包都包含为特定主题探索量身定制的数据集合。您也许已经注意到，此页面与"数据包"页面内容相同；您在两个地方都可以进行选择和设置。如需更详细的关于如何利用数据包的指导，请参阅帮助页面“导览”部分中的数据包导览。</v>
+        <v>在地图点设置中，您可以访问和管理不同位置的地理数据点。此功能允许您直接在交互式地图上查看特定位置的详细信息。您可以切换不同的地图层，并用详细描述（如纬度、经度和附加说明）可视化数据点。请注意，并非所有数据包都包含地图点。</v>
       </c>
     </row>
     <row r="452">
       <c r="A452" t="str">
-        <v>settings.column.tooltip.note-in-range</v>
+        <v>tours.settings.step7</v>
+      </c>
+      <c r="B452" t="str">
+        <v>In the Datapacks Settings, you can select the datapacks you wish to use for generating charts. We offer nine official datapacks, each comprising a curated collection of datasets tailored for specific thematic explorations. You might notice that this page resembles the Datapack page; selections can be configured here or there interchangeably. For more detailed guidance on how to utilize datapacks, please refer to the Datapacks Tour in the Help page "Tours" section.</v>
       </c>
       <c r="C452" t="str">
-        <v>数据不在所选时间区间内</v>
+        <v>在数据包设置中，您可以选择您希望用于生成图表的数据包。我们提供九个官方数据包，每个数据包都包含为特定主题探索量身定制的数据集合。您也许已经注意到，此页面与"数据包"页面内容相同；您在两个地方都可以进行选择和设置。如需更详细的关于如何利用数据包的指导，请参阅帮助页面“导览”部分中的数据包导览。</v>
       </c>
     </row>
     <row r="453">
       <c r="A453" t="str">
-        <v>language-names.en-US</v>
+        <v>settings.column.tooltip.note-in-range</v>
       </c>
       <c r="C453" t="str">
-        <v>English</v>
+        <v>数据不在所选时间区间内</v>
       </c>
     </row>
     <row r="454">
       <c r="A454" t="str">
-        <v>language-names.en</v>
+        <v>language-names.en-US</v>
       </c>
       <c r="C454" t="str">
         <v>English</v>
@@ -5034,15 +5034,23 @@
     </row>
     <row r="455">
       <c r="A455" t="str">
+        <v>language-names.en</v>
+      </c>
+      <c r="C455" t="str">
+        <v>English</v>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="str">
         <v>language-names.zh</v>
       </c>
-      <c r="C455" t="str">
+      <c r="C456" t="str">
         <v>中文</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C455"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C456"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
more work on establishing the uploaded datapack to a profile
</commit_message>
<xml_diff>
--- a/server/assets/translation.xlsx
+++ b/server/assets/translation.xlsx
@@ -375,7 +375,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C473"/>
+  <dimension ref="A1:C474"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3667,13 +3667,10 @@
     </row>
     <row r="325">
       <c r="A325" t="str">
-        <v>errors.title</v>
+        <v>errors.USER_DATAPACK_UPLOAD_FAILED</v>
       </c>
       <c r="B325" t="str">
-        <v>Error</v>
-      </c>
-      <c r="C325" t="str">
-        <v>错误</v>
+        <v>Unable to upload user datapack. Please try again later.</v>
       </c>
     </row>
     <row r="326">
@@ -4806,89 +4803,92 @@
     </row>
     <row r="437">
       <c r="A437" t="str">
-        <v>button.generate</v>
+        <v>errors.title</v>
       </c>
       <c r="B437" t="str">
-        <v>Generate</v>
+        <v>Error</v>
       </c>
       <c r="C437" t="str">
-        <v>绘制</v>
+        <v>错误</v>
       </c>
     </row>
     <row r="438">
       <c r="A438" t="str">
-        <v>button.generate-chart</v>
+        <v>button.generate</v>
       </c>
       <c r="B438" t="str">
-        <v>Generate Chart</v>
+        <v>Generate</v>
       </c>
       <c r="C438" t="str">
-        <v>绘制图表</v>
+        <v>绘制</v>
       </c>
     </row>
     <row r="439">
       <c r="A439" t="str">
-        <v>button.remove-cache</v>
+        <v>button.generate-chart</v>
       </c>
       <c r="B439" t="str">
-        <v>Remove Cache</v>
+        <v>Generate Chart</v>
       </c>
       <c r="C439" t="str">
-        <v>清除缓存</v>
+        <v>绘制图表</v>
       </c>
     </row>
     <row r="440">
       <c r="A440" t="str">
-        <v>button.confirm-selection</v>
+        <v>button.remove-cache</v>
       </c>
       <c r="B440" t="str">
-        <v>Confirm Selection</v>
+        <v>Remove Cache</v>
       </c>
       <c r="C440" t="str">
-        <v>确认选择</v>
+        <v>清除缓存</v>
       </c>
     </row>
     <row r="441">
       <c r="A441" t="str">
-        <v>button.generate-cross-plot</v>
+        <v>button.confirm-selection</v>
       </c>
       <c r="B441" t="str">
-        <v>Generate Cross Plot</v>
+        <v>Confirm Selection</v>
+      </c>
+      <c r="C441" t="str">
+        <v>确认选择</v>
       </c>
     </row>
     <row r="442">
       <c r="A442" t="str">
-        <v>yes</v>
+        <v>button.generate-cross-plot</v>
       </c>
       <c r="B442" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="C442" t="str">
-        <v>是</v>
+        <v>Generate Cross Plot</v>
       </c>
     </row>
     <row r="443">
       <c r="A443" t="str">
-        <v>no</v>
+        <v>yes</v>
       </c>
       <c r="B443" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="C443" t="str">
-        <v>否</v>
+        <v>是</v>
       </c>
     </row>
     <row r="444">
       <c r="A444" t="str">
-        <v>languageNames.en-US</v>
+        <v>no</v>
       </c>
       <c r="B444" t="str">
-        <v>English</v>
+        <v>No</v>
+      </c>
+      <c r="C444" t="str">
+        <v>否</v>
       </c>
     </row>
     <row r="445">
       <c r="A445" t="str">
-        <v>languageNames.en</v>
+        <v>languageNames.en-US</v>
       </c>
       <c r="B445" t="str">
         <v>English</v>
@@ -4896,284 +4896,284 @@
     </row>
     <row r="446">
       <c r="A446" t="str">
-        <v>languageNames.zh</v>
+        <v>languageNames.en</v>
       </c>
       <c r="B446" t="str">
-        <v>中文</v>
+        <v>English</v>
       </c>
     </row>
     <row r="447">
       <c r="A447" t="str">
-        <v>tours.quit</v>
+        <v>languageNames.zh</v>
       </c>
       <c r="B447" t="str">
-        <v>Quit Tour</v>
-      </c>
-      <c r="C447" t="str">
-        <v>退出导览</v>
+        <v>中文</v>
       </c>
     </row>
     <row r="448">
       <c r="A448" t="str">
-        <v>tours.finish</v>
+        <v>tours.quit</v>
       </c>
       <c r="B448" t="str">
-        <v>Finish Tour</v>
+        <v>Quit Tour</v>
       </c>
       <c r="C448" t="str">
-        <v>结束导览</v>
+        <v>退出导览</v>
       </c>
     </row>
     <row r="449">
       <c r="A449" t="str">
-        <v>tours.next</v>
+        <v>tours.finish</v>
       </c>
       <c r="B449" t="str">
-        <v>Next</v>
+        <v>Finish Tour</v>
       </c>
       <c r="C449" t="str">
-        <v>下一步</v>
+        <v>结束导览</v>
       </c>
     </row>
     <row r="450">
       <c r="A450" t="str">
-        <v>tours.back</v>
+        <v>tours.next</v>
       </c>
       <c r="B450" t="str">
-        <v>Back</v>
+        <v>Next</v>
       </c>
       <c r="C450" t="str">
-        <v>上一步</v>
+        <v>下一步</v>
       </c>
     </row>
     <row r="451">
       <c r="A451" t="str">
-        <v>tours.qsg.step1</v>
+        <v>tours.back</v>
       </c>
       <c r="B451" t="str">
-        <v>In the Presets page, we offer pre-configured settings that allow you to rapidly generate specific types of charts without configuring all options from the beginning. Each preset comes equipped with designated data packs, visual styles, and settings, enabling you to create charts with just a single click.</v>
+        <v>Back</v>
       </c>
       <c r="C451" t="str">
-        <v>在预设页面中，我们提供了预设置，允许您快速生成特定类型的图表，无需从头开始配置所有选项。每个预设都配备了指定的数据包、视觉样式和设置，使您能够一键创建图表</v>
+        <v>上一步</v>
       </c>
     </row>
     <row r="452">
       <c r="A452" t="str">
-        <v>tours.qsg.step2</v>
+        <v>tours.qsg.step1</v>
       </c>
       <c r="B452" t="str">
-        <v>In the Datapacks page, you can select the datapacks required to generate your charts. We offer nine official data packs, each containing a curated collection of datasets tailored for specific thematic explorations. For more detailed guidance on Datapacks, please refer to the Datapacks Tour under the "Tours" section</v>
+        <v>In the Presets page, we offer pre-configured settings that allow you to rapidly generate specific types of charts without configuring all options from the beginning. Each preset comes equipped with designated data packs, visual styles, and settings, enabling you to create charts with just a single click.</v>
       </c>
       <c r="C452" t="str">
-        <v>在数据包页面，您可以选择生成图表所需的数据包。我们提供九个官方数据包，每个数据包都包含为特定主题探索量身定制的数据集合集。如需更详细的数据包指导，请参考“导览”部分下的数据包导览。</v>
+        <v>在预设页面中，我们提供了预设置，允许您快速生成特定类型的图表，无需从头开始配置所有选项。每个预设都配备了指定的数据包、视觉样式和设置，使您能够一键创建图表</v>
       </c>
     </row>
     <row r="453">
       <c r="A453" t="str">
-        <v>tours.qsg.step3</v>
+        <v>tours.qsg.step2</v>
       </c>
       <c r="B453" t="str">
-        <v>In the Chart page, you can view the charts you have created and explore the detailed visualizations of geologic events. Additionally, you have the option to download and save these charts for your reference or further analysis.</v>
+        <v>In the Datapacks page, you can select the datapacks required to generate your charts. We offer nine official data packs, each containing a curated collection of datasets tailored for specific thematic explorations. For more detailed guidance on Datapacks, please refer to the Datapacks Tour under the "Tours" section</v>
       </c>
       <c r="C453" t="str">
-        <v>在图表页面，您可以查看已创建的图表并探索地质事件的详细可视化图。此外，您还可以下载并保存这些图表以供参考或进一步分析。</v>
+        <v>在数据包页面，您可以选择生成图表所需的数据包。我们提供九个官方数据包，每个数据包都包含为特定主题探索量身定制的数据集合集。如需更详细的数据包指导，请参考“导览”部分下的数据包导览。</v>
       </c>
     </row>
     <row r="454">
       <c r="A454" t="str">
-        <v>tours.qsg.step4</v>
+        <v>tours.qsg.step3</v>
       </c>
       <c r="B454" t="str">
-        <v>In the Settings page, you can customize all aspects of your charts. This includes adjusting the scale and time range, selecting which rows to display, setting the background color and font style, etc. Tailor your charts to meet your specific needs and preferences to optimize your visual analysis. For more detailed guidance on Settings, please refer to the Settings Tour under the "Tours" section</v>
+        <v>In the Chart page, you can view the charts you have created and explore the detailed visualizations of geologic events. Additionally, you have the option to download and save these charts for your reference or further analysis.</v>
       </c>
       <c r="C454" t="str">
-        <v>在设置页面，您可以自定义图表的所有方面。这包括调整比例和时间范围、选择显示哪些行、设置背景色和字体样式等。根据您的具体需求和偏好调整图表，以优化您的视觉分析。如需更详细的设置指导，请参考“导览”部分下的设置导览。</v>
+        <v>在图表页面，您可以查看已创建的图表并探索地质事件的详细可视化图。此外，您还可以下载并保存这些图表以供参考或进一步分析。</v>
       </c>
     </row>
     <row r="455">
       <c r="A455" t="str">
-        <v>tours.qsg.step5</v>
+        <v>tours.qsg.step4</v>
       </c>
       <c r="B455" t="str">
-        <v>In the Help Page, you can find detailed assistance and information on how to use the website.</v>
+        <v>In the Settings page, you can customize all aspects of your charts. This includes adjusting the scale and time range, selecting which rows to display, setting the background color and font style, etc. Tailor your charts to meet your specific needs and preferences to optimize your visual analysis. For more detailed guidance on Settings, please refer to the Settings Tour under the "Tours" section</v>
       </c>
       <c r="C455" t="str">
-        <v>在帮助页面，您可以找到关于如何使用网站的详细帮助和信息。</v>
+        <v>在设置页面，您可以自定义图表的所有方面。这包括调整比例和时间范围、选择显示哪些行、设置背景色和字体样式等。根据您的具体需求和偏好调整图表，以优化您的视觉分析。如需更详细的设置指导，请参考“导览”部分下的设置导览。</v>
       </c>
     </row>
     <row r="456">
       <c r="A456" t="str">
-        <v>tours.qsg.step6</v>
+        <v>tours.qsg.step5</v>
       </c>
       <c r="B456" t="str">
-        <v>In the Workshops Page, you can access a range of educational and experimental tutorials that offer in-depth guidance. Here, you can explore the workshops you have registered for, allowing you to engage with the content and enhance your skills in a hands-on learning environment.</v>
+        <v>In the Help Page, you can find detailed assistance and information on how to use the website.</v>
       </c>
       <c r="C456" t="str">
-        <v>在工作坊页面，您可以访问一系列提供深入指导的教育和实验教程。在这里，您可以探索已注册的研讨会，通过亲身实践的学习环境来提升您的技能。</v>
+        <v>在帮助页面，您可以找到关于如何使用网站的详细帮助和信息。</v>
       </c>
     </row>
     <row r="457">
       <c r="A457" t="str">
-        <v>tours.qsg.step7</v>
+        <v>tours.qsg.step6</v>
       </c>
       <c r="B457" t="str">
-        <v>The About Page provides information about our development team.</v>
+        <v>In the Workshops Page, you can access a range of educational and experimental tutorials that offer in-depth guidance. Here, you can explore the workshops you have registered for, allowing you to engage with the content and enhance your skills in a hands-on learning environment.</v>
       </c>
       <c r="C457" t="str">
-        <v>关于页面提供了我们开发团队的信息。</v>
+        <v>在工作坊页面，您可以访问一系列提供深入指导的教育和实验教程。在这里，您可以探索已注册的研讨会，通过亲身实践的学习环境来提升您的技能。</v>
       </c>
     </row>
     <row r="458">
       <c r="A458" t="str">
-        <v>tours.qsg.step8</v>
+        <v>tours.qsg.step7</v>
       </c>
       <c r="B458" t="str">
-        <v>Click here to sign in and unlock the features mentioned earlier, such as accessing registered workshops. Once logged in, you will also have the ability to upload datapacks and take full advantage of all functionalities.</v>
+        <v>The About Page provides information about our development team.</v>
       </c>
       <c r="C458" t="str">
-        <v>点击此处登录并解锁前面提到的功能，例如访问工作坊界面。登陆后，您还将能够上传数据包并充分利用所有功能。</v>
+        <v>关于页面提供了我们开发团队的信息。</v>
       </c>
     </row>
     <row r="459">
       <c r="A459" t="str">
-        <v>tours.datapack.step1</v>
+        <v>tours.qsg.step8</v>
       </c>
       <c r="B459" t="str">
-        <v>Switch between different display types for datapacks: rows, cards, or compact view.</v>
+        <v>Click here to sign in and unlock the features mentioned earlier, such as accessing registered workshops. Once logged in, you will also have the ability to upload datapacks and take full advantage of all functionalities.</v>
       </c>
       <c r="C459" t="str">
-        <v>在数据包显示类型之间切换：行视图、卡片视图或紧凑视图。</v>
+        <v>点击此处登录并解锁前面提到的功能，例如访问工作坊界面。登陆后，您还将能够上传数据包并充分利用所有功能。</v>
       </c>
     </row>
     <row r="460">
       <c r="A460" t="str">
-        <v>tours.datapack.step2</v>
+        <v>tours.datapack.step1</v>
       </c>
       <c r="B460" t="str">
-        <v>Add a datapack by clicking the checkbox</v>
+        <v>Switch between different display types for datapacks: rows, cards, or compact view.</v>
       </c>
       <c r="C460" t="str">
-        <v>勾选添加您想要的数据包</v>
+        <v>在数据包显示类型之间切换：行视图、卡片视图或紧凑视图。</v>
       </c>
     </row>
     <row r="461">
       <c r="A461" t="str">
-        <v>tours.datapack.step3</v>
+        <v>tours.datapack.step2</v>
       </c>
       <c r="B461" t="str">
-        <v>Click the deselect icon to deselect all datapacks</v>
+        <v>Add a datapack by clicking the checkbox</v>
       </c>
       <c r="C461" t="str">
-        <v>点此取消选择所有数据包</v>
+        <v>勾选添加您想要的数据包</v>
       </c>
     </row>
     <row r="462">
       <c r="A462" t="str">
-        <v>tours.datapack.step4</v>
+        <v>tours.datapack.step3</v>
       </c>
       <c r="B462" t="str">
-        <v>Remember to confirm your selection</v>
+        <v>Click the deselect icon to deselect all datapacks</v>
       </c>
       <c r="C462" t="str">
-        <v>记得确认您的选择</v>
+        <v>点此取消选择所有数据包</v>
       </c>
     </row>
     <row r="463">
       <c r="A463" t="str">
-        <v>tours.settings.step1</v>
+        <v>tours.datapack.step4</v>
       </c>
       <c r="B463" t="str">
-        <v>In the Time settings, you can Set the "Top of Interval" and "Base of Interval" for your data. These fields allow you to define the starting and ending ages or stages, which can be adjusted by entering values or using the dropdown selectors. Adjust the vertical scale to change how much vertical space each million years occupies on your charts. For example, setting it higher will spread the intervals further apart, making each period easier to examine closely.</v>
+        <v>Remember to confirm your selection</v>
       </c>
       <c r="C463" t="str">
-        <v>在时间设置中，您可以为您的数据设置“时间段顶部”和“时间段底部”。调整这两个值将改变图表的时间跨度，您可以通过输入值或使用下拉选择器进行调整。您还可以调整垂直比例，以改变图表中每百万年占据的垂直空间量。例如，将其设置得更高将使时间间隔进一步分开，使每个时期更易于仔细检查。</v>
+        <v>记得确认您的选择</v>
       </c>
     </row>
     <row r="464">
       <c r="A464" t="str">
-        <v>tours.settings.step2</v>
+        <v>tours.settings.step1</v>
       </c>
       <c r="B464" t="str">
-        <v>In the Preferences settings, you can customize the display options. For instance, you may choose to gray out columns with no data for selected time periods, add tooltips for additional information, or enable filtering and legend options for charts. Furthermore, you can load your settings from a file or save your current settings to a file. This feature is useful for backing up your configurations, sharing them with others, or quickly applying previously saved configurations to your chart.</v>
+        <v>In the Time settings, you can Set the "Top of Interval" and "Base of Interval" for your data. These fields allow you to define the starting and ending ages or stages, which can be adjusted by entering values or using the dropdown selectors. Adjust the vertical scale to change how much vertical space each million years occupies on your charts. For example, setting it higher will spread the intervals further apart, making each period easier to examine closely.</v>
       </c>
       <c r="C464" t="str">
-        <v>在偏好中，您可以自定义显示选项。例如，您可以选择在选定时间段内将无数据的列显示为灰色，添加工具提示以提供额外信息，或启用图表的筛选和图例选项。此外，您可以从文件加载您的设置或将当前设置保存到文件中。此功能使您可以备份设置、与他人分享或快速应用以前保存的设置到您的图表中。</v>
+        <v>在时间设置中，您可以为您的数据设置“时间段顶部”和“时间段底部”。调整这两个值将改变图表的时间跨度，您可以通过输入值或使用下拉选择器进行调整。您还可以调整垂直比例，以改变图表中每百万年占据的垂直空间量。例如，将其设置得更高将使时间间隔进一步分开，使每个时期更易于仔细检查。</v>
       </c>
     </row>
     <row r="465">
       <c r="A465" t="str">
-        <v>tours.settings.step3</v>
+        <v>tours.settings.step2</v>
       </c>
       <c r="B465" t="str">
-        <v>In Column Settings, you can deeply customize the appearance and organization of your charts.In the "Column Customization" area, you can adjust titles and shift row positions to streamline how data is displayed on your charts. Enable or disable specific elements like the chart title and Ma markers to suit your presentation needs. In the "Font Options" section, refine the appearance of your charts by choosing different fonts, sizes, and styles for headers and labels, ensuring important data stands out or meets formatting requirements. Please note that the advanced settings for columns can vary depending on the datapack you are working with, allowing for tailored configurations that best fit the data characteristics.</v>
+        <v>In the Preferences settings, you can customize the display options. For instance, you may choose to gray out columns with no data for selected time periods, add tooltips for additional information, or enable filtering and legend options for charts. Furthermore, you can load your settings from a file or save your current settings to a file. This feature is useful for backing up your configurations, sharing them with others, or quickly applying previously saved configurations to your chart.</v>
       </c>
       <c r="C465" t="str">
-        <v>在列设置中，您可以深度自定义图表的外观和组织。在“列自定义”区域，您可以调整标题和移动行位置，以简化图表上数据的显示方式。根据您的展示需求启用或禁用特定元素，如图表标题和百万年标记。在“字体选项”部分，通过选择不同的字体、大小和样式为标题和标签，细化您的图表外观，确保重要数据突出显示或符合格式要求。请注意，列高级设置可能根据您正在使用的数据包而有所不同，每个数据包都有最适合数据特性的列高级设置。</v>
+        <v>在偏好中，您可以自定义显示选项。例如，您可以选择在选定时间段内将无数据的列显示为灰色，添加工具提示以提供额外信息，或启用图表的筛选和图例选项。此外，您可以从文件加载您的设置或将当前设置保存到文件中。此功能使您可以备份设置、与他人分享或快速应用以前保存的设置到您的图表中。</v>
       </c>
     </row>
     <row r="466">
       <c r="A466" t="str">
-        <v>tours.settings.step4</v>
+        <v>tours.settings.step3</v>
       </c>
       <c r="B466" t="str">
-        <v>In the Search Settings, you can quickly locate specific columns by entering keywords and then directly add them to your chart. Simply enter a term related to the setting you are looking for, and the system will display all relevant results.This feature is particularly useful when managing numerous data points or when you need to make quick adjustments without browsing through extensive lists.</v>
+        <v>In Column Settings, you can deeply customize the appearance and organization of your charts.In the "Column Customization" area, you can adjust titles and shift row positions to streamline how data is displayed on your charts. Enable or disable specific elements like the chart title and Ma markers to suit your presentation needs. In the "Font Options" section, refine the appearance of your charts by choosing different fonts, sizes, and styles for headers and labels, ensuring important data stands out or meets formatting requirements. Please note that the advanced settings for columns can vary depending on the datapack you are working with, allowing for tailored configurations that best fit the data characteristics.</v>
       </c>
       <c r="C466" t="str">
-        <v>在搜索中，您可以通过输入关键词快速定位特定列，然后直接将其添加到您的图表中。只需输入一个与您正在寻找的设置相关的词语，系统便会显示所有相关结果。此功能可以帮助您管理众多数据点，或进行快速调整而无需浏览繁杂列表。请注意目前只支持英文搜索。</v>
+        <v>在列设置中，您可以深度自定义图表的外观和组织。在“列自定义”区域，您可以调整标题和移动行位置，以简化图表上数据的显示方式。根据您的展示需求启用或禁用特定元素，如图表标题和百万年标记。在“字体选项”部分，通过选择不同的字体、大小和样式为标题和标签，细化您的图表外观，确保重要数据突出显示或符合格式要求。请注意，列高级设置可能根据您正在使用的数据包而有所不同，每个数据包都有最适合数据特性的列高级设置。</v>
       </c>
     </row>
     <row r="467">
       <c r="A467" t="str">
-        <v>tours.settings.step5</v>
+        <v>tours.settings.step4</v>
       </c>
       <c r="B467" t="str">
-        <v>The Font Settings section allows you to customize the appearance of text within your charts. You can adjust font styles, sizes, and formatting for various elements such as column headers, age labels, and more. Each setting is inheritable, ensuring consistency across related elements unless specified otherwise. Changing a font setting here applies it system-wide, but you can override these for individual columns by using the "Change Font" option within each columns settings.Experiment with different fonts and sizes to enhance readability and visual appeal of your charts.</v>
+        <v>In the Search Settings, you can quickly locate specific columns by entering keywords and then directly add them to your chart. Simply enter a term related to the setting you are looking for, and the system will display all relevant results.This feature is particularly useful when managing numerous data points or when you need to make quick adjustments without browsing through extensive lists.</v>
       </c>
       <c r="C467" t="str">
-        <v>在字体设置中您可以自定义图表内的文本外观。您可以为各种元素如列标题、年龄标签等调整字体样式、大小和格式。每项设置都是可继承的，确保相关元素间的一致性，除非另行设置。在这里更改字体设置将系统范围内应用，但您可以使用每个列设置中的“更改字体”选项覆盖这些设置。尝试不同的字体和大小，以增强图表的可读性和视觉吸引力。</v>
+        <v>在搜索中，您可以通过输入关键词快速定位特定列，然后直接将其添加到您的图表中。只需输入一个与您正在寻找的设置相关的词语，系统便会显示所有相关结果。此功能可以帮助您管理众多数据点，或进行快速调整而无需浏览繁杂列表。请注意目前只支持英文搜索。</v>
       </c>
     </row>
     <row r="468">
       <c r="A468" t="str">
-        <v>tours.settings.step6</v>
+        <v>tours.settings.step5</v>
       </c>
       <c r="B468" t="str">
-        <v>In the Map Points Settings, you can access and manage geographic data points for different locations. This feature allows you to view specific location details directly on the interactive map. You can toggle different map layers and visualize data points with detailed descriptions, like latitude, longitude, and additional notes. Please note, however, that not all datapacks contain map points.</v>
+        <v>The Font Settings section allows you to customize the appearance of text within your charts. You can adjust font styles, sizes, and formatting for various elements such as column headers, age labels, and more. Each setting is inheritable, ensuring consistency across related elements unless specified otherwise. Changing a font setting here applies it system-wide, but you can override these for individual columns by using the "Change Font" option within each columns settings.Experiment with different fonts and sizes to enhance readability and visual appeal of your charts.</v>
       </c>
       <c r="C468" t="str">
-        <v>在地图点设置中，您可以访问和管理不同位置的地理数据点。此功能允许您直接在交互式地图上查看特定位置的详细信息。您可以切换不同的地图层，并用详细描述（如纬度、经度和附加说明）可视化数据点。请注意，并非所有数据包都包含地图点。</v>
+        <v>在字体设置中您可以自定义图表内的文本外观。您可以为各种元素如列标题、年龄标签等调整字体样式、大小和格式。每项设置都是可继承的，确保相关元素间的一致性，除非另行设置。在这里更改字体设置将系统范围内应用，但您可以使用每个列设置中的“更改字体”选项覆盖这些设置。尝试不同的字体和大小，以增强图表的可读性和视觉吸引力。</v>
       </c>
     </row>
     <row r="469">
       <c r="A469" t="str">
-        <v>tours.settings.step7</v>
+        <v>tours.settings.step6</v>
       </c>
       <c r="B469" t="str">
-        <v>In the Datapacks Settings, you can select the datapacks you wish to use for generating charts. We offer nine official datapacks, each comprising a curated collection of datasets tailored for specific thematic explorations. You might notice that this page resembles the Datapack page; selections can be configured here or there interchangeably. For more detailed guidance on how to utilize datapacks, please refer to the Datapacks Tour in the Help page "Tours" section.</v>
+        <v>In the Map Points Settings, you can access and manage geographic data points for different locations. This feature allows you to view specific location details directly on the interactive map. You can toggle different map layers and visualize data points with detailed descriptions, like latitude, longitude, and additional notes. Please note, however, that not all datapacks contain map points.</v>
       </c>
       <c r="C469" t="str">
-        <v>在数据包设置中，您可以选择您希望用于生成图表的数据包。我们提供九个官方数据包，每个数据包都包含为特定主题探索量身定制的数据集合。您也许已经注意到，此页面与"数据包"页面内容相同；您在两个地方都可以进行选择和设置。如需更详细的关于如何利用数据包的指导，请参阅帮助页面“导览”部分中的数据包导览。</v>
+        <v>在地图点设置中，您可以访问和管理不同位置的地理数据点。此功能允许您直接在交互式地图上查看特定位置的详细信息。您可以切换不同的地图层，并用详细描述（如纬度、经度和附加说明）可视化数据点。请注意，并非所有数据包都包含地图点。</v>
       </c>
     </row>
     <row r="470">
       <c r="A470" t="str">
-        <v>settings.column.tooltip.note-in-range</v>
+        <v>tours.settings.step7</v>
+      </c>
+      <c r="B470" t="str">
+        <v>In the Datapacks Settings, you can select the datapacks you wish to use for generating charts. We offer nine official datapacks, each comprising a curated collection of datasets tailored for specific thematic explorations. You might notice that this page resembles the Datapack page; selections can be configured here or there interchangeably. For more detailed guidance on how to utilize datapacks, please refer to the Datapacks Tour in the Help page "Tours" section.</v>
       </c>
       <c r="C470" t="str">
-        <v>数据不在所选时间区间内</v>
+        <v>在数据包设置中，您可以选择您希望用于生成图表的数据包。我们提供九个官方数据包，每个数据包都包含为特定主题探索量身定制的数据集合。您也许已经注意到，此页面与"数据包"页面内容相同；您在两个地方都可以进行选择和设置。如需更详细的关于如何利用数据包的指导，请参阅帮助页面“导览”部分中的数据包导览。</v>
       </c>
     </row>
     <row r="471">
       <c r="A471" t="str">
-        <v>language-names.en-US</v>
+        <v>settings.column.tooltip.note-in-range</v>
       </c>
       <c r="C471" t="str">
-        <v>English</v>
+        <v>数据不在所选时间区间内</v>
       </c>
     </row>
     <row r="472">
       <c r="A472" t="str">
-        <v>language-names.en</v>
+        <v>language-names.en-US</v>
       </c>
       <c r="C472" t="str">
         <v>English</v>
@@ -5181,15 +5181,23 @@
     </row>
     <row r="473">
       <c r="A473" t="str">
+        <v>language-names.en</v>
+      </c>
+      <c r="C473" t="str">
+        <v>English</v>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="str">
         <v>language-names.zh</v>
       </c>
-      <c r="C473" t="str">
+      <c r="C474" t="str">
         <v>中文</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C473"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C474"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>